<commit_message>
Include SpaceX (consolidated SpaceX/xAI) in AI infra financing model
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AI_Infrastructure_Financing_2025-2030.xlsx
+++ b/AI_Infrastructure_Financing_2025-2030.xlsx
@@ -1196,7 +1196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B51"/>
+  <dimension ref="B2:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1276,236 +1276,250 @@
     <row r="14">
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>• Neoclouds / AI-native infra: GPU-cloud &amp; AI-native data-center builders (CoreWeave, xAI,</t>
+          <t>• Neoclouds / AI-native infra: GPU-cloud &amp; AI-native data-center builders (CoreWeave,</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Nebius, IREN, Crusoe, Lambda, Fluidstack, Nscale, + an 'Other' aggregate).</t>
+          <t xml:space="preserve">   SpaceX/xAI, Nebius, IREN, Crusoe, Lambda, Fluidstack, Nscale, + an 'Other' aggregate).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>• 'Equity / internal funding' = operating cash flow / free cash flow allocated to AI capex</t>
+          <t>• SpaceX acquired xAI (effective 2 Feb 2026), so Colossus I &amp; II are now SpaceX-owned; the two</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   PLUS external equity (IPOs, strategic stakes e.g. NVIDIA, ATM programs, mandatory</t>
+          <t xml:space="preserve">   are shown as one consolidated 'SpaceX / xAI' line to avoid double-counting the same clusters.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   convertible PREFERRED treated as equity). Hyperscalers self-fund the majority via FCF.</t>
+          <t>• 'Equity / internal funding' = operating cash flow / free cash flow allocated to AI capex</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">   PLUS external equity (IPOs, strategic stakes e.g. NVIDIA, ATM programs, mandatory</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   convertible PREFERRED treated as equity). Hyperscalers self-fund the majority via FCF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="5" t="inlineStr">
+        <is>
           <t>• 'Debt financing' = external borrowing, split by instrument (see below).</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="7" t="inlineStr">
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Debt instrument buckets (mutually exclusive — they sum to total debt)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>1. Corporate bonds (public IG/HY) — on-balance-sheet senior notes sold in public markets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>2. Bank &amp; syndicated loans — term loans, revolvers, delayed-draw term loans (incl. GPU-backed DDTLs).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>3. Alternate private credit — direct lending / private placements by credit funds (Blackstone,</t>
+          <t>1. Corporate bonds (public IG/HY) — on-balance-sheet senior notes sold in public markets.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Apollo, Blue Owl, PIMCO, Magnetar, etc.), including privately-placed SPV/project debt.</t>
+          <t>2. Bank &amp; syndicated loans — term loans, revolvers, delayed-draw term loans (incl. GPU-backed DDTLs).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>4. Insurance-linked lending — debt funded off insurer/annuity balance sheets (Athene/Apollo,</t>
+          <t>3. Alternate private credit — direct lending / private placements by credit funds (Blackstone,</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Global Atlantic/KKR, MetLife, Brookfield, etc.). NOTE: large overlap with private credit &amp;</t>
+          <t xml:space="preserve">   Apollo, Blue Owl, PIMCO, Magnetar, etc.), including privately-placed SPV/project debt.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   bonds; shown separately to size the insurance channel — see double-counting note below.</t>
+          <t>4. Insurance-linked lending — debt funded off insurer/annuity balance sheets (Athene/Apollo,</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>5. Securitization / ABS / CMBS — secured data-center bonds &amp; GPU-backed asset-backed securities.</t>
+          <t xml:space="preserve">   Global Atlantic/KKR, MetLife, Brookfield, etc.). NOTE: large overlap with private credit &amp;</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>6. Convertibles / equity-linked debt — convertible notes (excludes mandatory convert. PREFERRED).</t>
+          <t xml:space="preserve">   bonds; shown separately to size the insurance channel — see double-counting note below.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>7. Vendor &amp; equipment-lease financing — chip/equipment leases &amp; sale-leasebacks (e.g. NVIDIA</t>
+          <t>5. Securitization / ABS / CMBS — secured data-center bonds &amp; GPU-backed asset-backed securities.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   chip-lease SPVs, finance leases). Microsoft's large finance-lease book sits largely here.</t>
+          <t>6. Convertibles / equity-linked debt — convertible notes (excludes mandatory convert. PREFERRED).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Memo: 'Off-B/S SPV / JV (memo)' flags the portion routed through special-purpose vehicles /</t>
+          <t>7. Vendor &amp; equipment-lease financing — chip/equipment leases &amp; sale-leasebacks (e.g. NVIDIA</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   joint ventures (e.g. Meta-Hyperion, xAI Colossus 2, Oracle project SPVs). It OVERLAPS the</t>
+          <t xml:space="preserve">   chip-lease SPVs, finance leases). Microsoft's large finance-lease book sits largely here.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="5" t="inlineStr">
         <is>
+          <t>Memo: 'Off-B/S SPV / JV (memo)' flags the portion routed through special-purpose vehicles /</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   joint ventures (e.g. Meta-Hyperion, xAI Colossus 2, Oracle project SPVs). It OVERLAPS the</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">   buckets above and is therefore NOT added into the debt total.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="B37" s="8" t="inlineStr">
+    <row r="39" ht="20" customHeight="1">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>Methodology &amp; caveats</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>• Figures are RESEARCH ESTIMATES for the cumulative 2025-2030 buildout. They blend disclosed</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  transactions (2023-early 2026) with forward projections; they are illustrative, not audited.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>• Aggregate cross-check: total financing ≈ $5.25tn, consistent with Goldman Sachs' ~$5.3tn</t>
+          <t>• Figures are RESEARCH ESTIMATES for the cumulative 2025-2030 buildout. They blend disclosed</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2025-2030 AI + data-center capex estimate; aggregate debt ≈ $1.8tn, consistent with Morgan</t>
+          <t xml:space="preserve">  transactions (2023-early 2026) with forward projections; they are illustrative, not audited.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stanley / BofA projections of $1-2tn of debt financing for the buildout.</t>
+          <t>• Aggregate cross-check: total financing ≈ $5.25tn, consistent with Goldman Sachs' ~$5.3tn</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>• Insurance-linked lending double counts with private credit/bonds at the capital-source level;</t>
+          <t xml:space="preserve">  2025-2030 AI + data-center capex estimate; aggregate debt ≈ $1.8tn, consistent with Morgan</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  to avoid inflating totals, each dollar of debt is classified ONCE by its primary instrument and</t>
+          <t xml:space="preserve">  Stanley / BofA projections of $1-2tn of debt financing for the buildout.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  the insurance bucket captures only directly insurer-originated / insurance-balance-sheet debt.</t>
+          <t>• Insurance-linked lending double counts with private credit/bonds at the capital-source level;</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>• Company splits reflect observed behavior: Microsoft/Alphabet/Amazon are FCF-heavy with</t>
+          <t xml:space="preserve">  to avoid inflating totals, each dollar of debt is classified ONCE by its primary instrument and</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  selective bonds; Meta &amp; Oracle lean more on debt &amp; SPVs; neoclouds are debt-heavy (asset-backed).</t>
+          <t xml:space="preserve">  the insurance bucket captures only directly insurer-originated / insurance-balance-sheet debt.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="5" t="inlineStr">
         <is>
+          <t>• Company splits reflect observed behavior: Microsoft/Alphabet/Amazon are FCF-heavy with</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  selective bonds; Meta &amp; Oracle lean more on debt &amp; SPVs; neoclouds are debt-heavy (asset-backed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="5" t="inlineStr">
+        <is>
           <t>• Built with openpyxl. See Key Deals &amp; Sources sheet for citations.</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="B51" s="9" t="inlineStr">
+    <row r="53" ht="30" customHeight="1">
+      <c r="B53" s="9" t="inlineStr">
         <is>
           <t>Disclaimer: For analytical/illustrative purposes only. Not investment advice and not a representation of any company's actual financing. Verify against primary filings before use.</t>
         </is>
@@ -1850,14 +1864,14 @@
       </c>
       <c r="I11" s="16" t="inlineStr">
         <is>
-          <t>xAI (Colossus)</t>
+          <t>SpaceX / xAI (Colossus)</t>
         </is>
       </c>
       <c r="J11" s="17" t="n">
-        <v>55</v>
+        <v>140</v>
       </c>
       <c r="K11" s="17" t="n">
-        <v>70</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12">
@@ -1887,7 +1901,7 @@
     <row r="13">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>CoreWeave</t>
+          <t>SpaceX / xAI (Colossus)</t>
         </is>
       </c>
       <c r="B13" s="27" t="inlineStr">
@@ -1896,19 +1910,19 @@
         </is>
       </c>
       <c r="C13" s="28" t="n">
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>145</v>
+        <v>245</v>
       </c>
       <c r="F13" s="29" t="n">
-        <v>0.8275862068965517</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="I13" s="16" t="inlineStr">
         <is>
@@ -1925,7 +1939,7 @@
     <row r="14">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>xAI (Colossus)</t>
+          <t>CoreWeave</t>
         </is>
       </c>
       <c r="B14" s="27" t="inlineStr">
@@ -1934,19 +1948,19 @@
         </is>
       </c>
       <c r="C14" s="28" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="E14" s="28" t="n">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="F14" s="29" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.8275862068965517</v>
       </c>
       <c r="G14" s="28" t="n">
-        <v>45</v>
+        <v>95</v>
       </c>
       <c r="I14" s="16" t="inlineStr">
         <is>
@@ -2701,7 +2715,7 @@
     <row r="14">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>xAI (Colossus)</t>
+          <t>SpaceX / xAI (Colossus)</t>
         </is>
       </c>
       <c r="B14" s="39" t="inlineStr">
@@ -2710,35 +2724,35 @@
         </is>
       </c>
       <c r="C14" s="28" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D14" s="28" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="E14" s="28" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F14" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" s="28" t="n">
         <v>3</v>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>2</v>
       </c>
       <c r="H14" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I14" s="28" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="J14" s="40">
         <f>SUM(C14:I14)</f>
         <v/>
       </c>
       <c r="K14" s="41" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="L14" s="42" t="n">
-        <v>55</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15">
@@ -3411,22 +3425,22 @@
         </is>
       </c>
       <c r="B10" s="28" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="C10" s="28" t="n">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="E10" s="28" t="n">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="F10" s="28" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="G10" s="28" t="n">
-        <v>96</v>
+        <v>126</v>
       </c>
       <c r="H10" s="40">
         <f>SUM(B10:G10)</f>
@@ -3480,7 +3494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3956,44 +3970,44 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="50" t="inlineStr">
         <is>
-          <t>xAI (Colossus)</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="B18" s="51" t="inlineStr">
         <is>
-          <t>$10bn raise ($5bn secured notes/term loans + $5bn equity) via Morgan Stanley</t>
+          <t>SpaceX acquired xAI effective Feb 2, 2026; Colossus I &amp; II now SpaceX-owned (vertically-integrated AI platform; Terafab chip JV w/ Tesla &amp; Intel)</t>
         </is>
       </c>
       <c r="C18" s="51" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D18" s="51" t="inlineStr">
         <is>
-          <t>$10bn</t>
+          <t>merger</t>
         </is>
       </c>
       <c r="E18" s="51" t="inlineStr">
         <is>
-          <t>Loans + equity</t>
+          <t>Equity / M&amp;A</t>
         </is>
       </c>
       <c r="F18" s="52" t="inlineStr">
         <is>
-          <t>CNBC</t>
+          <t>SpaceX S-1</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="47" t="inlineStr">
         <is>
-          <t>xAI (Colossus)</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="B19" s="48" t="inlineStr">
         <is>
-          <t>Colossus 2 SPV (Valor Equity): ~$12.5bn debt + ~$7.5bn equity (NVIDIA up to $2bn) to buy &amp; lease GPUs</t>
+          <t>SpaceX AI capex $12.7bn in 2025 (~61% of total) + $7.7bn in Q1 2026; AI buildout funded by Starlink FCF, private raises, planned IPO</t>
         </is>
       </c>
       <c r="C19" s="48" t="inlineStr">
@@ -4003,61 +4017,61 @@
       </c>
       <c r="D19" s="48" t="inlineStr">
         <is>
-          <t>~$20bn</t>
+          <t>$20bn+ capex</t>
         </is>
       </c>
       <c r="E19" s="48" t="inlineStr">
         <is>
-          <t>SPV / vendor lease</t>
+          <t>Internal / equity</t>
         </is>
       </c>
       <c r="F19" s="49" t="inlineStr">
         <is>
-          <t>The Information; Yahoo</t>
+          <t>SpaceX S-1; The Verge</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="50" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="B20" s="51" t="inlineStr">
         <is>
-          <t>$3bn+ convertibles + bank lines; lighter balance sheet; Yandex spin-off cash ~$2.5bn; NVIDIA ~$2bn equity; Microsoft ~$7bn prepay</t>
+          <t>Anthropic compute contract: $1.25bn/month (~$45bn) through May 2029 for Colossus I &amp; II — anchor revenue underwriting infra financing</t>
         </is>
       </c>
       <c r="C20" s="51" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026-29</t>
         </is>
       </c>
       <c r="D20" s="51" t="inlineStr">
         <is>
-          <t>$3bn+</t>
+          <t>~$45bn</t>
         </is>
       </c>
       <c r="E20" s="51" t="inlineStr">
         <is>
-          <t>Convertibles</t>
+          <t>Take-or-pay (demand)</t>
         </is>
       </c>
       <c r="F20" s="52" t="inlineStr">
         <is>
-          <t>frankk research</t>
+          <t>SpaceX S-1; The Verge</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="47" t="inlineStr">
         <is>
-          <t>Lambda</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="B21" s="48" t="inlineStr">
         <is>
-          <t>$500m GPU-backed facility from Macquarie</t>
+          <t>xAI $10bn raise ($5bn secured notes/term loans incl. Apollo $5bn facility + $5bn equity) via Morgan Stanley</t>
         </is>
       </c>
       <c r="C21" s="48" t="inlineStr">
@@ -4067,270 +4081,366 @@
       </c>
       <c r="D21" s="48" t="inlineStr">
         <is>
-          <t>$0.5bn</t>
+          <t>$10bn</t>
         </is>
       </c>
       <c r="E21" s="48" t="inlineStr">
         <is>
-          <t>Bank / GPU-backed loan</t>
+          <t>Loans + equity</t>
         </is>
       </c>
       <c r="F21" s="49" t="inlineStr">
         <is>
-          <t>theaiinsider</t>
+          <t>CNBC</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="50" t="inlineStr">
         <is>
-          <t>Nscale</t>
+          <t>SpaceX / xAI</t>
         </is>
       </c>
       <c r="B22" s="51" t="inlineStr">
         <is>
-          <t>$1.4bn term loan</t>
+          <t>Colossus 2 SPV (Valor Equity): ~$12.5bn debt + ~$7.5bn equity (NVIDIA up to $2bn) to buy &amp; lease GPUs</t>
         </is>
       </c>
       <c r="C22" s="51" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025-26</t>
         </is>
       </c>
       <c r="D22" s="51" t="inlineStr">
         <is>
-          <t>$1.4bn</t>
+          <t>~$20bn</t>
         </is>
       </c>
       <c r="E22" s="51" t="inlineStr">
         <is>
-          <t>Bank loan</t>
+          <t>SPV / vendor lease</t>
         </is>
       </c>
       <c r="F22" s="52" t="inlineStr">
         <is>
-          <t>theaiinsider</t>
+          <t>The Information; Yahoo</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="47" t="inlineStr">
         <is>
-          <t>Fluidstack</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="B23" s="48" t="inlineStr">
         <is>
-          <t>Facility backed by ~$6.7bn Google-contracted revenue (Google lease backstop)</t>
+          <t>$3bn+ convertibles + bank lines; lighter balance sheet; Yandex spin-off cash ~$2.5bn; NVIDIA ~$2bn equity; Microsoft ~$7bn prepay</t>
         </is>
       </c>
       <c r="C23" s="48" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025-26</t>
         </is>
       </c>
       <c r="D23" s="48" t="inlineStr">
         <is>
-          <t>~$6.7bn</t>
+          <t>$3bn+</t>
         </is>
       </c>
       <c r="E23" s="48" t="inlineStr">
         <is>
-          <t>SPV / private credit</t>
+          <t>Convertibles</t>
         </is>
       </c>
       <c r="F23" s="49" t="inlineStr">
         <is>
-          <t>theaiinsider</t>
+          <t>frankk research</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="50" t="inlineStr">
         <is>
-          <t>Applied Digital</t>
+          <t>Lambda</t>
         </is>
       </c>
       <c r="B24" s="51" t="inlineStr">
         <is>
-          <t>$1.59bn high-yield bond (7%) for CoreWeave-leased campus (Polaris Forge 1)</t>
+          <t>$500m GPU-backed facility from Macquarie</t>
         </is>
       </c>
       <c r="C24" s="51" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D24" s="51" t="inlineStr">
         <is>
-          <t>$1.59bn</t>
+          <t>$0.5bn</t>
         </is>
       </c>
       <c r="E24" s="51" t="inlineStr">
         <is>
-          <t>Securitization / HY bond</t>
+          <t>Bank / GPU-backed loan</t>
         </is>
       </c>
       <c r="F24" s="52" t="inlineStr">
         <is>
-          <t>TNW</t>
+          <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="47" t="inlineStr">
         <is>
-          <t>Sector-wide</t>
+          <t>Nscale</t>
         </is>
       </c>
       <c r="B25" s="48" t="inlineStr">
         <is>
-          <t>HY/unrated AI-infra issuers raised ~$107bn funded+committed debt by ~May 2026 ($68.7bn neoclouds / $38.7bn AI-native DCs)</t>
+          <t>$1.4bn term loan</t>
         </is>
       </c>
       <c r="C25" s="48" t="inlineStr">
         <is>
-          <t>to 2026</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D25" s="48" t="inlineStr">
         <is>
-          <t>~$107bn</t>
+          <t>$1.4bn</t>
         </is>
       </c>
       <c r="E25" s="48" t="inlineStr">
         <is>
-          <t>All debt</t>
+          <t>Bank loan</t>
         </is>
       </c>
       <c r="F25" s="49" t="inlineStr">
         <is>
-          <t>Octus</t>
+          <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="50" t="inlineStr">
         <is>
-          <t>Sector-wide</t>
+          <t>Fluidstack</t>
         </is>
       </c>
       <c r="B26" s="51" t="inlineStr">
         <is>
-          <t>Insurance-linked platforms deployed ~$180bn into private credit in 2025 (~25% of global private credit AUM)</t>
+          <t>Facility backed by ~$6.7bn Google-contracted revenue (Google lease backstop)</t>
         </is>
       </c>
       <c r="C26" s="51" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D26" s="51" t="inlineStr">
         <is>
-          <t>~$180bn</t>
+          <t>~$6.7bn</t>
         </is>
       </c>
       <c r="E26" s="51" t="inlineStr">
         <is>
-          <t>Insurance / private credit</t>
+          <t>SPV / private credit</t>
         </is>
       </c>
       <c r="F26" s="52" t="inlineStr">
         <is>
-          <t>McKinsey; ABF Journal</t>
+          <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="47" t="inlineStr">
         <is>
+          <t>Applied Digital</t>
+        </is>
+      </c>
+      <c r="B27" s="48" t="inlineStr">
+        <is>
+          <t>$1.59bn high-yield bond (7%) for CoreWeave-leased campus (Polaris Forge 1)</t>
+        </is>
+      </c>
+      <c r="C27" s="48" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D27" s="48" t="inlineStr">
+        <is>
+          <t>$1.59bn</t>
+        </is>
+      </c>
+      <c r="E27" s="48" t="inlineStr">
+        <is>
+          <t>Securitization / HY bond</t>
+        </is>
+      </c>
+      <c r="F27" s="49" t="inlineStr">
+        <is>
+          <t>TNW</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="50" t="inlineStr">
+        <is>
           <t>Sector-wide</t>
         </is>
       </c>
-      <c r="B27" s="48" t="inlineStr">
+      <c r="B28" s="51" t="inlineStr">
+        <is>
+          <t>HY/unrated AI-infra issuers raised ~$107bn funded+committed debt by ~May 2026 ($68.7bn neoclouds / $38.7bn AI-native DCs)</t>
+        </is>
+      </c>
+      <c r="C28" s="51" t="inlineStr">
+        <is>
+          <t>to 2026</t>
+        </is>
+      </c>
+      <c r="D28" s="51" t="inlineStr">
+        <is>
+          <t>~$107bn</t>
+        </is>
+      </c>
+      <c r="E28" s="51" t="inlineStr">
+        <is>
+          <t>All debt</t>
+        </is>
+      </c>
+      <c r="F28" s="52" t="inlineStr">
+        <is>
+          <t>Octus</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="47" t="inlineStr">
+        <is>
+          <t>Sector-wide</t>
+        </is>
+      </c>
+      <c r="B29" s="48" t="inlineStr">
+        <is>
+          <t>Insurance-linked platforms deployed ~$180bn into private credit in 2025 (~25% of global private credit AUM)</t>
+        </is>
+      </c>
+      <c r="C29" s="48" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D29" s="48" t="inlineStr">
+        <is>
+          <t>~$180bn</t>
+        </is>
+      </c>
+      <c r="E29" s="48" t="inlineStr">
+        <is>
+          <t>Insurance / private credit</t>
+        </is>
+      </c>
+      <c r="F29" s="49" t="inlineStr">
+        <is>
+          <t>McKinsey; ABF Journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="50" t="inlineStr">
+        <is>
+          <t>Sector-wide</t>
+        </is>
+      </c>
+      <c r="B30" s="51" t="inlineStr">
         <is>
           <t>Goldman Sachs: ~$5.3tn AI + data-center capex 2025-2030; Morgan Stanley: ~$800bn private credit for AI DCs 2025-28</t>
         </is>
       </c>
-      <c r="C27" s="48" t="inlineStr">
+      <c r="C30" s="51" t="inlineStr">
         <is>
           <t>2025-30</t>
         </is>
       </c>
-      <c r="D27" s="48" t="inlineStr">
+      <c r="D30" s="51" t="inlineStr">
         <is>
           <t>$5.3tn capex</t>
         </is>
       </c>
-      <c r="E27" s="48" t="inlineStr">
+      <c r="E30" s="51" t="inlineStr">
         <is>
           <t>Context</t>
         </is>
       </c>
-      <c r="F27" s="49" t="inlineStr">
+      <c r="F30" s="52" t="inlineStr">
         <is>
           <t>Goldman; Morgan Stanley</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="53" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="53" t="inlineStr">
         <is>
           <t>Selected sources:</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="54" t="inlineStr">
-        <is>
-          <t>Goldman Sachs Research — ~$5.3tn AI + data-center capex 2025-2030; private markets in DC financing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="54" t="inlineStr">
-        <is>
-          <t>Morgan Stanley — ~$2tn capex 2025-28 with &gt;$1tn debt; ~$800bn private credit for AI DCs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="54" t="inlineStr">
-        <is>
-          <t>Bank of America / BofA Securities — hyperscaler bond issuance ($121bn 2025; ~$175bn 2026E).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="54" t="inlineStr">
         <is>
-          <t>Moody's Ratings — hyperscaler capex (~$785bn 2026, ~$1tn 2027); $662bn off-B/S DC leases.</t>
+          <t>Goldman Sachs Research — ~$5.3tn AI + data-center capex 2025-2030; private markets in DC financing.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="54" t="inlineStr">
         <is>
-          <t>McKinsey — ~$2.7tn US (5.2tn global) data-center capex by 2030; insurance-linked private credit.</t>
+          <t>Morgan Stanley — ~$2tn capex 2025-28 with &gt;$1tn debt; ~$800bn private credit for AI DCs.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="54" t="inlineStr">
         <is>
-          <t>Octus — HY/unrated AI-infra debt (~$107bn to ~May 2026); ~14GW unfunded ≈ $344bn need.</t>
+          <t>Bank of America / BofA Securities — hyperscaler bond issuance ($121bn 2025; ~$175bn 2026E).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="54" t="inlineStr">
         <is>
-          <t>Company disclosures &amp; press: Meta IR / FT / S&amp;P (Hyperion); Oracle IR / IFR / Reuters; CoreWeave IR;</t>
+          <t>Moody's Ratings — hyperscaler capex (~$785bn 2026, ~$1tn 2027); $662bn off-B/S DC leases.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="54" t="inlineStr">
+        <is>
+          <t>McKinsey — ~$2.7tn US (5.2tn global) data-center capex by 2030; insurance-linked private credit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="54" t="inlineStr">
+        <is>
+          <t>Octus — HY/unrated AI-infra debt (~$107bn to ~May 2026); ~14GW unfunded ≈ $344bn need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="54" t="inlineStr">
+        <is>
+          <t>Company disclosures &amp; press: Meta IR / FT / S&amp;P (Hyperion); Oracle IR / IFR / Reuters; CoreWeave IR;</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="54" t="inlineStr">
         <is>
           <t xml:space="preserve">  CNBC / WSJ / The Information (xAI); Blackstone; Apollo Academy; MUFG; CreditSights; CNA.</t>
         </is>

</xml_diff>

<commit_message>
Add colocation/data-center REIT and sovereign cloud segments
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AI_Infrastructure_Financing_2025-2030.xlsx
+++ b/AI_Infrastructure_Financing_2025-2030.xlsx
@@ -141,7 +141,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -190,6 +190,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F4E9DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDE4F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
@@ -220,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -277,6 +287,22 @@
     <xf numFmtId="9" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -306,6 +332,26 @@
     <xf numFmtId="3" fontId="20" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="18" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="19" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="18" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="19" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -314,13 +360,13 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -447,12 +493,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Summary (by Company)'!$I$5:$I$18</f>
+              <f>'Summary (by Company)'!$I$5:$I$34</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary (by Company)'!$J$5:$J$18</f>
+              <f>'Summary (by Company)'!$J$5:$J$34</f>
             </numRef>
           </val>
         </ser>
@@ -471,12 +517,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Summary (by Company)'!$I$5:$I$18</f>
+              <f>'Summary (by Company)'!$I$5:$I$34</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary (by Company)'!$K$5:$K$18</f>
+              <f>'Summary (by Company)'!$K$5:$K$34</f>
             </numRef>
           </val>
         </ser>
@@ -571,7 +617,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Debt by Type'!$C$23:$I$23</f>
+              <f>'Debt by Type'!$C$43:$I$43</f>
             </numRef>
           </val>
         </ser>
@@ -774,6 +820,54 @@
             </numRef>
           </val>
         </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <strRef>
+              <f>'Capex Projections'!A11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Capex Projections'!$B$4:$G$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Capex Projections'!$B$11:$G$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <strRef>
+              <f>'Capex Projections'!A12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Capex Projections'!$B$4:$G$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Capex Projections'!$B$12:$G$12</f>
+            </numRef>
+          </val>
+        </ser>
         <gapWidth val="150"/>
         <overlap val="100"/>
         <axId val="10"/>
@@ -832,7 +926,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>25</row>
+      <row>45</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9360000" cy="3240000"/>
@@ -859,7 +953,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>46</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="2880000"/>
@@ -886,7 +980,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>15</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -1196,7 +1290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B53"/>
+  <dimension ref="B2:B65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1304,222 +1398,306 @@
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>• 'Equity / internal funding' = operating cash flow / free cash flow allocated to AI capex</t>
+          <t>• Colocation / data-center REITs: wholesale &amp; retail colo / powered-shell owners (Equinix,</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   PLUS external equity (IPOs, strategic stakes e.g. NVIDIA, ATM programs, mandatory</t>
+          <t xml:space="preserve">   Digital Realty, QTS, Vantage, Aligned, CyrusOne, Switch, Stack, + 'Other') that build campuses</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   convertible PREFERRED treated as equity). Hyperscalers self-fund the majority via FCF.</t>
+          <t xml:space="preserve">   and lease them to hyperscalers / neoclouds; heavy users of ABS/CMBS securitization &amp; infra equity.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>• 'Debt financing' = external borrowing, split by instrument (see below).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Debt instrument buckets (mutually exclusive — they sum to total debt)</t>
+          <t>• Sovereign clouds: state / sovereign-wealth-funded national AI infrastructure (HUMAIN-Saudi PIF,</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   MGX/Mubadala, Stargate UAE/G42/Khazna, Qatar QIA, EU/France, India, + 'Other'); mostly equity-funded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>• 'Equity / internal funding' = operating cash flow / free cash flow allocated to AI capex</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>1. Corporate bonds (public IG/HY) — on-balance-sheet senior notes sold in public markets.</t>
+          <t xml:space="preserve">   PLUS external equity (IPOs, strategic stakes e.g. NVIDIA, ATM programs, mandatory</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2. Bank &amp; syndicated loans — term loans, revolvers, delayed-draw term loans (incl. GPU-backed DDTLs).</t>
+          <t xml:space="preserve">   convertible PREFERRED treated as equity). Hyperscalers self-fund the majority via FCF.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>3. Alternate private credit — direct lending / private placements by credit funds (Blackstone,</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Apollo, Blue Owl, PIMCO, Magnetar, etc.), including privately-placed SPV/project debt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>4. Insurance-linked lending — debt funded off insurer/annuity balance sheets (Athene/Apollo,</t>
+          <t>• 'Debt financing' = external borrowing, split by instrument (see below).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Debt instrument buckets (mutually exclusive — they sum to total debt)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Global Atlantic/KKR, MetLife, Brookfield, etc.). NOTE: large overlap with private credit &amp;</t>
+          <t>1. Corporate bonds (public IG/HY) — on-balance-sheet senior notes sold in public markets.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   bonds; shown separately to size the insurance channel — see double-counting note below.</t>
+          <t>2. Bank &amp; syndicated loans — term loans, revolvers, delayed-draw term loans (incl. GPU-backed DDTLs).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>5. Securitization / ABS / CMBS — secured data-center bonds &amp; GPU-backed asset-backed securities.</t>
+          <t>3. Alternate private credit — direct lending / private placements by credit funds (Blackstone,</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>6. Convertibles / equity-linked debt — convertible notes (excludes mandatory convert. PREFERRED).</t>
+          <t xml:space="preserve">   Apollo, Blue Owl, PIMCO, Magnetar, etc.), including privately-placed SPV/project debt.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>7. Vendor &amp; equipment-lease financing — chip/equipment leases &amp; sale-leasebacks (e.g. NVIDIA</t>
+          <t>4. Insurance-linked lending — debt funded off insurer/annuity balance sheets (Athene/Apollo,</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   chip-lease SPVs, finance leases). Microsoft's large finance-lease book sits largely here.</t>
+          <t xml:space="preserve">   Global Atlantic/KKR, MetLife, Brookfield, etc.). NOTE: large overlap with private credit &amp;</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Memo: 'Off-B/S SPV / JV (memo)' flags the portion routed through special-purpose vehicles /</t>
+          <t xml:space="preserve">   bonds; shown separately to size the insurance channel — see double-counting note below.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   joint ventures (e.g. Meta-Hyperion, xAI Colossus 2, Oracle project SPVs). It OVERLAPS the</t>
+          <t>5. Securitization / ABS / CMBS — secured data-center bonds &amp; GPU-backed asset-backed securities.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   buckets above and is therefore NOT added into the debt total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>Methodology &amp; caveats</t>
+          <t>6. Convertibles / equity-linked debt — convertible notes (excludes mandatory convert. PREFERRED).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>7. Vendor &amp; equipment-lease financing — chip/equipment leases &amp; sale-leasebacks (e.g. NVIDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   chip-lease SPVs, finance leases). Microsoft's large finance-lease book sits largely here.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>• Figures are RESEARCH ESTIMATES for the cumulative 2025-2030 buildout. They blend disclosed</t>
+          <t>Memo: 'Off-B/S SPV / JV (memo)' flags the portion routed through special-purpose vehicles /</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  transactions (2023-early 2026) with forward projections; they are illustrative, not audited.</t>
+          <t xml:space="preserve">   joint ventures (e.g. Meta-Hyperion, xAI Colossus 2, Oracle project SPVs). It OVERLAPS the</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>• Aggregate cross-check: total financing ≈ $5.25tn, consistent with Goldman Sachs' ~$5.3tn</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2025-2030 AI + data-center capex estimate; aggregate debt ≈ $1.8tn, consistent with Morgan</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Stanley / BofA projections of $1-2tn of debt financing for the buildout.</t>
+          <t xml:space="preserve">   buckets above and is therefore NOT added into the debt total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>Methodology &amp; caveats</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>• Insurance-linked lending double counts with private credit/bonds at the capital-source level;</t>
+          <t>• Figures are RESEARCH ESTIMATES for the cumulative 2025-2030 buildout. They blend disclosed</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  to avoid inflating totals, each dollar of debt is classified ONCE by its primary instrument and</t>
+          <t xml:space="preserve">  transactions (2023-early 2026) with forward projections; they are illustrative, not audited.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  the insurance bucket captures only directly insurer-originated / insurance-balance-sheet debt.</t>
+          <t>• Aggregate cross-check: total financing ≈ $5.25tn, consistent with Goldman Sachs' ~$5.3tn</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>• Company splits reflect observed behavior: Microsoft/Alphabet/Amazon are FCF-heavy with</t>
+          <t xml:space="preserve">  2025-2030 AI + data-center capex estimate; aggregate debt ≈ $1.8tn, consistent with Morgan</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  selective bonds; Meta &amp; Oracle lean more on debt &amp; SPVs; neoclouds are debt-heavy (asset-backed).</t>
+          <t xml:space="preserve">  Stanley / BofA projections of $1-2tn of debt financing for the buildout.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="5" t="inlineStr">
         <is>
+          <t>• CROSS-SEGMENT OVERLAP: hyperscalers LEASE much colocation capacity (so colo financing partly</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  funds the same capacity hyperscalers report as off-B/S leases), and sovereign-wealth funds</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (MGX, PIF, QIA) also INVEST in neoclouds/labs and colo (e.g. MGX/BlackRock bought Aligned; PIF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  put ~$3bn into xAI). The all-segment 'grand total' is therefore a GROSS figure of capital raised</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  across distinct balance sheets and is not strictly additive; treat it as an upper-bound view.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Hyperscaler + Neocloud financing (~$5.4tn) ties to Goldman's ~$5.3tn big-tech capex; adding</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  third-party colo + sovereign brings the gross total toward broader ~$6-7tn AI-infra estimates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>• Insurance-linked lending double counts with private credit/bonds at the capital-source level;</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  to avoid inflating totals, each dollar of debt is classified ONCE by its primary instrument and</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  the insurance bucket captures only directly insurer-originated / insurance-balance-sheet debt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>• Company splits reflect observed behavior: Microsoft/Alphabet/Amazon are FCF-heavy with</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  selective bonds; Meta &amp; Oracle lean more on debt &amp; SPVs; neoclouds are debt-heavy (asset-backed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="5" t="inlineStr">
+        <is>
           <t>• Built with openpyxl. See Key Deals &amp; Sources sheet for citations.</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="30" customHeight="1">
-      <c r="B53" s="9" t="inlineStr">
+    <row r="65" ht="30" customHeight="1">
+      <c r="B65" s="9" t="inlineStr">
         <is>
           <t>Disclaimer: For analytical/illustrative purposes only. Not investment advice and not a representation of any company's actual financing. Verify against primary filings before use.</t>
         </is>
@@ -1539,7 +1717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2152,6 +2330,17 @@
       <c r="G19" s="28" t="n">
         <v>10</v>
       </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Equinix</t>
+        </is>
+      </c>
+      <c r="J19" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="K19" s="17" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="26" t="inlineStr">
@@ -2179,6 +2368,17 @@
       <c r="G20" s="28" t="n">
         <v>14</v>
       </c>
+      <c r="I20" s="16" t="inlineStr">
+        <is>
+          <t>Digital Realty</t>
+        </is>
+      </c>
+      <c r="J20" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="K20" s="17" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="26" t="inlineStr">
@@ -2205,6 +2405,17 @@
       </c>
       <c r="G21" s="28" t="n">
         <v>8</v>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>QTS (Blackstone)</t>
+        </is>
+      </c>
+      <c r="J21" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="K21" s="17" t="n">
+        <v>42</v>
       </c>
     </row>
     <row r="22">
@@ -2234,32 +2445,689 @@
         <f>SUM(G13:G21)</f>
         <v/>
       </c>
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <t>Vantage Data Centers</t>
+        </is>
+      </c>
+      <c r="J22" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="K22" s="17" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="30" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>COLOCATION / DATA-CENTER REIT</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>Aligned Data Centers (MGX/BlackRock)</t>
+        </is>
+      </c>
+      <c r="J23" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="K23" s="17" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>Other colo &amp; powered-shell owners</t>
+        </is>
+      </c>
+      <c r="B24" s="31" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C24" s="32" t="n">
+        <v>30</v>
+      </c>
+      <c r="D24" s="32" t="n">
+        <v>55</v>
+      </c>
+      <c r="E24" s="32" t="n">
+        <v>85</v>
+      </c>
+      <c r="F24" s="33" t="n">
+        <v>0.6470588235294118</v>
+      </c>
+      <c r="G24" s="32" t="n">
+        <v>30</v>
+      </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>CyrusOne (KKR/GIP)</t>
+        </is>
+      </c>
+      <c r="J24" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="K24" s="17" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>Equinix</t>
+        </is>
+      </c>
+      <c r="B25" s="31" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="n">
+        <v>25</v>
+      </c>
+      <c r="D25" s="32" t="n">
+        <v>45</v>
+      </c>
+      <c r="E25" s="32" t="n">
+        <v>70</v>
+      </c>
+      <c r="F25" s="33" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="G25" s="32" t="n">
+        <v>20</v>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>Switch (DigitalBridge)</t>
+        </is>
+      </c>
+      <c r="J25" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="K25" s="17" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>Digital Realty</t>
+        </is>
+      </c>
+      <c r="B26" s="31" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C26" s="32" t="n">
+        <v>20</v>
+      </c>
+      <c r="D26" s="32" t="n">
+        <v>40</v>
+      </c>
+      <c r="E26" s="32" t="n">
+        <v>60</v>
+      </c>
+      <c r="F26" s="33" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="G26" s="32" t="n">
+        <v>18</v>
+      </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>Stack Infrastructure</t>
+        </is>
+      </c>
+      <c r="J26" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="K26" s="17" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>QTS (Blackstone)</t>
+        </is>
+      </c>
+      <c r="B27" s="31" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C27" s="32" t="n">
+        <v>18</v>
+      </c>
+      <c r="D27" s="32" t="n">
+        <v>42</v>
+      </c>
+      <c r="E27" s="32" t="n">
+        <v>60</v>
+      </c>
+      <c r="F27" s="33" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G27" s="32" t="n">
+        <v>35</v>
+      </c>
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <t>Other colo &amp; powered-shell owners</t>
+        </is>
+      </c>
+      <c r="J27" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="K27" s="17" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Vantage Data Centers</t>
+        </is>
+      </c>
+      <c r="B28" s="31" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C28" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="D28" s="32" t="n">
+        <v>35</v>
+      </c>
+      <c r="E28" s="32" t="n">
+        <v>50</v>
+      </c>
+      <c r="F28" s="33" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G28" s="32" t="n">
+        <v>28</v>
+      </c>
+      <c r="I28" s="16" t="inlineStr">
+        <is>
+          <t>HUMAIN (Saudi PIF)</t>
+        </is>
+      </c>
+      <c r="J28" s="17" t="n">
+        <v>80</v>
+      </c>
+      <c r="K28" s="17" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>Aligned Data Centers (MGX/BlackRock)</t>
+        </is>
+      </c>
+      <c r="B29" s="31" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C29" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="D29" s="32" t="n">
+        <v>28</v>
+      </c>
+      <c r="E29" s="32" t="n">
+        <v>40</v>
+      </c>
+      <c r="F29" s="33" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G29" s="32" t="n">
+        <v>22</v>
+      </c>
+      <c r="I29" s="16" t="inlineStr">
+        <is>
+          <t>MGX / Mubadala (UAE)</t>
+        </is>
+      </c>
+      <c r="J29" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="K29" s="17" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>CyrusOne (KKR/GIP)</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C30" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="D30" s="32" t="n">
+        <v>28</v>
+      </c>
+      <c r="E30" s="32" t="n">
+        <v>40</v>
+      </c>
+      <c r="F30" s="33" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G30" s="32" t="n">
+        <v>22</v>
+      </c>
+      <c r="I30" s="16" t="inlineStr">
+        <is>
+          <t>Stargate UAE / G42 / Khazna</t>
+        </is>
+      </c>
+      <c r="J30" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="K30" s="17" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>Switch (DigitalBridge)</t>
+        </is>
+      </c>
+      <c r="B31" s="31" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C31" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="D31" s="32" t="n">
+        <v>22</v>
+      </c>
+      <c r="E31" s="32" t="n">
+        <v>30</v>
+      </c>
+      <c r="F31" s="33" t="n">
+        <v>0.7333333333333333</v>
+      </c>
+      <c r="G31" s="32" t="n">
+        <v>16</v>
+      </c>
+      <c r="I31" s="16" t="inlineStr">
+        <is>
+          <t>Qatar (QIA / Qai + Brookfield JV)</t>
+        </is>
+      </c>
+      <c r="J31" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="K31" s="17" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Stack Infrastructure</t>
+        </is>
+      </c>
+      <c r="B32" s="31" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C32" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="D32" s="32" t="n">
+        <v>17</v>
+      </c>
+      <c r="E32" s="32" t="n">
+        <v>25</v>
+      </c>
+      <c r="F32" s="33" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G32" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="I32" s="16" t="inlineStr">
+        <is>
+          <t>EU / France (Mistral, sovereign cloud)</t>
+        </is>
+      </c>
+      <c r="J32" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="K32" s="17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT subtotal</t>
+        </is>
+      </c>
+      <c r="B33" s="23" t="n"/>
+      <c r="C33" s="24">
+        <f>SUM(C24:C32)</f>
+        <v/>
+      </c>
+      <c r="D33" s="24">
+        <f>SUM(D24:D32)</f>
+        <v/>
+      </c>
+      <c r="E33" s="24">
+        <f>SUM(E24:E32)</f>
+        <v/>
+      </c>
+      <c r="F33" s="25">
+        <f>D33/E33</f>
+        <v/>
+      </c>
+      <c r="G33" s="24">
+        <f>SUM(G24:G32)</f>
+        <v/>
+      </c>
+      <c r="I33" s="16" t="inlineStr">
+        <is>
+          <t>India (IndiaAI Mission)</t>
+        </is>
+      </c>
+      <c r="J33" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="K33" s="17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>SOVEREIGN CLOUD</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="n"/>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="15" t="n"/>
+      <c r="F34" s="15" t="n"/>
+      <c r="G34" s="15" t="n"/>
+      <c r="I34" s="16" t="inlineStr">
+        <is>
+          <t>Other sovereign AI (Japan, Korea, Singapore, etc.)</t>
+        </is>
+      </c>
+      <c r="J34" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="K34" s="17" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="34" t="inlineStr">
+        <is>
+          <t>HUMAIN (Saudi PIF)</t>
+        </is>
+      </c>
+      <c r="B35" s="35" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C35" s="36" t="n">
+        <v>80</v>
+      </c>
+      <c r="D35" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="E35" s="36" t="n">
+        <v>100</v>
+      </c>
+      <c r="F35" s="37" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G35" s="36" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="34" t="inlineStr">
+        <is>
+          <t>MGX / Mubadala (UAE)</t>
+        </is>
+      </c>
+      <c r="B36" s="35" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C36" s="36" t="n">
+        <v>30</v>
+      </c>
+      <c r="D36" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="E36" s="36" t="n">
+        <v>40</v>
+      </c>
+      <c r="F36" s="37" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G36" s="36" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="34" t="inlineStr">
+        <is>
+          <t>Other sovereign AI (Japan, Korea, Singapore, etc.)</t>
+        </is>
+      </c>
+      <c r="B37" s="35" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C37" s="36" t="n">
+        <v>25</v>
+      </c>
+      <c r="D37" s="36" t="n">
+        <v>8</v>
+      </c>
+      <c r="E37" s="36" t="n">
+        <v>33</v>
+      </c>
+      <c r="F37" s="37" t="n">
+        <v>0.2424242424242424</v>
+      </c>
+      <c r="G37" s="36" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="34" t="inlineStr">
+        <is>
+          <t>Stargate UAE / G42 / Khazna</t>
+        </is>
+      </c>
+      <c r="B38" s="35" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C38" s="36" t="n">
+        <v>22</v>
+      </c>
+      <c r="D38" s="36" t="n">
+        <v>8</v>
+      </c>
+      <c r="E38" s="36" t="n">
+        <v>30</v>
+      </c>
+      <c r="F38" s="37" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="G38" s="36" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="34" t="inlineStr">
+        <is>
+          <t>Qatar (QIA / Qai + Brookfield JV)</t>
+        </is>
+      </c>
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C39" s="36" t="n">
+        <v>14</v>
+      </c>
+      <c r="D39" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="E39" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="F39" s="37" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G39" s="36" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="34" t="inlineStr">
+        <is>
+          <t>EU / France (Mistral, sovereign cloud)</t>
+        </is>
+      </c>
+      <c r="B40" s="35" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C40" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="D40" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="E40" s="36" t="n">
+        <v>17</v>
+      </c>
+      <c r="F40" s="37" t="n">
+        <v>0.2941176470588235</v>
+      </c>
+      <c r="G40" s="36" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="34" t="inlineStr">
+        <is>
+          <t>India (IndiaAI Mission)</t>
+        </is>
+      </c>
+      <c r="B41" s="35" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C41" s="36" t="n">
+        <v>8</v>
+      </c>
+      <c r="D41" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="F41" s="37" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G41" s="36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="22" t="inlineStr">
+        <is>
+          <t>Sovereign cloud subtotal</t>
+        </is>
+      </c>
+      <c r="B42" s="23" t="n"/>
+      <c r="C42" s="24">
+        <f>SUM(C35:C41)</f>
+        <v/>
+      </c>
+      <c r="D42" s="24">
+        <f>SUM(D35:D41)</f>
+        <v/>
+      </c>
+      <c r="E42" s="24">
+        <f>SUM(E35:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="25">
+        <f>D42/E42</f>
+        <v/>
+      </c>
+      <c r="G42" s="24">
+        <f>SUM(G35:G41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="38" t="inlineStr">
         <is>
           <t>GRAND TOTAL — all companies</t>
         </is>
       </c>
-      <c r="B23" s="31" t="n"/>
-      <c r="C23" s="32">
-        <f>SUM(C6,C7,C8,C9,C10,C13,C14,C15,C16,C17,C18,C19,C20,C21)</f>
-        <v/>
-      </c>
-      <c r="D23" s="32">
-        <f>SUM(D6,D7,D8,D9,D10,D13,D14,D15,D16,D17,D18,D19,D20,D21)</f>
-        <v/>
-      </c>
-      <c r="E23" s="32">
-        <f>SUM(E6,E7,E8,E9,E10,E13,E14,E15,E16,E17,E18,E19,E20,E21)</f>
-        <v/>
-      </c>
-      <c r="F23" s="33">
-        <f>D23/E23</f>
-        <v/>
-      </c>
-      <c r="G23" s="32">
-        <f>SUM(G6,G7,G8,G9,G10,G13,G14,G15,G16,G17,G18,G19,G20,G21)</f>
+      <c r="B43" s="39" t="n"/>
+      <c r="C43" s="40">
+        <f>SUM(C6,C7,C8,C9,C10,C13,C14,C15,C16,C17,C18,C19,C20,C21,C24,C25,C26,C27,C28,C29,C30,C31,C32,C35,C36,C37,C38,C39,C40,C41)</f>
+        <v/>
+      </c>
+      <c r="D43" s="40">
+        <f>SUM(D6,D7,D8,D9,D10,D13,D14,D15,D16,D17,D18,D19,D20,D21,D24,D25,D26,D27,D28,D29,D30,D31,D32,D35,D36,D37,D38,D39,D40,D41)</f>
+        <v/>
+      </c>
+      <c r="E43" s="40">
+        <f>SUM(E6,E7,E8,E9,E10,E13,E14,E15,E16,E17,E18,E19,E20,E21,E24,E25,E26,E27,E28,E29,E30,E31,E32,E35,E36,E37,E38,E39,E40,E41)</f>
+        <v/>
+      </c>
+      <c r="F43" s="41">
+        <f>D43/E43</f>
+        <v/>
+      </c>
+      <c r="G43" s="40">
+        <f>SUM(G6,G7,G8,G9,G10,G13,G14,G15,G16,G17,G18,G19,G20,G21,G24,G25,G26,G27,G28,G29,G30,G31,G32,G35,G36,G37,G38,G39,G40,G41)</f>
         <v/>
       </c>
     </row>
@@ -2275,7 +3143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2394,7 +3262,7 @@
           <t>Meta Platforms</t>
         </is>
       </c>
-      <c r="B6" s="34" t="inlineStr">
+      <c r="B6" s="42" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
@@ -2420,14 +3288,14 @@
       <c r="I6" s="20" t="n">
         <v>20</v>
       </c>
-      <c r="J6" s="35">
+      <c r="J6" s="43">
         <f>SUM(C6:I6)</f>
         <v/>
       </c>
-      <c r="K6" s="36" t="n">
+      <c r="K6" s="44" t="n">
         <v>180</v>
       </c>
-      <c r="L6" s="37" t="n">
+      <c r="L6" s="45" t="n">
         <v>487</v>
       </c>
     </row>
@@ -2437,7 +3305,7 @@
           <t>Amazon (AWS)</t>
         </is>
       </c>
-      <c r="B7" s="34" t="inlineStr">
+      <c r="B7" s="42" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
@@ -2463,14 +3331,14 @@
       <c r="I7" s="20" t="n">
         <v>30</v>
       </c>
-      <c r="J7" s="35">
+      <c r="J7" s="43">
         <f>SUM(C7:I7)</f>
         <v/>
       </c>
-      <c r="K7" s="36" t="n">
+      <c r="K7" s="44" t="n">
         <v>50</v>
       </c>
-      <c r="L7" s="37" t="n">
+      <c r="L7" s="45" t="n">
         <v>950</v>
       </c>
     </row>
@@ -2480,7 +3348,7 @@
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="B8" s="34" t="inlineStr">
+      <c r="B8" s="42" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
@@ -2506,14 +3374,14 @@
       <c r="I8" s="20" t="n">
         <v>35</v>
       </c>
-      <c r="J8" s="35">
+      <c r="J8" s="43">
         <f>SUM(C8:I8)</f>
         <v/>
       </c>
-      <c r="K8" s="36" t="n">
+      <c r="K8" s="44" t="n">
         <v>70</v>
       </c>
-      <c r="L8" s="37" t="n">
+      <c r="L8" s="45" t="n">
         <v>750</v>
       </c>
     </row>
@@ -2523,7 +3391,7 @@
           <t>Alphabet (Google)</t>
         </is>
       </c>
-      <c r="B9" s="34" t="inlineStr">
+      <c r="B9" s="42" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
@@ -2549,14 +3417,14 @@
       <c r="I9" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="J9" s="35">
+      <c r="J9" s="43">
         <f>SUM(C9:I9)</f>
         <v/>
       </c>
-      <c r="K9" s="36" t="n">
+      <c r="K9" s="44" t="n">
         <v>30</v>
       </c>
-      <c r="L9" s="37" t="n">
+      <c r="L9" s="45" t="n">
         <v>931</v>
       </c>
     </row>
@@ -2566,7 +3434,7 @@
           <t>Oracle (OCI)</t>
         </is>
       </c>
-      <c r="B10" s="34" t="inlineStr">
+      <c r="B10" s="42" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
@@ -2592,19 +3460,19 @@
       <c r="I10" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="J10" s="35">
+      <c r="J10" s="43">
         <f>SUM(C10:I10)</f>
         <v/>
       </c>
-      <c r="K10" s="36" t="n">
+      <c r="K10" s="44" t="n">
         <v>45</v>
       </c>
-      <c r="L10" s="37" t="n">
+      <c r="L10" s="45" t="n">
         <v>175</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="38" t="inlineStr">
+      <c r="A11" s="46" t="inlineStr">
         <is>
           <t>Hyperscaler subtotal</t>
         </is>
@@ -2675,7 +3543,7 @@
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="B13" s="39" t="inlineStr">
+      <c r="B13" s="47" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
@@ -2701,14 +3569,14 @@
       <c r="I13" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="J13" s="40">
+      <c r="J13" s="48">
         <f>SUM(C13:I13)</f>
         <v/>
       </c>
-      <c r="K13" s="41" t="n">
+      <c r="K13" s="49" t="n">
         <v>95</v>
       </c>
-      <c r="L13" s="42" t="n">
+      <c r="L13" s="50" t="n">
         <v>25</v>
       </c>
     </row>
@@ -2718,7 +3586,7 @@
           <t>SpaceX / xAI (Colossus)</t>
         </is>
       </c>
-      <c r="B14" s="39" t="inlineStr">
+      <c r="B14" s="47" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
@@ -2744,14 +3612,14 @@
       <c r="I14" s="28" t="n">
         <v>27</v>
       </c>
-      <c r="J14" s="40">
+      <c r="J14" s="48">
         <f>SUM(C14:I14)</f>
         <v/>
       </c>
-      <c r="K14" s="41" t="n">
+      <c r="K14" s="49" t="n">
         <v>70</v>
       </c>
-      <c r="L14" s="42" t="n">
+      <c r="L14" s="50" t="n">
         <v>140</v>
       </c>
     </row>
@@ -2761,7 +3629,7 @@
           <t>Other neoclouds &amp; AI-native DCs</t>
         </is>
       </c>
-      <c r="B15" s="39" t="inlineStr">
+      <c r="B15" s="47" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
@@ -2787,14 +3655,14 @@
       <c r="I15" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="J15" s="40">
+      <c r="J15" s="48">
         <f>SUM(C15:I15)</f>
         <v/>
       </c>
-      <c r="K15" s="41" t="n">
+      <c r="K15" s="49" t="n">
         <v>25</v>
       </c>
-      <c r="L15" s="42" t="n">
+      <c r="L15" s="50" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2804,7 +3672,7 @@
           <t>Nebius</t>
         </is>
       </c>
-      <c r="B16" s="39" t="inlineStr">
+      <c r="B16" s="47" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
@@ -2830,14 +3698,14 @@
       <c r="I16" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="J16" s="40">
+      <c r="J16" s="48">
         <f>SUM(C16:I16)</f>
         <v/>
       </c>
-      <c r="K16" s="41" t="n">
+      <c r="K16" s="49" t="n">
         <v>10</v>
       </c>
-      <c r="L16" s="42" t="n">
+      <c r="L16" s="50" t="n">
         <v>18</v>
       </c>
     </row>
@@ -2847,7 +3715,7 @@
           <t>IREN</t>
         </is>
       </c>
-      <c r="B17" s="39" t="inlineStr">
+      <c r="B17" s="47" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
@@ -2873,14 +3741,14 @@
       <c r="I17" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="40">
+      <c r="J17" s="48">
         <f>SUM(C17:I17)</f>
         <v/>
       </c>
-      <c r="K17" s="41" t="n">
+      <c r="K17" s="49" t="n">
         <v>8</v>
       </c>
-      <c r="L17" s="42" t="n">
+      <c r="L17" s="50" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2890,7 +3758,7 @@
           <t>Crusoe</t>
         </is>
       </c>
-      <c r="B18" s="39" t="inlineStr">
+      <c r="B18" s="47" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
@@ -2916,14 +3784,14 @@
       <c r="I18" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="J18" s="40">
+      <c r="J18" s="48">
         <f>SUM(C18:I18)</f>
         <v/>
       </c>
-      <c r="K18" s="41" t="n">
+      <c r="K18" s="49" t="n">
         <v>12</v>
       </c>
-      <c r="L18" s="42" t="n">
+      <c r="L18" s="50" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2933,7 +3801,7 @@
           <t>Fluidstack</t>
         </is>
       </c>
-      <c r="B19" s="39" t="inlineStr">
+      <c r="B19" s="47" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
@@ -2959,14 +3827,14 @@
       <c r="I19" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="J19" s="40">
+      <c r="J19" s="48">
         <f>SUM(C19:I19)</f>
         <v/>
       </c>
-      <c r="K19" s="41" t="n">
+      <c r="K19" s="49" t="n">
         <v>14</v>
       </c>
-      <c r="L19" s="42" t="n">
+      <c r="L19" s="50" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2976,7 +3844,7 @@
           <t>Lambda</t>
         </is>
       </c>
-      <c r="B20" s="39" t="inlineStr">
+      <c r="B20" s="47" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
@@ -3002,14 +3870,14 @@
       <c r="I20" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="J20" s="40">
+      <c r="J20" s="48">
         <f>SUM(C20:I20)</f>
         <v/>
       </c>
-      <c r="K20" s="41" t="n">
+      <c r="K20" s="49" t="n">
         <v>10</v>
       </c>
-      <c r="L20" s="42" t="n">
+      <c r="L20" s="50" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3019,7 +3887,7 @@
           <t>Nscale</t>
         </is>
       </c>
-      <c r="B21" s="39" t="inlineStr">
+      <c r="B21" s="47" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
@@ -3045,19 +3913,19 @@
       <c r="I21" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="J21" s="40">
+      <c r="J21" s="48">
         <f>SUM(C21:I21)</f>
         <v/>
       </c>
-      <c r="K21" s="41" t="n">
+      <c r="K21" s="49" t="n">
         <v>8</v>
       </c>
-      <c r="L21" s="42" t="n">
+      <c r="L21" s="50" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="38" t="inlineStr">
+      <c r="A22" s="46" t="inlineStr">
         <is>
           <t>Neocloud / AI-native subtotal</t>
         </is>
@@ -3105,89 +3973,909 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="30" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>COLOCATION / DATA-CENTER REIT</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
+      <c r="L23" s="15" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>Other colo &amp; powered-shell owners</t>
+        </is>
+      </c>
+      <c r="B24" s="51" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C24" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="D24" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="E24" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="F24" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="G24" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="H24" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="J24" s="52">
+        <f>SUM(C24:I24)</f>
+        <v/>
+      </c>
+      <c r="K24" s="53" t="n">
+        <v>30</v>
+      </c>
+      <c r="L24" s="54" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>Equinix</t>
+        </is>
+      </c>
+      <c r="B25" s="51" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="n">
+        <v>18</v>
+      </c>
+      <c r="D25" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="H25" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" s="52">
+        <f>SUM(C25:I25)</f>
+        <v/>
+      </c>
+      <c r="K25" s="53" t="n">
+        <v>20</v>
+      </c>
+      <c r="L25" s="54" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>QTS (Blackstone)</t>
+        </is>
+      </c>
+      <c r="B26" s="51" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C26" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="F26" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="G26" s="32" t="n">
+        <v>19</v>
+      </c>
+      <c r="H26" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="52">
+        <f>SUM(C26:I26)</f>
+        <v/>
+      </c>
+      <c r="K26" s="53" t="n">
+        <v>35</v>
+      </c>
+      <c r="L26" s="54" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>Digital Realty</t>
+        </is>
+      </c>
+      <c r="B27" s="51" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C27" s="32" t="n">
+        <v>16</v>
+      </c>
+      <c r="D27" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F27" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="H27" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" s="52">
+        <f>SUM(C27:I27)</f>
+        <v/>
+      </c>
+      <c r="K27" s="53" t="n">
+        <v>18</v>
+      </c>
+      <c r="L27" s="54" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Vantage Data Centers</t>
+        </is>
+      </c>
+      <c r="B28" s="51" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C28" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="E28" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="F28" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G28" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="H28" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J28" s="52">
+        <f>SUM(C28:I28)</f>
+        <v/>
+      </c>
+      <c r="K28" s="53" t="n">
+        <v>28</v>
+      </c>
+      <c r="L28" s="54" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>Aligned Data Centers (MGX/BlackRock)</t>
+        </is>
+      </c>
+      <c r="B29" s="51" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C29" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="F29" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G29" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="H29" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J29" s="52">
+        <f>SUM(C29:I29)</f>
+        <v/>
+      </c>
+      <c r="K29" s="53" t="n">
+        <v>22</v>
+      </c>
+      <c r="L29" s="54" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>CyrusOne (KKR/GIP)</t>
+        </is>
+      </c>
+      <c r="B30" s="51" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C30" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E30" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="F30" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G30" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="H30" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" s="52">
+        <f>SUM(C30:I30)</f>
+        <v/>
+      </c>
+      <c r="K30" s="53" t="n">
+        <v>22</v>
+      </c>
+      <c r="L30" s="54" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>Switch (DigitalBridge)</t>
+        </is>
+      </c>
+      <c r="B31" s="51" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C31" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E31" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="F31" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="H31" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" s="52">
+        <f>SUM(C31:I31)</f>
+        <v/>
+      </c>
+      <c r="K31" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="L31" s="54" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Stack Infrastructure</t>
+        </is>
+      </c>
+      <c r="B32" s="51" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C32" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="F32" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="G32" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="H32" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="52">
+        <f>SUM(C32:I32)</f>
+        <v/>
+      </c>
+      <c r="K32" s="53" t="n">
+        <v>12</v>
+      </c>
+      <c r="L32" s="54" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="46" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT subtotal</t>
+        </is>
+      </c>
+      <c r="B33" s="23" t="n"/>
+      <c r="C33" s="24">
+        <f>SUM(C24:C32)</f>
+        <v/>
+      </c>
+      <c r="D33" s="24">
+        <f>SUM(D24:D32)</f>
+        <v/>
+      </c>
+      <c r="E33" s="24">
+        <f>SUM(E24:E32)</f>
+        <v/>
+      </c>
+      <c r="F33" s="24">
+        <f>SUM(F24:F32)</f>
+        <v/>
+      </c>
+      <c r="G33" s="24">
+        <f>SUM(G24:G32)</f>
+        <v/>
+      </c>
+      <c r="H33" s="24">
+        <f>SUM(H24:H32)</f>
+        <v/>
+      </c>
+      <c r="I33" s="24">
+        <f>SUM(I24:I32)</f>
+        <v/>
+      </c>
+      <c r="J33" s="24">
+        <f>SUM(J24:J32)</f>
+        <v/>
+      </c>
+      <c r="K33" s="24">
+        <f>SUM(K24:K32)</f>
+        <v/>
+      </c>
+      <c r="L33" s="24">
+        <f>SUM(L24:L32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>SOVEREIGN CLOUD</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="n"/>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="15" t="n"/>
+      <c r="F34" s="15" t="n"/>
+      <c r="G34" s="15" t="n"/>
+      <c r="H34" s="15" t="n"/>
+      <c r="I34" s="15" t="n"/>
+      <c r="J34" s="15" t="n"/>
+      <c r="K34" s="15" t="n"/>
+      <c r="L34" s="15" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="34" t="inlineStr">
+        <is>
+          <t>HUMAIN (Saudi PIF)</t>
+        </is>
+      </c>
+      <c r="B35" s="55" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C35" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="D35" s="36" t="n">
+        <v>8</v>
+      </c>
+      <c r="E35" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="F35" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="J35" s="56">
+        <f>SUM(C35:I35)</f>
+        <v/>
+      </c>
+      <c r="K35" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="L35" s="58" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="34" t="inlineStr">
+        <is>
+          <t>MGX / Mubadala (UAE)</t>
+        </is>
+      </c>
+      <c r="B36" s="55" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C36" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="E36" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="F36" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="J36" s="56">
+        <f>SUM(C36:I36)</f>
+        <v/>
+      </c>
+      <c r="K36" s="57" t="n">
+        <v>8</v>
+      </c>
+      <c r="L36" s="58" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="34" t="inlineStr">
+        <is>
+          <t>Stargate UAE / G42 / Khazna</t>
+        </is>
+      </c>
+      <c r="B37" s="55" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C37" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F37" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="J37" s="56">
+        <f>SUM(C37:I37)</f>
+        <v/>
+      </c>
+      <c r="K37" s="57" t="n">
+        <v>6</v>
+      </c>
+      <c r="L37" s="58" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="34" t="inlineStr">
+        <is>
+          <t>Other sovereign AI (Japan, Korea, Singapore, etc.)</t>
+        </is>
+      </c>
+      <c r="B38" s="55" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C38" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="J38" s="56">
+        <f>SUM(C38:I38)</f>
+        <v/>
+      </c>
+      <c r="K38" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="L38" s="58" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="34" t="inlineStr">
+        <is>
+          <t>Qatar (QIA / Qai + Brookfield JV)</t>
+        </is>
+      </c>
+      <c r="B39" s="55" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C39" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="56">
+        <f>SUM(C39:I39)</f>
+        <v/>
+      </c>
+      <c r="K39" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="L39" s="58" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="34" t="inlineStr">
+        <is>
+          <t>EU / France (Mistral, sovereign cloud)</t>
+        </is>
+      </c>
+      <c r="B40" s="55" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C40" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" s="56">
+        <f>SUM(C40:I40)</f>
+        <v/>
+      </c>
+      <c r="K40" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="L40" s="58" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="34" t="inlineStr">
+        <is>
+          <t>India (IndiaAI Mission)</t>
+        </is>
+      </c>
+      <c r="B41" s="55" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C41" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="J41" s="56">
+        <f>SUM(C41:I41)</f>
+        <v/>
+      </c>
+      <c r="K41" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="L41" s="58" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="46" t="inlineStr">
+        <is>
+          <t>Sovereign cloud subtotal</t>
+        </is>
+      </c>
+      <c r="B42" s="23" t="n"/>
+      <c r="C42" s="24">
+        <f>SUM(C35:C41)</f>
+        <v/>
+      </c>
+      <c r="D42" s="24">
+        <f>SUM(D35:D41)</f>
+        <v/>
+      </c>
+      <c r="E42" s="24">
+        <f>SUM(E35:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="24">
+        <f>SUM(F35:F41)</f>
+        <v/>
+      </c>
+      <c r="G42" s="24">
+        <f>SUM(G35:G41)</f>
+        <v/>
+      </c>
+      <c r="H42" s="24">
+        <f>SUM(H35:H41)</f>
+        <v/>
+      </c>
+      <c r="I42" s="24">
+        <f>SUM(I35:I41)</f>
+        <v/>
+      </c>
+      <c r="J42" s="24">
+        <f>SUM(J35:J41)</f>
+        <v/>
+      </c>
+      <c r="K42" s="24">
+        <f>SUM(K35:K41)</f>
+        <v/>
+      </c>
+      <c r="L42" s="24">
+        <f>SUM(L35:L41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="38" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B23" s="31" t="n"/>
-      <c r="C23" s="32">
-        <f>SUM(C6,C7,C8,C9,C10,C13,C14,C15,C16,C17,C18,C19,C20,C21)</f>
-        <v/>
-      </c>
-      <c r="D23" s="32">
-        <f>SUM(D6,D7,D8,D9,D10,D13,D14,D15,D16,D17,D18,D19,D20,D21)</f>
-        <v/>
-      </c>
-      <c r="E23" s="32">
-        <f>SUM(E6,E7,E8,E9,E10,E13,E14,E15,E16,E17,E18,E19,E20,E21)</f>
-        <v/>
-      </c>
-      <c r="F23" s="32">
-        <f>SUM(F6,F7,F8,F9,F10,F13,F14,F15,F16,F17,F18,F19,F20,F21)</f>
-        <v/>
-      </c>
-      <c r="G23" s="32">
-        <f>SUM(G6,G7,G8,G9,G10,G13,G14,G15,G16,G17,G18,G19,G20,G21)</f>
-        <v/>
-      </c>
-      <c r="H23" s="32">
-        <f>SUM(H6,H7,H8,H9,H10,H13,H14,H15,H16,H17,H18,H19,H20,H21)</f>
-        <v/>
-      </c>
-      <c r="I23" s="32">
-        <f>SUM(I6,I7,I8,I9,I10,I13,I14,I15,I16,I17,I18,I19,I20,I21)</f>
-        <v/>
-      </c>
-      <c r="J23" s="32">
-        <f>SUM(J6,J7,J8,J9,J10,J13,J14,J15,J16,J17,J18,J19,J20,J21)</f>
-        <v/>
-      </c>
-      <c r="K23" s="32">
-        <f>SUM(K6,K7,K8,K9,K10,K13,K14,K15,K16,K17,K18,K19,K20,K21)</f>
-        <v/>
-      </c>
-      <c r="L23" s="32">
-        <f>SUM(L6,L7,L8,L9,L10,L13,L14,L15,L16,L17,L18,L19,L20,L21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="43" t="inlineStr">
+      <c r="B43" s="39" t="n"/>
+      <c r="C43" s="40">
+        <f>SUM(C6,C7,C8,C9,C10,C13,C14,C15,C16,C17,C18,C19,C20,C21,C24,C25,C26,C27,C28,C29,C30,C31,C32,C35,C36,C37,C38,C39,C40,C41)</f>
+        <v/>
+      </c>
+      <c r="D43" s="40">
+        <f>SUM(D6,D7,D8,D9,D10,D13,D14,D15,D16,D17,D18,D19,D20,D21,D24,D25,D26,D27,D28,D29,D30,D31,D32,D35,D36,D37,D38,D39,D40,D41)</f>
+        <v/>
+      </c>
+      <c r="E43" s="40">
+        <f>SUM(E6,E7,E8,E9,E10,E13,E14,E15,E16,E17,E18,E19,E20,E21,E24,E25,E26,E27,E28,E29,E30,E31,E32,E35,E36,E37,E38,E39,E40,E41)</f>
+        <v/>
+      </c>
+      <c r="F43" s="40">
+        <f>SUM(F6,F7,F8,F9,F10,F13,F14,F15,F16,F17,F18,F19,F20,F21,F24,F25,F26,F27,F28,F29,F30,F31,F32,F35,F36,F37,F38,F39,F40,F41)</f>
+        <v/>
+      </c>
+      <c r="G43" s="40">
+        <f>SUM(G6,G7,G8,G9,G10,G13,G14,G15,G16,G17,G18,G19,G20,G21,G24,G25,G26,G27,G28,G29,G30,G31,G32,G35,G36,G37,G38,G39,G40,G41)</f>
+        <v/>
+      </c>
+      <c r="H43" s="40">
+        <f>SUM(H6,H7,H8,H9,H10,H13,H14,H15,H16,H17,H18,H19,H20,H21,H24,H25,H26,H27,H28,H29,H30,H31,H32,H35,H36,H37,H38,H39,H40,H41)</f>
+        <v/>
+      </c>
+      <c r="I43" s="40">
+        <f>SUM(I6,I7,I8,I9,I10,I13,I14,I15,I16,I17,I18,I19,I20,I21,I24,I25,I26,I27,I28,I29,I30,I31,I32,I35,I36,I37,I38,I39,I40,I41)</f>
+        <v/>
+      </c>
+      <c r="J43" s="40">
+        <f>SUM(J6,J7,J8,J9,J10,J13,J14,J15,J16,J17,J18,J19,J20,J21,J24,J25,J26,J27,J28,J29,J30,J31,J32,J35,J36,J37,J38,J39,J40,J41)</f>
+        <v/>
+      </c>
+      <c r="K43" s="40">
+        <f>SUM(K6,K7,K8,K9,K10,K13,K14,K15,K16,K17,K18,K19,K20,K21,K24,K25,K26,K27,K28,K29,K30,K31,K32,K35,K36,K37,K38,K39,K40,K41)</f>
+        <v/>
+      </c>
+      <c r="L43" s="40">
+        <f>SUM(L6,L7,L8,L9,L10,L13,L14,L15,L16,L17,L18,L19,L20,L21,L24,L25,L26,L27,L28,L29,L30,L31,L32,L35,L36,L37,L38,L39,L40,L41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="59" t="inlineStr">
         <is>
           <t>% of total debt</t>
         </is>
       </c>
-      <c r="C24" s="44">
-        <f>C23/$J$23</f>
-        <v/>
-      </c>
-      <c r="D24" s="44">
-        <f>D23/$J$23</f>
-        <v/>
-      </c>
-      <c r="E24" s="44">
-        <f>E23/$J$23</f>
-        <v/>
-      </c>
-      <c r="F24" s="44">
-        <f>F23/$J$23</f>
-        <v/>
-      </c>
-      <c r="G24" s="44">
-        <f>G23/$J$23</f>
-        <v/>
-      </c>
-      <c r="H24" s="44">
-        <f>H23/$J$23</f>
-        <v/>
-      </c>
-      <c r="I24" s="44">
-        <f>I23/$J$23</f>
-        <v/>
-      </c>
-      <c r="J24" s="45">
-        <f>J23/J23</f>
+      <c r="C44" s="60">
+        <f>C43/$J$43</f>
+        <v/>
+      </c>
+      <c r="D44" s="60">
+        <f>D43/$J$43</f>
+        <v/>
+      </c>
+      <c r="E44" s="60">
+        <f>E43/$J$43</f>
+        <v/>
+      </c>
+      <c r="F44" s="60">
+        <f>F43/$J$43</f>
+        <v/>
+      </c>
+      <c r="G44" s="60">
+        <f>G43/$J$43</f>
+        <v/>
+      </c>
+      <c r="H44" s="60">
+        <f>H43/$J$43</f>
+        <v/>
+      </c>
+      <c r="I44" s="60">
+        <f>I43/$J$43</f>
+        <v/>
+      </c>
+      <c r="J44" s="61">
+        <f>J43/J43</f>
         <v/>
       </c>
     </row>
@@ -3203,7 +4891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3297,7 +4985,7 @@
       <c r="G5" s="20" t="n">
         <v>215</v>
       </c>
-      <c r="H5" s="35">
+      <c r="H5" s="43">
         <f>SUM(B5:G5)</f>
         <v/>
       </c>
@@ -3326,7 +5014,7 @@
       <c r="G6" s="20" t="n">
         <v>255</v>
       </c>
-      <c r="H6" s="35">
+      <c r="H6" s="43">
         <f>SUM(B6:G6)</f>
         <v/>
       </c>
@@ -3355,7 +5043,7 @@
       <c r="G7" s="20" t="n">
         <v>245</v>
       </c>
-      <c r="H7" s="35">
+      <c r="H7" s="43">
         <f>SUM(B7:G7)</f>
         <v/>
       </c>
@@ -3384,7 +5072,7 @@
       <c r="G8" s="20" t="n">
         <v>195</v>
       </c>
-      <c r="H8" s="35">
+      <c r="H8" s="43">
         <f>SUM(B8:G8)</f>
         <v/>
       </c>
@@ -3413,7 +5101,7 @@
       <c r="G9" s="20" t="n">
         <v>90</v>
       </c>
-      <c r="H9" s="35">
+      <c r="H9" s="43">
         <f>SUM(B9:G9)</f>
         <v/>
       </c>
@@ -3442,43 +5130,101 @@
       <c r="G10" s="28" t="n">
         <v>126</v>
       </c>
-      <c r="H10" s="40">
+      <c r="H10" s="48">
         <f>SUM(B10:G10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="46" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REITs (aggregate)</t>
+        </is>
+      </c>
+      <c r="B11" s="32" t="n">
+        <v>55</v>
+      </c>
+      <c r="C11" s="32" t="n">
+        <v>70</v>
+      </c>
+      <c r="D11" s="32" t="n">
+        <v>80</v>
+      </c>
+      <c r="E11" s="32" t="n">
+        <v>85</v>
+      </c>
+      <c r="F11" s="32" t="n">
+        <v>85</v>
+      </c>
+      <c r="G11" s="32" t="n">
+        <v>85</v>
+      </c>
+      <c r="H11" s="52">
+        <f>SUM(B11:G11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t>Sovereign clouds (aggregate)</t>
+        </is>
+      </c>
+      <c r="B12" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="C12" s="36" t="n">
+        <v>35</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>45</v>
+      </c>
+      <c r="E12" s="36" t="n">
+        <v>50</v>
+      </c>
+      <c r="F12" s="36" t="n">
+        <v>50</v>
+      </c>
+      <c r="G12" s="36" t="n">
+        <v>50</v>
+      </c>
+      <c r="H12" s="56">
+        <f>SUM(B12:G12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="62" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="32">
-        <f>SUM(B5:B10)</f>
-        <v/>
-      </c>
-      <c r="C11" s="32">
-        <f>SUM(C5:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="32">
-        <f>SUM(D5:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="32">
-        <f>SUM(E5:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="32">
-        <f>SUM(F5:F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="32">
-        <f>SUM(G5:G10)</f>
-        <v/>
-      </c>
-      <c r="H11" s="32">
-        <f>SUM(H5:H10)</f>
+      <c r="B13" s="40">
+        <f>SUM(B5:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="40">
+        <f>SUM(C5:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="40">
+        <f>SUM(D5:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="40">
+        <f>SUM(E5:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="40">
+        <f>SUM(F5:F12)</f>
+        <v/>
+      </c>
+      <c r="G13" s="40">
+        <f>SUM(G5:G12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="40">
+        <f>SUM(H5:H12)</f>
         <v/>
       </c>
     </row>
@@ -3494,7 +5240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3552,895 +5298,1183 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="47" t="inlineStr">
+      <c r="A5" s="63" t="inlineStr">
         <is>
           <t>Meta Platforms</t>
         </is>
       </c>
-      <c r="B5" s="48" t="inlineStr">
+      <c r="B5" s="64" t="inlineStr">
         <is>
           <t>Hyperion JV (Beignet Investor LLC) — Blue Owl 80% / Meta 20%; $27.3bn A+ private bond led by PIMCO (~$18bn) &amp; BlackRock; off-B/S SPV w/ residual-value guarantee</t>
         </is>
       </c>
-      <c r="C5" s="48" t="inlineStr">
+      <c r="C5" s="64" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D5" s="48" t="inlineStr">
+      <c r="D5" s="64" t="inlineStr">
         <is>
           <t>$27.3bn debt</t>
         </is>
       </c>
-      <c r="E5" s="48" t="inlineStr">
+      <c r="E5" s="64" t="inlineStr">
         <is>
           <t>SPV / private credit / insurance</t>
         </is>
       </c>
-      <c r="F5" s="49" t="inlineStr">
+      <c r="F5" s="65" t="inlineStr">
         <is>
           <t>Meta IR; FT; S&amp;P</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="50" t="inlineStr">
+      <c r="A6" s="66" t="inlineStr">
         <is>
           <t>Meta Platforms</t>
         </is>
       </c>
-      <c r="B6" s="51" t="inlineStr">
+      <c r="B6" s="67" t="inlineStr">
         <is>
           <t>$30bn multi-tranche IG corporate bond (largest 2025 IG deal), maturities to 2063</t>
         </is>
       </c>
-      <c r="C6" s="51" t="inlineStr">
+      <c r="C6" s="67" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D6" s="51" t="inlineStr">
+      <c r="D6" s="67" t="inlineStr">
         <is>
           <t>$30bn</t>
         </is>
       </c>
-      <c r="E6" s="51" t="inlineStr">
+      <c r="E6" s="67" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F6" s="52" t="inlineStr">
+      <c r="F6" s="68" t="inlineStr">
         <is>
           <t>BofA; MUFG</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="47" t="inlineStr">
+      <c r="A7" s="63" t="inlineStr">
         <is>
           <t>Amazon (AWS)</t>
         </is>
       </c>
-      <c r="B7" s="48" t="inlineStr">
+      <c r="B7" s="64" t="inlineStr">
         <is>
           <t>~$54bn USD + €14.5bn (~$16.8bn) IG bonds (near-record), ~4x oversubscribed</t>
         </is>
       </c>
-      <c r="C7" s="48" t="inlineStr">
+      <c r="C7" s="64" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D7" s="48" t="inlineStr">
+      <c r="D7" s="64" t="inlineStr">
         <is>
           <t>~$71bn</t>
         </is>
       </c>
-      <c r="E7" s="48" t="inlineStr">
+      <c r="E7" s="64" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F7" s="49" t="inlineStr">
+      <c r="F7" s="65" t="inlineStr">
         <is>
           <t>CNA; Reuters</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="50" t="inlineStr">
+      <c r="A8" s="66" t="inlineStr">
         <is>
           <t>Amazon (AWS)</t>
         </is>
       </c>
-      <c r="B8" s="51" t="inlineStr">
+      <c r="B8" s="67" t="inlineStr">
         <is>
           <t>$15bn IG bond</t>
         </is>
       </c>
-      <c r="C8" s="51" t="inlineStr">
+      <c r="C8" s="67" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D8" s="51" t="inlineStr">
+      <c r="D8" s="67" t="inlineStr">
         <is>
           <t>$15bn</t>
         </is>
       </c>
-      <c r="E8" s="51" t="inlineStr">
+      <c r="E8" s="67" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F8" s="52" t="inlineStr">
+      <c r="F8" s="68" t="inlineStr">
         <is>
           <t>CNA</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="47" t="inlineStr">
+      <c r="A9" s="63" t="inlineStr">
         <is>
           <t>Alphabet (Google)</t>
         </is>
       </c>
-      <c r="B9" s="48" t="inlineStr">
+      <c r="B9" s="64" t="inlineStr">
         <is>
           <t>~$32bn multi-currency bond incl. rare 100-yr tranche; plus $17.5bn Nov 2025</t>
         </is>
       </c>
-      <c r="C9" s="48" t="inlineStr">
+      <c r="C9" s="64" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D9" s="48" t="inlineStr">
+      <c r="D9" s="64" t="inlineStr">
         <is>
           <t>~$50bn</t>
         </is>
       </c>
-      <c r="E9" s="48" t="inlineStr">
+      <c r="E9" s="64" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F9" s="49" t="inlineStr">
+      <c r="F9" s="65" t="inlineStr">
         <is>
           <t>ConstructConnect; CNA</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="50" t="inlineStr">
+      <c r="A10" s="66" t="inlineStr">
         <is>
           <t>Oracle (OCI)</t>
         </is>
       </c>
-      <c r="B10" s="51" t="inlineStr">
+      <c r="B10" s="67" t="inlineStr">
         <is>
           <t>$25bn 8-part IG bond (Feb 2026) within $45-50bn CY26 debt+equity plan; $20bn ATM + mandatory convertible preferred (equity)</t>
         </is>
       </c>
-      <c r="C10" s="51" t="inlineStr">
+      <c r="C10" s="67" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D10" s="51" t="inlineStr">
+      <c r="D10" s="67" t="inlineStr">
         <is>
           <t>$25bn debt</t>
         </is>
       </c>
-      <c r="E10" s="51" t="inlineStr">
+      <c r="E10" s="67" t="inlineStr">
         <is>
           <t>Corporate bonds + equity</t>
         </is>
       </c>
-      <c r="F10" s="52" t="inlineStr">
+      <c r="F10" s="68" t="inlineStr">
         <is>
           <t>Oracle IR; IFR</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="47" t="inlineStr">
+      <c r="A11" s="63" t="inlineStr">
         <is>
           <t>Oracle (OCI)</t>
         </is>
       </c>
-      <c r="B11" s="48" t="inlineStr">
+      <c r="B11" s="64" t="inlineStr">
         <is>
           <t>$18bn 6-part IG bond (Sep 2025)</t>
         </is>
       </c>
-      <c r="C11" s="48" t="inlineStr">
+      <c r="C11" s="64" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D11" s="48" t="inlineStr">
+      <c r="D11" s="64" t="inlineStr">
         <is>
           <t>$18bn</t>
         </is>
       </c>
-      <c r="E11" s="48" t="inlineStr">
+      <c r="E11" s="64" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F11" s="49" t="inlineStr">
+      <c r="F11" s="65" t="inlineStr">
         <is>
           <t>Reuters/CNA</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="50" t="inlineStr">
+      <c r="A12" s="66" t="inlineStr">
         <is>
           <t>Oracle (OCI)</t>
         </is>
       </c>
-      <c r="B12" s="51" t="inlineStr">
+      <c r="B12" s="67" t="inlineStr">
         <is>
           <t>Project-level SPV financing: ~$16.3bn Michigan campus; further Texas / Wisconsin deals</t>
         </is>
       </c>
-      <c r="C12" s="51" t="inlineStr">
+      <c r="C12" s="67" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D12" s="51" t="inlineStr">
+      <c r="D12" s="67" t="inlineStr">
         <is>
           <t>~$25bn+</t>
         </is>
       </c>
-      <c r="E12" s="51" t="inlineStr">
+      <c r="E12" s="67" t="inlineStr">
         <is>
           <t>SPV / project finance</t>
         </is>
       </c>
-      <c r="F12" s="52" t="inlineStr">
+      <c r="F12" s="68" t="inlineStr">
         <is>
           <t>Press reports</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="47" t="inlineStr">
+      <c r="A13" s="63" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="B13" s="48" t="inlineStr">
+      <c r="B13" s="64" t="inlineStr">
         <is>
           <t>Finance-lease driven build (~$108bn uncommenced finance leases as of 9/30/24; commence FY25-FY30)</t>
         </is>
       </c>
-      <c r="C13" s="48" t="inlineStr">
+      <c r="C13" s="64" t="inlineStr">
         <is>
           <t>2024-30</t>
         </is>
       </c>
-      <c r="D13" s="48" t="inlineStr">
+      <c r="D13" s="64" t="inlineStr">
         <is>
           <t>$100bn+ leases</t>
         </is>
       </c>
-      <c r="E13" s="48" t="inlineStr">
+      <c r="E13" s="64" t="inlineStr">
         <is>
           <t>Vendor / lease / SPV</t>
         </is>
       </c>
-      <c r="F13" s="49" t="inlineStr">
+      <c r="F13" s="65" t="inlineStr">
         <is>
           <t>MSFT 10-Q; CNBC</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="50" t="inlineStr">
+      <c r="A14" s="66" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="B14" s="51" t="inlineStr">
+      <c r="B14" s="67" t="inlineStr">
         <is>
           <t>DDTL 4.0 — $8.5bn delayed-draw term loan; first IG-rated (Moody's A3 / DBRS A-low) GPU-backed financing; SOFR+225 / ~5.9%</t>
         </is>
       </c>
-      <c r="C14" s="51" t="inlineStr">
+      <c r="C14" s="67" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D14" s="51" t="inlineStr">
+      <c r="D14" s="67" t="inlineStr">
         <is>
           <t>$8.5bn</t>
         </is>
       </c>
-      <c r="E14" s="51" t="inlineStr">
+      <c r="E14" s="67" t="inlineStr">
         <is>
           <t>Bank / GPU-backed loan</t>
         </is>
       </c>
-      <c r="F14" s="52" t="inlineStr">
+      <c r="F14" s="68" t="inlineStr">
         <is>
           <t>CoreWeave IR</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="47" t="inlineStr">
+      <c r="A15" s="63" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="B15" s="48" t="inlineStr">
+      <c r="B15" s="64" t="inlineStr">
         <is>
           <t>$7.5bn debt facility led by Blackstone &amp; Magnetar (largest private debt deal at the time)</t>
         </is>
       </c>
-      <c r="C15" s="48" t="inlineStr">
+      <c r="C15" s="64" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D15" s="48" t="inlineStr">
+      <c r="D15" s="64" t="inlineStr">
         <is>
           <t>$7.5bn</t>
         </is>
       </c>
-      <c r="E15" s="48" t="inlineStr">
+      <c r="E15" s="64" t="inlineStr">
         <is>
           <t>Private credit / loan</t>
         </is>
       </c>
-      <c r="F15" s="49" t="inlineStr">
+      <c r="F15" s="65" t="inlineStr">
         <is>
           <t>Blackstone</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="50" t="inlineStr">
+      <c r="A16" s="66" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="B16" s="51" t="inlineStr">
+      <c r="B16" s="67" t="inlineStr">
         <is>
           <t>$2.7bn 1.75% convertible notes; ~$30bn total debt by early 2026; ~$28bn debt+equity raised in 12 mos</t>
         </is>
       </c>
-      <c r="C16" s="51" t="inlineStr">
+      <c r="C16" s="67" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D16" s="51" t="inlineStr">
+      <c r="D16" s="67" t="inlineStr">
         <is>
           <t>$2.7bn conv.</t>
         </is>
       </c>
-      <c r="E16" s="51" t="inlineStr">
+      <c r="E16" s="67" t="inlineStr">
         <is>
           <t>Convertibles</t>
         </is>
       </c>
-      <c r="F16" s="52" t="inlineStr">
+      <c r="F16" s="68" t="inlineStr">
         <is>
           <t>thedig; CoreWeave</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="47" t="inlineStr">
+      <c r="A17" s="63" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="B17" s="48" t="inlineStr">
+      <c r="B17" s="64" t="inlineStr">
         <is>
           <t>$2bn strategic equity from NVIDIA; IPO Mar 2025 raised ~$1.5bn</t>
         </is>
       </c>
-      <c r="C17" s="48" t="inlineStr">
+      <c r="C17" s="64" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D17" s="48" t="inlineStr">
+      <c r="D17" s="64" t="inlineStr">
         <is>
           <t>$3.5bn equity</t>
         </is>
       </c>
-      <c r="E17" s="48" t="inlineStr">
+      <c r="E17" s="64" t="inlineStr">
         <is>
           <t>Equity</t>
         </is>
       </c>
-      <c r="F17" s="49" t="inlineStr">
+      <c r="F17" s="65" t="inlineStr">
         <is>
           <t>CNBC; CoreWeave</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="50" t="inlineStr">
+      <c r="A18" s="66" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B18" s="51" t="inlineStr">
+      <c r="B18" s="67" t="inlineStr">
         <is>
           <t>SpaceX acquired xAI effective Feb 2, 2026; Colossus I &amp; II now SpaceX-owned (vertically-integrated AI platform; Terafab chip JV w/ Tesla &amp; Intel)</t>
         </is>
       </c>
-      <c r="C18" s="51" t="inlineStr">
+      <c r="C18" s="67" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D18" s="51" t="inlineStr">
+      <c r="D18" s="67" t="inlineStr">
         <is>
           <t>merger</t>
         </is>
       </c>
-      <c r="E18" s="51" t="inlineStr">
+      <c r="E18" s="67" t="inlineStr">
         <is>
           <t>Equity / M&amp;A</t>
         </is>
       </c>
-      <c r="F18" s="52" t="inlineStr">
+      <c r="F18" s="68" t="inlineStr">
         <is>
           <t>SpaceX S-1</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="47" t="inlineStr">
+      <c r="A19" s="63" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B19" s="48" t="inlineStr">
+      <c r="B19" s="64" t="inlineStr">
         <is>
           <t>SpaceX AI capex $12.7bn in 2025 (~61% of total) + $7.7bn in Q1 2026; AI buildout funded by Starlink FCF, private raises, planned IPO</t>
         </is>
       </c>
-      <c r="C19" s="48" t="inlineStr">
+      <c r="C19" s="64" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D19" s="48" t="inlineStr">
+      <c r="D19" s="64" t="inlineStr">
         <is>
           <t>$20bn+ capex</t>
         </is>
       </c>
-      <c r="E19" s="48" t="inlineStr">
+      <c r="E19" s="64" t="inlineStr">
         <is>
           <t>Internal / equity</t>
         </is>
       </c>
-      <c r="F19" s="49" t="inlineStr">
+      <c r="F19" s="65" t="inlineStr">
         <is>
           <t>SpaceX S-1; The Verge</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="50" t="inlineStr">
+      <c r="A20" s="66" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B20" s="51" t="inlineStr">
+      <c r="B20" s="67" t="inlineStr">
         <is>
           <t>Anthropic compute contract: $1.25bn/month (~$45bn) through May 2029 for Colossus I &amp; II — anchor revenue underwriting infra financing</t>
         </is>
       </c>
-      <c r="C20" s="51" t="inlineStr">
+      <c r="C20" s="67" t="inlineStr">
         <is>
           <t>2026-29</t>
         </is>
       </c>
-      <c r="D20" s="51" t="inlineStr">
+      <c r="D20" s="67" t="inlineStr">
         <is>
           <t>~$45bn</t>
         </is>
       </c>
-      <c r="E20" s="51" t="inlineStr">
+      <c r="E20" s="67" t="inlineStr">
         <is>
           <t>Take-or-pay (demand)</t>
         </is>
       </c>
-      <c r="F20" s="52" t="inlineStr">
+      <c r="F20" s="68" t="inlineStr">
         <is>
           <t>SpaceX S-1; The Verge</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="47" t="inlineStr">
+      <c r="A21" s="63" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B21" s="48" t="inlineStr">
+      <c r="B21" s="64" t="inlineStr">
         <is>
           <t>xAI $10bn raise ($5bn secured notes/term loans incl. Apollo $5bn facility + $5bn equity) via Morgan Stanley</t>
         </is>
       </c>
-      <c r="C21" s="48" t="inlineStr">
+      <c r="C21" s="64" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D21" s="48" t="inlineStr">
+      <c r="D21" s="64" t="inlineStr">
         <is>
           <t>$10bn</t>
         </is>
       </c>
-      <c r="E21" s="48" t="inlineStr">
+      <c r="E21" s="64" t="inlineStr">
         <is>
           <t>Loans + equity</t>
         </is>
       </c>
-      <c r="F21" s="49" t="inlineStr">
+      <c r="F21" s="65" t="inlineStr">
         <is>
           <t>CNBC</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="50" t="inlineStr">
+      <c r="A22" s="66" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B22" s="51" t="inlineStr">
+      <c r="B22" s="67" t="inlineStr">
         <is>
           <t>Colossus 2 SPV (Valor Equity): ~$12.5bn debt + ~$7.5bn equity (NVIDIA up to $2bn) to buy &amp; lease GPUs</t>
         </is>
       </c>
-      <c r="C22" s="51" t="inlineStr">
+      <c r="C22" s="67" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D22" s="51" t="inlineStr">
+      <c r="D22" s="67" t="inlineStr">
         <is>
           <t>~$20bn</t>
         </is>
       </c>
-      <c r="E22" s="51" t="inlineStr">
+      <c r="E22" s="67" t="inlineStr">
         <is>
           <t>SPV / vendor lease</t>
         </is>
       </c>
-      <c r="F22" s="52" t="inlineStr">
+      <c r="F22" s="68" t="inlineStr">
         <is>
           <t>The Information; Yahoo</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="47" t="inlineStr">
+      <c r="A23" s="63" t="inlineStr">
         <is>
           <t>Nebius</t>
         </is>
       </c>
-      <c r="B23" s="48" t="inlineStr">
+      <c r="B23" s="64" t="inlineStr">
         <is>
           <t>$3bn+ convertibles + bank lines; lighter balance sheet; Yandex spin-off cash ~$2.5bn; NVIDIA ~$2bn equity; Microsoft ~$7bn prepay</t>
         </is>
       </c>
-      <c r="C23" s="48" t="inlineStr">
+      <c r="C23" s="64" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D23" s="48" t="inlineStr">
+      <c r="D23" s="64" t="inlineStr">
         <is>
           <t>$3bn+</t>
         </is>
       </c>
-      <c r="E23" s="48" t="inlineStr">
+      <c r="E23" s="64" t="inlineStr">
         <is>
           <t>Convertibles</t>
         </is>
       </c>
-      <c r="F23" s="49" t="inlineStr">
+      <c r="F23" s="65" t="inlineStr">
         <is>
           <t>frankk research</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="50" t="inlineStr">
+      <c r="A24" s="66" t="inlineStr">
         <is>
           <t>Lambda</t>
         </is>
       </c>
-      <c r="B24" s="51" t="inlineStr">
+      <c r="B24" s="67" t="inlineStr">
         <is>
           <t>$500m GPU-backed facility from Macquarie</t>
         </is>
       </c>
-      <c r="C24" s="51" t="inlineStr">
+      <c r="C24" s="67" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D24" s="51" t="inlineStr">
+      <c r="D24" s="67" t="inlineStr">
         <is>
           <t>$0.5bn</t>
         </is>
       </c>
-      <c r="E24" s="51" t="inlineStr">
+      <c r="E24" s="67" t="inlineStr">
         <is>
           <t>Bank / GPU-backed loan</t>
         </is>
       </c>
-      <c r="F24" s="52" t="inlineStr">
+      <c r="F24" s="68" t="inlineStr">
         <is>
           <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="47" t="inlineStr">
+      <c r="A25" s="63" t="inlineStr">
         <is>
           <t>Nscale</t>
         </is>
       </c>
-      <c r="B25" s="48" t="inlineStr">
+      <c r="B25" s="64" t="inlineStr">
         <is>
           <t>$1.4bn term loan</t>
         </is>
       </c>
-      <c r="C25" s="48" t="inlineStr">
+      <c r="C25" s="64" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D25" s="48" t="inlineStr">
+      <c r="D25" s="64" t="inlineStr">
         <is>
           <t>$1.4bn</t>
         </is>
       </c>
-      <c r="E25" s="48" t="inlineStr">
+      <c r="E25" s="64" t="inlineStr">
         <is>
           <t>Bank loan</t>
         </is>
       </c>
-      <c r="F25" s="49" t="inlineStr">
+      <c r="F25" s="65" t="inlineStr">
         <is>
           <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="50" t="inlineStr">
+      <c r="A26" s="66" t="inlineStr">
         <is>
           <t>Fluidstack</t>
         </is>
       </c>
-      <c r="B26" s="51" t="inlineStr">
+      <c r="B26" s="67" t="inlineStr">
         <is>
           <t>Facility backed by ~$6.7bn Google-contracted revenue (Google lease backstop)</t>
         </is>
       </c>
-      <c r="C26" s="51" t="inlineStr">
+      <c r="C26" s="67" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D26" s="51" t="inlineStr">
+      <c r="D26" s="67" t="inlineStr">
         <is>
           <t>~$6.7bn</t>
         </is>
       </c>
-      <c r="E26" s="51" t="inlineStr">
+      <c r="E26" s="67" t="inlineStr">
         <is>
           <t>SPV / private credit</t>
         </is>
       </c>
-      <c r="F26" s="52" t="inlineStr">
+      <c r="F26" s="68" t="inlineStr">
         <is>
           <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="47" t="inlineStr">
+      <c r="A27" s="63" t="inlineStr">
         <is>
           <t>Applied Digital</t>
         </is>
       </c>
-      <c r="B27" s="48" t="inlineStr">
+      <c r="B27" s="64" t="inlineStr">
         <is>
           <t>$1.59bn high-yield bond (7%) for CoreWeave-leased campus (Polaris Forge 1)</t>
         </is>
       </c>
-      <c r="C27" s="48" t="inlineStr">
+      <c r="C27" s="64" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D27" s="48" t="inlineStr">
+      <c r="D27" s="64" t="inlineStr">
         <is>
           <t>$1.59bn</t>
         </is>
       </c>
-      <c r="E27" s="48" t="inlineStr">
+      <c r="E27" s="64" t="inlineStr">
         <is>
           <t>Securitization / HY bond</t>
         </is>
       </c>
-      <c r="F27" s="49" t="inlineStr">
+      <c r="F27" s="65" t="inlineStr">
         <is>
           <t>TNW</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="50" t="inlineStr">
+      <c r="A28" s="66" t="inlineStr">
+        <is>
+          <t>Aligned Data Centers</t>
+        </is>
+      </c>
+      <c r="B28" s="67" t="inlineStr">
+        <is>
+          <t>$12bn capital raise ($5bn+ new equity + $7bn debt commitments) led by Macquarie (early 2025); later acquired by MGX/BlackRock consortium (~$40bn)</t>
+        </is>
+      </c>
+      <c r="C28" s="67" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D28" s="67" t="inlineStr">
+        <is>
+          <t>$12bn / $40bn</t>
+        </is>
+      </c>
+      <c r="E28" s="67" t="inlineStr">
+        <is>
+          <t>Infra equity + debt</t>
+        </is>
+      </c>
+      <c r="F28" s="68" t="inlineStr">
+        <is>
+          <t>SFA; NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="63" t="inlineStr">
+        <is>
+          <t>QTS (Blackstone)</t>
+        </is>
+      </c>
+      <c r="B29" s="64" t="inlineStr">
+        <is>
+          <t>BX 2025-VOLT SASB CMBS $3.5bn (~10 QTS DCs); + Phoenix ABS (QTS Issuer 2025-1)</t>
+        </is>
+      </c>
+      <c r="C29" s="64" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D29" s="64" t="inlineStr">
+        <is>
+          <t>$3.5bn+</t>
+        </is>
+      </c>
+      <c r="E29" s="64" t="inlineStr">
+        <is>
+          <t>Securitization (CMBS/ABS)</t>
+        </is>
+      </c>
+      <c r="F29" s="65" t="inlineStr">
+        <is>
+          <t>CREFC; SFA</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="66" t="inlineStr">
+        <is>
+          <t>Switch (DigitalBridge)</t>
+        </is>
+      </c>
+      <c r="B30" s="67" t="inlineStr">
+        <is>
+          <t>$2.4bn SASB CMBS (SWCH 2025-DATA) + $1.1bn ABS — green bonds</t>
+        </is>
+      </c>
+      <c r="C30" s="67" t="inlineStr">
+        <is>
+          <t>2024-25</t>
+        </is>
+      </c>
+      <c r="D30" s="67" t="inlineStr">
+        <is>
+          <t>$3.5bn</t>
+        </is>
+      </c>
+      <c r="E30" s="67" t="inlineStr">
+        <is>
+          <t>Securitization (CMBS/ABS)</t>
+        </is>
+      </c>
+      <c r="F30" s="68" t="inlineStr">
+        <is>
+          <t>SFA; CREFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="63" t="inlineStr">
+        <is>
+          <t>Vantage Data Centers</t>
+        </is>
+      </c>
+      <c r="B31" s="64" t="inlineStr">
+        <is>
+          <t>First public data-center ABS (2024); ongoing multi-billion securitization &amp; infra-equity program</t>
+        </is>
+      </c>
+      <c r="C31" s="64" t="inlineStr">
+        <is>
+          <t>2024-26</t>
+        </is>
+      </c>
+      <c r="D31" s="64" t="inlineStr">
+        <is>
+          <t>multi-$bn</t>
+        </is>
+      </c>
+      <c r="E31" s="64" t="inlineStr">
+        <is>
+          <t>Securitization / equity</t>
+        </is>
+      </c>
+      <c r="F31" s="65" t="inlineStr">
+        <is>
+          <t>Dentons</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="66" t="inlineStr">
+        <is>
+          <t>Colocation sector</t>
+        </is>
+      </c>
+      <c r="B32" s="67" t="inlineStr">
+        <is>
+          <t>US data-center ABS+CMBS issuance ~$26bn in 2025 (~10x 2020); ~$57bn since 2021; Morgan Stanley ~$130bn securitized net issuance 2026-28; ~$150bn permanent financing need 2026-27</t>
+        </is>
+      </c>
+      <c r="C32" s="67" t="inlineStr">
+        <is>
+          <t>2025-28</t>
+        </is>
+      </c>
+      <c r="D32" s="67" t="inlineStr">
+        <is>
+          <t>~$130bn</t>
+        </is>
+      </c>
+      <c r="E32" s="67" t="inlineStr">
+        <is>
+          <t>Securitization (ABS/CMBS)</t>
+        </is>
+      </c>
+      <c r="F32" s="68" t="inlineStr">
+        <is>
+          <t>Impax; CREFC; Morgan Stanley</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="63" t="inlineStr">
+        <is>
+          <t>HUMAIN (Saudi PIF)</t>
+        </is>
+      </c>
+      <c r="B33" s="64" t="inlineStr">
+        <is>
+          <t>PIF national AI champion (announced 13 May 2025): ~$100bn across 11 data centers / 2.2 GW; ~600k NVIDIA GPUs; ALLAM Arabic LLM</t>
+        </is>
+      </c>
+      <c r="C33" s="64" t="inlineStr">
+        <is>
+          <t>2025-30</t>
+        </is>
+      </c>
+      <c r="D33" s="64" t="inlineStr">
+        <is>
+          <t>~$100bn</t>
+        </is>
+      </c>
+      <c r="E33" s="64" t="inlineStr">
+        <is>
+          <t>Sovereign equity</t>
+        </is>
+      </c>
+      <c r="F33" s="65" t="inlineStr">
+        <is>
+          <t>Presenc AI; NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="66" t="inlineStr">
+        <is>
+          <t>Stargate UAE / G42</t>
+        </is>
+      </c>
+      <c r="B34" s="67" t="inlineStr">
+        <is>
+          <t>$30bn+ 5GW Abu Dhabi campus (Khazna/G42 w/ OpenAI, Oracle, NVIDIA, Cisco, SoftBank); Phase 1 200MW Q3 2026; Microsoft ~$1.5bn equity</t>
+        </is>
+      </c>
+      <c r="C34" s="67" t="inlineStr">
+        <is>
+          <t>2025-30</t>
+        </is>
+      </c>
+      <c r="D34" s="67" t="inlineStr">
+        <is>
+          <t>~$30bn+</t>
+        </is>
+      </c>
+      <c r="E34" s="67" t="inlineStr">
+        <is>
+          <t>Sovereign equity + JV</t>
+        </is>
+      </c>
+      <c r="F34" s="68" t="inlineStr">
+        <is>
+          <t>Khaleej Times; dcpulse</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="63" t="inlineStr">
+        <is>
+          <t>MGX / Mubadala (UAE)</t>
+        </is>
+      </c>
+      <c r="B35" s="64" t="inlineStr">
+        <is>
+          <t>Anchored Stargate; co-led ~$40bn Aligned Data Centers acquisition w/ BlackRock; AIP (BlackRock-Microsoft) targets up to $100bn global AI infra</t>
+        </is>
+      </c>
+      <c r="C35" s="64" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="D35" s="64" t="inlineStr">
+        <is>
+          <t>~$40bn+</t>
+        </is>
+      </c>
+      <c r="E35" s="64" t="inlineStr">
+        <is>
+          <t>Sovereign equity / infra</t>
+        </is>
+      </c>
+      <c r="F35" s="65" t="inlineStr">
+        <is>
+          <t>NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="66" t="inlineStr">
+        <is>
+          <t>Qatar (QIA / Qai)</t>
+        </is>
+      </c>
+      <c r="B36" s="67" t="inlineStr">
+        <is>
+          <t>~$20bn AI-infrastructure JV with Brookfield (late 2025); earlier positions in xAI &amp; Databricks</t>
+        </is>
+      </c>
+      <c r="C36" s="67" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D36" s="67" t="inlineStr">
+        <is>
+          <t>~$20bn</t>
+        </is>
+      </c>
+      <c r="E36" s="67" t="inlineStr">
+        <is>
+          <t>Sovereign equity + JV</t>
+        </is>
+      </c>
+      <c r="F36" s="68" t="inlineStr">
+        <is>
+          <t>NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="63" t="inlineStr">
         <is>
           <t>Sector-wide</t>
         </is>
       </c>
-      <c r="B28" s="51" t="inlineStr">
+      <c r="B37" s="64" t="inlineStr">
         <is>
           <t>HY/unrated AI-infra issuers raised ~$107bn funded+committed debt by ~May 2026 ($68.7bn neoclouds / $38.7bn AI-native DCs)</t>
         </is>
       </c>
-      <c r="C28" s="51" t="inlineStr">
+      <c r="C37" s="64" t="inlineStr">
         <is>
           <t>to 2026</t>
         </is>
       </c>
-      <c r="D28" s="51" t="inlineStr">
+      <c r="D37" s="64" t="inlineStr">
         <is>
           <t>~$107bn</t>
         </is>
       </c>
-      <c r="E28" s="51" t="inlineStr">
+      <c r="E37" s="64" t="inlineStr">
         <is>
           <t>All debt</t>
         </is>
       </c>
-      <c r="F28" s="52" t="inlineStr">
+      <c r="F37" s="65" t="inlineStr">
         <is>
           <t>Octus</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="47" t="inlineStr">
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="66" t="inlineStr">
         <is>
           <t>Sector-wide</t>
         </is>
       </c>
-      <c r="B29" s="48" t="inlineStr">
+      <c r="B38" s="67" t="inlineStr">
         <is>
           <t>Insurance-linked platforms deployed ~$180bn into private credit in 2025 (~25% of global private credit AUM)</t>
         </is>
       </c>
-      <c r="C29" s="48" t="inlineStr">
+      <c r="C38" s="67" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D29" s="48" t="inlineStr">
+      <c r="D38" s="67" t="inlineStr">
         <is>
           <t>~$180bn</t>
         </is>
       </c>
-      <c r="E29" s="48" t="inlineStr">
+      <c r="E38" s="67" t="inlineStr">
         <is>
           <t>Insurance / private credit</t>
         </is>
       </c>
-      <c r="F29" s="49" t="inlineStr">
+      <c r="F38" s="68" t="inlineStr">
         <is>
           <t>McKinsey; ABF Journal</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="50" t="inlineStr">
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="63" t="inlineStr">
         <is>
           <t>Sector-wide</t>
         </is>
       </c>
-      <c r="B30" s="51" t="inlineStr">
+      <c r="B39" s="64" t="inlineStr">
         <is>
           <t>Goldman Sachs: ~$5.3tn AI + data-center capex 2025-2030; Morgan Stanley: ~$800bn private credit for AI DCs 2025-28</t>
         </is>
       </c>
-      <c r="C30" s="51" t="inlineStr">
+      <c r="C39" s="64" t="inlineStr">
         <is>
           <t>2025-30</t>
         </is>
       </c>
-      <c r="D30" s="51" t="inlineStr">
+      <c r="D39" s="64" t="inlineStr">
         <is>
           <t>$5.3tn capex</t>
         </is>
       </c>
-      <c r="E30" s="51" t="inlineStr">
+      <c r="E39" s="64" t="inlineStr">
         <is>
           <t>Context</t>
         </is>
       </c>
-      <c r="F30" s="52" t="inlineStr">
+      <c r="F39" s="65" t="inlineStr">
         <is>
           <t>Goldman; Morgan Stanley</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="53" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="69" t="inlineStr">
         <is>
           <t>Selected sources:</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="54" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="70" t="inlineStr">
         <is>
           <t>Goldman Sachs Research — ~$5.3tn AI + data-center capex 2025-2030; private markets in DC financing.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="54" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="70" t="inlineStr">
         <is>
           <t>Morgan Stanley — ~$2tn capex 2025-28 with &gt;$1tn debt; ~$800bn private credit for AI DCs.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="54" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="70" t="inlineStr">
         <is>
           <t>Bank of America / BofA Securities — hyperscaler bond issuance ($121bn 2025; ~$175bn 2026E).</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="54" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="70" t="inlineStr">
         <is>
           <t>Moody's Ratings — hyperscaler capex (~$785bn 2026, ~$1tn 2027); $662bn off-B/S DC leases.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="54" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="70" t="inlineStr">
         <is>
           <t>McKinsey — ~$2.7tn US (5.2tn global) data-center capex by 2030; insurance-linked private credit.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="54" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="70" t="inlineStr">
         <is>
           <t>Octus — HY/unrated AI-infra debt (~$107bn to ~May 2026); ~14GW unfunded ≈ $344bn need.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="54" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="70" t="inlineStr">
         <is>
           <t>Company disclosures &amp; press: Meta IR / FT / S&amp;P (Hyperion); Oracle IR / IFR / Reuters; CoreWeave IR;</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="54" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="70" t="inlineStr">
         <is>
           <t xml:space="preserve">  CNBC / WSJ / The Information (xAI); Blackstone; Apollo Academy; MUFG; CreditSights; CNA.</t>
         </is>

</xml_diff>

<commit_message>
List all companies separately in Capex Projections tab (grouped by segment)
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AI_Infrastructure_Financing_2025-2030.xlsx
+++ b/AI_Infrastructure_Financing_2025-2030.xlsx
@@ -239,7 +239,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -397,7 +397,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="25" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -726,7 +725,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Annual AI-Infrastructure Capex by Company ($bn)</a:t>
+              <a:t>Annual AI-Infrastructure Capex by Segment ($bn)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -741,7 +740,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Capex Projections'!A5</f>
+              <f>'Capex Projections'!$A$11</f>
             </strRef>
           </tx>
           <spPr>
@@ -751,12 +750,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Capex Projections'!$B$4:$G$4</f>
+              <f>'Capex Projections'!$C$4:$H$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Capex Projections'!$B$5:$G$5</f>
+              <f>'Capex Projections'!$C$11:$H$11</f>
             </numRef>
           </val>
         </ser>
@@ -765,7 +764,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Capex Projections'!A6</f>
+              <f>'Capex Projections'!$A$22</f>
             </strRef>
           </tx>
           <spPr>
@@ -775,12 +774,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Capex Projections'!$B$4:$G$4</f>
+              <f>'Capex Projections'!$C$4:$H$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Capex Projections'!$B$6:$G$6</f>
+              <f>'Capex Projections'!$C$22:$H$22</f>
             </numRef>
           </val>
         </ser>
@@ -789,7 +788,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Capex Projections'!A7</f>
+              <f>'Capex Projections'!$A$33</f>
             </strRef>
           </tx>
           <spPr>
@@ -799,12 +798,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Capex Projections'!$B$4:$G$4</f>
+              <f>'Capex Projections'!$C$4:$H$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Capex Projections'!$B$7:$G$7</f>
+              <f>'Capex Projections'!$C$33:$H$33</f>
             </numRef>
           </val>
         </ser>
@@ -813,7 +812,7 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Capex Projections'!A8</f>
+              <f>'Capex Projections'!$A$42</f>
             </strRef>
           </tx>
           <spPr>
@@ -823,108 +822,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Capex Projections'!$B$4:$G$4</f>
+              <f>'Capex Projections'!$C$4:$H$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Capex Projections'!$B$8:$G$8</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="4"/>
-          <order val="4"/>
-          <tx>
-            <strRef>
-              <f>'Capex Projections'!A9</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Capex Projections'!$B$4:$G$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Capex Projections'!$B$9:$G$9</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="5"/>
-          <order val="5"/>
-          <tx>
-            <strRef>
-              <f>'Capex Projections'!A10</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Capex Projections'!$B$4:$G$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Capex Projections'!$B$10:$G$10</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="6"/>
-          <order val="6"/>
-          <tx>
-            <strRef>
-              <f>'Capex Projections'!A11</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Capex Projections'!$B$4:$G$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Capex Projections'!$B$11:$G$11</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="7"/>
-          <order val="7"/>
-          <tx>
-            <strRef>
-              <f>'Capex Projections'!A12</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Capex Projections'!$B$4:$G$4</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Capex Projections'!$B$12:$G$12</f>
+              <f>'Capex Projections'!$C$42:$H$42</f>
             </numRef>
           </val>
         </ser>
@@ -1040,7 +943,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>15</row>
+      <row>45</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="8640000" cy="3240000"/>
@@ -6804,17 +6707,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6839,35 +6743,40 @@
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>2028</t>
         </is>
       </c>
-      <c r="F4" s="12" t="inlineStr">
+      <c r="G4" s="12" t="inlineStr">
         <is>
           <t>2029</t>
         </is>
       </c>
-      <c r="G4" s="12" t="inlineStr">
+      <c r="H4" s="12" t="inlineStr">
         <is>
           <t>2030</t>
         </is>
       </c>
-      <c r="H4" s="12" t="inlineStr">
+      <c r="I4" s="12" t="inlineStr">
         <is>
           <t>Cumulative
 2025-30</t>
@@ -6875,33 +6784,19 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="B5" s="22" t="n">
-        <v>95</v>
-      </c>
-      <c r="C5" s="22" t="n">
-        <v>140</v>
-      </c>
-      <c r="D5" s="22" t="n">
-        <v>165</v>
-      </c>
-      <c r="E5" s="22" t="n">
-        <v>185</v>
-      </c>
-      <c r="F5" s="22" t="n">
-        <v>200</v>
-      </c>
-      <c r="G5" s="22" t="n">
-        <v>215</v>
-      </c>
-      <c r="H5" s="23">
-        <f>SUM(B5:G5)</f>
-        <v/>
-      </c>
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>HYPERSCALER</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n"/>
+      <c r="C5" s="15" t="n"/>
+      <c r="D5" s="15" t="n"/>
+      <c r="E5" s="15" t="n"/>
+      <c r="F5" s="15" t="n"/>
+      <c r="G5" s="15" t="n"/>
+      <c r="H5" s="15" t="n"/>
+      <c r="I5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="18" t="inlineStr">
@@ -6909,26 +6804,31 @@
           <t>Amazon (AWS)</t>
         </is>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="C6" s="22" t="n">
+      <c r="D6" s="22" t="n">
         <v>200</v>
       </c>
-      <c r="D6" s="22" t="n">
+      <c r="E6" s="22" t="n">
         <v>225</v>
       </c>
-      <c r="E6" s="22" t="n">
+      <c r="F6" s="22" t="n">
         <v>240</v>
       </c>
-      <c r="F6" s="22" t="n">
+      <c r="G6" s="22" t="n">
         <v>250</v>
       </c>
-      <c r="G6" s="22" t="n">
+      <c r="H6" s="22" t="n">
         <v>255</v>
       </c>
-      <c r="H6" s="23">
-        <f>SUM(B6:G6)</f>
+      <c r="I6" s="23">
+        <f>SUM(C6:H6)</f>
         <v/>
       </c>
     </row>
@@ -6938,206 +6838,1208 @@
           <t>Alphabet (Google)</t>
         </is>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="n">
         <v>91</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="D7" s="22" t="n">
         <v>180</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="E7" s="22" t="n">
         <v>200</v>
       </c>
-      <c r="E7" s="22" t="n">
+      <c r="F7" s="22" t="n">
         <v>215</v>
       </c>
-      <c r="F7" s="22" t="n">
+      <c r="G7" s="22" t="n">
         <v>230</v>
       </c>
-      <c r="G7" s="22" t="n">
+      <c r="H7" s="22" t="n">
         <v>245</v>
       </c>
-      <c r="H7" s="23">
-        <f>SUM(B7:G7)</f>
+      <c r="I7" s="23">
+        <f>SUM(C7:H7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="18" t="inlineStr">
         <is>
-          <t>Meta Platforms</t>
-        </is>
-      </c>
-      <c r="B8" s="22" t="n">
-        <v>72</v>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
       </c>
       <c r="C8" s="22" t="n">
-        <v>125</v>
+        <v>95</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="E8" s="22" t="n">
         <v>165</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>195</v>
-      </c>
-      <c r="H8" s="23">
-        <f>SUM(B8:G8)</f>
+        <v>200</v>
+      </c>
+      <c r="H8" s="22" t="n">
+        <v>215</v>
+      </c>
+      <c r="I8" s="23">
+        <f>SUM(C8:H8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="18" t="inlineStr">
         <is>
+          <t>Meta Platforms</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>72</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>125</v>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>150</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>165</v>
+      </c>
+      <c r="G9" s="22" t="n">
+        <v>180</v>
+      </c>
+      <c r="H9" s="22" t="n">
+        <v>195</v>
+      </c>
+      <c r="I9" s="23">
+        <f>SUM(C9:H9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
           <t>Oracle (OCI)</t>
         </is>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="D10" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="D9" s="22" t="n">
+      <c r="E10" s="22" t="n">
         <v>65</v>
       </c>
-      <c r="E9" s="22" t="n">
+      <c r="F10" s="22" t="n">
         <v>75</v>
       </c>
-      <c r="F9" s="22" t="n">
+      <c r="G10" s="22" t="n">
         <v>85</v>
       </c>
-      <c r="G9" s="22" t="n">
+      <c r="H10" s="22" t="n">
         <v>90</v>
       </c>
-      <c r="H9" s="23">
-        <f>SUM(B9:G9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="30" t="inlineStr">
-        <is>
-          <t>Neoclouds / AI-native (aggregate)</t>
-        </is>
-      </c>
-      <c r="B10" s="34" t="n">
-        <v>70</v>
-      </c>
-      <c r="C10" s="34" t="n">
-        <v>110</v>
-      </c>
-      <c r="D10" s="34" t="n">
-        <v>125</v>
-      </c>
-      <c r="E10" s="34" t="n">
-        <v>115</v>
-      </c>
-      <c r="F10" s="34" t="n">
-        <v>120</v>
-      </c>
-      <c r="G10" s="34" t="n">
-        <v>126</v>
-      </c>
-      <c r="H10" s="35">
-        <f>SUM(B10:G10)</f>
+      <c r="I10" s="23">
+        <f>SUM(C10:H10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="38" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REITs (aggregate)</t>
-        </is>
-      </c>
-      <c r="B11" s="42" t="n">
-        <v>55</v>
-      </c>
-      <c r="C11" s="42" t="n">
-        <v>70</v>
-      </c>
-      <c r="D11" s="42" t="n">
-        <v>80</v>
-      </c>
-      <c r="E11" s="42" t="n">
-        <v>85</v>
-      </c>
-      <c r="F11" s="42" t="n">
-        <v>85</v>
-      </c>
-      <c r="G11" s="42" t="n">
-        <v>85</v>
-      </c>
-      <c r="H11" s="43">
-        <f>SUM(B11:G11)</f>
+      <c r="A11" s="58" t="inlineStr">
+        <is>
+          <t>Hyperscaler subtotal</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="n"/>
+      <c r="C11" s="28">
+        <f>SUM(C6:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="28">
+        <f>SUM(D6:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="28">
+        <f>SUM(E6:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="28">
+        <f>SUM(F6:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="28">
+        <f>SUM(G6:G10)</f>
+        <v/>
+      </c>
+      <c r="H11" s="28">
+        <f>SUM(H6:H10)</f>
+        <v/>
+      </c>
+      <c r="I11" s="28">
+        <f>SUM(I6:I10)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="46" t="inlineStr">
-        <is>
-          <t>Sovereign clouds (aggregate)</t>
-        </is>
-      </c>
-      <c r="B12" s="50" t="n">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>NEOCLOUD / AI-NATIVE</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="15" t="n"/>
+      <c r="I12" s="15" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>SpaceX / xAI (Colossus)</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="C13" s="34" t="n">
+        <v>24</v>
+      </c>
+      <c r="D13" s="34" t="n">
+        <v>39</v>
+      </c>
+      <c r="E13" s="34" t="n">
+        <v>47</v>
+      </c>
+      <c r="F13" s="34" t="n">
+        <v>44</v>
+      </c>
+      <c r="G13" s="34" t="n">
+        <v>44</v>
+      </c>
+      <c r="H13" s="34" t="n">
+        <v>47</v>
+      </c>
+      <c r="I13" s="35">
+        <f>SUM(C13:H13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>CoreWeave</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="C14" s="34" t="n">
+        <v>14</v>
+      </c>
+      <c r="D14" s="34" t="n">
+        <v>23</v>
+      </c>
+      <c r="E14" s="34" t="n">
+        <v>28</v>
+      </c>
+      <c r="F14" s="34" t="n">
+        <v>26</v>
+      </c>
+      <c r="G14" s="34" t="n">
+        <v>26</v>
+      </c>
+      <c r="H14" s="34" t="n">
+        <v>28</v>
+      </c>
+      <c r="I14" s="35">
+        <f>SUM(C14:H14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>Other neoclouds &amp; AI-native DCs</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="C15" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="D15" s="34" t="n">
+        <v>13</v>
+      </c>
+      <c r="E15" s="34" t="n">
+        <v>15</v>
+      </c>
+      <c r="F15" s="34" t="n">
+        <v>15</v>
+      </c>
+      <c r="G15" s="34" t="n">
+        <v>14</v>
+      </c>
+      <c r="H15" s="34" t="n">
+        <v>15</v>
+      </c>
+      <c r="I15" s="35">
+        <f>SUM(C15:H15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="B16" s="31" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="C16" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="E16" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="F16" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="G16" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="H16" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="I16" s="35">
+        <f>SUM(C16:H16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>IREN</t>
+        </is>
+      </c>
+      <c r="B17" s="31" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="C17" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="F17" s="34" t="n">
+        <v>7</v>
+      </c>
+      <c r="G17" s="34" t="n">
+        <v>7</v>
+      </c>
+      <c r="H17" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="I17" s="35">
+        <f>SUM(C17:H17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>Crusoe</t>
+        </is>
+      </c>
+      <c r="B18" s="31" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="C18" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="E18" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="F18" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="G18" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="H18" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="I18" s="35">
+        <f>SUM(C18:H18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>Lambda</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="C19" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="H19" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="I19" s="35">
+        <f>SUM(C19:H19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>Fluidstack</t>
+        </is>
+      </c>
+      <c r="B20" s="31" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="C20" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="G20" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" s="35">
+        <f>SUM(C20:H20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>Nscale</t>
+        </is>
+      </c>
+      <c r="B21" s="31" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="C21" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="I21" s="35">
+        <f>SUM(C21:H21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="58" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native subtotal</t>
+        </is>
+      </c>
+      <c r="B22" s="27" t="n"/>
+      <c r="C22" s="28">
+        <f>SUM(C13:C21)</f>
+        <v/>
+      </c>
+      <c r="D22" s="28">
+        <f>SUM(D13:D21)</f>
+        <v/>
+      </c>
+      <c r="E22" s="28">
+        <f>SUM(E13:E21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="28">
+        <f>SUM(F13:F21)</f>
+        <v/>
+      </c>
+      <c r="G22" s="28">
+        <f>SUM(G13:G21)</f>
+        <v/>
+      </c>
+      <c r="H22" s="28">
+        <f>SUM(H13:H21)</f>
+        <v/>
+      </c>
+      <c r="I22" s="28">
+        <f>SUM(I13:I21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>COLOCATION / DATA-CENTER REIT</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="15" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="38" t="inlineStr">
+        <is>
+          <t>Other colo &amp; powered-shell owners</t>
+        </is>
+      </c>
+      <c r="B24" s="39" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C24" s="42" t="n">
+        <v>10</v>
+      </c>
+      <c r="D24" s="42" t="n">
+        <v>13</v>
+      </c>
+      <c r="E24" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="F24" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="G24" s="42" t="n">
+        <v>16</v>
+      </c>
+      <c r="H24" s="42" t="n">
+        <v>16</v>
+      </c>
+      <c r="I24" s="43">
+        <f>SUM(C24:H24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="38" t="inlineStr">
+        <is>
+          <t>Equinix</t>
+        </is>
+      </c>
+      <c r="B25" s="39" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C25" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="D25" s="42" t="n">
+        <v>11</v>
+      </c>
+      <c r="E25" s="42" t="n">
+        <v>12</v>
+      </c>
+      <c r="F25" s="42" t="n">
+        <v>13</v>
+      </c>
+      <c r="G25" s="42" t="n">
+        <v>13</v>
+      </c>
+      <c r="H25" s="42" t="n">
+        <v>13</v>
+      </c>
+      <c r="I25" s="43">
+        <f>SUM(C25:H25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="38" t="inlineStr">
+        <is>
+          <t>Digital Realty</t>
+        </is>
+      </c>
+      <c r="B26" s="39" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C26" s="42" t="n">
+        <v>7</v>
+      </c>
+      <c r="D26" s="42" t="n">
+        <v>9</v>
+      </c>
+      <c r="E26" s="42" t="n">
+        <v>10</v>
+      </c>
+      <c r="F26" s="42" t="n">
+        <v>11</v>
+      </c>
+      <c r="G26" s="42" t="n">
+        <v>12</v>
+      </c>
+      <c r="H26" s="42" t="n">
+        <v>11</v>
+      </c>
+      <c r="I26" s="43">
+        <f>SUM(C26:H26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="38" t="inlineStr">
+        <is>
+          <t>QTS (Blackstone)</t>
+        </is>
+      </c>
+      <c r="B27" s="39" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C27" s="42" t="n">
+        <v>7</v>
+      </c>
+      <c r="D27" s="42" t="n">
+        <v>9</v>
+      </c>
+      <c r="E27" s="42" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" s="42" t="n">
+        <v>11</v>
+      </c>
+      <c r="G27" s="42" t="n">
+        <v>12</v>
+      </c>
+      <c r="H27" s="42" t="n">
+        <v>11</v>
+      </c>
+      <c r="I27" s="43">
+        <f>SUM(C27:H27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="38" t="inlineStr">
+        <is>
+          <t>Vantage Data Centers</t>
+        </is>
+      </c>
+      <c r="B28" s="39" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C28" s="42" t="n">
+        <v>6</v>
+      </c>
+      <c r="D28" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="E28" s="42" t="n">
+        <v>9</v>
+      </c>
+      <c r="F28" s="42" t="n">
+        <v>9</v>
+      </c>
+      <c r="G28" s="42" t="n">
+        <v>9</v>
+      </c>
+      <c r="H28" s="42" t="n">
+        <v>9</v>
+      </c>
+      <c r="I28" s="43">
+        <f>SUM(C28:H28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="38" t="inlineStr">
+        <is>
+          <t>Aligned Data Centers (MGX/BlackRock)</t>
+        </is>
+      </c>
+      <c r="B29" s="39" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C29" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="D29" s="42" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" s="42" t="n">
+        <v>7</v>
+      </c>
+      <c r="F29" s="42" t="n">
+        <v>7</v>
+      </c>
+      <c r="G29" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="H29" s="42" t="n">
+        <v>7</v>
+      </c>
+      <c r="I29" s="43">
+        <f>SUM(C29:H29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="38" t="inlineStr">
+        <is>
+          <t>CyrusOne (KKR/GIP)</t>
+        </is>
+      </c>
+      <c r="B30" s="39" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C30" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="D30" s="42" t="n">
+        <v>6</v>
+      </c>
+      <c r="E30" s="42" t="n">
+        <v>7</v>
+      </c>
+      <c r="F30" s="42" t="n">
+        <v>7</v>
+      </c>
+      <c r="G30" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="H30" s="42" t="n">
+        <v>7</v>
+      </c>
+      <c r="I30" s="43">
+        <f>SUM(C30:H30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="38" t="inlineStr">
+        <is>
+          <t>Switch (DigitalBridge)</t>
+        </is>
+      </c>
+      <c r="B31" s="39" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C31" s="42" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" s="42" t="n">
+        <v>4</v>
+      </c>
+      <c r="E31" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="F31" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="G31" s="42" t="n">
+        <v>6</v>
+      </c>
+      <c r="H31" s="42" t="n">
+        <v>6</v>
+      </c>
+      <c r="I31" s="43">
+        <f>SUM(C31:H31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="38" t="inlineStr">
+        <is>
+          <t>Stack Infrastructure</t>
+        </is>
+      </c>
+      <c r="B32" s="39" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="C32" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" s="42" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" s="42" t="n">
+        <v>4</v>
+      </c>
+      <c r="F32" s="42" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="H32" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="I32" s="43">
+        <f>SUM(C32:H32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="58" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT subtotal</t>
+        </is>
+      </c>
+      <c r="B33" s="27" t="n"/>
+      <c r="C33" s="28">
+        <f>SUM(C24:C32)</f>
+        <v/>
+      </c>
+      <c r="D33" s="28">
+        <f>SUM(D24:D32)</f>
+        <v/>
+      </c>
+      <c r="E33" s="28">
+        <f>SUM(E24:E32)</f>
+        <v/>
+      </c>
+      <c r="F33" s="28">
+        <f>SUM(F24:F32)</f>
+        <v/>
+      </c>
+      <c r="G33" s="28">
+        <f>SUM(G24:G32)</f>
+        <v/>
+      </c>
+      <c r="H33" s="28">
+        <f>SUM(H24:H32)</f>
+        <v/>
+      </c>
+      <c r="I33" s="28">
+        <f>SUM(I24:I32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>SOVEREIGN CLOUD</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="n"/>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="15" t="n"/>
+      <c r="F34" s="15" t="n"/>
+      <c r="G34" s="15" t="n"/>
+      <c r="H34" s="15" t="n"/>
+      <c r="I34" s="15" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="46" t="inlineStr">
+        <is>
+          <t>HUMAIN (Saudi PIF)</t>
+        </is>
+      </c>
+      <c r="B35" s="47" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C35" s="50" t="n">
+        <v>8</v>
+      </c>
+      <c r="D35" s="50" t="n">
+        <v>14</v>
+      </c>
+      <c r="E35" s="50" t="n">
+        <v>18</v>
+      </c>
+      <c r="F35" s="50" t="n">
         <v>20</v>
       </c>
-      <c r="C12" s="50" t="n">
-        <v>35</v>
-      </c>
-      <c r="D12" s="50" t="n">
-        <v>45</v>
-      </c>
-      <c r="E12" s="50" t="n">
-        <v>50</v>
-      </c>
-      <c r="F12" s="50" t="n">
-        <v>50</v>
-      </c>
-      <c r="G12" s="50" t="n">
-        <v>50</v>
-      </c>
-      <c r="H12" s="51">
-        <f>SUM(B12:G12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="69" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B13" s="56">
-        <f>SUM(B5:B12)</f>
-        <v/>
-      </c>
-      <c r="C13" s="56">
-        <f>SUM(C5:C12)</f>
-        <v/>
-      </c>
-      <c r="D13" s="56">
-        <f>SUM(D5:D12)</f>
-        <v/>
-      </c>
-      <c r="E13" s="56">
-        <f>SUM(E5:E12)</f>
-        <v/>
-      </c>
-      <c r="F13" s="56">
-        <f>SUM(F5:F12)</f>
-        <v/>
-      </c>
-      <c r="G13" s="56">
-        <f>SUM(G5:G12)</f>
-        <v/>
-      </c>
-      <c r="H13" s="56">
-        <f>SUM(H5:H12)</f>
+      <c r="G35" s="50" t="n">
+        <v>20</v>
+      </c>
+      <c r="H35" s="50" t="n">
+        <v>20</v>
+      </c>
+      <c r="I35" s="51">
+        <f>SUM(C35:H35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="46" t="inlineStr">
+        <is>
+          <t>MGX / Mubadala (UAE)</t>
+        </is>
+      </c>
+      <c r="B36" s="47" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C36" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" s="50" t="n">
+        <v>6</v>
+      </c>
+      <c r="E36" s="50" t="n">
+        <v>7</v>
+      </c>
+      <c r="F36" s="50" t="n">
+        <v>8</v>
+      </c>
+      <c r="G36" s="50" t="n">
+        <v>8</v>
+      </c>
+      <c r="H36" s="50" t="n">
+        <v>8</v>
+      </c>
+      <c r="I36" s="51">
+        <f>SUM(C36:H36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="46" t="inlineStr">
+        <is>
+          <t>Other sovereign AI (Japan, Korea, Singapore, etc.)</t>
+        </is>
+      </c>
+      <c r="B37" s="47" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C37" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" s="50" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" s="50" t="n">
+        <v>6</v>
+      </c>
+      <c r="F37" s="50" t="n">
+        <v>7</v>
+      </c>
+      <c r="G37" s="50" t="n">
+        <v>6</v>
+      </c>
+      <c r="H37" s="50" t="n">
+        <v>6</v>
+      </c>
+      <c r="I37" s="51">
+        <f>SUM(C37:H37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="46" t="inlineStr">
+        <is>
+          <t>Stargate UAE / G42 / Khazna</t>
+        </is>
+      </c>
+      <c r="B38" s="47" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C38" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="E38" s="50" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" s="50" t="n">
+        <v>6</v>
+      </c>
+      <c r="G38" s="50" t="n">
+        <v>6</v>
+      </c>
+      <c r="H38" s="50" t="n">
+        <v>6</v>
+      </c>
+      <c r="I38" s="51">
+        <f>SUM(C38:H38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="46" t="inlineStr">
+        <is>
+          <t>Qatar (QIA / Qai + Brookfield JV)</t>
+        </is>
+      </c>
+      <c r="B39" s="47" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C39" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="F39" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="G39" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="H39" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="I39" s="51">
+        <f>SUM(C39:H39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="46" t="inlineStr">
+        <is>
+          <t>EU / France (Mistral, sovereign cloud)</t>
+        </is>
+      </c>
+      <c r="B40" s="47" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C40" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="G40" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="H40" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="I40" s="51">
+        <f>SUM(C40:H40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="46" t="inlineStr">
+        <is>
+          <t>India (IndiaAI Mission)</t>
+        </is>
+      </c>
+      <c r="B41" s="47" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="C41" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="G41" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="H41" s="50" t="n">
+        <v>2</v>
+      </c>
+      <c r="I41" s="51">
+        <f>SUM(C41:H41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="58" t="inlineStr">
+        <is>
+          <t>Sovereign cloud subtotal</t>
+        </is>
+      </c>
+      <c r="B42" s="27" t="n"/>
+      <c r="C42" s="28">
+        <f>SUM(C35:C41)</f>
+        <v/>
+      </c>
+      <c r="D42" s="28">
+        <f>SUM(D35:D41)</f>
+        <v/>
+      </c>
+      <c r="E42" s="28">
+        <f>SUM(E35:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="28">
+        <f>SUM(F35:F41)</f>
+        <v/>
+      </c>
+      <c r="G42" s="28">
+        <f>SUM(G35:G41)</f>
+        <v/>
+      </c>
+      <c r="H42" s="28">
+        <f>SUM(H35:H41)</f>
+        <v/>
+      </c>
+      <c r="I42" s="28">
+        <f>SUM(I35:I41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="54" t="inlineStr">
+        <is>
+          <t>TOTAL — all companies</t>
+        </is>
+      </c>
+      <c r="B43" s="55" t="n"/>
+      <c r="C43" s="56">
+        <f>SUM(C6,C7,C8,C9,C10,C13,C14,C15,C16,C17,C18,C19,C20,C21,C24,C25,C26,C27,C28,C29,C30,C31,C32,C35,C36,C37,C38,C39,C40,C41)</f>
+        <v/>
+      </c>
+      <c r="D43" s="56">
+        <f>SUM(D6,D7,D8,D9,D10,D13,D14,D15,D16,D17,D18,D19,D20,D21,D24,D25,D26,D27,D28,D29,D30,D31,D32,D35,D36,D37,D38,D39,D40,D41)</f>
+        <v/>
+      </c>
+      <c r="E43" s="56">
+        <f>SUM(E6,E7,E8,E9,E10,E13,E14,E15,E16,E17,E18,E19,E20,E21,E24,E25,E26,E27,E28,E29,E30,E31,E32,E35,E36,E37,E38,E39,E40,E41)</f>
+        <v/>
+      </c>
+      <c r="F43" s="56">
+        <f>SUM(F6,F7,F8,F9,F10,F13,F14,F15,F16,F17,F18,F19,F20,F21,F24,F25,F26,F27,F28,F29,F30,F31,F32,F35,F36,F37,F38,F39,F40,F41)</f>
+        <v/>
+      </c>
+      <c r="G43" s="56">
+        <f>SUM(G6,G7,G8,G9,G10,G13,G14,G15,G16,G17,G18,G19,G20,G21,G24,G25,G26,G27,G28,G29,G30,G31,G32,G35,G36,G37,G38,G39,G40,G41)</f>
+        <v/>
+      </c>
+      <c r="H43" s="56">
+        <f>SUM(H6,H7,H8,H9,H10,H13,H14,H15,H16,H17,H18,H19,H20,H21,H24,H25,H26,H27,H28,H29,H30,H31,H32,H35,H36,H37,H38,H39,H40,H41)</f>
+        <v/>
+      </c>
+      <c r="I43" s="56">
+        <f>SUM(I6,I7,I8,I9,I10,I13,I14,I15,I16,I17,I18,I19,I20,I21,I24,I25,I26,I27,I28,I29,I30,I31,I32,I35,I36,I37,I38,I39,I40,I41)</f>
         <v/>
       </c>
     </row>
@@ -7211,1183 +8113,1183 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="70" t="inlineStr">
+      <c r="A5" s="69" t="inlineStr">
         <is>
           <t>Meta Platforms</t>
         </is>
       </c>
-      <c r="B5" s="71" t="inlineStr">
+      <c r="B5" s="70" t="inlineStr">
         <is>
           <t>Hyperion JV (Beignet Investor LLC) — Blue Owl 80% / Meta 20%; $27.3bn A+ private bond led by PIMCO (~$18bn) &amp; BlackRock; off-B/S SPV w/ residual-value guarantee</t>
         </is>
       </c>
-      <c r="C5" s="71" t="inlineStr">
+      <c r="C5" s="70" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D5" s="71" t="inlineStr">
+      <c r="D5" s="70" t="inlineStr">
         <is>
           <t>$27.3bn debt</t>
         </is>
       </c>
-      <c r="E5" s="71" t="inlineStr">
+      <c r="E5" s="70" t="inlineStr">
         <is>
           <t>SPV / private credit / insurance</t>
         </is>
       </c>
-      <c r="F5" s="72" t="inlineStr">
+      <c r="F5" s="71" t="inlineStr">
         <is>
           <t>Meta IR; FT; S&amp;P</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="73" t="inlineStr">
+      <c r="A6" s="72" t="inlineStr">
         <is>
           <t>Meta Platforms</t>
         </is>
       </c>
-      <c r="B6" s="74" t="inlineStr">
+      <c r="B6" s="73" t="inlineStr">
         <is>
           <t>$30bn multi-tranche IG corporate bond (largest 2025 IG deal), maturities to 2063</t>
         </is>
       </c>
-      <c r="C6" s="74" t="inlineStr">
+      <c r="C6" s="73" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D6" s="74" t="inlineStr">
+      <c r="D6" s="73" t="inlineStr">
         <is>
           <t>$30bn</t>
         </is>
       </c>
-      <c r="E6" s="74" t="inlineStr">
+      <c r="E6" s="73" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F6" s="75" t="inlineStr">
+      <c r="F6" s="74" t="inlineStr">
         <is>
           <t>BofA; MUFG</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="70" t="inlineStr">
+      <c r="A7" s="69" t="inlineStr">
         <is>
           <t>Amazon (AWS)</t>
         </is>
       </c>
-      <c r="B7" s="71" t="inlineStr">
+      <c r="B7" s="70" t="inlineStr">
         <is>
           <t>~$54bn USD + €14.5bn (~$16.8bn) IG bonds (near-record), ~4x oversubscribed</t>
         </is>
       </c>
-      <c r="C7" s="71" t="inlineStr">
+      <c r="C7" s="70" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D7" s="71" t="inlineStr">
+      <c r="D7" s="70" t="inlineStr">
         <is>
           <t>~$71bn</t>
         </is>
       </c>
-      <c r="E7" s="71" t="inlineStr">
+      <c r="E7" s="70" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F7" s="72" t="inlineStr">
+      <c r="F7" s="71" t="inlineStr">
         <is>
           <t>CNA; Reuters</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="73" t="inlineStr">
+      <c r="A8" s="72" t="inlineStr">
         <is>
           <t>Amazon (AWS)</t>
         </is>
       </c>
-      <c r="B8" s="74" t="inlineStr">
+      <c r="B8" s="73" t="inlineStr">
         <is>
           <t>$15bn IG bond</t>
         </is>
       </c>
-      <c r="C8" s="74" t="inlineStr">
+      <c r="C8" s="73" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D8" s="74" t="inlineStr">
+      <c r="D8" s="73" t="inlineStr">
         <is>
           <t>$15bn</t>
         </is>
       </c>
-      <c r="E8" s="74" t="inlineStr">
+      <c r="E8" s="73" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F8" s="75" t="inlineStr">
+      <c r="F8" s="74" t="inlineStr">
         <is>
           <t>CNA</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="70" t="inlineStr">
+      <c r="A9" s="69" t="inlineStr">
         <is>
           <t>Alphabet (Google)</t>
         </is>
       </c>
-      <c r="B9" s="71" t="inlineStr">
+      <c r="B9" s="70" t="inlineStr">
         <is>
           <t>~$32bn multi-currency bond incl. rare 100-yr tranche; plus $17.5bn Nov 2025</t>
         </is>
       </c>
-      <c r="C9" s="71" t="inlineStr">
+      <c r="C9" s="70" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D9" s="71" t="inlineStr">
+      <c r="D9" s="70" t="inlineStr">
         <is>
           <t>~$50bn</t>
         </is>
       </c>
-      <c r="E9" s="71" t="inlineStr">
+      <c r="E9" s="70" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F9" s="72" t="inlineStr">
+      <c r="F9" s="71" t="inlineStr">
         <is>
           <t>ConstructConnect; CNA</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="73" t="inlineStr">
+      <c r="A10" s="72" t="inlineStr">
         <is>
           <t>Oracle (OCI)</t>
         </is>
       </c>
-      <c r="B10" s="74" t="inlineStr">
+      <c r="B10" s="73" t="inlineStr">
         <is>
           <t>$25bn 8-part IG bond (Feb 2026) within $45-50bn CY26 debt+equity plan; $20bn ATM + mandatory convertible preferred (equity)</t>
         </is>
       </c>
-      <c r="C10" s="74" t="inlineStr">
+      <c r="C10" s="73" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D10" s="74" t="inlineStr">
+      <c r="D10" s="73" t="inlineStr">
         <is>
           <t>$25bn debt</t>
         </is>
       </c>
-      <c r="E10" s="74" t="inlineStr">
+      <c r="E10" s="73" t="inlineStr">
         <is>
           <t>Corporate bonds + equity</t>
         </is>
       </c>
-      <c r="F10" s="75" t="inlineStr">
+      <c r="F10" s="74" t="inlineStr">
         <is>
           <t>Oracle IR; IFR</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="70" t="inlineStr">
+      <c r="A11" s="69" t="inlineStr">
         <is>
           <t>Oracle (OCI)</t>
         </is>
       </c>
-      <c r="B11" s="71" t="inlineStr">
+      <c r="B11" s="70" t="inlineStr">
         <is>
           <t>$18bn 6-part IG bond (Sep 2025)</t>
         </is>
       </c>
-      <c r="C11" s="71" t="inlineStr">
+      <c r="C11" s="70" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D11" s="71" t="inlineStr">
+      <c r="D11" s="70" t="inlineStr">
         <is>
           <t>$18bn</t>
         </is>
       </c>
-      <c r="E11" s="71" t="inlineStr">
+      <c r="E11" s="70" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F11" s="72" t="inlineStr">
+      <c r="F11" s="71" t="inlineStr">
         <is>
           <t>Reuters/CNA</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="73" t="inlineStr">
+      <c r="A12" s="72" t="inlineStr">
         <is>
           <t>Oracle (OCI)</t>
         </is>
       </c>
-      <c r="B12" s="74" t="inlineStr">
+      <c r="B12" s="73" t="inlineStr">
         <is>
           <t>Project-level SPV financing: ~$16.3bn Michigan campus; further Texas / Wisconsin deals</t>
         </is>
       </c>
-      <c r="C12" s="74" t="inlineStr">
+      <c r="C12" s="73" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D12" s="74" t="inlineStr">
+      <c r="D12" s="73" t="inlineStr">
         <is>
           <t>~$25bn+</t>
         </is>
       </c>
-      <c r="E12" s="74" t="inlineStr">
+      <c r="E12" s="73" t="inlineStr">
         <is>
           <t>SPV / project finance</t>
         </is>
       </c>
-      <c r="F12" s="75" t="inlineStr">
+      <c r="F12" s="74" t="inlineStr">
         <is>
           <t>Press reports</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="70" t="inlineStr">
+      <c r="A13" s="69" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="B13" s="71" t="inlineStr">
+      <c r="B13" s="70" t="inlineStr">
         <is>
           <t>Finance-lease driven build (~$108bn uncommenced finance leases as of 9/30/24; commence FY25-FY30)</t>
         </is>
       </c>
-      <c r="C13" s="71" t="inlineStr">
+      <c r="C13" s="70" t="inlineStr">
         <is>
           <t>2024-30</t>
         </is>
       </c>
-      <c r="D13" s="71" t="inlineStr">
+      <c r="D13" s="70" t="inlineStr">
         <is>
           <t>$100bn+ leases</t>
         </is>
       </c>
-      <c r="E13" s="71" t="inlineStr">
+      <c r="E13" s="70" t="inlineStr">
         <is>
           <t>Vendor / lease / SPV</t>
         </is>
       </c>
-      <c r="F13" s="72" t="inlineStr">
+      <c r="F13" s="71" t="inlineStr">
         <is>
           <t>MSFT 10-Q; CNBC</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="73" t="inlineStr">
+      <c r="A14" s="72" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="B14" s="74" t="inlineStr">
+      <c r="B14" s="73" t="inlineStr">
         <is>
           <t>DDTL 4.0 — $8.5bn delayed-draw term loan; first IG-rated (Moody's A3 / DBRS A-low) GPU-backed financing; SOFR+225 / ~5.9%</t>
         </is>
       </c>
-      <c r="C14" s="74" t="inlineStr">
+      <c r="C14" s="73" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D14" s="74" t="inlineStr">
+      <c r="D14" s="73" t="inlineStr">
         <is>
           <t>$8.5bn</t>
         </is>
       </c>
-      <c r="E14" s="74" t="inlineStr">
+      <c r="E14" s="73" t="inlineStr">
         <is>
           <t>Bank / GPU-backed loan</t>
         </is>
       </c>
-      <c r="F14" s="75" t="inlineStr">
+      <c r="F14" s="74" t="inlineStr">
         <is>
           <t>CoreWeave IR</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="70" t="inlineStr">
+      <c r="A15" s="69" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="B15" s="71" t="inlineStr">
+      <c r="B15" s="70" t="inlineStr">
         <is>
           <t>$7.5bn debt facility led by Blackstone &amp; Magnetar (largest private debt deal at the time)</t>
         </is>
       </c>
-      <c r="C15" s="71" t="inlineStr">
+      <c r="C15" s="70" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D15" s="71" t="inlineStr">
+      <c r="D15" s="70" t="inlineStr">
         <is>
           <t>$7.5bn</t>
         </is>
       </c>
-      <c r="E15" s="71" t="inlineStr">
+      <c r="E15" s="70" t="inlineStr">
         <is>
           <t>Private credit / loan</t>
         </is>
       </c>
-      <c r="F15" s="72" t="inlineStr">
+      <c r="F15" s="71" t="inlineStr">
         <is>
           <t>Blackstone</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="73" t="inlineStr">
+      <c r="A16" s="72" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="B16" s="74" t="inlineStr">
+      <c r="B16" s="73" t="inlineStr">
         <is>
           <t>$2.7bn 1.75% convertible notes; ~$30bn total debt by early 2026; ~$28bn debt+equity raised in 12 mos</t>
         </is>
       </c>
-      <c r="C16" s="74" t="inlineStr">
+      <c r="C16" s="73" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D16" s="74" t="inlineStr">
+      <c r="D16" s="73" t="inlineStr">
         <is>
           <t>$2.7bn conv.</t>
         </is>
       </c>
-      <c r="E16" s="74" t="inlineStr">
+      <c r="E16" s="73" t="inlineStr">
         <is>
           <t>Convertibles</t>
         </is>
       </c>
-      <c r="F16" s="75" t="inlineStr">
+      <c r="F16" s="74" t="inlineStr">
         <is>
           <t>thedig; CoreWeave</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="70" t="inlineStr">
+      <c r="A17" s="69" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="B17" s="71" t="inlineStr">
+      <c r="B17" s="70" t="inlineStr">
         <is>
           <t>$2bn strategic equity from NVIDIA; IPO Mar 2025 raised ~$1.5bn</t>
         </is>
       </c>
-      <c r="C17" s="71" t="inlineStr">
+      <c r="C17" s="70" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D17" s="71" t="inlineStr">
+      <c r="D17" s="70" t="inlineStr">
         <is>
           <t>$3.5bn equity</t>
         </is>
       </c>
-      <c r="E17" s="71" t="inlineStr">
+      <c r="E17" s="70" t="inlineStr">
         <is>
           <t>Equity</t>
         </is>
       </c>
-      <c r="F17" s="72" t="inlineStr">
+      <c r="F17" s="71" t="inlineStr">
         <is>
           <t>CNBC; CoreWeave</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="73" t="inlineStr">
+      <c r="A18" s="72" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B18" s="74" t="inlineStr">
+      <c r="B18" s="73" t="inlineStr">
         <is>
           <t>SpaceX acquired xAI effective Feb 2, 2026; Colossus I &amp; II now SpaceX-owned (vertically-integrated AI platform; Terafab chip JV w/ Tesla &amp; Intel)</t>
         </is>
       </c>
-      <c r="C18" s="74" t="inlineStr">
+      <c r="C18" s="73" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D18" s="74" t="inlineStr">
+      <c r="D18" s="73" t="inlineStr">
         <is>
           <t>merger</t>
         </is>
       </c>
-      <c r="E18" s="74" t="inlineStr">
+      <c r="E18" s="73" t="inlineStr">
         <is>
           <t>Equity / M&amp;A</t>
         </is>
       </c>
-      <c r="F18" s="75" t="inlineStr">
+      <c r="F18" s="74" t="inlineStr">
         <is>
           <t>SpaceX S-1</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="70" t="inlineStr">
+      <c r="A19" s="69" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B19" s="71" t="inlineStr">
+      <c r="B19" s="70" t="inlineStr">
         <is>
           <t>SpaceX AI capex $12.7bn in 2025 (~61% of total) + $7.7bn in Q1 2026; AI buildout funded by Starlink FCF, private raises, planned IPO</t>
         </is>
       </c>
-      <c r="C19" s="71" t="inlineStr">
+      <c r="C19" s="70" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D19" s="71" t="inlineStr">
+      <c r="D19" s="70" t="inlineStr">
         <is>
           <t>$20bn+ capex</t>
         </is>
       </c>
-      <c r="E19" s="71" t="inlineStr">
+      <c r="E19" s="70" t="inlineStr">
         <is>
           <t>Internal / equity</t>
         </is>
       </c>
-      <c r="F19" s="72" t="inlineStr">
+      <c r="F19" s="71" t="inlineStr">
         <is>
           <t>SpaceX S-1; The Verge</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="73" t="inlineStr">
+      <c r="A20" s="72" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B20" s="74" t="inlineStr">
+      <c r="B20" s="73" t="inlineStr">
         <is>
           <t>Anthropic compute contract: $1.25bn/month (~$45bn) through May 2029 for Colossus I &amp; II — anchor revenue underwriting infra financing</t>
         </is>
       </c>
-      <c r="C20" s="74" t="inlineStr">
+      <c r="C20" s="73" t="inlineStr">
         <is>
           <t>2026-29</t>
         </is>
       </c>
-      <c r="D20" s="74" t="inlineStr">
+      <c r="D20" s="73" t="inlineStr">
         <is>
           <t>~$45bn</t>
         </is>
       </c>
-      <c r="E20" s="74" t="inlineStr">
+      <c r="E20" s="73" t="inlineStr">
         <is>
           <t>Take-or-pay (demand)</t>
         </is>
       </c>
-      <c r="F20" s="75" t="inlineStr">
+      <c r="F20" s="74" t="inlineStr">
         <is>
           <t>SpaceX S-1; The Verge</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="70" t="inlineStr">
+      <c r="A21" s="69" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B21" s="71" t="inlineStr">
+      <c r="B21" s="70" t="inlineStr">
         <is>
           <t>xAI $10bn raise ($5bn secured notes/term loans incl. Apollo $5bn facility + $5bn equity) via Morgan Stanley</t>
         </is>
       </c>
-      <c r="C21" s="71" t="inlineStr">
+      <c r="C21" s="70" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D21" s="71" t="inlineStr">
+      <c r="D21" s="70" t="inlineStr">
         <is>
           <t>$10bn</t>
         </is>
       </c>
-      <c r="E21" s="71" t="inlineStr">
+      <c r="E21" s="70" t="inlineStr">
         <is>
           <t>Loans + equity</t>
         </is>
       </c>
-      <c r="F21" s="72" t="inlineStr">
+      <c r="F21" s="71" t="inlineStr">
         <is>
           <t>CNBC</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="73" t="inlineStr">
+      <c r="A22" s="72" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B22" s="74" t="inlineStr">
+      <c r="B22" s="73" t="inlineStr">
         <is>
           <t>Colossus 2 SPV (Valor Equity): ~$12.5bn debt + ~$7.5bn equity (NVIDIA up to $2bn) to buy &amp; lease GPUs</t>
         </is>
       </c>
-      <c r="C22" s="74" t="inlineStr">
+      <c r="C22" s="73" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D22" s="74" t="inlineStr">
+      <c r="D22" s="73" t="inlineStr">
         <is>
           <t>~$20bn</t>
         </is>
       </c>
-      <c r="E22" s="74" t="inlineStr">
+      <c r="E22" s="73" t="inlineStr">
         <is>
           <t>SPV / vendor lease</t>
         </is>
       </c>
-      <c r="F22" s="75" t="inlineStr">
+      <c r="F22" s="74" t="inlineStr">
         <is>
           <t>The Information; Yahoo</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="70" t="inlineStr">
+      <c r="A23" s="69" t="inlineStr">
         <is>
           <t>Nebius</t>
         </is>
       </c>
-      <c r="B23" s="71" t="inlineStr">
+      <c r="B23" s="70" t="inlineStr">
         <is>
           <t>$3bn+ convertibles + bank lines; lighter balance sheet; Yandex spin-off cash ~$2.5bn; NVIDIA ~$2bn equity; Microsoft ~$7bn prepay</t>
         </is>
       </c>
-      <c r="C23" s="71" t="inlineStr">
+      <c r="C23" s="70" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D23" s="71" t="inlineStr">
+      <c r="D23" s="70" t="inlineStr">
         <is>
           <t>$3bn+</t>
         </is>
       </c>
-      <c r="E23" s="71" t="inlineStr">
+      <c r="E23" s="70" t="inlineStr">
         <is>
           <t>Convertibles</t>
         </is>
       </c>
-      <c r="F23" s="72" t="inlineStr">
+      <c r="F23" s="71" t="inlineStr">
         <is>
           <t>frankk research</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="73" t="inlineStr">
+      <c r="A24" s="72" t="inlineStr">
         <is>
           <t>Lambda</t>
         </is>
       </c>
-      <c r="B24" s="74" t="inlineStr">
+      <c r="B24" s="73" t="inlineStr">
         <is>
           <t>$500m GPU-backed facility from Macquarie</t>
         </is>
       </c>
-      <c r="C24" s="74" t="inlineStr">
+      <c r="C24" s="73" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D24" s="74" t="inlineStr">
+      <c r="D24" s="73" t="inlineStr">
         <is>
           <t>$0.5bn</t>
         </is>
       </c>
-      <c r="E24" s="74" t="inlineStr">
+      <c r="E24" s="73" t="inlineStr">
         <is>
           <t>Bank / GPU-backed loan</t>
         </is>
       </c>
-      <c r="F24" s="75" t="inlineStr">
+      <c r="F24" s="74" t="inlineStr">
         <is>
           <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="70" t="inlineStr">
+      <c r="A25" s="69" t="inlineStr">
         <is>
           <t>Nscale</t>
         </is>
       </c>
-      <c r="B25" s="71" t="inlineStr">
+      <c r="B25" s="70" t="inlineStr">
         <is>
           <t>$1.4bn term loan</t>
         </is>
       </c>
-      <c r="C25" s="71" t="inlineStr">
+      <c r="C25" s="70" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D25" s="71" t="inlineStr">
+      <c r="D25" s="70" t="inlineStr">
         <is>
           <t>$1.4bn</t>
         </is>
       </c>
-      <c r="E25" s="71" t="inlineStr">
+      <c r="E25" s="70" t="inlineStr">
         <is>
           <t>Bank loan</t>
         </is>
       </c>
-      <c r="F25" s="72" t="inlineStr">
+      <c r="F25" s="71" t="inlineStr">
         <is>
           <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="73" t="inlineStr">
+      <c r="A26" s="72" t="inlineStr">
         <is>
           <t>Fluidstack</t>
         </is>
       </c>
-      <c r="B26" s="74" t="inlineStr">
+      <c r="B26" s="73" t="inlineStr">
         <is>
           <t>Facility backed by ~$6.7bn Google-contracted revenue (Google lease backstop)</t>
         </is>
       </c>
-      <c r="C26" s="74" t="inlineStr">
+      <c r="C26" s="73" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D26" s="74" t="inlineStr">
+      <c r="D26" s="73" t="inlineStr">
         <is>
           <t>~$6.7bn</t>
         </is>
       </c>
-      <c r="E26" s="74" t="inlineStr">
+      <c r="E26" s="73" t="inlineStr">
         <is>
           <t>SPV / private credit</t>
         </is>
       </c>
-      <c r="F26" s="75" t="inlineStr">
+      <c r="F26" s="74" t="inlineStr">
         <is>
           <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="70" t="inlineStr">
+      <c r="A27" s="69" t="inlineStr">
         <is>
           <t>Applied Digital</t>
         </is>
       </c>
-      <c r="B27" s="71" t="inlineStr">
+      <c r="B27" s="70" t="inlineStr">
         <is>
           <t>$1.59bn high-yield bond (7%) for CoreWeave-leased campus (Polaris Forge 1)</t>
         </is>
       </c>
-      <c r="C27" s="71" t="inlineStr">
+      <c r="C27" s="70" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D27" s="71" t="inlineStr">
+      <c r="D27" s="70" t="inlineStr">
         <is>
           <t>$1.59bn</t>
         </is>
       </c>
-      <c r="E27" s="71" t="inlineStr">
+      <c r="E27" s="70" t="inlineStr">
         <is>
           <t>Securitization / HY bond</t>
         </is>
       </c>
-      <c r="F27" s="72" t="inlineStr">
+      <c r="F27" s="71" t="inlineStr">
         <is>
           <t>TNW</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="73" t="inlineStr">
+      <c r="A28" s="72" t="inlineStr">
         <is>
           <t>Aligned Data Centers</t>
         </is>
       </c>
-      <c r="B28" s="74" t="inlineStr">
+      <c r="B28" s="73" t="inlineStr">
         <is>
           <t>$12bn capital raise ($5bn+ new equity + $7bn debt commitments) led by Macquarie (early 2025); later acquired by MGX/BlackRock consortium (~$40bn)</t>
         </is>
       </c>
-      <c r="C28" s="74" t="inlineStr">
+      <c r="C28" s="73" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D28" s="74" t="inlineStr">
+      <c r="D28" s="73" t="inlineStr">
         <is>
           <t>$12bn / $40bn</t>
         </is>
       </c>
-      <c r="E28" s="74" t="inlineStr">
+      <c r="E28" s="73" t="inlineStr">
         <is>
           <t>Infra equity + debt</t>
         </is>
       </c>
-      <c r="F28" s="75" t="inlineStr">
+      <c r="F28" s="74" t="inlineStr">
         <is>
           <t>SFA; NYU DRI</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="70" t="inlineStr">
+      <c r="A29" s="69" t="inlineStr">
         <is>
           <t>QTS (Blackstone)</t>
         </is>
       </c>
-      <c r="B29" s="71" t="inlineStr">
+      <c r="B29" s="70" t="inlineStr">
         <is>
           <t>BX 2025-VOLT SASB CMBS $3.5bn (~10 QTS DCs); + Phoenix ABS (QTS Issuer 2025-1)</t>
         </is>
       </c>
-      <c r="C29" s="71" t="inlineStr">
+      <c r="C29" s="70" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D29" s="71" t="inlineStr">
+      <c r="D29" s="70" t="inlineStr">
         <is>
           <t>$3.5bn+</t>
         </is>
       </c>
-      <c r="E29" s="71" t="inlineStr">
+      <c r="E29" s="70" t="inlineStr">
         <is>
           <t>Securitization (CMBS/ABS)</t>
         </is>
       </c>
-      <c r="F29" s="72" t="inlineStr">
+      <c r="F29" s="71" t="inlineStr">
         <is>
           <t>CREFC; SFA</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="73" t="inlineStr">
+      <c r="A30" s="72" t="inlineStr">
         <is>
           <t>Switch (DigitalBridge)</t>
         </is>
       </c>
-      <c r="B30" s="74" t="inlineStr">
+      <c r="B30" s="73" t="inlineStr">
         <is>
           <t>$2.4bn SASB CMBS (SWCH 2025-DATA) + $1.1bn ABS — green bonds</t>
         </is>
       </c>
-      <c r="C30" s="74" t="inlineStr">
+      <c r="C30" s="73" t="inlineStr">
         <is>
           <t>2024-25</t>
         </is>
       </c>
-      <c r="D30" s="74" t="inlineStr">
+      <c r="D30" s="73" t="inlineStr">
         <is>
           <t>$3.5bn</t>
         </is>
       </c>
-      <c r="E30" s="74" t="inlineStr">
+      <c r="E30" s="73" t="inlineStr">
         <is>
           <t>Securitization (CMBS/ABS)</t>
         </is>
       </c>
-      <c r="F30" s="75" t="inlineStr">
+      <c r="F30" s="74" t="inlineStr">
         <is>
           <t>SFA; CREFC</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="70" t="inlineStr">
+      <c r="A31" s="69" t="inlineStr">
         <is>
           <t>Vantage Data Centers</t>
         </is>
       </c>
-      <c r="B31" s="71" t="inlineStr">
+      <c r="B31" s="70" t="inlineStr">
         <is>
           <t>First public data-center ABS (2024); ongoing multi-billion securitization &amp; infra-equity program</t>
         </is>
       </c>
-      <c r="C31" s="71" t="inlineStr">
+      <c r="C31" s="70" t="inlineStr">
         <is>
           <t>2024-26</t>
         </is>
       </c>
-      <c r="D31" s="71" t="inlineStr">
+      <c r="D31" s="70" t="inlineStr">
         <is>
           <t>multi-$bn</t>
         </is>
       </c>
-      <c r="E31" s="71" t="inlineStr">
+      <c r="E31" s="70" t="inlineStr">
         <is>
           <t>Securitization / equity</t>
         </is>
       </c>
-      <c r="F31" s="72" t="inlineStr">
+      <c r="F31" s="71" t="inlineStr">
         <is>
           <t>Dentons</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="73" t="inlineStr">
+      <c r="A32" s="72" t="inlineStr">
         <is>
           <t>Colocation sector</t>
         </is>
       </c>
-      <c r="B32" s="74" t="inlineStr">
+      <c r="B32" s="73" t="inlineStr">
         <is>
           <t>US data-center ABS+CMBS issuance ~$26bn in 2025 (~10x 2020); ~$57bn since 2021; Morgan Stanley ~$130bn securitized net issuance 2026-28; ~$150bn permanent financing need 2026-27</t>
         </is>
       </c>
-      <c r="C32" s="74" t="inlineStr">
+      <c r="C32" s="73" t="inlineStr">
         <is>
           <t>2025-28</t>
         </is>
       </c>
-      <c r="D32" s="74" t="inlineStr">
+      <c r="D32" s="73" t="inlineStr">
         <is>
           <t>~$130bn</t>
         </is>
       </c>
-      <c r="E32" s="74" t="inlineStr">
+      <c r="E32" s="73" t="inlineStr">
         <is>
           <t>Securitization (ABS/CMBS)</t>
         </is>
       </c>
-      <c r="F32" s="75" t="inlineStr">
+      <c r="F32" s="74" t="inlineStr">
         <is>
           <t>Impax; CREFC; Morgan Stanley</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="70" t="inlineStr">
+      <c r="A33" s="69" t="inlineStr">
         <is>
           <t>HUMAIN (Saudi PIF)</t>
         </is>
       </c>
-      <c r="B33" s="71" t="inlineStr">
+      <c r="B33" s="70" t="inlineStr">
         <is>
           <t>PIF national AI champion (announced 13 May 2025): ~$100bn across 11 data centers / 2.2 GW; ~600k NVIDIA GPUs; ALLAM Arabic LLM</t>
         </is>
       </c>
-      <c r="C33" s="71" t="inlineStr">
+      <c r="C33" s="70" t="inlineStr">
         <is>
           <t>2025-30</t>
         </is>
       </c>
-      <c r="D33" s="71" t="inlineStr">
+      <c r="D33" s="70" t="inlineStr">
         <is>
           <t>~$100bn</t>
         </is>
       </c>
-      <c r="E33" s="71" t="inlineStr">
+      <c r="E33" s="70" t="inlineStr">
         <is>
           <t>Sovereign equity</t>
         </is>
       </c>
-      <c r="F33" s="72" t="inlineStr">
+      <c r="F33" s="71" t="inlineStr">
         <is>
           <t>Presenc AI; NYU DRI</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="73" t="inlineStr">
+      <c r="A34" s="72" t="inlineStr">
         <is>
           <t>Stargate UAE / G42</t>
         </is>
       </c>
-      <c r="B34" s="74" t="inlineStr">
+      <c r="B34" s="73" t="inlineStr">
         <is>
           <t>$30bn+ 5GW Abu Dhabi campus (Khazna/G42 w/ OpenAI, Oracle, NVIDIA, Cisco, SoftBank); Phase 1 200MW Q3 2026; Microsoft ~$1.5bn equity</t>
         </is>
       </c>
-      <c r="C34" s="74" t="inlineStr">
+      <c r="C34" s="73" t="inlineStr">
         <is>
           <t>2025-30</t>
         </is>
       </c>
-      <c r="D34" s="74" t="inlineStr">
+      <c r="D34" s="73" t="inlineStr">
         <is>
           <t>~$30bn+</t>
         </is>
       </c>
-      <c r="E34" s="74" t="inlineStr">
+      <c r="E34" s="73" t="inlineStr">
         <is>
           <t>Sovereign equity + JV</t>
         </is>
       </c>
-      <c r="F34" s="75" t="inlineStr">
+      <c r="F34" s="74" t="inlineStr">
         <is>
           <t>Khaleej Times; dcpulse</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="70" t="inlineStr">
+      <c r="A35" s="69" t="inlineStr">
         <is>
           <t>MGX / Mubadala (UAE)</t>
         </is>
       </c>
-      <c r="B35" s="71" t="inlineStr">
+      <c r="B35" s="70" t="inlineStr">
         <is>
           <t>Anchored Stargate; co-led ~$40bn Aligned Data Centers acquisition w/ BlackRock; AIP (BlackRock-Microsoft) targets up to $100bn global AI infra</t>
         </is>
       </c>
-      <c r="C35" s="71" t="inlineStr">
+      <c r="C35" s="70" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D35" s="71" t="inlineStr">
+      <c r="D35" s="70" t="inlineStr">
         <is>
           <t>~$40bn+</t>
         </is>
       </c>
-      <c r="E35" s="71" t="inlineStr">
+      <c r="E35" s="70" t="inlineStr">
         <is>
           <t>Sovereign equity / infra</t>
         </is>
       </c>
-      <c r="F35" s="72" t="inlineStr">
+      <c r="F35" s="71" t="inlineStr">
         <is>
           <t>NYU DRI</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="73" t="inlineStr">
+      <c r="A36" s="72" t="inlineStr">
         <is>
           <t>Qatar (QIA / Qai)</t>
         </is>
       </c>
-      <c r="B36" s="74" t="inlineStr">
+      <c r="B36" s="73" t="inlineStr">
         <is>
           <t>~$20bn AI-infrastructure JV with Brookfield (late 2025); earlier positions in xAI &amp; Databricks</t>
         </is>
       </c>
-      <c r="C36" s="74" t="inlineStr">
+      <c r="C36" s="73" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D36" s="74" t="inlineStr">
+      <c r="D36" s="73" t="inlineStr">
         <is>
           <t>~$20bn</t>
         </is>
       </c>
-      <c r="E36" s="74" t="inlineStr">
+      <c r="E36" s="73" t="inlineStr">
         <is>
           <t>Sovereign equity + JV</t>
         </is>
       </c>
-      <c r="F36" s="75" t="inlineStr">
+      <c r="F36" s="74" t="inlineStr">
         <is>
           <t>NYU DRI</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="70" t="inlineStr">
+      <c r="A37" s="69" t="inlineStr">
         <is>
           <t>Sector-wide</t>
         </is>
       </c>
-      <c r="B37" s="71" t="inlineStr">
+      <c r="B37" s="70" t="inlineStr">
         <is>
           <t>HY/unrated AI-infra issuers raised ~$107bn funded+committed debt by ~May 2026 ($68.7bn neoclouds / $38.7bn AI-native DCs)</t>
         </is>
       </c>
-      <c r="C37" s="71" t="inlineStr">
+      <c r="C37" s="70" t="inlineStr">
         <is>
           <t>to 2026</t>
         </is>
       </c>
-      <c r="D37" s="71" t="inlineStr">
+      <c r="D37" s="70" t="inlineStr">
         <is>
           <t>~$107bn</t>
         </is>
       </c>
-      <c r="E37" s="71" t="inlineStr">
+      <c r="E37" s="70" t="inlineStr">
         <is>
           <t>All debt</t>
         </is>
       </c>
-      <c r="F37" s="72" t="inlineStr">
+      <c r="F37" s="71" t="inlineStr">
         <is>
           <t>Octus</t>
         </is>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="73" t="inlineStr">
+      <c r="A38" s="72" t="inlineStr">
         <is>
           <t>Sector-wide</t>
         </is>
       </c>
-      <c r="B38" s="74" t="inlineStr">
+      <c r="B38" s="73" t="inlineStr">
         <is>
           <t>Insurance-linked platforms deployed ~$180bn into private credit in 2025 (~25% of global private credit AUM)</t>
         </is>
       </c>
-      <c r="C38" s="74" t="inlineStr">
+      <c r="C38" s="73" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D38" s="74" t="inlineStr">
+      <c r="D38" s="73" t="inlineStr">
         <is>
           <t>~$180bn</t>
         </is>
       </c>
-      <c r="E38" s="74" t="inlineStr">
+      <c r="E38" s="73" t="inlineStr">
         <is>
           <t>Insurance / private credit</t>
         </is>
       </c>
-      <c r="F38" s="75" t="inlineStr">
+      <c r="F38" s="74" t="inlineStr">
         <is>
           <t>McKinsey; ABF Journal</t>
         </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="70" t="inlineStr">
+      <c r="A39" s="69" t="inlineStr">
         <is>
           <t>Sector-wide</t>
         </is>
       </c>
-      <c r="B39" s="71" t="inlineStr">
+      <c r="B39" s="70" t="inlineStr">
         <is>
           <t>Goldman Sachs: ~$5.3tn AI + data-center capex 2025-2030; Morgan Stanley: ~$800bn private credit for AI DCs 2025-28</t>
         </is>
       </c>
-      <c r="C39" s="71" t="inlineStr">
+      <c r="C39" s="70" t="inlineStr">
         <is>
           <t>2025-30</t>
         </is>
       </c>
-      <c r="D39" s="71" t="inlineStr">
+      <c r="D39" s="70" t="inlineStr">
         <is>
           <t>$5.3tn capex</t>
         </is>
       </c>
-      <c r="E39" s="71" t="inlineStr">
+      <c r="E39" s="70" t="inlineStr">
         <is>
           <t>Context</t>
         </is>
       </c>
-      <c r="F39" s="72" t="inlineStr">
+      <c r="F39" s="71" t="inlineStr">
         <is>
           <t>Goldman; Morgan Stanley</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="76" t="inlineStr">
+      <c r="A41" s="75" t="inlineStr">
         <is>
           <t>Selected sources:</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="77" t="inlineStr">
+      <c r="A42" s="76" t="inlineStr">
         <is>
           <t>Goldman Sachs Research — ~$5.3tn AI + data-center capex 2025-2030; private markets in DC financing.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="77" t="inlineStr">
+      <c r="A43" s="76" t="inlineStr">
         <is>
           <t>Morgan Stanley — ~$2tn capex 2025-28 with &gt;$1tn debt; ~$800bn private credit for AI DCs.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="77" t="inlineStr">
+      <c r="A44" s="76" t="inlineStr">
         <is>
           <t>Bank of America / BofA Securities — hyperscaler bond issuance ($121bn 2025; ~$175bn 2026E).</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="77" t="inlineStr">
+      <c r="A45" s="76" t="inlineStr">
         <is>
           <t>Moody's Ratings — hyperscaler capex (~$785bn 2026, ~$1tn 2027); $662bn off-B/S DC leases.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="77" t="inlineStr">
+      <c r="A46" s="76" t="inlineStr">
         <is>
           <t>McKinsey — ~$2.7tn US (5.2tn global) data-center capex by 2030; insurance-linked private credit.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="77" t="inlineStr">
+      <c r="A47" s="76" t="inlineStr">
         <is>
           <t>Octus — HY/unrated AI-infra debt (~$107bn to ~May 2026); ~14GW unfunded ≈ $344bn need.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="77" t="inlineStr">
+      <c r="A48" s="76" t="inlineStr">
         <is>
           <t>Company disclosures &amp; press: Meta IR / FT / S&amp;P (Hyperion); Oracle IR / IFR / Reuters; CoreWeave IR;</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="77" t="inlineStr">
+      <c r="A49" s="76" t="inlineStr">
         <is>
           <t xml:space="preserve">  CNBC / WSJ / The Information (xAI); Blackstone; Apollo Academy; MUFG; CreditSights; CNA.</t>
         </is>

</xml_diff>

<commit_message>
Add Private Credit Deals transaction-log tab
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AI_Infrastructure_Financing_2025-2030.xlsx
+++ b/AI_Infrastructure_Financing_2025-2030.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Debt by Type" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Cash-Flow Bridge" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Capex Projections" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Key Deals &amp; Sources" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Private Credit Deals" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Key Deals &amp; Sources" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1"/>
@@ -21,10 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0)"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -135,11 +137,15 @@
       <color rgb="00B00020"/>
     </font>
     <font>
+      <sz val="9"/>
+    </font>
+    <font>
       <b val="1"/>
       <sz val="9"/>
     </font>
     <font>
-      <sz val="9"/>
+      <color rgb="005A5A5A"/>
+      <sz val="8"/>
     </font>
     <font>
       <color rgb="002E5A9C"/>
@@ -150,7 +156,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -209,6 +215,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FCEFC7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
@@ -239,7 +255,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -397,26 +413,91 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="26" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="26" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="26" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1253,7 +1334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B70"/>
+  <dimension ref="B2:B72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1305,397 +1386,411 @@
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>• Capex Projections: annual AI-infrastructure capex 2025-2030 by company.</t>
+          <t>• Cash-Flow Bridge: operating cash flow -&gt; free cash flow -&gt; external funding gap.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="5" t="inlineStr">
         <is>
+          <t>• Capex Projections: annual AI-infrastructure capex 2025-2030 by company.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>• Private Credit Deals: transaction log of private-credit / SPV / 144A debt for AI infra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="5" t="inlineStr">
+        <is>
           <t>• Key Deals &amp; Sources: notable disclosed transactions underpinning the estimates.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="6" t="inlineStr">
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Scope &amp; definitions</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>• Hyperscalers: Microsoft, Amazon (AWS), Alphabet (Google), Meta, Oracle (OCI).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>• Neoclouds / AI-native infra: GPU-cloud &amp; AI-native data-center builders (CoreWeave,</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   SpaceX/xAI, Nebius, IREN, Crusoe, Lambda, Fluidstack, Nscale, + an 'Other' aggregate).</t>
+          <t>• Hyperscalers: Microsoft, Amazon (AWS), Alphabet (Google), Meta, Oracle (OCI).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>• SpaceX acquired xAI (effective 2 Feb 2026), so Colossus I &amp; II are now SpaceX-owned; the two</t>
+          <t>• Neoclouds / AI-native infra: GPU-cloud &amp; AI-native data-center builders (CoreWeave,</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   are shown as one consolidated 'SpaceX / xAI' line to avoid double-counting the same clusters.</t>
+          <t xml:space="preserve">   SpaceX/xAI, Nebius, IREN, Crusoe, Lambda, Fluidstack, Nscale, + an 'Other' aggregate).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>• Colocation / data-center REITs: wholesale &amp; retail colo / powered-shell owners (Equinix,</t>
+          <t>• SpaceX acquired xAI (effective 2 Feb 2026), so Colossus I &amp; II are now SpaceX-owned; the two</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Digital Realty, QTS, Vantage, Aligned, CyrusOne, Switch, Stack, + 'Other') that build campuses</t>
+          <t xml:space="preserve">   are shown as one consolidated 'SpaceX / xAI' line to avoid double-counting the same clusters.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   and lease them to hyperscalers / neoclouds; heavy users of ABS/CMBS securitization &amp; infra equity.</t>
+          <t>• Colocation / data-center REITs: wholesale &amp; retail colo / powered-shell owners (Equinix,</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>• Sovereign clouds: state / sovereign-wealth-funded national AI infrastructure (HUMAIN-Saudi PIF,</t>
+          <t xml:space="preserve">   Digital Realty, QTS, Vantage, Aligned, CyrusOne, Switch, Stack, + 'Other') that build campuses</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   MGX/Mubadala, Stargate UAE/G42/Khazna, Qatar QIA, EU/France, India, + 'Other'); mostly equity-funded.</t>
+          <t xml:space="preserve">   and lease them to hyperscalers / neoclouds; heavy users of ABS/CMBS securitization &amp; infra equity.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>• Funding sources now split three ways:  Capex = Operating cash flow (self-funded) +</t>
+          <t>• Sovereign clouds: state / sovereign-wealth-funded national AI infrastructure (HUMAIN-Saudi PIF,</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   External equity + Total debt.</t>
+          <t xml:space="preserve">   MGX/Mubadala, Stargate UAE/G42/Khazna, Qatar QIA, EU/France, India, + 'Other'); mostly equity-funded.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Operating cash flow (self-funded): internally-generated cash (CFO) reinvested into AI capex.</t>
+          <t>• Funding sources now split three ways:  Capex = Operating cash flow (self-funded) +</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - External equity: IPOs, secondaries, strategic stakes (e.g. NVIDIA), ATM programs, sovereign-</t>
+          <t xml:space="preserve">   External equity + Total debt.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">     wealth equity and mandatory convertible PREFERRED (treated as equity).</t>
+          <t xml:space="preserve">   - Operating cash flow (self-funded): internally-generated cash (CFO) reinvested into AI capex.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Total debt: external borrowing, split by instrument (see below).</t>
+          <t xml:space="preserve">   - External equity: IPOs, secondaries, strategic stakes (e.g. NVIDIA), ATM programs, sovereign-</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>• The 'Cash-Flow Bridge' sheet separates OPERATING CASH FLOW (CFO) and FREE CASH FLOW from the</t>
+          <t xml:space="preserve">     wealth equity and mandatory convertible PREFERRED (treated as equity).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   equity portion:  CFO - dividends/buybacks/other = self-funded capex; FREE CASH FLOW = CFO -</t>
+          <t xml:space="preserve">   - Total debt: external borrowing, split by instrument (see below).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="5" t="inlineStr">
         <is>
+          <t>• The 'Cash-Flow Bridge' sheet separates OPERATING CASH FLOW (CFO) and FREE CASH FLOW from the</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   equity portion:  CFO - dividends/buybacks/other = self-funded capex; FREE CASH FLOW = CFO -</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">   AI capex (negative for most builders, which is what drives external equity + debt issuance).</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="B33" s="7" t="inlineStr">
+    <row r="35" ht="20" customHeight="1">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>Debt instrument buckets (mutually exclusive — they sum to total debt)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>1. Corporate bonds (public IG/HY) — on-balance-sheet senior notes sold in public markets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>2. Bank &amp; syndicated loans — term loans, revolvers, delayed-draw term loans (incl. GPU-backed DDTLs).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>3. Alternate private credit — direct lending / private placements by credit funds (Blackstone,</t>
+          <t>1. Corporate bonds (public IG/HY) — on-balance-sheet senior notes sold in public markets.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Apollo, Blue Owl, PIMCO, Magnetar, etc.), including privately-placed SPV/project debt.</t>
+          <t>2. Bank &amp; syndicated loans — term loans, revolvers, delayed-draw term loans (incl. GPU-backed DDTLs).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>4. Insurance-linked lending — debt funded off insurer/annuity balance sheets (Athene/Apollo,</t>
+          <t>3. Alternate private credit — direct lending / private placements by credit funds (Blackstone,</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Global Atlantic/KKR, MetLife, Brookfield, etc.). NOTE: large overlap with private credit &amp;</t>
+          <t xml:space="preserve">   Apollo, Blue Owl, PIMCO, Magnetar, etc.), including privately-placed SPV/project debt.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   bonds; shown separately to size the insurance channel — see double-counting note below.</t>
+          <t>4. Insurance-linked lending — debt funded off insurer/annuity balance sheets (Athene/Apollo,</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>5. Securitization / ABS / CMBS — secured data-center bonds &amp; GPU-backed asset-backed securities.</t>
+          <t xml:space="preserve">   Global Atlantic/KKR, MetLife, Brookfield, etc.). NOTE: large overlap with private credit &amp;</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>6. Convertibles / equity-linked debt — convertible notes (excludes mandatory convert. PREFERRED).</t>
+          <t xml:space="preserve">   bonds; shown separately to size the insurance channel — see double-counting note below.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>7. Vendor &amp; equipment-lease financing — chip/equipment leases &amp; sale-leasebacks (e.g. NVIDIA</t>
+          <t>5. Securitization / ABS / CMBS — secured data-center bonds &amp; GPU-backed asset-backed securities.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   chip-lease SPVs, finance leases). Microsoft's large finance-lease book sits largely here.</t>
+          <t>6. Convertibles / equity-linked debt — convertible notes (excludes mandatory convert. PREFERRED).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Memo: 'Off-B/S SPV / JV (memo)' flags the portion routed through special-purpose vehicles /</t>
+          <t>7. Vendor &amp; equipment-lease financing — chip/equipment leases &amp; sale-leasebacks (e.g. NVIDIA</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   joint ventures (e.g. Meta-Hyperion, xAI Colossus 2, Oracle project SPVs). It OVERLAPS the</t>
+          <t xml:space="preserve">   chip-lease SPVs, finance leases). Microsoft's large finance-lease book sits largely here.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="5" t="inlineStr">
         <is>
+          <t>Memo: 'Off-B/S SPV / JV (memo)' flags the portion routed through special-purpose vehicles /</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   joint ventures (e.g. Meta-Hyperion, xAI Colossus 2, Oracle project SPVs). It OVERLAPS the</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">   buckets above and is therefore NOT added into the debt total.</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="B49" s="8" t="inlineStr">
+    <row r="51" ht="20" customHeight="1">
+      <c r="B51" s="8" t="inlineStr">
         <is>
           <t>Methodology &amp; caveats</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>• Figures are RESEARCH ESTIMATES for the cumulative 2025-2030 buildout. They blend disclosed</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  transactions (2023-early 2026) with forward projections; they are illustrative, not audited.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>• Aggregate cross-check: total financing ≈ $5.25tn, consistent with Goldman Sachs' ~$5.3tn</t>
+          <t>• Figures are RESEARCH ESTIMATES for the cumulative 2025-2030 buildout. They blend disclosed</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2025-2030 AI + data-center capex estimate; aggregate debt ≈ $1.8tn, consistent with Morgan</t>
+          <t xml:space="preserve">  transactions (2023-early 2026) with forward projections; they are illustrative, not audited.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stanley / BofA projections of $1-2tn of debt financing for the buildout.</t>
+          <t>• Aggregate cross-check: total financing ≈ $5.25tn, consistent with Goldman Sachs' ~$5.3tn</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>• CROSS-SEGMENT OVERLAP: hyperscalers LEASE much colocation capacity (so colo financing partly</t>
+          <t xml:space="preserve">  2025-2030 AI + data-center capex estimate; aggregate debt ≈ $1.8tn, consistent with Morgan</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  funds the same capacity hyperscalers report as off-B/S leases), and sovereign-wealth funds</t>
+          <t xml:space="preserve">  Stanley / BofA projections of $1-2tn of debt financing for the buildout.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (MGX, PIF, QIA) also INVEST in neoclouds/labs and colo (e.g. MGX/BlackRock bought Aligned; PIF</t>
+          <t>• CROSS-SEGMENT OVERLAP: hyperscalers LEASE much colocation capacity (so colo financing partly</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  put ~$3bn into xAI). The all-segment 'grand total' is therefore a GROSS figure of capital raised</t>
+          <t xml:space="preserve">  funds the same capacity hyperscalers report as off-B/S leases), and sovereign-wealth funds</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  across distinct balance sheets and is not strictly additive; treat it as an upper-bound view.</t>
+          <t xml:space="preserve">  (MGX, PIF, QIA) also INVEST in neoclouds/labs and colo (e.g. MGX/BlackRock bought Aligned; PIF</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Hyperscaler + Neocloud financing (~$5.4tn) ties to Goldman's ~$5.3tn big-tech capex; adding</t>
+          <t xml:space="preserve">  put ~$3bn into xAI). The all-segment 'grand total' is therefore a GROSS figure of capital raised</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  third-party colo + sovereign brings the gross total toward broader ~$6-7tn AI-infra estimates.</t>
+          <t xml:space="preserve">  across distinct balance sheets and is not strictly additive; treat it as an upper-bound view.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>• Insurance-linked lending double counts with private credit/bonds at the capital-source level;</t>
+          <t xml:space="preserve">  Hyperscaler + Neocloud financing (~$5.4tn) ties to Goldman's ~$5.3tn big-tech capex; adding</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  to avoid inflating totals, each dollar of debt is classified ONCE by its primary instrument and</t>
+          <t xml:space="preserve">  third-party colo + sovereign brings the gross total toward broader ~$6-7tn AI-infra estimates.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  the insurance bucket captures only directly insurer-originated / insurance-balance-sheet debt.</t>
+          <t>• Insurance-linked lending double counts with private credit/bonds at the capital-source level;</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>• Company splits reflect observed behavior: Microsoft/Alphabet/Amazon are FCF-heavy with</t>
+          <t xml:space="preserve">  to avoid inflating totals, each dollar of debt is classified ONCE by its primary instrument and</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  selective bonds; Meta &amp; Oracle lean more on debt &amp; SPVs; neoclouds are debt-heavy (asset-backed).</t>
+          <t xml:space="preserve">  the insurance bucket captures only directly insurer-originated / insurance-balance-sheet debt.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="B67" s="5" t="inlineStr">
         <is>
+          <t>• Company splits reflect observed behavior: Microsoft/Alphabet/Amazon are FCF-heavy with</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  selective bonds; Meta &amp; Oracle lean more on debt &amp; SPVs; neoclouds are debt-heavy (asset-backed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="5" t="inlineStr">
+        <is>
           <t>• Built with openpyxl. See Key Deals &amp; Sources sheet for citations.</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="30" customHeight="1">
-      <c r="B70" s="9" t="inlineStr">
+    <row r="72" ht="30" customHeight="1">
+      <c r="B72" s="9" t="inlineStr">
         <is>
           <t>Disclaimer: For analytical/illustrative purposes only. Not investment advice and not a representation of any company's actual financing. Verify against primary filings before use.</t>
         </is>
@@ -8055,6 +8150,1245 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Private Credit Transactions — AI Infrastructure (US$bn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Transaction log of private-credit / SPV / private-placement (144A) debt for AI infra. Itemized deals are summed; 'Context / market' rows (frameworks, projections) are not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="69" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B4" s="69" t="inlineStr">
+        <is>
+          <t>Borrower / Project</t>
+        </is>
+      </c>
+      <c r="C4" s="69" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="D4" s="69" t="inlineStr">
+        <is>
+          <t>Lead lenders / arrangers</t>
+        </is>
+      </c>
+      <c r="E4" s="69" t="inlineStr">
+        <is>
+          <t>Debt amount
+($bn)</t>
+        </is>
+      </c>
+      <c r="F4" s="69" t="inlineStr">
+        <is>
+          <t>Structure / instrument</t>
+        </is>
+      </c>
+      <c r="G4" s="69" t="inlineStr">
+        <is>
+          <t>Pricing</t>
+        </is>
+      </c>
+      <c r="H4" s="69" t="inlineStr">
+        <is>
+          <t>Tenor /
+maturity</t>
+        </is>
+      </c>
+      <c r="I4" s="69" t="inlineStr">
+        <is>
+          <t>Collateral / notes</t>
+        </is>
+      </c>
+      <c r="J4" s="69" t="inlineStr">
+        <is>
+          <t>Source(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="70" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B5" s="71" t="inlineStr">
+        <is>
+          <t>Oracle — Texas + Wisconsin data centers</t>
+        </is>
+      </c>
+      <c r="C5" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D5" s="70" t="inlineStr">
+        <is>
+          <t>Private credit consortium</t>
+        </is>
+      </c>
+      <c r="E5" s="73" t="n">
+        <v>38</v>
+      </c>
+      <c r="F5" s="70" t="inlineStr">
+        <is>
+          <t>SPV debt package</t>
+        </is>
+      </c>
+      <c r="G5" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H5" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I5" s="70" t="inlineStr">
+        <is>
+          <t>Two-site off-B/S financing</t>
+        </is>
+      </c>
+      <c r="J5" s="74" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="75" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B6" s="76" t="inlineStr">
+        <is>
+          <t>Anthropic — Google TPU chip SPV</t>
+        </is>
+      </c>
+      <c r="C6" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D6" s="75" t="inlineStr">
+        <is>
+          <t>Apollo (Atlas SP $0.8bn equity; Athene), Blackstone; Broadcom RVG</t>
+        </is>
+      </c>
+      <c r="E6" s="78" t="n">
+        <v>35</v>
+      </c>
+      <c r="F6" s="75" t="inlineStr">
+        <is>
+          <t>Chip-leasing SPV; 3 tranches; ~half syndicated</t>
+        </is>
+      </c>
+      <c r="G6" s="75" t="inlineStr">
+        <is>
+          <t>A1 T+100bp; A2 5.75%; B 8.5%</t>
+        </is>
+      </c>
+      <c r="H6" s="75" t="inlineStr">
+        <is>
+          <t>~5y</t>
+        </is>
+      </c>
+      <c r="I6" s="75" t="inlineStr">
+        <is>
+          <t>Buys Google TPUs leased to Anthropic; Broadcom residual-value support</t>
+        </is>
+      </c>
+      <c r="J6" s="79" t="inlineStr">
+        <is>
+          <t>privatedebtnews; Build.inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="70" t="inlineStr">
+        <is>
+          <t>Oct 2025</t>
+        </is>
+      </c>
+      <c r="B7" s="71" t="inlineStr">
+        <is>
+          <t>Meta — Hyperion (Beignet Investor LLC), Louisiana</t>
+        </is>
+      </c>
+      <c r="C7" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D7" s="70" t="inlineStr">
+        <is>
+          <t>PIMCO (~$18bn), BlackRock, Apollo (debt); Blue Owl (equity); MS adviser</t>
+        </is>
+      </c>
+      <c r="E7" s="73" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="F7" s="70" t="inlineStr">
+        <is>
+          <t>Off-B/S SPV; 144A senior secured bond</t>
+        </is>
+      </c>
+      <c r="G7" s="70" t="inlineStr">
+        <is>
+          <t>6.581% / T+225bp</t>
+        </is>
+      </c>
+      <c r="H7" s="70" t="inlineStr">
+        <is>
+          <t>Due May 2049 (~23.6y)</t>
+        </is>
+      </c>
+      <c r="I7" s="70" t="inlineStr">
+        <is>
+          <t>2.1GW campus; Meta lease + residual-value guarantee (up to ~$28bn); A+ (S&amp;P)</t>
+        </is>
+      </c>
+      <c r="J7" s="74" t="inlineStr">
+        <is>
+          <t>IFR; FT; Quinn Emanuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="70" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B8" s="71" t="inlineStr">
+        <is>
+          <t>Oracle — New Mexico site</t>
+        </is>
+      </c>
+      <c r="C8" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D8" s="70" t="inlineStr">
+        <is>
+          <t>Private credit lenders</t>
+        </is>
+      </c>
+      <c r="E8" s="73" t="n">
+        <v>18</v>
+      </c>
+      <c r="F8" s="70" t="inlineStr">
+        <is>
+          <t>SPV / project loan</t>
+        </is>
+      </c>
+      <c r="G8" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H8" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I8" s="70" t="inlineStr">
+        <is>
+          <t>Single-site project loan</t>
+        </is>
+      </c>
+      <c r="J8" s="74" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B9" s="71" t="inlineStr">
+        <is>
+          <t>Oracle — Michigan campus</t>
+        </is>
+      </c>
+      <c r="C9" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D9" s="70" t="inlineStr">
+        <is>
+          <t>Project-finance lenders</t>
+        </is>
+      </c>
+      <c r="E9" s="73" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="F9" s="70" t="inlineStr">
+        <is>
+          <t>Project-level SPV financing</t>
+        </is>
+      </c>
+      <c r="G9" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H9" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I9" s="70" t="inlineStr">
+        <is>
+          <t>OCI capacity build</t>
+        </is>
+      </c>
+      <c r="J9" s="74" t="inlineStr">
+        <is>
+          <t>Press reports</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="75" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B10" s="76" t="inlineStr">
+        <is>
+          <t>xAI — Colossus 2 chip SPV (Memphis/Southaven)</t>
+        </is>
+      </c>
+      <c r="C10" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D10" s="75" t="inlineStr">
+        <is>
+          <t>Valor Equity (lead), Apollo, Diameter (debt); NVIDIA up to $2bn equity</t>
+        </is>
+      </c>
+      <c r="E10" s="78" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F10" s="75" t="inlineStr">
+        <is>
+          <t>SPV; debt + ~$7.5bn equity to buy &amp; lease GPUs</t>
+        </is>
+      </c>
+      <c r="G10" s="75" t="inlineStr">
+        <is>
+          <t>~10.5%</t>
+        </is>
+      </c>
+      <c r="H10" s="75" t="inlineStr">
+        <is>
+          <t>5y (~2.5y avg life)</t>
+        </is>
+      </c>
+      <c r="I10" s="75" t="inlineStr">
+        <is>
+          <t>Buys NVIDIA GPUs leased to xAI; chips as collateral</t>
+        </is>
+      </c>
+      <c r="J10" s="79" t="inlineStr">
+        <is>
+          <t>FT; WSJ; AAE filing</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B11" s="71" t="inlineStr">
+        <is>
+          <t>Oracle/OpenAI — Abilene, TX (Stargate; Crusoe developer)</t>
+        </is>
+      </c>
+      <c r="C11" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D11" s="70" t="inlineStr">
+        <is>
+          <t>Blue Owl + JPMorgan (incl. Crusoe, Primary Digital Infrastructure)</t>
+        </is>
+      </c>
+      <c r="E11" s="73" t="n">
+        <v>10</v>
+      </c>
+      <c r="F11" s="70" t="inlineStr">
+        <is>
+          <t>Off-B/S SPV (~$13bn incl. equity)</t>
+        </is>
+      </c>
+      <c r="G11" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H11" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I11" s="70" t="inlineStr">
+        <is>
+          <t>SPV owns OpenAI Abilene facility</t>
+        </is>
+      </c>
+      <c r="J11" s="74" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="75" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B12" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — DDTL 4.0 (Compute Acq. Co. VIII)</t>
+        </is>
+      </c>
+      <c r="C12" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D12" s="75" t="inlineStr">
+        <is>
+          <t>Blackstone Credit &amp; Insurance (anchor); MUFG, MS, GS, JPM</t>
+        </is>
+      </c>
+      <c r="E12" s="78" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="F12" s="75" t="inlineStr">
+        <is>
+          <t>Non-recourse GPU-backed delayed-draw term loan</t>
+        </is>
+      </c>
+      <c r="G12" s="75" t="inlineStr">
+        <is>
+          <t>SOFR+225 / ~5.9% fixed</t>
+        </is>
+      </c>
+      <c r="H12" s="75" t="inlineStr">
+        <is>
+          <t>Mar 2032</t>
+        </is>
+      </c>
+      <c r="I12" s="75" t="inlineStr">
+        <is>
+          <t>First IG-rated (A3 / A low) HPC-collateralized loan</t>
+        </is>
+      </c>
+      <c r="J12" s="79" t="inlineStr">
+        <is>
+          <t>CoreWeave IR</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="75" t="inlineStr">
+        <is>
+          <t>May 2024</t>
+        </is>
+      </c>
+      <c r="B13" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — $7.5bn debt facility</t>
+        </is>
+      </c>
+      <c r="C13" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D13" s="75" t="inlineStr">
+        <is>
+          <t>Blackstone, Magnetar (co-leads), Coatue, Carlyle, CDPQ, BlackRock, Eldridge</t>
+        </is>
+      </c>
+      <c r="E13" s="78" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F13" s="75" t="inlineStr">
+        <is>
+          <t>GPU + customer-contract secured facility</t>
+        </is>
+      </c>
+      <c r="G13" s="75" t="inlineStr">
+        <is>
+          <t>~10%+ (at issue)</t>
+        </is>
+      </c>
+      <c r="H13" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I13" s="75" t="inlineStr">
+        <is>
+          <t>Largest private debt deal at the time</t>
+        </is>
+      </c>
+      <c r="J13" s="79" t="inlineStr">
+        <is>
+          <t>Blackstone</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="80" t="inlineStr">
+        <is>
+          <t>Early 2025</t>
+        </is>
+      </c>
+      <c r="B14" s="81" t="inlineStr">
+        <is>
+          <t>Aligned Data Centers — debt commitments</t>
+        </is>
+      </c>
+      <c r="C14" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D14" s="80" t="inlineStr">
+        <is>
+          <t>Macquarie + global investors</t>
+        </is>
+      </c>
+      <c r="E14" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="F14" s="80" t="inlineStr">
+        <is>
+          <t>Debt within $12bn raise (+$5bn equity)</t>
+        </is>
+      </c>
+      <c r="G14" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H14" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I14" s="80" t="inlineStr">
+        <is>
+          <t>Later acquired by MGX/BlackRock (~$40bn)</t>
+        </is>
+      </c>
+      <c r="J14" s="84" t="inlineStr">
+        <is>
+          <t>SFA; NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="75" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B15" s="76" t="inlineStr">
+        <is>
+          <t>Fluidstack — Google-backed facility</t>
+        </is>
+      </c>
+      <c r="C15" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D15" s="75" t="inlineStr">
+        <is>
+          <t>Private credit (Google lease backstop)</t>
+        </is>
+      </c>
+      <c r="E15" s="78" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="F15" s="75" t="inlineStr">
+        <is>
+          <t>SPV backed by contracted revenue</t>
+        </is>
+      </c>
+      <c r="G15" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H15" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I15" s="75" t="inlineStr">
+        <is>
+          <t>~$6.7bn Google-contracted revenue backstop</t>
+        </is>
+      </c>
+      <c r="J15" s="79" t="inlineStr">
+        <is>
+          <t>theaiinsider</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="75" t="inlineStr">
+        <is>
+          <t>Jun-Jul 2025</t>
+        </is>
+      </c>
+      <c r="B16" s="76" t="inlineStr">
+        <is>
+          <t>xAI — secured notes / term loan (part of $10bn raise)</t>
+        </is>
+      </c>
+      <c r="C16" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D16" s="75" t="inlineStr">
+        <is>
+          <t>Apollo, Diameter; Morgan Stanley arranger</t>
+        </is>
+      </c>
+      <c r="E16" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" s="75" t="inlineStr">
+        <is>
+          <t>Secured notes + term loan</t>
+        </is>
+      </c>
+      <c r="G16" s="75" t="inlineStr">
+        <is>
+          <t>up to ~12.5%</t>
+        </is>
+      </c>
+      <c r="H16" s="75" t="inlineStr">
+        <is>
+          <t>~3-5y</t>
+        </is>
+      </c>
+      <c r="I16" s="75" t="inlineStr">
+        <is>
+          <t>Lenders can seize/operate Colossus on default</t>
+        </is>
+      </c>
+      <c r="J16" s="79" t="inlineStr">
+        <is>
+          <t>CNBC; ciphertalk</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="80" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="B17" s="81" t="inlineStr">
+        <is>
+          <t>Applied Digital — Macquarie financing</t>
+        </is>
+      </c>
+      <c r="C17" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D17" s="80" t="inlineStr">
+        <is>
+          <t>Macquarie</t>
+        </is>
+      </c>
+      <c r="E17" s="83" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" s="80" t="inlineStr">
+        <is>
+          <t>Perpetual/structured HPC financing</t>
+        </is>
+      </c>
+      <c r="G17" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H17" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I17" s="80" t="inlineStr">
+        <is>
+          <t>Powered-shell build for CoreWeave (Polaris Forge)</t>
+        </is>
+      </c>
+      <c r="J17" s="84" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="75" t="inlineStr">
+        <is>
+          <t>Jul 2025</t>
+        </is>
+      </c>
+      <c r="B18" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — OpenAI contract financing</t>
+        </is>
+      </c>
+      <c r="C18" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D18" s="75" t="inlineStr">
+        <is>
+          <t>Private lenders (SPV)</t>
+        </is>
+      </c>
+      <c r="E18" s="78" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F18" s="75" t="inlineStr">
+        <is>
+          <t>SPV debt vs. $11.9bn OpenAI contract</t>
+        </is>
+      </c>
+      <c r="G18" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H18" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I18" s="75" t="inlineStr">
+        <is>
+          <t>Funds CoreWeave's OpenAI compute obligations</t>
+        </is>
+      </c>
+      <c r="J18" s="79" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="75" t="inlineStr">
+        <is>
+          <t>Aug 2023</t>
+        </is>
+      </c>
+      <c r="B19" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — $2.3bn debt facility</t>
+        </is>
+      </c>
+      <c r="C19" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D19" s="75" t="inlineStr">
+        <is>
+          <t>Blackstone, Magnetar</t>
+        </is>
+      </c>
+      <c r="E19" s="78" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F19" s="75" t="inlineStr">
+        <is>
+          <t>GPU-backed facility</t>
+        </is>
+      </c>
+      <c r="G19" s="75" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H19" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I19" s="75" t="inlineStr">
+        <is>
+          <t>Early template for GPU-collateralized debt</t>
+        </is>
+      </c>
+      <c r="J19" s="79" t="inlineStr">
+        <is>
+          <t>Blackstone</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="75" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B20" s="76" t="inlineStr">
+        <is>
+          <t>Nscale — term loan</t>
+        </is>
+      </c>
+      <c r="C20" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D20" s="75" t="inlineStr">
+        <is>
+          <t>Private credit</t>
+        </is>
+      </c>
+      <c r="E20" s="78" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F20" s="75" t="inlineStr">
+        <is>
+          <t>Term loan</t>
+        </is>
+      </c>
+      <c r="G20" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H20" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I20" s="75" t="inlineStr">
+        <is>
+          <t>GPU-cloud build</t>
+        </is>
+      </c>
+      <c r="J20" s="79" t="inlineStr">
+        <is>
+          <t>theaiinsider</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="75" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B21" s="76" t="inlineStr">
+        <is>
+          <t>Lambda — GPU-backed facility</t>
+        </is>
+      </c>
+      <c r="C21" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D21" s="75" t="inlineStr">
+        <is>
+          <t>Macquarie</t>
+        </is>
+      </c>
+      <c r="E21" s="78" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F21" s="75" t="inlineStr">
+        <is>
+          <t>GPU-backed facility</t>
+        </is>
+      </c>
+      <c r="G21" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H21" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I21" s="75" t="inlineStr">
+        <is>
+          <t>GPU-cloud build</t>
+        </is>
+      </c>
+      <c r="J21" s="79" t="inlineStr">
+        <is>
+          <t>theaiinsider</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="85" t="n"/>
+      <c r="B22" s="86" t="inlineStr">
+        <is>
+          <t>Total — itemized private credit deals</t>
+        </is>
+      </c>
+      <c r="C22" s="85" t="n"/>
+      <c r="D22" s="85" t="n"/>
+      <c r="E22" s="87">
+        <f>SUM(E5:E21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="85" t="n"/>
+      <c r="G22" s="85" t="n"/>
+      <c r="H22" s="85" t="n"/>
+      <c r="I22" s="85" t="n"/>
+      <c r="J22" s="85" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>CONTEXT / FRAMEWORKS / PROJECTIONS (not summed)</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n"/>
+      <c r="C24" s="15" t="n"/>
+      <c r="D24" s="15" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="15" t="n"/>
+      <c r="G24" s="15" t="n"/>
+      <c r="H24" s="15" t="n"/>
+      <c r="I24" s="15" t="n"/>
+      <c r="J24" s="15" t="n"/>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="88" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="B25" s="88" t="inlineStr">
+        <is>
+          <t>KKR + Energy Capital Partners — AI infrastructure partnership</t>
+        </is>
+      </c>
+      <c r="C25" s="89" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D25" s="88" t="inlineStr">
+        <is>
+          <t>KKR, Energy Capital Partners</t>
+        </is>
+      </c>
+      <c r="E25" s="90" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" s="88" t="inlineStr">
+        <is>
+          <t>Strategic partnership/commitment</t>
+        </is>
+      </c>
+      <c r="G25" s="88" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H25" s="88" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I25" s="88" t="inlineStr">
+        <is>
+          <t>~$50bn to accelerate AI infrastructure</t>
+        </is>
+      </c>
+      <c r="J25" s="91" t="inlineStr">
+        <is>
+          <t>Business Times</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="88" t="inlineStr">
+        <is>
+          <t>Late 2025</t>
+        </is>
+      </c>
+      <c r="B26" s="88" t="inlineStr">
+        <is>
+          <t>Qatar (QIA / Qai) + Brookfield — AI infrastructure JV</t>
+        </is>
+      </c>
+      <c r="C26" s="89" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D26" s="88" t="inlineStr">
+        <is>
+          <t>QIA / Qai, Brookfield</t>
+        </is>
+      </c>
+      <c r="E26" s="90" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F26" s="88" t="inlineStr">
+        <is>
+          <t>Joint venture / infra credit</t>
+        </is>
+      </c>
+      <c r="G26" s="88" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H26" s="88" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I26" s="88" t="inlineStr">
+        <is>
+          <t>~$20bn JV</t>
+        </is>
+      </c>
+      <c r="J26" s="91" t="inlineStr">
+        <is>
+          <t>NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="88" t="inlineStr">
+        <is>
+          <t>2025-28</t>
+        </is>
+      </c>
+      <c r="B27" s="88" t="inlineStr">
+        <is>
+          <t>Broadcom + Apollo + Blackstone — AI compute platform</t>
+        </is>
+      </c>
+      <c r="C27" s="89" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D27" s="88" t="inlineStr">
+        <is>
+          <t>Apollo, Blackstone, Broadcom</t>
+        </is>
+      </c>
+      <c r="E27" s="90" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F27" s="88" t="inlineStr">
+        <is>
+          <t>Platform framework</t>
+        </is>
+      </c>
+      <c r="G27" s="88" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H27" s="88" t="inlineStr">
+        <is>
+          <t>through 2028</t>
+        </is>
+      </c>
+      <c r="I27" s="88" t="inlineStr">
+        <is>
+          <t>&gt;20 GW of compute to be deployed</t>
+        </is>
+      </c>
+      <c r="J27" s="91" t="inlineStr">
+        <is>
+          <t>privatedebtnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="88" t="inlineStr">
+        <is>
+          <t>from Nov 2025</t>
+        </is>
+      </c>
+      <c r="B28" s="88" t="inlineStr">
+        <is>
+          <t>Sector — 144A private placements (data centers)</t>
+        </is>
+      </c>
+      <c r="C28" s="89" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D28" s="88" t="inlineStr">
+        <is>
+          <t>Multiple (Blue Owl, PIMCO, etc.)</t>
+        </is>
+      </c>
+      <c r="E28" s="90" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F28" s="88" t="inlineStr">
+        <is>
+          <t>144A private placement bonds</t>
+        </is>
+      </c>
+      <c r="G28" s="88" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H28" s="88" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I28" s="88" t="inlineStr">
+        <is>
+          <t>&gt;$40bn by Applied Digital, CoreWeave, Hut 8, Related since Nov 2025</t>
+        </is>
+      </c>
+      <c r="J28" s="91" t="inlineStr">
+        <is>
+          <t>Bisnow</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="88" t="inlineStr">
+        <is>
+          <t>2025-28</t>
+        </is>
+      </c>
+      <c r="B29" s="88" t="inlineStr">
+        <is>
+          <t>Market — projected private credit for AI data centers</t>
+        </is>
+      </c>
+      <c r="C29" s="89" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D29" s="88" t="inlineStr">
+        <is>
+          <t>Industry-wide</t>
+        </is>
+      </c>
+      <c r="E29" s="90" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F29" s="88" t="inlineStr">
+        <is>
+          <t>Projection</t>
+        </is>
+      </c>
+      <c r="G29" s="88" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H29" s="88" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I29" s="88" t="inlineStr">
+        <is>
+          <t>Morgan Stanley: ~$800bn over next 2 years; &gt;$200bn already outstanding</t>
+        </is>
+      </c>
+      <c r="J29" s="91" t="inlineStr">
+        <is>
+          <t>Morgan Stanley; Quinn Emanuel</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8113,1183 +9447,1183 @@
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="69" t="inlineStr">
+      <c r="A5" s="92" t="inlineStr">
         <is>
           <t>Meta Platforms</t>
         </is>
       </c>
-      <c r="B5" s="70" t="inlineStr">
+      <c r="B5" s="93" t="inlineStr">
         <is>
           <t>Hyperion JV (Beignet Investor LLC) — Blue Owl 80% / Meta 20%; $27.3bn A+ private bond led by PIMCO (~$18bn) &amp; BlackRock; off-B/S SPV w/ residual-value guarantee</t>
         </is>
       </c>
-      <c r="C5" s="70" t="inlineStr">
+      <c r="C5" s="93" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D5" s="70" t="inlineStr">
+      <c r="D5" s="93" t="inlineStr">
         <is>
           <t>$27.3bn debt</t>
         </is>
       </c>
-      <c r="E5" s="70" t="inlineStr">
+      <c r="E5" s="93" t="inlineStr">
         <is>
           <t>SPV / private credit / insurance</t>
         </is>
       </c>
-      <c r="F5" s="71" t="inlineStr">
+      <c r="F5" s="94" t="inlineStr">
         <is>
           <t>Meta IR; FT; S&amp;P</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="72" t="inlineStr">
+      <c r="A6" s="95" t="inlineStr">
         <is>
           <t>Meta Platforms</t>
         </is>
       </c>
-      <c r="B6" s="73" t="inlineStr">
+      <c r="B6" s="96" t="inlineStr">
         <is>
           <t>$30bn multi-tranche IG corporate bond (largest 2025 IG deal), maturities to 2063</t>
         </is>
       </c>
-      <c r="C6" s="73" t="inlineStr">
+      <c r="C6" s="96" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D6" s="73" t="inlineStr">
+      <c r="D6" s="96" t="inlineStr">
         <is>
           <t>$30bn</t>
         </is>
       </c>
-      <c r="E6" s="73" t="inlineStr">
+      <c r="E6" s="96" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F6" s="74" t="inlineStr">
+      <c r="F6" s="97" t="inlineStr">
         <is>
           <t>BofA; MUFG</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="69" t="inlineStr">
+      <c r="A7" s="92" t="inlineStr">
         <is>
           <t>Amazon (AWS)</t>
         </is>
       </c>
-      <c r="B7" s="70" t="inlineStr">
+      <c r="B7" s="93" t="inlineStr">
         <is>
           <t>~$54bn USD + €14.5bn (~$16.8bn) IG bonds (near-record), ~4x oversubscribed</t>
         </is>
       </c>
-      <c r="C7" s="70" t="inlineStr">
+      <c r="C7" s="93" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D7" s="70" t="inlineStr">
+      <c r="D7" s="93" t="inlineStr">
         <is>
           <t>~$71bn</t>
         </is>
       </c>
-      <c r="E7" s="70" t="inlineStr">
+      <c r="E7" s="93" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F7" s="71" t="inlineStr">
+      <c r="F7" s="94" t="inlineStr">
         <is>
           <t>CNA; Reuters</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="72" t="inlineStr">
+      <c r="A8" s="95" t="inlineStr">
         <is>
           <t>Amazon (AWS)</t>
         </is>
       </c>
-      <c r="B8" s="73" t="inlineStr">
+      <c r="B8" s="96" t="inlineStr">
         <is>
           <t>$15bn IG bond</t>
         </is>
       </c>
-      <c r="C8" s="73" t="inlineStr">
+      <c r="C8" s="96" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D8" s="73" t="inlineStr">
+      <c r="D8" s="96" t="inlineStr">
         <is>
           <t>$15bn</t>
         </is>
       </c>
-      <c r="E8" s="73" t="inlineStr">
+      <c r="E8" s="96" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F8" s="74" t="inlineStr">
+      <c r="F8" s="97" t="inlineStr">
         <is>
           <t>CNA</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="69" t="inlineStr">
+      <c r="A9" s="92" t="inlineStr">
         <is>
           <t>Alphabet (Google)</t>
         </is>
       </c>
-      <c r="B9" s="70" t="inlineStr">
+      <c r="B9" s="93" t="inlineStr">
         <is>
           <t>~$32bn multi-currency bond incl. rare 100-yr tranche; plus $17.5bn Nov 2025</t>
         </is>
       </c>
-      <c r="C9" s="70" t="inlineStr">
+      <c r="C9" s="93" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D9" s="70" t="inlineStr">
+      <c r="D9" s="93" t="inlineStr">
         <is>
           <t>~$50bn</t>
         </is>
       </c>
-      <c r="E9" s="70" t="inlineStr">
+      <c r="E9" s="93" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F9" s="71" t="inlineStr">
+      <c r="F9" s="94" t="inlineStr">
         <is>
           <t>ConstructConnect; CNA</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="72" t="inlineStr">
+      <c r="A10" s="95" t="inlineStr">
         <is>
           <t>Oracle (OCI)</t>
         </is>
       </c>
-      <c r="B10" s="73" t="inlineStr">
+      <c r="B10" s="96" t="inlineStr">
         <is>
           <t>$25bn 8-part IG bond (Feb 2026) within $45-50bn CY26 debt+equity plan; $20bn ATM + mandatory convertible preferred (equity)</t>
         </is>
       </c>
-      <c r="C10" s="73" t="inlineStr">
+      <c r="C10" s="96" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D10" s="73" t="inlineStr">
+      <c r="D10" s="96" t="inlineStr">
         <is>
           <t>$25bn debt</t>
         </is>
       </c>
-      <c r="E10" s="73" t="inlineStr">
+      <c r="E10" s="96" t="inlineStr">
         <is>
           <t>Corporate bonds + equity</t>
         </is>
       </c>
-      <c r="F10" s="74" t="inlineStr">
+      <c r="F10" s="97" t="inlineStr">
         <is>
           <t>Oracle IR; IFR</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="69" t="inlineStr">
+      <c r="A11" s="92" t="inlineStr">
         <is>
           <t>Oracle (OCI)</t>
         </is>
       </c>
-      <c r="B11" s="70" t="inlineStr">
+      <c r="B11" s="93" t="inlineStr">
         <is>
           <t>$18bn 6-part IG bond (Sep 2025)</t>
         </is>
       </c>
-      <c r="C11" s="70" t="inlineStr">
+      <c r="C11" s="93" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D11" s="70" t="inlineStr">
+      <c r="D11" s="93" t="inlineStr">
         <is>
           <t>$18bn</t>
         </is>
       </c>
-      <c r="E11" s="70" t="inlineStr">
+      <c r="E11" s="93" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F11" s="71" t="inlineStr">
+      <c r="F11" s="94" t="inlineStr">
         <is>
           <t>Reuters/CNA</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="72" t="inlineStr">
+      <c r="A12" s="95" t="inlineStr">
         <is>
           <t>Oracle (OCI)</t>
         </is>
       </c>
-      <c r="B12" s="73" t="inlineStr">
+      <c r="B12" s="96" t="inlineStr">
         <is>
           <t>Project-level SPV financing: ~$16.3bn Michigan campus; further Texas / Wisconsin deals</t>
         </is>
       </c>
-      <c r="C12" s="73" t="inlineStr">
+      <c r="C12" s="96" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D12" s="73" t="inlineStr">
+      <c r="D12" s="96" t="inlineStr">
         <is>
           <t>~$25bn+</t>
         </is>
       </c>
-      <c r="E12" s="73" t="inlineStr">
+      <c r="E12" s="96" t="inlineStr">
         <is>
           <t>SPV / project finance</t>
         </is>
       </c>
-      <c r="F12" s="74" t="inlineStr">
+      <c r="F12" s="97" t="inlineStr">
         <is>
           <t>Press reports</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="69" t="inlineStr">
+      <c r="A13" s="92" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="B13" s="70" t="inlineStr">
+      <c r="B13" s="93" t="inlineStr">
         <is>
           <t>Finance-lease driven build (~$108bn uncommenced finance leases as of 9/30/24; commence FY25-FY30)</t>
         </is>
       </c>
-      <c r="C13" s="70" t="inlineStr">
+      <c r="C13" s="93" t="inlineStr">
         <is>
           <t>2024-30</t>
         </is>
       </c>
-      <c r="D13" s="70" t="inlineStr">
+      <c r="D13" s="93" t="inlineStr">
         <is>
           <t>$100bn+ leases</t>
         </is>
       </c>
-      <c r="E13" s="70" t="inlineStr">
+      <c r="E13" s="93" t="inlineStr">
         <is>
           <t>Vendor / lease / SPV</t>
         </is>
       </c>
-      <c r="F13" s="71" t="inlineStr">
+      <c r="F13" s="94" t="inlineStr">
         <is>
           <t>MSFT 10-Q; CNBC</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="72" t="inlineStr">
+      <c r="A14" s="95" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="B14" s="73" t="inlineStr">
+      <c r="B14" s="96" t="inlineStr">
         <is>
           <t>DDTL 4.0 — $8.5bn delayed-draw term loan; first IG-rated (Moody's A3 / DBRS A-low) GPU-backed financing; SOFR+225 / ~5.9%</t>
         </is>
       </c>
-      <c r="C14" s="73" t="inlineStr">
+      <c r="C14" s="96" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D14" s="73" t="inlineStr">
+      <c r="D14" s="96" t="inlineStr">
         <is>
           <t>$8.5bn</t>
         </is>
       </c>
-      <c r="E14" s="73" t="inlineStr">
+      <c r="E14" s="96" t="inlineStr">
         <is>
           <t>Bank / GPU-backed loan</t>
         </is>
       </c>
-      <c r="F14" s="74" t="inlineStr">
+      <c r="F14" s="97" t="inlineStr">
         <is>
           <t>CoreWeave IR</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="69" t="inlineStr">
+      <c r="A15" s="92" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="B15" s="70" t="inlineStr">
+      <c r="B15" s="93" t="inlineStr">
         <is>
           <t>$7.5bn debt facility led by Blackstone &amp; Magnetar (largest private debt deal at the time)</t>
         </is>
       </c>
-      <c r="C15" s="70" t="inlineStr">
+      <c r="C15" s="93" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D15" s="70" t="inlineStr">
+      <c r="D15" s="93" t="inlineStr">
         <is>
           <t>$7.5bn</t>
         </is>
       </c>
-      <c r="E15" s="70" t="inlineStr">
+      <c r="E15" s="93" t="inlineStr">
         <is>
           <t>Private credit / loan</t>
         </is>
       </c>
-      <c r="F15" s="71" t="inlineStr">
+      <c r="F15" s="94" t="inlineStr">
         <is>
           <t>Blackstone</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="72" t="inlineStr">
+      <c r="A16" s="95" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="B16" s="73" t="inlineStr">
+      <c r="B16" s="96" t="inlineStr">
         <is>
           <t>$2.7bn 1.75% convertible notes; ~$30bn total debt by early 2026; ~$28bn debt+equity raised in 12 mos</t>
         </is>
       </c>
-      <c r="C16" s="73" t="inlineStr">
+      <c r="C16" s="96" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D16" s="73" t="inlineStr">
+      <c r="D16" s="96" t="inlineStr">
         <is>
           <t>$2.7bn conv.</t>
         </is>
       </c>
-      <c r="E16" s="73" t="inlineStr">
+      <c r="E16" s="96" t="inlineStr">
         <is>
           <t>Convertibles</t>
         </is>
       </c>
-      <c r="F16" s="74" t="inlineStr">
+      <c r="F16" s="97" t="inlineStr">
         <is>
           <t>thedig; CoreWeave</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="69" t="inlineStr">
+      <c r="A17" s="92" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="B17" s="70" t="inlineStr">
+      <c r="B17" s="93" t="inlineStr">
         <is>
           <t>$2bn strategic equity from NVIDIA; IPO Mar 2025 raised ~$1.5bn</t>
         </is>
       </c>
-      <c r="C17" s="70" t="inlineStr">
+      <c r="C17" s="93" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D17" s="70" t="inlineStr">
+      <c r="D17" s="93" t="inlineStr">
         <is>
           <t>$3.5bn equity</t>
         </is>
       </c>
-      <c r="E17" s="70" t="inlineStr">
+      <c r="E17" s="93" t="inlineStr">
         <is>
           <t>Equity</t>
         </is>
       </c>
-      <c r="F17" s="71" t="inlineStr">
+      <c r="F17" s="94" t="inlineStr">
         <is>
           <t>CNBC; CoreWeave</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="72" t="inlineStr">
+      <c r="A18" s="95" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B18" s="73" t="inlineStr">
+      <c r="B18" s="96" t="inlineStr">
         <is>
           <t>SpaceX acquired xAI effective Feb 2, 2026; Colossus I &amp; II now SpaceX-owned (vertically-integrated AI platform; Terafab chip JV w/ Tesla &amp; Intel)</t>
         </is>
       </c>
-      <c r="C18" s="73" t="inlineStr">
+      <c r="C18" s="96" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D18" s="73" t="inlineStr">
+      <c r="D18" s="96" t="inlineStr">
         <is>
           <t>merger</t>
         </is>
       </c>
-      <c r="E18" s="73" t="inlineStr">
+      <c r="E18" s="96" t="inlineStr">
         <is>
           <t>Equity / M&amp;A</t>
         </is>
       </c>
-      <c r="F18" s="74" t="inlineStr">
+      <c r="F18" s="97" t="inlineStr">
         <is>
           <t>SpaceX S-1</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="69" t="inlineStr">
+      <c r="A19" s="92" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B19" s="70" t="inlineStr">
+      <c r="B19" s="93" t="inlineStr">
         <is>
           <t>SpaceX AI capex $12.7bn in 2025 (~61% of total) + $7.7bn in Q1 2026; AI buildout funded by Starlink FCF, private raises, planned IPO</t>
         </is>
       </c>
-      <c r="C19" s="70" t="inlineStr">
+      <c r="C19" s="93" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D19" s="70" t="inlineStr">
+      <c r="D19" s="93" t="inlineStr">
         <is>
           <t>$20bn+ capex</t>
         </is>
       </c>
-      <c r="E19" s="70" t="inlineStr">
+      <c r="E19" s="93" t="inlineStr">
         <is>
           <t>Internal / equity</t>
         </is>
       </c>
-      <c r="F19" s="71" t="inlineStr">
+      <c r="F19" s="94" t="inlineStr">
         <is>
           <t>SpaceX S-1; The Verge</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="72" t="inlineStr">
+      <c r="A20" s="95" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B20" s="73" t="inlineStr">
+      <c r="B20" s="96" t="inlineStr">
         <is>
           <t>Anthropic compute contract: $1.25bn/month (~$45bn) through May 2029 for Colossus I &amp; II — anchor revenue underwriting infra financing</t>
         </is>
       </c>
-      <c r="C20" s="73" t="inlineStr">
+      <c r="C20" s="96" t="inlineStr">
         <is>
           <t>2026-29</t>
         </is>
       </c>
-      <c r="D20" s="73" t="inlineStr">
+      <c r="D20" s="96" t="inlineStr">
         <is>
           <t>~$45bn</t>
         </is>
       </c>
-      <c r="E20" s="73" t="inlineStr">
+      <c r="E20" s="96" t="inlineStr">
         <is>
           <t>Take-or-pay (demand)</t>
         </is>
       </c>
-      <c r="F20" s="74" t="inlineStr">
+      <c r="F20" s="97" t="inlineStr">
         <is>
           <t>SpaceX S-1; The Verge</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="69" t="inlineStr">
+      <c r="A21" s="92" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B21" s="70" t="inlineStr">
+      <c r="B21" s="93" t="inlineStr">
         <is>
           <t>xAI $10bn raise ($5bn secured notes/term loans incl. Apollo $5bn facility + $5bn equity) via Morgan Stanley</t>
         </is>
       </c>
-      <c r="C21" s="70" t="inlineStr">
+      <c r="C21" s="93" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D21" s="70" t="inlineStr">
+      <c r="D21" s="93" t="inlineStr">
         <is>
           <t>$10bn</t>
         </is>
       </c>
-      <c r="E21" s="70" t="inlineStr">
+      <c r="E21" s="93" t="inlineStr">
         <is>
           <t>Loans + equity</t>
         </is>
       </c>
-      <c r="F21" s="71" t="inlineStr">
+      <c r="F21" s="94" t="inlineStr">
         <is>
           <t>CNBC</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="72" t="inlineStr">
+      <c r="A22" s="95" t="inlineStr">
         <is>
           <t>SpaceX / xAI</t>
         </is>
       </c>
-      <c r="B22" s="73" t="inlineStr">
+      <c r="B22" s="96" t="inlineStr">
         <is>
           <t>Colossus 2 SPV (Valor Equity): ~$12.5bn debt + ~$7.5bn equity (NVIDIA up to $2bn) to buy &amp; lease GPUs</t>
         </is>
       </c>
-      <c r="C22" s="73" t="inlineStr">
+      <c r="C22" s="96" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D22" s="73" t="inlineStr">
+      <c r="D22" s="96" t="inlineStr">
         <is>
           <t>~$20bn</t>
         </is>
       </c>
-      <c r="E22" s="73" t="inlineStr">
+      <c r="E22" s="96" t="inlineStr">
         <is>
           <t>SPV / vendor lease</t>
         </is>
       </c>
-      <c r="F22" s="74" t="inlineStr">
+      <c r="F22" s="97" t="inlineStr">
         <is>
           <t>The Information; Yahoo</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="69" t="inlineStr">
+      <c r="A23" s="92" t="inlineStr">
         <is>
           <t>Nebius</t>
         </is>
       </c>
-      <c r="B23" s="70" t="inlineStr">
+      <c r="B23" s="93" t="inlineStr">
         <is>
           <t>$3bn+ convertibles + bank lines; lighter balance sheet; Yandex spin-off cash ~$2.5bn; NVIDIA ~$2bn equity; Microsoft ~$7bn prepay</t>
         </is>
       </c>
-      <c r="C23" s="70" t="inlineStr">
+      <c r="C23" s="93" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D23" s="70" t="inlineStr">
+      <c r="D23" s="93" t="inlineStr">
         <is>
           <t>$3bn+</t>
         </is>
       </c>
-      <c r="E23" s="70" t="inlineStr">
+      <c r="E23" s="93" t="inlineStr">
         <is>
           <t>Convertibles</t>
         </is>
       </c>
-      <c r="F23" s="71" t="inlineStr">
+      <c r="F23" s="94" t="inlineStr">
         <is>
           <t>frankk research</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="72" t="inlineStr">
+      <c r="A24" s="95" t="inlineStr">
         <is>
           <t>Lambda</t>
         </is>
       </c>
-      <c r="B24" s="73" t="inlineStr">
+      <c r="B24" s="96" t="inlineStr">
         <is>
           <t>$500m GPU-backed facility from Macquarie</t>
         </is>
       </c>
-      <c r="C24" s="73" t="inlineStr">
+      <c r="C24" s="96" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D24" s="73" t="inlineStr">
+      <c r="D24" s="96" t="inlineStr">
         <is>
           <t>$0.5bn</t>
         </is>
       </c>
-      <c r="E24" s="73" t="inlineStr">
+      <c r="E24" s="96" t="inlineStr">
         <is>
           <t>Bank / GPU-backed loan</t>
         </is>
       </c>
-      <c r="F24" s="74" t="inlineStr">
+      <c r="F24" s="97" t="inlineStr">
         <is>
           <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="69" t="inlineStr">
+      <c r="A25" s="92" t="inlineStr">
         <is>
           <t>Nscale</t>
         </is>
       </c>
-      <c r="B25" s="70" t="inlineStr">
+      <c r="B25" s="93" t="inlineStr">
         <is>
           <t>$1.4bn term loan</t>
         </is>
       </c>
-      <c r="C25" s="70" t="inlineStr">
+      <c r="C25" s="93" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D25" s="70" t="inlineStr">
+      <c r="D25" s="93" t="inlineStr">
         <is>
           <t>$1.4bn</t>
         </is>
       </c>
-      <c r="E25" s="70" t="inlineStr">
+      <c r="E25" s="93" t="inlineStr">
         <is>
           <t>Bank loan</t>
         </is>
       </c>
-      <c r="F25" s="71" t="inlineStr">
+      <c r="F25" s="94" t="inlineStr">
         <is>
           <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="72" t="inlineStr">
+      <c r="A26" s="95" t="inlineStr">
         <is>
           <t>Fluidstack</t>
         </is>
       </c>
-      <c r="B26" s="73" t="inlineStr">
+      <c r="B26" s="96" t="inlineStr">
         <is>
           <t>Facility backed by ~$6.7bn Google-contracted revenue (Google lease backstop)</t>
         </is>
       </c>
-      <c r="C26" s="73" t="inlineStr">
+      <c r="C26" s="96" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D26" s="73" t="inlineStr">
+      <c r="D26" s="96" t="inlineStr">
         <is>
           <t>~$6.7bn</t>
         </is>
       </c>
-      <c r="E26" s="73" t="inlineStr">
+      <c r="E26" s="96" t="inlineStr">
         <is>
           <t>SPV / private credit</t>
         </is>
       </c>
-      <c r="F26" s="74" t="inlineStr">
+      <c r="F26" s="97" t="inlineStr">
         <is>
           <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="69" t="inlineStr">
+      <c r="A27" s="92" t="inlineStr">
         <is>
           <t>Applied Digital</t>
         </is>
       </c>
-      <c r="B27" s="70" t="inlineStr">
+      <c r="B27" s="93" t="inlineStr">
         <is>
           <t>$1.59bn high-yield bond (7%) for CoreWeave-leased campus (Polaris Forge 1)</t>
         </is>
       </c>
-      <c r="C27" s="70" t="inlineStr">
+      <c r="C27" s="93" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D27" s="70" t="inlineStr">
+      <c r="D27" s="93" t="inlineStr">
         <is>
           <t>$1.59bn</t>
         </is>
       </c>
-      <c r="E27" s="70" t="inlineStr">
+      <c r="E27" s="93" t="inlineStr">
         <is>
           <t>Securitization / HY bond</t>
         </is>
       </c>
-      <c r="F27" s="71" t="inlineStr">
+      <c r="F27" s="94" t="inlineStr">
         <is>
           <t>TNW</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="72" t="inlineStr">
+      <c r="A28" s="95" t="inlineStr">
         <is>
           <t>Aligned Data Centers</t>
         </is>
       </c>
-      <c r="B28" s="73" t="inlineStr">
+      <c r="B28" s="96" t="inlineStr">
         <is>
           <t>$12bn capital raise ($5bn+ new equity + $7bn debt commitments) led by Macquarie (early 2025); later acquired by MGX/BlackRock consortium (~$40bn)</t>
         </is>
       </c>
-      <c r="C28" s="73" t="inlineStr">
+      <c r="C28" s="96" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D28" s="73" t="inlineStr">
+      <c r="D28" s="96" t="inlineStr">
         <is>
           <t>$12bn / $40bn</t>
         </is>
       </c>
-      <c r="E28" s="73" t="inlineStr">
+      <c r="E28" s="96" t="inlineStr">
         <is>
           <t>Infra equity + debt</t>
         </is>
       </c>
-      <c r="F28" s="74" t="inlineStr">
+      <c r="F28" s="97" t="inlineStr">
         <is>
           <t>SFA; NYU DRI</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="69" t="inlineStr">
+      <c r="A29" s="92" t="inlineStr">
         <is>
           <t>QTS (Blackstone)</t>
         </is>
       </c>
-      <c r="B29" s="70" t="inlineStr">
+      <c r="B29" s="93" t="inlineStr">
         <is>
           <t>BX 2025-VOLT SASB CMBS $3.5bn (~10 QTS DCs); + Phoenix ABS (QTS Issuer 2025-1)</t>
         </is>
       </c>
-      <c r="C29" s="70" t="inlineStr">
+      <c r="C29" s="93" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D29" s="70" t="inlineStr">
+      <c r="D29" s="93" t="inlineStr">
         <is>
           <t>$3.5bn+</t>
         </is>
       </c>
-      <c r="E29" s="70" t="inlineStr">
+      <c r="E29" s="93" t="inlineStr">
         <is>
           <t>Securitization (CMBS/ABS)</t>
         </is>
       </c>
-      <c r="F29" s="71" t="inlineStr">
+      <c r="F29" s="94" t="inlineStr">
         <is>
           <t>CREFC; SFA</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="72" t="inlineStr">
+      <c r="A30" s="95" t="inlineStr">
         <is>
           <t>Switch (DigitalBridge)</t>
         </is>
       </c>
-      <c r="B30" s="73" t="inlineStr">
+      <c r="B30" s="96" t="inlineStr">
         <is>
           <t>$2.4bn SASB CMBS (SWCH 2025-DATA) + $1.1bn ABS — green bonds</t>
         </is>
       </c>
-      <c r="C30" s="73" t="inlineStr">
+      <c r="C30" s="96" t="inlineStr">
         <is>
           <t>2024-25</t>
         </is>
       </c>
-      <c r="D30" s="73" t="inlineStr">
+      <c r="D30" s="96" t="inlineStr">
         <is>
           <t>$3.5bn</t>
         </is>
       </c>
-      <c r="E30" s="73" t="inlineStr">
+      <c r="E30" s="96" t="inlineStr">
         <is>
           <t>Securitization (CMBS/ABS)</t>
         </is>
       </c>
-      <c r="F30" s="74" t="inlineStr">
+      <c r="F30" s="97" t="inlineStr">
         <is>
           <t>SFA; CREFC</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="69" t="inlineStr">
+      <c r="A31" s="92" t="inlineStr">
         <is>
           <t>Vantage Data Centers</t>
         </is>
       </c>
-      <c r="B31" s="70" t="inlineStr">
+      <c r="B31" s="93" t="inlineStr">
         <is>
           <t>First public data-center ABS (2024); ongoing multi-billion securitization &amp; infra-equity program</t>
         </is>
       </c>
-      <c r="C31" s="70" t="inlineStr">
+      <c r="C31" s="93" t="inlineStr">
         <is>
           <t>2024-26</t>
         </is>
       </c>
-      <c r="D31" s="70" t="inlineStr">
+      <c r="D31" s="93" t="inlineStr">
         <is>
           <t>multi-$bn</t>
         </is>
       </c>
-      <c r="E31" s="70" t="inlineStr">
+      <c r="E31" s="93" t="inlineStr">
         <is>
           <t>Securitization / equity</t>
         </is>
       </c>
-      <c r="F31" s="71" t="inlineStr">
+      <c r="F31" s="94" t="inlineStr">
         <is>
           <t>Dentons</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="72" t="inlineStr">
+      <c r="A32" s="95" t="inlineStr">
         <is>
           <t>Colocation sector</t>
         </is>
       </c>
-      <c r="B32" s="73" t="inlineStr">
+      <c r="B32" s="96" t="inlineStr">
         <is>
           <t>US data-center ABS+CMBS issuance ~$26bn in 2025 (~10x 2020); ~$57bn since 2021; Morgan Stanley ~$130bn securitized net issuance 2026-28; ~$150bn permanent financing need 2026-27</t>
         </is>
       </c>
-      <c r="C32" s="73" t="inlineStr">
+      <c r="C32" s="96" t="inlineStr">
         <is>
           <t>2025-28</t>
         </is>
       </c>
-      <c r="D32" s="73" t="inlineStr">
+      <c r="D32" s="96" t="inlineStr">
         <is>
           <t>~$130bn</t>
         </is>
       </c>
-      <c r="E32" s="73" t="inlineStr">
+      <c r="E32" s="96" t="inlineStr">
         <is>
           <t>Securitization (ABS/CMBS)</t>
         </is>
       </c>
-      <c r="F32" s="74" t="inlineStr">
+      <c r="F32" s="97" t="inlineStr">
         <is>
           <t>Impax; CREFC; Morgan Stanley</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="69" t="inlineStr">
+      <c r="A33" s="92" t="inlineStr">
         <is>
           <t>HUMAIN (Saudi PIF)</t>
         </is>
       </c>
-      <c r="B33" s="70" t="inlineStr">
+      <c r="B33" s="93" t="inlineStr">
         <is>
           <t>PIF national AI champion (announced 13 May 2025): ~$100bn across 11 data centers / 2.2 GW; ~600k NVIDIA GPUs; ALLAM Arabic LLM</t>
         </is>
       </c>
-      <c r="C33" s="70" t="inlineStr">
+      <c r="C33" s="93" t="inlineStr">
         <is>
           <t>2025-30</t>
         </is>
       </c>
-      <c r="D33" s="70" t="inlineStr">
+      <c r="D33" s="93" t="inlineStr">
         <is>
           <t>~$100bn</t>
         </is>
       </c>
-      <c r="E33" s="70" t="inlineStr">
+      <c r="E33" s="93" t="inlineStr">
         <is>
           <t>Sovereign equity</t>
         </is>
       </c>
-      <c r="F33" s="71" t="inlineStr">
+      <c r="F33" s="94" t="inlineStr">
         <is>
           <t>Presenc AI; NYU DRI</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="72" t="inlineStr">
+      <c r="A34" s="95" t="inlineStr">
         <is>
           <t>Stargate UAE / G42</t>
         </is>
       </c>
-      <c r="B34" s="73" t="inlineStr">
+      <c r="B34" s="96" t="inlineStr">
         <is>
           <t>$30bn+ 5GW Abu Dhabi campus (Khazna/G42 w/ OpenAI, Oracle, NVIDIA, Cisco, SoftBank); Phase 1 200MW Q3 2026; Microsoft ~$1.5bn equity</t>
         </is>
       </c>
-      <c r="C34" s="73" t="inlineStr">
+      <c r="C34" s="96" t="inlineStr">
         <is>
           <t>2025-30</t>
         </is>
       </c>
-      <c r="D34" s="73" t="inlineStr">
+      <c r="D34" s="96" t="inlineStr">
         <is>
           <t>~$30bn+</t>
         </is>
       </c>
-      <c r="E34" s="73" t="inlineStr">
+      <c r="E34" s="96" t="inlineStr">
         <is>
           <t>Sovereign equity + JV</t>
         </is>
       </c>
-      <c r="F34" s="74" t="inlineStr">
+      <c r="F34" s="97" t="inlineStr">
         <is>
           <t>Khaleej Times; dcpulse</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="69" t="inlineStr">
+      <c r="A35" s="92" t="inlineStr">
         <is>
           <t>MGX / Mubadala (UAE)</t>
         </is>
       </c>
-      <c r="B35" s="70" t="inlineStr">
+      <c r="B35" s="93" t="inlineStr">
         <is>
           <t>Anchored Stargate; co-led ~$40bn Aligned Data Centers acquisition w/ BlackRock; AIP (BlackRock-Microsoft) targets up to $100bn global AI infra</t>
         </is>
       </c>
-      <c r="C35" s="70" t="inlineStr">
+      <c r="C35" s="93" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D35" s="70" t="inlineStr">
+      <c r="D35" s="93" t="inlineStr">
         <is>
           <t>~$40bn+</t>
         </is>
       </c>
-      <c r="E35" s="70" t="inlineStr">
+      <c r="E35" s="93" t="inlineStr">
         <is>
           <t>Sovereign equity / infra</t>
         </is>
       </c>
-      <c r="F35" s="71" t="inlineStr">
+      <c r="F35" s="94" t="inlineStr">
         <is>
           <t>NYU DRI</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="72" t="inlineStr">
+      <c r="A36" s="95" t="inlineStr">
         <is>
           <t>Qatar (QIA / Qai)</t>
         </is>
       </c>
-      <c r="B36" s="73" t="inlineStr">
+      <c r="B36" s="96" t="inlineStr">
         <is>
           <t>~$20bn AI-infrastructure JV with Brookfield (late 2025); earlier positions in xAI &amp; Databricks</t>
         </is>
       </c>
-      <c r="C36" s="73" t="inlineStr">
+      <c r="C36" s="96" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D36" s="73" t="inlineStr">
+      <c r="D36" s="96" t="inlineStr">
         <is>
           <t>~$20bn</t>
         </is>
       </c>
-      <c r="E36" s="73" t="inlineStr">
+      <c r="E36" s="96" t="inlineStr">
         <is>
           <t>Sovereign equity + JV</t>
         </is>
       </c>
-      <c r="F36" s="74" t="inlineStr">
+      <c r="F36" s="97" t="inlineStr">
         <is>
           <t>NYU DRI</t>
         </is>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="69" t="inlineStr">
+      <c r="A37" s="92" t="inlineStr">
         <is>
           <t>Sector-wide</t>
         </is>
       </c>
-      <c r="B37" s="70" t="inlineStr">
+      <c r="B37" s="93" t="inlineStr">
         <is>
           <t>HY/unrated AI-infra issuers raised ~$107bn funded+committed debt by ~May 2026 ($68.7bn neoclouds / $38.7bn AI-native DCs)</t>
         </is>
       </c>
-      <c r="C37" s="70" t="inlineStr">
+      <c r="C37" s="93" t="inlineStr">
         <is>
           <t>to 2026</t>
         </is>
       </c>
-      <c r="D37" s="70" t="inlineStr">
+      <c r="D37" s="93" t="inlineStr">
         <is>
           <t>~$107bn</t>
         </is>
       </c>
-      <c r="E37" s="70" t="inlineStr">
+      <c r="E37" s="93" t="inlineStr">
         <is>
           <t>All debt</t>
         </is>
       </c>
-      <c r="F37" s="71" t="inlineStr">
+      <c r="F37" s="94" t="inlineStr">
         <is>
           <t>Octus</t>
         </is>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="72" t="inlineStr">
+      <c r="A38" s="95" t="inlineStr">
         <is>
           <t>Sector-wide</t>
         </is>
       </c>
-      <c r="B38" s="73" t="inlineStr">
+      <c r="B38" s="96" t="inlineStr">
         <is>
           <t>Insurance-linked platforms deployed ~$180bn into private credit in 2025 (~25% of global private credit AUM)</t>
         </is>
       </c>
-      <c r="C38" s="73" t="inlineStr">
+      <c r="C38" s="96" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D38" s="73" t="inlineStr">
+      <c r="D38" s="96" t="inlineStr">
         <is>
           <t>~$180bn</t>
         </is>
       </c>
-      <c r="E38" s="73" t="inlineStr">
+      <c r="E38" s="96" t="inlineStr">
         <is>
           <t>Insurance / private credit</t>
         </is>
       </c>
-      <c r="F38" s="74" t="inlineStr">
+      <c r="F38" s="97" t="inlineStr">
         <is>
           <t>McKinsey; ABF Journal</t>
         </is>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="69" t="inlineStr">
+      <c r="A39" s="92" t="inlineStr">
         <is>
           <t>Sector-wide</t>
         </is>
       </c>
-      <c r="B39" s="70" t="inlineStr">
+      <c r="B39" s="93" t="inlineStr">
         <is>
           <t>Goldman Sachs: ~$5.3tn AI + data-center capex 2025-2030; Morgan Stanley: ~$800bn private credit for AI DCs 2025-28</t>
         </is>
       </c>
-      <c r="C39" s="70" t="inlineStr">
+      <c r="C39" s="93" t="inlineStr">
         <is>
           <t>2025-30</t>
         </is>
       </c>
-      <c r="D39" s="70" t="inlineStr">
+      <c r="D39" s="93" t="inlineStr">
         <is>
           <t>$5.3tn capex</t>
         </is>
       </c>
-      <c r="E39" s="70" t="inlineStr">
+      <c r="E39" s="93" t="inlineStr">
         <is>
           <t>Context</t>
         </is>
       </c>
-      <c r="F39" s="71" t="inlineStr">
+      <c r="F39" s="94" t="inlineStr">
         <is>
           <t>Goldman; Morgan Stanley</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="75" t="inlineStr">
+      <c r="A41" s="98" t="inlineStr">
         <is>
           <t>Selected sources:</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="76" t="inlineStr">
+      <c r="A42" s="99" t="inlineStr">
         <is>
           <t>Goldman Sachs Research — ~$5.3tn AI + data-center capex 2025-2030; private markets in DC financing.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="76" t="inlineStr">
+      <c r="A43" s="99" t="inlineStr">
         <is>
           <t>Morgan Stanley — ~$2tn capex 2025-28 with &gt;$1tn debt; ~$800bn private credit for AI DCs.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="76" t="inlineStr">
+      <c r="A44" s="99" t="inlineStr">
         <is>
           <t>Bank of America / BofA Securities — hyperscaler bond issuance ($121bn 2025; ~$175bn 2026E).</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="76" t="inlineStr">
+      <c r="A45" s="99" t="inlineStr">
         <is>
           <t>Moody's Ratings — hyperscaler capex (~$785bn 2026, ~$1tn 2027); $662bn off-B/S DC leases.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="76" t="inlineStr">
+      <c r="A46" s="99" t="inlineStr">
         <is>
           <t>McKinsey — ~$2.7tn US (5.2tn global) data-center capex by 2030; insurance-linked private credit.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="76" t="inlineStr">
+      <c r="A47" s="99" t="inlineStr">
         <is>
           <t>Octus — HY/unrated AI-infra debt (~$107bn to ~May 2026); ~14GW unfunded ≈ $344bn need.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="76" t="inlineStr">
+      <c r="A48" s="99" t="inlineStr">
         <is>
           <t>Company disclosures &amp; press: Meta IR / FT / S&amp;P (Hyperion); Oracle IR / IFR / Reuters; CoreWeave IR;</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="76" t="inlineStr">
+      <c r="A49" s="99" t="inlineStr">
         <is>
           <t xml:space="preserve">  CNBC / WSJ / The Information (xAI); Blackstone; Apollo Academy; MUFG; CreditSights; CNA.</t>
         </is>

</xml_diff>

<commit_message>
Merge Private Credit and Key Deals tabs into unified Deals & Sources tab
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AI_Infrastructure_Financing_2025-2030.xlsx
+++ b/AI_Infrastructure_Financing_2025-2030.xlsx
@@ -12,8 +12,7 @@
     <sheet name="Debt by Type" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Cash-Flow Bridge" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Capex Projections" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Private Credit Deals" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Key Deals &amp; Sources" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Deals &amp; Sources" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1"/>
@@ -156,7 +155,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -223,11 +222,6 @@
         <fgColor rgb="00F0F0F0"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -255,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -478,23 +472,29 @@
     <xf numFmtId="0" fontId="28" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1334,7 +1334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B72"/>
+  <dimension ref="B2:B71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1400,397 +1400,390 @@
     <row r="11">
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>• Private Credit Deals: transaction log of private-credit / SPV / 144A debt for AI infra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>• Key Deals &amp; Sources: notable disclosed transactions underpinning the estimates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="6" t="inlineStr">
+          <t>• Deals &amp; Sources: private-credit transactions + other key deals (bonds, equity, etc.) + sources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Scope &amp; definitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>• Hyperscalers: Microsoft, Amazon (AWS), Alphabet (Google), Meta, Oracle (OCI).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>• Hyperscalers: Microsoft, Amazon (AWS), Alphabet (Google), Meta, Oracle (OCI).</t>
+          <t>• Neoclouds / AI-native infra: GPU-cloud &amp; AI-native data-center builders (CoreWeave,</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>• Neoclouds / AI-native infra: GPU-cloud &amp; AI-native data-center builders (CoreWeave,</t>
+          <t xml:space="preserve">   SpaceX/xAI, Nebius, IREN, Crusoe, Lambda, Fluidstack, Nscale, + an 'Other' aggregate).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   SpaceX/xAI, Nebius, IREN, Crusoe, Lambda, Fluidstack, Nscale, + an 'Other' aggregate).</t>
+          <t>• SpaceX acquired xAI (effective 2 Feb 2026), so Colossus I &amp; II are now SpaceX-owned; the two</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>• SpaceX acquired xAI (effective 2 Feb 2026), so Colossus I &amp; II are now SpaceX-owned; the two</t>
+          <t xml:space="preserve">   are shown as one consolidated 'SpaceX / xAI' line to avoid double-counting the same clusters.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   are shown as one consolidated 'SpaceX / xAI' line to avoid double-counting the same clusters.</t>
+          <t>• Colocation / data-center REITs: wholesale &amp; retail colo / powered-shell owners (Equinix,</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>• Colocation / data-center REITs: wholesale &amp; retail colo / powered-shell owners (Equinix,</t>
+          <t xml:space="preserve">   Digital Realty, QTS, Vantage, Aligned, CyrusOne, Switch, Stack, + 'Other') that build campuses</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Digital Realty, QTS, Vantage, Aligned, CyrusOne, Switch, Stack, + 'Other') that build campuses</t>
+          <t xml:space="preserve">   and lease them to hyperscalers / neoclouds; heavy users of ABS/CMBS securitization &amp; infra equity.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   and lease them to hyperscalers / neoclouds; heavy users of ABS/CMBS securitization &amp; infra equity.</t>
+          <t>• Sovereign clouds: state / sovereign-wealth-funded national AI infrastructure (HUMAIN-Saudi PIF,</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>• Sovereign clouds: state / sovereign-wealth-funded national AI infrastructure (HUMAIN-Saudi PIF,</t>
+          <t xml:space="preserve">   MGX/Mubadala, Stargate UAE/G42/Khazna, Qatar QIA, EU/France, India, + 'Other'); mostly equity-funded.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   MGX/Mubadala, Stargate UAE/G42/Khazna, Qatar QIA, EU/France, India, + 'Other'); mostly equity-funded.</t>
+          <t>• Funding sources now split three ways:  Capex = Operating cash flow (self-funded) +</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>• Funding sources now split three ways:  Capex = Operating cash flow (self-funded) +</t>
+          <t xml:space="preserve">   External equity + Total debt.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   External equity + Total debt.</t>
+          <t xml:space="preserve">   - Operating cash flow (self-funded): internally-generated cash (CFO) reinvested into AI capex.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Operating cash flow (self-funded): internally-generated cash (CFO) reinvested into AI capex.</t>
+          <t xml:space="preserve">   - External equity: IPOs, secondaries, strategic stakes (e.g. NVIDIA), ATM programs, sovereign-</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - External equity: IPOs, secondaries, strategic stakes (e.g. NVIDIA), ATM programs, sovereign-</t>
+          <t xml:space="preserve">     wealth equity and mandatory convertible PREFERRED (treated as equity).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">     wealth equity and mandatory convertible PREFERRED (treated as equity).</t>
+          <t xml:space="preserve">   - Total debt: external borrowing, split by instrument (see below).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Total debt: external borrowing, split by instrument (see below).</t>
+          <t>• The 'Cash-Flow Bridge' sheet separates OPERATING CASH FLOW (CFO) and FREE CASH FLOW from the</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>• The 'Cash-Flow Bridge' sheet separates OPERATING CASH FLOW (CFO) and FREE CASH FLOW from the</t>
+          <t xml:space="preserve">   equity portion:  CFO - dividends/buybacks/other = self-funded capex; FREE CASH FLOW = CFO -</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   equity portion:  CFO - dividends/buybacks/other = self-funded capex; FREE CASH FLOW = CFO -</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="5" t="inlineStr">
-        <is>
           <t xml:space="preserve">   AI capex (negative for most builders, which is what drives external equity + debt issuance).</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="B35" s="7" t="inlineStr">
+    <row r="34" ht="20" customHeight="1">
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>Debt instrument buckets (mutually exclusive — they sum to total debt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>1. Corporate bonds (public IG/HY) — on-balance-sheet senior notes sold in public markets.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>1. Corporate bonds (public IG/HY) — on-balance-sheet senior notes sold in public markets.</t>
+          <t>2. Bank &amp; syndicated loans — term loans, revolvers, delayed-draw term loans (incl. GPU-backed DDTLs).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2. Bank &amp; syndicated loans — term loans, revolvers, delayed-draw term loans (incl. GPU-backed DDTLs).</t>
+          <t>3. Alternate private credit — direct lending / private placements by credit funds (Blackstone,</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>3. Alternate private credit — direct lending / private placements by credit funds (Blackstone,</t>
+          <t xml:space="preserve">   Apollo, Blue Owl, PIMCO, Magnetar, etc.), including privately-placed SPV/project debt.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Apollo, Blue Owl, PIMCO, Magnetar, etc.), including privately-placed SPV/project debt.</t>
+          <t>4. Insurance-linked lending — debt funded off insurer/annuity balance sheets (Athene/Apollo,</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>4. Insurance-linked lending — debt funded off insurer/annuity balance sheets (Athene/Apollo,</t>
+          <t xml:space="preserve">   Global Atlantic/KKR, MetLife, Brookfield, etc.). NOTE: large overlap with private credit &amp;</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Global Atlantic/KKR, MetLife, Brookfield, etc.). NOTE: large overlap with private credit &amp;</t>
+          <t xml:space="preserve">   bonds; shown separately to size the insurance channel — see double-counting note below.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   bonds; shown separately to size the insurance channel — see double-counting note below.</t>
+          <t>5. Securitization / ABS / CMBS — secured data-center bonds &amp; GPU-backed asset-backed securities.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>5. Securitization / ABS / CMBS — secured data-center bonds &amp; GPU-backed asset-backed securities.</t>
+          <t>6. Convertibles / equity-linked debt — convertible notes (excludes mandatory convert. PREFERRED).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>6. Convertibles / equity-linked debt — convertible notes (excludes mandatory convert. PREFERRED).</t>
+          <t>7. Vendor &amp; equipment-lease financing — chip/equipment leases &amp; sale-leasebacks (e.g. NVIDIA</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>7. Vendor &amp; equipment-lease financing — chip/equipment leases &amp; sale-leasebacks (e.g. NVIDIA</t>
+          <t xml:space="preserve">   chip-lease SPVs, finance leases). Microsoft's large finance-lease book sits largely here.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   chip-lease SPVs, finance leases). Microsoft's large finance-lease book sits largely here.</t>
+          <t>Memo: 'Off-B/S SPV / JV (memo)' flags the portion routed through special-purpose vehicles /</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Memo: 'Off-B/S SPV / JV (memo)' flags the portion routed through special-purpose vehicles /</t>
+          <t xml:space="preserve">   joint ventures (e.g. Meta-Hyperion, xAI Colossus 2, Oracle project SPVs). It OVERLAPS the</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   joint ventures (e.g. Meta-Hyperion, xAI Colossus 2, Oracle project SPVs). It OVERLAPS the</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="5" t="inlineStr">
-        <is>
           <t xml:space="preserve">   buckets above and is therefore NOT added into the debt total.</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="B51" s="8" t="inlineStr">
+    <row r="50" ht="20" customHeight="1">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>Methodology &amp; caveats</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>• Figures are RESEARCH ESTIMATES for the cumulative 2025-2030 buildout. They blend disclosed</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>• Figures are RESEARCH ESTIMATES for the cumulative 2025-2030 buildout. They blend disclosed</t>
+          <t xml:space="preserve">  transactions (2023-early 2026) with forward projections; they are illustrative, not audited.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  transactions (2023-early 2026) with forward projections; they are illustrative, not audited.</t>
+          <t>• Aggregate cross-check: total financing ≈ $5.25tn, consistent with Goldman Sachs' ~$5.3tn</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>• Aggregate cross-check: total financing ≈ $5.25tn, consistent with Goldman Sachs' ~$5.3tn</t>
+          <t xml:space="preserve">  2025-2030 AI + data-center capex estimate; aggregate debt ≈ $1.8tn, consistent with Morgan</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2025-2030 AI + data-center capex estimate; aggregate debt ≈ $1.8tn, consistent with Morgan</t>
+          <t xml:space="preserve">  Stanley / BofA projections of $1-2tn of debt financing for the buildout.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stanley / BofA projections of $1-2tn of debt financing for the buildout.</t>
+          <t>• CROSS-SEGMENT OVERLAP: hyperscalers LEASE much colocation capacity (so colo financing partly</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>• CROSS-SEGMENT OVERLAP: hyperscalers LEASE much colocation capacity (so colo financing partly</t>
+          <t xml:space="preserve">  funds the same capacity hyperscalers report as off-B/S leases), and sovereign-wealth funds</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  funds the same capacity hyperscalers report as off-B/S leases), and sovereign-wealth funds</t>
+          <t xml:space="preserve">  (MGX, PIF, QIA) also INVEST in neoclouds/labs and colo (e.g. MGX/BlackRock bought Aligned; PIF</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (MGX, PIF, QIA) also INVEST in neoclouds/labs and colo (e.g. MGX/BlackRock bought Aligned; PIF</t>
+          <t xml:space="preserve">  put ~$3bn into xAI). The all-segment 'grand total' is therefore a GROSS figure of capital raised</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  put ~$3bn into xAI). The all-segment 'grand total' is therefore a GROSS figure of capital raised</t>
+          <t xml:space="preserve">  across distinct balance sheets and is not strictly additive; treat it as an upper-bound view.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  across distinct balance sheets and is not strictly additive; treat it as an upper-bound view.</t>
+          <t xml:space="preserve">  Hyperscaler + Neocloud financing (~$5.4tn) ties to Goldman's ~$5.3tn big-tech capex; adding</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Hyperscaler + Neocloud financing (~$5.4tn) ties to Goldman's ~$5.3tn big-tech capex; adding</t>
+          <t xml:space="preserve">  third-party colo + sovereign brings the gross total toward broader ~$6-7tn AI-infra estimates.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  third-party colo + sovereign brings the gross total toward broader ~$6-7tn AI-infra estimates.</t>
+          <t>• Insurance-linked lending double counts with private credit/bonds at the capital-source level;</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>• Insurance-linked lending double counts with private credit/bonds at the capital-source level;</t>
+          <t xml:space="preserve">  to avoid inflating totals, each dollar of debt is classified ONCE by its primary instrument and</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  to avoid inflating totals, each dollar of debt is classified ONCE by its primary instrument and</t>
+          <t xml:space="preserve">  the insurance bucket captures only directly insurer-originated / insurance-balance-sheet debt.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  the insurance bucket captures only directly insurer-originated / insurance-balance-sheet debt.</t>
+          <t>• Company splits reflect observed behavior: Microsoft/Alphabet/Amazon are FCF-heavy with</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>• Company splits reflect observed behavior: Microsoft/Alphabet/Amazon are FCF-heavy with</t>
+          <t xml:space="preserve">  selective bonds; Meta &amp; Oracle lean more on debt &amp; SPVs; neoclouds are debt-heavy (asset-backed).</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  selective bonds; Meta &amp; Oracle lean more on debt &amp; SPVs; neoclouds are debt-heavy (asset-backed).</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" s="5" t="inlineStr">
-        <is>
           <t>• Built with openpyxl. See Key Deals &amp; Sources sheet for citations.</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="30" customHeight="1">
-      <c r="B72" s="9" t="inlineStr">
+    <row r="71" ht="30" customHeight="1">
+      <c r="B71" s="9" t="inlineStr">
         <is>
           <t>Disclaimer: For analytical/illustrative purposes only. Not investment advice and not a representation of any company's actual financing. Verify against primary filings before use.</t>
         </is>
@@ -8150,32 +8143,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>Private Credit Transactions — AI Infrastructure (US$bn)</t>
+          <t>AI-Infrastructure Deals — Private Credit &amp; Other Key Transactions (US$bn)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Transaction log of private-credit / SPV / private-placement (144A) debt for AI infra. Itemized deals are summed; 'Context / market' rows (frameworks, projections) are not.</t>
+          <t>Unified transaction log. Section 1: private-credit / SPV / 144A debt (itemized deals summed). Section 2: context/frameworks. Section 3: other key deals (bonds, equity, securitization, sovereign, leases). Amounts '~' = approximate.</t>
         </is>
       </c>
     </row>
@@ -8233,165 +8226,131 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="70" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>1) PRIVATE CREDIT TRANSACTIONS (itemized — summed below)</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n"/>
+      <c r="C5" s="15" t="n"/>
+      <c r="D5" s="15" t="n"/>
+      <c r="E5" s="15" t="n"/>
+      <c r="F5" s="15" t="n"/>
+      <c r="G5" s="15" t="n"/>
+      <c r="H5" s="15" t="n"/>
+      <c r="I5" s="15" t="n"/>
+      <c r="J5" s="15" t="n"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="70" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="B5" s="71" t="inlineStr">
+      <c r="B6" s="71" t="inlineStr">
         <is>
           <t>Oracle — Texas + Wisconsin data centers</t>
         </is>
       </c>
-      <c r="C5" s="72" t="inlineStr">
+      <c r="C6" s="72" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="D5" s="70" t="inlineStr">
+      <c r="D6" s="70" t="inlineStr">
         <is>
           <t>Private credit consortium</t>
         </is>
       </c>
-      <c r="E5" s="73" t="n">
+      <c r="E6" s="73" t="n">
         <v>38</v>
       </c>
-      <c r="F5" s="70" t="inlineStr">
+      <c r="F6" s="70" t="inlineStr">
         <is>
           <t>SPV debt package</t>
         </is>
       </c>
-      <c r="G5" s="70" t="inlineStr">
+      <c r="G6" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H5" s="70" t="inlineStr">
+      <c r="H6" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I5" s="70" t="inlineStr">
+      <c r="I6" s="70" t="inlineStr">
         <is>
           <t>Two-site off-B/S financing</t>
         </is>
       </c>
-      <c r="J5" s="74" t="inlineStr">
+      <c r="J6" s="74" t="inlineStr">
         <is>
           <t>FT</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="75" t="inlineStr">
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="75" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="B6" s="76" t="inlineStr">
+      <c r="B7" s="76" t="inlineStr">
         <is>
           <t>Anthropic — Google TPU chip SPV</t>
         </is>
       </c>
-      <c r="C6" s="77" t="inlineStr">
+      <c r="C7" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D6" s="75" t="inlineStr">
+      <c r="D7" s="75" t="inlineStr">
         <is>
           <t>Apollo (Atlas SP $0.8bn equity; Athene), Blackstone; Broadcom RVG</t>
         </is>
       </c>
-      <c r="E6" s="78" t="n">
+      <c r="E7" s="78" t="n">
         <v>35</v>
       </c>
-      <c r="F6" s="75" t="inlineStr">
+      <c r="F7" s="75" t="inlineStr">
         <is>
           <t>Chip-leasing SPV; 3 tranches; ~half syndicated</t>
         </is>
       </c>
-      <c r="G6" s="75" t="inlineStr">
+      <c r="G7" s="75" t="inlineStr">
         <is>
           <t>A1 T+100bp; A2 5.75%; B 8.5%</t>
         </is>
       </c>
-      <c r="H6" s="75" t="inlineStr">
+      <c r="H7" s="75" t="inlineStr">
         <is>
           <t>~5y</t>
         </is>
       </c>
-      <c r="I6" s="75" t="inlineStr">
+      <c r="I7" s="75" t="inlineStr">
         <is>
           <t>Buys Google TPUs leased to Anthropic; Broadcom residual-value support</t>
         </is>
       </c>
-      <c r="J6" s="79" t="inlineStr">
+      <c r="J7" s="79" t="inlineStr">
         <is>
           <t>privatedebtnews; Build.inc</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="70" t="inlineStr">
-        <is>
-          <t>Oct 2025</t>
-        </is>
-      </c>
-      <c r="B7" s="71" t="inlineStr">
-        <is>
-          <t>Meta — Hyperion (Beignet Investor LLC), Louisiana</t>
-        </is>
-      </c>
-      <c r="C7" s="72" t="inlineStr">
-        <is>
-          <t>Hyperscaler</t>
-        </is>
-      </c>
-      <c r="D7" s="70" t="inlineStr">
-        <is>
-          <t>PIMCO (~$18bn), BlackRock, Apollo (debt); Blue Owl (equity); MS adviser</t>
-        </is>
-      </c>
-      <c r="E7" s="73" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="F7" s="70" t="inlineStr">
-        <is>
-          <t>Off-B/S SPV; 144A senior secured bond</t>
-        </is>
-      </c>
-      <c r="G7" s="70" t="inlineStr">
-        <is>
-          <t>6.581% / T+225bp</t>
-        </is>
-      </c>
-      <c r="H7" s="70" t="inlineStr">
-        <is>
-          <t>Due May 2049 (~23.6y)</t>
-        </is>
-      </c>
-      <c r="I7" s="70" t="inlineStr">
-        <is>
-          <t>2.1GW campus; Meta lease + residual-value guarantee (up to ~$28bn); A+ (S&amp;P)</t>
-        </is>
-      </c>
-      <c r="J7" s="74" t="inlineStr">
-        <is>
-          <t>IFR; FT; Quinn Emanuel</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="70" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>Oct 2025</t>
         </is>
       </c>
       <c r="B8" s="71" t="inlineStr">
         <is>
-          <t>Oracle — New Mexico site</t>
+          <t>Meta — Hyperion (Beignet Investor LLC), Louisiana</t>
         </is>
       </c>
       <c r="C8" s="72" t="inlineStr">
@@ -8401,547 +8360,547 @@
       </c>
       <c r="D8" s="70" t="inlineStr">
         <is>
-          <t>Private credit lenders</t>
+          <t>PIMCO (~$18bn), BlackRock, Apollo (debt); Blue Owl (equity); MS adviser</t>
         </is>
       </c>
       <c r="E8" s="73" t="n">
-        <v>18</v>
+        <v>27.3</v>
       </c>
       <c r="F8" s="70" t="inlineStr">
         <is>
-          <t>SPV / project loan</t>
+          <t>Off-B/S SPV; 144A senior secured bond</t>
         </is>
       </c>
       <c r="G8" s="70" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>6.581% / T+225bp</t>
         </is>
       </c>
       <c r="H8" s="70" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Due May 2049 (~23.6y)</t>
         </is>
       </c>
       <c r="I8" s="70" t="inlineStr">
         <is>
-          <t>Single-site project loan</t>
+          <t>2.1GW campus; Meta lease + residual-value guarantee (up to ~$28bn); A+ (S&amp;P)</t>
         </is>
       </c>
       <c r="J8" s="74" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>IFR; FT; Quinn Emanuel</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="70" t="inlineStr">
         <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B9" s="71" t="inlineStr">
+        <is>
+          <t>Oracle — New Mexico site</t>
+        </is>
+      </c>
+      <c r="C9" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D9" s="70" t="inlineStr">
+        <is>
+          <t>Private credit lenders</t>
+        </is>
+      </c>
+      <c r="E9" s="73" t="n">
+        <v>18</v>
+      </c>
+      <c r="F9" s="70" t="inlineStr">
+        <is>
+          <t>SPV / project loan</t>
+        </is>
+      </c>
+      <c r="G9" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H9" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I9" s="70" t="inlineStr">
+        <is>
+          <t>Single-site project loan</t>
+        </is>
+      </c>
+      <c r="J9" s="74" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="70" t="inlineStr">
+        <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B9" s="71" t="inlineStr">
+      <c r="B10" s="71" t="inlineStr">
         <is>
           <t>Oracle — Michigan campus</t>
         </is>
       </c>
-      <c r="C9" s="72" t="inlineStr">
+      <c r="C10" s="72" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="D9" s="70" t="inlineStr">
+      <c r="D10" s="70" t="inlineStr">
         <is>
           <t>Project-finance lenders</t>
         </is>
       </c>
-      <c r="E9" s="73" t="n">
+      <c r="E10" s="73" t="n">
         <v>16.3</v>
       </c>
-      <c r="F9" s="70" t="inlineStr">
+      <c r="F10" s="70" t="inlineStr">
         <is>
           <t>Project-level SPV financing</t>
         </is>
       </c>
-      <c r="G9" s="70" t="inlineStr">
+      <c r="G10" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H9" s="70" t="inlineStr">
+      <c r="H10" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I9" s="70" t="inlineStr">
+      <c r="I10" s="70" t="inlineStr">
         <is>
           <t>OCI capacity build</t>
         </is>
       </c>
-      <c r="J9" s="74" t="inlineStr">
+      <c r="J10" s="74" t="inlineStr">
         <is>
           <t>Press reports</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="75" t="inlineStr">
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="75" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="B10" s="76" t="inlineStr">
+      <c r="B11" s="76" t="inlineStr">
         <is>
           <t>xAI — Colossus 2 chip SPV (Memphis/Southaven)</t>
         </is>
       </c>
-      <c r="C10" s="77" t="inlineStr">
+      <c r="C11" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D10" s="75" t="inlineStr">
+      <c r="D11" s="75" t="inlineStr">
         <is>
           <t>Valor Equity (lead), Apollo, Diameter (debt); NVIDIA up to $2bn equity</t>
         </is>
       </c>
-      <c r="E10" s="78" t="n">
+      <c r="E11" s="78" t="n">
         <v>12.5</v>
       </c>
-      <c r="F10" s="75" t="inlineStr">
+      <c r="F11" s="75" t="inlineStr">
         <is>
           <t>SPV; debt + ~$7.5bn equity to buy &amp; lease GPUs</t>
         </is>
       </c>
-      <c r="G10" s="75" t="inlineStr">
+      <c r="G11" s="75" t="inlineStr">
         <is>
           <t>~10.5%</t>
         </is>
       </c>
-      <c r="H10" s="75" t="inlineStr">
+      <c r="H11" s="75" t="inlineStr">
         <is>
           <t>5y (~2.5y avg life)</t>
         </is>
       </c>
-      <c r="I10" s="75" t="inlineStr">
+      <c r="I11" s="75" t="inlineStr">
         <is>
           <t>Buys NVIDIA GPUs leased to xAI; chips as collateral</t>
         </is>
       </c>
-      <c r="J10" s="79" t="inlineStr">
+      <c r="J11" s="79" t="inlineStr">
         <is>
           <t>FT; WSJ; AAE filing</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="70" t="inlineStr">
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="70" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B11" s="71" t="inlineStr">
+      <c r="B12" s="71" t="inlineStr">
         <is>
           <t>Oracle/OpenAI — Abilene, TX (Stargate; Crusoe developer)</t>
         </is>
       </c>
-      <c r="C11" s="72" t="inlineStr">
+      <c r="C12" s="72" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="D11" s="70" t="inlineStr">
+      <c r="D12" s="70" t="inlineStr">
         <is>
           <t>Blue Owl + JPMorgan (incl. Crusoe, Primary Digital Infrastructure)</t>
         </is>
       </c>
-      <c r="E11" s="73" t="n">
+      <c r="E12" s="73" t="n">
         <v>10</v>
       </c>
-      <c r="F11" s="70" t="inlineStr">
+      <c r="F12" s="70" t="inlineStr">
         <is>
           <t>Off-B/S SPV (~$13bn incl. equity)</t>
         </is>
       </c>
-      <c r="G11" s="70" t="inlineStr">
+      <c r="G12" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H11" s="70" t="inlineStr">
+      <c r="H12" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I11" s="70" t="inlineStr">
+      <c r="I12" s="70" t="inlineStr">
         <is>
           <t>SPV owns OpenAI Abilene facility</t>
         </is>
       </c>
-      <c r="J11" s="74" t="inlineStr">
+      <c r="J12" s="74" t="inlineStr">
         <is>
           <t>FT</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="75" t="inlineStr">
-        <is>
-          <t>Mar 2026</t>
-        </is>
-      </c>
-      <c r="B12" s="76" t="inlineStr">
-        <is>
-          <t>CoreWeave — DDTL 4.0 (Compute Acq. Co. VIII)</t>
-        </is>
-      </c>
-      <c r="C12" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D12" s="75" t="inlineStr">
-        <is>
-          <t>Blackstone Credit &amp; Insurance (anchor); MUFG, MS, GS, JPM</t>
-        </is>
-      </c>
-      <c r="E12" s="78" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="F12" s="75" t="inlineStr">
-        <is>
-          <t>Non-recourse GPU-backed delayed-draw term loan</t>
-        </is>
-      </c>
-      <c r="G12" s="75" t="inlineStr">
-        <is>
-          <t>SOFR+225 / ~5.9% fixed</t>
-        </is>
-      </c>
-      <c r="H12" s="75" t="inlineStr">
-        <is>
-          <t>Mar 2032</t>
-        </is>
-      </c>
-      <c r="I12" s="75" t="inlineStr">
-        <is>
-          <t>First IG-rated (A3 / A low) HPC-collateralized loan</t>
-        </is>
-      </c>
-      <c r="J12" s="79" t="inlineStr">
-        <is>
-          <t>CoreWeave IR</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="75" t="inlineStr">
         <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B13" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — DDTL 4.0 (Compute Acq. Co. VIII)</t>
+        </is>
+      </c>
+      <c r="C13" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D13" s="75" t="inlineStr">
+        <is>
+          <t>Blackstone Credit &amp; Insurance (anchor); MUFG, MS, GS, JPM</t>
+        </is>
+      </c>
+      <c r="E13" s="78" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="F13" s="75" t="inlineStr">
+        <is>
+          <t>Non-recourse GPU-backed delayed-draw term loan</t>
+        </is>
+      </c>
+      <c r="G13" s="75" t="inlineStr">
+        <is>
+          <t>SOFR+225 / ~5.9% fixed</t>
+        </is>
+      </c>
+      <c r="H13" s="75" t="inlineStr">
+        <is>
+          <t>Mar 2032</t>
+        </is>
+      </c>
+      <c r="I13" s="75" t="inlineStr">
+        <is>
+          <t>First IG-rated (A3 / A low) HPC-collateralized loan</t>
+        </is>
+      </c>
+      <c r="J13" s="79" t="inlineStr">
+        <is>
+          <t>CoreWeave IR</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="75" t="inlineStr">
+        <is>
           <t>May 2024</t>
         </is>
       </c>
-      <c r="B13" s="76" t="inlineStr">
+      <c r="B14" s="76" t="inlineStr">
         <is>
           <t>CoreWeave — $7.5bn debt facility</t>
         </is>
       </c>
-      <c r="C13" s="77" t="inlineStr">
+      <c r="C14" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D13" s="75" t="inlineStr">
+      <c r="D14" s="75" t="inlineStr">
         <is>
           <t>Blackstone, Magnetar (co-leads), Coatue, Carlyle, CDPQ, BlackRock, Eldridge</t>
         </is>
       </c>
-      <c r="E13" s="78" t="n">
+      <c r="E14" s="78" t="n">
         <v>7.5</v>
       </c>
-      <c r="F13" s="75" t="inlineStr">
+      <c r="F14" s="75" t="inlineStr">
         <is>
           <t>GPU + customer-contract secured facility</t>
         </is>
       </c>
-      <c r="G13" s="75" t="inlineStr">
+      <c r="G14" s="75" t="inlineStr">
         <is>
           <t>~10%+ (at issue)</t>
         </is>
       </c>
-      <c r="H13" s="75" t="inlineStr">
+      <c r="H14" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I13" s="75" t="inlineStr">
+      <c r="I14" s="75" t="inlineStr">
         <is>
           <t>Largest private debt deal at the time</t>
         </is>
       </c>
-      <c r="J13" s="79" t="inlineStr">
+      <c r="J14" s="79" t="inlineStr">
         <is>
           <t>Blackstone</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="80" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="80" t="inlineStr">
         <is>
           <t>Early 2025</t>
         </is>
       </c>
-      <c r="B14" s="81" t="inlineStr">
+      <c r="B15" s="81" t="inlineStr">
         <is>
           <t>Aligned Data Centers — debt commitments</t>
         </is>
       </c>
-      <c r="C14" s="82" t="inlineStr">
+      <c r="C15" s="82" t="inlineStr">
         <is>
           <t>Colocation / data-center REIT</t>
         </is>
       </c>
-      <c r="D14" s="80" t="inlineStr">
+      <c r="D15" s="80" t="inlineStr">
         <is>
           <t>Macquarie + global investors</t>
         </is>
       </c>
-      <c r="E14" s="83" t="n">
+      <c r="E15" s="83" t="n">
         <v>7</v>
       </c>
-      <c r="F14" s="80" t="inlineStr">
+      <c r="F15" s="80" t="inlineStr">
         <is>
           <t>Debt within $12bn raise (+$5bn equity)</t>
         </is>
       </c>
-      <c r="G14" s="80" t="inlineStr">
+      <c r="G15" s="80" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H14" s="80" t="inlineStr">
+      <c r="H15" s="80" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I14" s="80" t="inlineStr">
+      <c r="I15" s="80" t="inlineStr">
         <is>
           <t>Later acquired by MGX/BlackRock (~$40bn)</t>
         </is>
       </c>
-      <c r="J14" s="84" t="inlineStr">
+      <c r="J15" s="84" t="inlineStr">
         <is>
           <t>SFA; NYU DRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="75" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B15" s="76" t="inlineStr">
-        <is>
-          <t>Fluidstack — Google-backed facility</t>
-        </is>
-      </c>
-      <c r="C15" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D15" s="75" t="inlineStr">
-        <is>
-          <t>Private credit (Google lease backstop)</t>
-        </is>
-      </c>
-      <c r="E15" s="78" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="F15" s="75" t="inlineStr">
-        <is>
-          <t>SPV backed by contracted revenue</t>
-        </is>
-      </c>
-      <c r="G15" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H15" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I15" s="75" t="inlineStr">
-        <is>
-          <t>~$6.7bn Google-contracted revenue backstop</t>
-        </is>
-      </c>
-      <c r="J15" s="79" t="inlineStr">
-        <is>
-          <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="75" t="inlineStr">
         <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B16" s="76" t="inlineStr">
+        <is>
+          <t>Fluidstack — Google-backed facility</t>
+        </is>
+      </c>
+      <c r="C16" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D16" s="75" t="inlineStr">
+        <is>
+          <t>Private credit (Google lease backstop)</t>
+        </is>
+      </c>
+      <c r="E16" s="78" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="F16" s="75" t="inlineStr">
+        <is>
+          <t>SPV backed by contracted revenue</t>
+        </is>
+      </c>
+      <c r="G16" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H16" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I16" s="75" t="inlineStr">
+        <is>
+          <t>~$6.7bn Google-contracted revenue backstop</t>
+        </is>
+      </c>
+      <c r="J16" s="79" t="inlineStr">
+        <is>
+          <t>theaiinsider</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="75" t="inlineStr">
+        <is>
           <t>Jun-Jul 2025</t>
         </is>
       </c>
-      <c r="B16" s="76" t="inlineStr">
+      <c r="B17" s="76" t="inlineStr">
         <is>
           <t>xAI — secured notes / term loan (part of $10bn raise)</t>
         </is>
       </c>
-      <c r="C16" s="77" t="inlineStr">
+      <c r="C17" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D16" s="75" t="inlineStr">
+      <c r="D17" s="75" t="inlineStr">
         <is>
           <t>Apollo, Diameter; Morgan Stanley arranger</t>
         </is>
       </c>
-      <c r="E16" s="78" t="n">
+      <c r="E17" s="78" t="n">
         <v>5</v>
       </c>
-      <c r="F16" s="75" t="inlineStr">
+      <c r="F17" s="75" t="inlineStr">
         <is>
           <t>Secured notes + term loan</t>
         </is>
       </c>
-      <c r="G16" s="75" t="inlineStr">
+      <c r="G17" s="75" t="inlineStr">
         <is>
           <t>up to ~12.5%</t>
         </is>
       </c>
-      <c r="H16" s="75" t="inlineStr">
+      <c r="H17" s="75" t="inlineStr">
         <is>
           <t>~3-5y</t>
         </is>
       </c>
-      <c r="I16" s="75" t="inlineStr">
+      <c r="I17" s="75" t="inlineStr">
         <is>
           <t>Lenders can seize/operate Colossus on default</t>
         </is>
       </c>
-      <c r="J16" s="79" t="inlineStr">
+      <c r="J17" s="79" t="inlineStr">
         <is>
           <t>CNBC; ciphertalk</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="80" t="inlineStr">
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="80" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="B17" s="81" t="inlineStr">
+      <c r="B18" s="81" t="inlineStr">
         <is>
           <t>Applied Digital — Macquarie financing</t>
         </is>
       </c>
-      <c r="C17" s="82" t="inlineStr">
+      <c r="C18" s="82" t="inlineStr">
         <is>
           <t>Colocation / data-center REIT</t>
         </is>
       </c>
-      <c r="D17" s="80" t="inlineStr">
+      <c r="D18" s="80" t="inlineStr">
         <is>
           <t>Macquarie</t>
         </is>
       </c>
-      <c r="E17" s="83" t="n">
+      <c r="E18" s="83" t="n">
         <v>5</v>
       </c>
-      <c r="F17" s="80" t="inlineStr">
+      <c r="F18" s="80" t="inlineStr">
         <is>
           <t>Perpetual/structured HPC financing</t>
         </is>
       </c>
-      <c r="G17" s="80" t="inlineStr">
+      <c r="G18" s="80" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H17" s="80" t="inlineStr">
+      <c r="H18" s="80" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I17" s="80" t="inlineStr">
+      <c r="I18" s="80" t="inlineStr">
         <is>
           <t>Powered-shell build for CoreWeave (Polaris Forge)</t>
         </is>
       </c>
-      <c r="J17" s="84" t="inlineStr">
+      <c r="J18" s="84" t="inlineStr">
         <is>
           <t>press</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="75" t="inlineStr">
-        <is>
-          <t>Jul 2025</t>
-        </is>
-      </c>
-      <c r="B18" s="76" t="inlineStr">
-        <is>
-          <t>CoreWeave — OpenAI contract financing</t>
-        </is>
-      </c>
-      <c r="C18" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D18" s="75" t="inlineStr">
-        <is>
-          <t>Private lenders (SPV)</t>
-        </is>
-      </c>
-      <c r="E18" s="78" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="F18" s="75" t="inlineStr">
-        <is>
-          <t>SPV debt vs. $11.9bn OpenAI contract</t>
-        </is>
-      </c>
-      <c r="G18" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H18" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I18" s="75" t="inlineStr">
-        <is>
-          <t>Funds CoreWeave's OpenAI compute obligations</t>
-        </is>
-      </c>
-      <c r="J18" s="79" t="inlineStr">
-        <is>
-          <t>FT</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="75" t="inlineStr">
         <is>
-          <t>Aug 2023</t>
+          <t>Jul 2025</t>
         </is>
       </c>
       <c r="B19" s="76" t="inlineStr">
         <is>
-          <t>CoreWeave — $2.3bn debt facility</t>
+          <t>CoreWeave — OpenAI contract financing</t>
         </is>
       </c>
       <c r="C19" s="77" t="inlineStr">
@@ -8951,20 +8910,20 @@
       </c>
       <c r="D19" s="75" t="inlineStr">
         <is>
-          <t>Blackstone, Magnetar</t>
+          <t>Private lenders (SPV)</t>
         </is>
       </c>
       <c r="E19" s="78" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
       <c r="F19" s="75" t="inlineStr">
         <is>
-          <t>GPU-backed facility</t>
+          <t>SPV debt vs. $11.9bn OpenAI contract</t>
         </is>
       </c>
       <c r="G19" s="75" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H19" s="75" t="inlineStr">
@@ -8974,24 +8933,24 @@
       </c>
       <c r="I19" s="75" t="inlineStr">
         <is>
-          <t>Early template for GPU-collateralized debt</t>
+          <t>Funds CoreWeave's OpenAI compute obligations</t>
         </is>
       </c>
       <c r="J19" s="79" t="inlineStr">
         <is>
-          <t>Blackstone</t>
+          <t>FT</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="75" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Aug 2023</t>
         </is>
       </c>
       <c r="B20" s="76" t="inlineStr">
         <is>
-          <t>Nscale — term loan</t>
+          <t>CoreWeave — $2.3bn debt facility</t>
         </is>
       </c>
       <c r="C20" s="77" t="inlineStr">
@@ -9001,184 +8960,182 @@
       </c>
       <c r="D20" s="75" t="inlineStr">
         <is>
-          <t>Private credit</t>
+          <t>Blackstone, Magnetar</t>
         </is>
       </c>
       <c r="E20" s="78" t="n">
-        <v>1.4</v>
+        <v>2.3</v>
       </c>
       <c r="F20" s="75" t="inlineStr">
         <is>
-          <t>Term loan</t>
+          <t>GPU-backed facility</t>
         </is>
       </c>
       <c r="G20" s="75" t="inlineStr">
         <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H20" s="75" t="inlineStr">
+        <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H20" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
       <c r="I20" s="75" t="inlineStr">
         <is>
-          <t>GPU-cloud build</t>
+          <t>Early template for GPU-collateralized debt</t>
         </is>
       </c>
       <c r="J20" s="79" t="inlineStr">
         <is>
-          <t>theaiinsider</t>
+          <t>Blackstone</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="75" t="inlineStr">
         <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B21" s="76" t="inlineStr">
+        <is>
+          <t>Nscale — term loan</t>
+        </is>
+      </c>
+      <c r="C21" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D21" s="75" t="inlineStr">
+        <is>
+          <t>Private credit</t>
+        </is>
+      </c>
+      <c r="E21" s="78" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F21" s="75" t="inlineStr">
+        <is>
+          <t>Term loan</t>
+        </is>
+      </c>
+      <c r="G21" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H21" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I21" s="75" t="inlineStr">
+        <is>
+          <t>GPU-cloud build</t>
+        </is>
+      </c>
+      <c r="J21" s="79" t="inlineStr">
+        <is>
+          <t>theaiinsider</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="75" t="inlineStr">
+        <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B21" s="76" t="inlineStr">
+      <c r="B22" s="76" t="inlineStr">
         <is>
           <t>Lambda — GPU-backed facility</t>
         </is>
       </c>
-      <c r="C21" s="77" t="inlineStr">
+      <c r="C22" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D21" s="75" t="inlineStr">
+      <c r="D22" s="75" t="inlineStr">
         <is>
           <t>Macquarie</t>
         </is>
       </c>
-      <c r="E21" s="78" t="n">
+      <c r="E22" s="78" t="n">
         <v>0.5</v>
       </c>
-      <c r="F21" s="75" t="inlineStr">
+      <c r="F22" s="75" t="inlineStr">
         <is>
           <t>GPU-backed facility</t>
         </is>
       </c>
-      <c r="G21" s="75" t="inlineStr">
+      <c r="G22" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H21" s="75" t="inlineStr">
+      <c r="H22" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I21" s="75" t="inlineStr">
+      <c r="I22" s="75" t="inlineStr">
         <is>
           <t>GPU-cloud build</t>
         </is>
       </c>
-      <c r="J21" s="79" t="inlineStr">
+      <c r="J22" s="79" t="inlineStr">
         <is>
           <t>theaiinsider</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="85" t="n"/>
-      <c r="B22" s="86" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="85" t="n"/>
+      <c r="B23" s="86" t="inlineStr">
         <is>
           <t>Total — itemized private credit deals</t>
         </is>
       </c>
-      <c r="C22" s="85" t="n"/>
-      <c r="D22" s="85" t="n"/>
-      <c r="E22" s="87">
-        <f>SUM(E5:E21)</f>
-        <v/>
-      </c>
-      <c r="F22" s="85" t="n"/>
-      <c r="G22" s="85" t="n"/>
-      <c r="H22" s="85" t="n"/>
-      <c r="I22" s="85" t="n"/>
-      <c r="J22" s="85" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>CONTEXT / FRAMEWORKS / PROJECTIONS (not summed)</t>
-        </is>
-      </c>
-      <c r="B24" s="15" t="n"/>
-      <c r="C24" s="15" t="n"/>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15" t="n"/>
-      <c r="G24" s="15" t="n"/>
-      <c r="H24" s="15" t="n"/>
-      <c r="I24" s="15" t="n"/>
-      <c r="J24" s="15" t="n"/>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="88" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B25" s="88" t="inlineStr">
-        <is>
-          <t>KKR + Energy Capital Partners — AI infrastructure partnership</t>
-        </is>
-      </c>
-      <c r="C25" s="89" t="inlineStr">
-        <is>
-          <t>Context / market</t>
-        </is>
-      </c>
-      <c r="D25" s="88" t="inlineStr">
-        <is>
-          <t>KKR, Energy Capital Partners</t>
-        </is>
-      </c>
-      <c r="E25" s="90" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F25" s="88" t="inlineStr">
-        <is>
-          <t>Strategic partnership/commitment</t>
-        </is>
-      </c>
-      <c r="G25" s="88" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H25" s="88" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I25" s="88" t="inlineStr">
-        <is>
-          <t>~$50bn to accelerate AI infrastructure</t>
-        </is>
-      </c>
-      <c r="J25" s="91" t="inlineStr">
-        <is>
-          <t>Business Times</t>
-        </is>
-      </c>
+      <c r="C23" s="85" t="n"/>
+      <c r="D23" s="85" t="n"/>
+      <c r="E23" s="87">
+        <f>SUM(E6:E22)</f>
+        <v/>
+      </c>
+      <c r="F23" s="85" t="n"/>
+      <c r="G23" s="85" t="n"/>
+      <c r="H23" s="85" t="n"/>
+      <c r="I23" s="85" t="n"/>
+      <c r="J23" s="85" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>2) CONTEXT / FRAMEWORKS / PROJECTIONS (not summed)</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n"/>
+      <c r="C25" s="15" t="n"/>
+      <c r="D25" s="15" t="n"/>
+      <c r="E25" s="15" t="n"/>
+      <c r="F25" s="15" t="n"/>
+      <c r="G25" s="15" t="n"/>
+      <c r="H25" s="15" t="n"/>
+      <c r="I25" s="15" t="n"/>
+      <c r="J25" s="15" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="88" t="inlineStr">
         <is>
-          <t>Late 2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="B26" s="88" t="inlineStr">
         <is>
-          <t>Qatar (QIA / Qai) + Brookfield — AI infrastructure JV</t>
+          <t>KKR + Energy Capital Partners — AI infrastructure partnership</t>
         </is>
       </c>
       <c r="C26" s="89" t="inlineStr">
@@ -9188,7 +9145,7 @@
       </c>
       <c r="D26" s="88" t="inlineStr">
         <is>
-          <t>QIA / Qai, Brookfield</t>
+          <t>KKR, Energy Capital Partners</t>
         </is>
       </c>
       <c r="E26" s="90" t="inlineStr">
@@ -9198,7 +9155,7 @@
       </c>
       <c r="F26" s="88" t="inlineStr">
         <is>
-          <t>Joint venture / infra credit</t>
+          <t>Strategic partnership/commitment</t>
         </is>
       </c>
       <c r="G26" s="88" t="inlineStr">
@@ -9213,24 +9170,24 @@
       </c>
       <c r="I26" s="88" t="inlineStr">
         <is>
-          <t>~$20bn JV</t>
+          <t>~$50bn to accelerate AI infrastructure</t>
         </is>
       </c>
       <c r="J26" s="91" t="inlineStr">
         <is>
-          <t>NYU DRI</t>
+          <t>Business Times</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="88" t="inlineStr">
         <is>
-          <t>2025-28</t>
+          <t>Late 2025</t>
         </is>
       </c>
       <c r="B27" s="88" t="inlineStr">
         <is>
-          <t>Broadcom + Apollo + Blackstone — AI compute platform</t>
+          <t>Qatar (QIA / Qai) + Brookfield — AI infrastructure JV</t>
         </is>
       </c>
       <c r="C27" s="89" t="inlineStr">
@@ -9240,7 +9197,7 @@
       </c>
       <c r="D27" s="88" t="inlineStr">
         <is>
-          <t>Apollo, Blackstone, Broadcom</t>
+          <t>QIA / Qai, Brookfield</t>
         </is>
       </c>
       <c r="E27" s="90" t="inlineStr">
@@ -9250,7 +9207,7 @@
       </c>
       <c r="F27" s="88" t="inlineStr">
         <is>
-          <t>Platform framework</t>
+          <t>Joint venture / infra credit</t>
         </is>
       </c>
       <c r="G27" s="88" t="inlineStr">
@@ -9260,29 +9217,29 @@
       </c>
       <c r="H27" s="88" t="inlineStr">
         <is>
-          <t>through 2028</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I27" s="88" t="inlineStr">
         <is>
-          <t>&gt;20 GW of compute to be deployed</t>
+          <t>~$20bn JV</t>
         </is>
       </c>
       <c r="J27" s="91" t="inlineStr">
         <is>
-          <t>privatedebtnews</t>
+          <t>NYU DRI</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="88" t="inlineStr">
         <is>
-          <t>from Nov 2025</t>
+          <t>2025-28</t>
         </is>
       </c>
       <c r="B28" s="88" t="inlineStr">
         <is>
-          <t>Sector — 144A private placements (data centers)</t>
+          <t>Broadcom + Apollo + Blackstone — AI compute platform</t>
         </is>
       </c>
       <c r="C28" s="89" t="inlineStr">
@@ -9292,7 +9249,7 @@
       </c>
       <c r="D28" s="88" t="inlineStr">
         <is>
-          <t>Multiple (Blue Owl, PIMCO, etc.)</t>
+          <t>Apollo, Blackstone, Broadcom</t>
         </is>
       </c>
       <c r="E28" s="90" t="inlineStr">
@@ -9302,7 +9259,7 @@
       </c>
       <c r="F28" s="88" t="inlineStr">
         <is>
-          <t>144A private placement bonds</t>
+          <t>Platform framework</t>
         </is>
       </c>
       <c r="G28" s="88" t="inlineStr">
@@ -9312,1320 +9269,1240 @@
       </c>
       <c r="H28" s="88" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>through 2028</t>
         </is>
       </c>
       <c r="I28" s="88" t="inlineStr">
         <is>
-          <t>&gt;$40bn by Applied Digital, CoreWeave, Hut 8, Related since Nov 2025</t>
+          <t>&gt;20 GW of compute to be deployed</t>
         </is>
       </c>
       <c r="J28" s="91" t="inlineStr">
         <is>
-          <t>Bisnow</t>
+          <t>privatedebtnews</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="88" t="inlineStr">
         <is>
+          <t>from Nov 2025</t>
+        </is>
+      </c>
+      <c r="B29" s="88" t="inlineStr">
+        <is>
+          <t>Sector — 144A private placements (data centers)</t>
+        </is>
+      </c>
+      <c r="C29" s="89" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D29" s="88" t="inlineStr">
+        <is>
+          <t>Multiple (Blue Owl, PIMCO, etc.)</t>
+        </is>
+      </c>
+      <c r="E29" s="90" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F29" s="88" t="inlineStr">
+        <is>
+          <t>144A private placement bonds</t>
+        </is>
+      </c>
+      <c r="G29" s="88" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H29" s="88" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I29" s="88" t="inlineStr">
+        <is>
+          <t>&gt;$40bn by Applied Digital, CoreWeave, Hut 8, Related since Nov 2025</t>
+        </is>
+      </c>
+      <c r="J29" s="91" t="inlineStr">
+        <is>
+          <t>Bisnow</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="88" t="inlineStr">
+        <is>
           <t>2025-28</t>
         </is>
       </c>
-      <c r="B29" s="88" t="inlineStr">
+      <c r="B30" s="88" t="inlineStr">
         <is>
           <t>Market — projected private credit for AI data centers</t>
         </is>
       </c>
-      <c r="C29" s="89" t="inlineStr">
+      <c r="C30" s="89" t="inlineStr">
         <is>
           <t>Context / market</t>
         </is>
       </c>
-      <c r="D29" s="88" t="inlineStr">
+      <c r="D30" s="88" t="inlineStr">
         <is>
           <t>Industry-wide</t>
         </is>
       </c>
-      <c r="E29" s="90" t="inlineStr">
+      <c r="E30" s="90" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F29" s="88" t="inlineStr">
+      <c r="F30" s="88" t="inlineStr">
         <is>
           <t>Projection</t>
         </is>
       </c>
-      <c r="G29" s="88" t="inlineStr">
+      <c r="G30" s="88" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H29" s="88" t="inlineStr">
+      <c r="H30" s="88" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I29" s="88" t="inlineStr">
+      <c r="I30" s="88" t="inlineStr">
         <is>
           <t>Morgan Stanley: ~$800bn over next 2 years; &gt;$200bn already outstanding</t>
         </is>
       </c>
-      <c r="J29" s="91" t="inlineStr">
+      <c r="J30" s="91" t="inlineStr">
         <is>
           <t>Morgan Stanley; Quinn Emanuel</t>
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F49"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="64" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Key Disclosed Transactions &amp; Sources</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="11" t="inlineStr">
-        <is>
-          <t>Representative deals underpinning the estimates. Amounts as reported; '~' denotes approximate/announced figures. Not exhaustive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Company / Group</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Transaction</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Primary instrument</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
-        <is>
-          <t>Source(s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="92" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>3) OTHER KEY DEALS — bonds · equity · securitization · sovereign · leases</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="15" t="n"/>
+      <c r="G32" s="15" t="n"/>
+      <c r="H32" s="15" t="n"/>
+      <c r="I32" s="15" t="n"/>
+      <c r="J32" s="15" t="n"/>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B33" s="70" t="inlineStr">
         <is>
           <t>Meta Platforms</t>
         </is>
       </c>
-      <c r="B5" s="93" t="inlineStr">
-        <is>
-          <t>Hyperion JV (Beignet Investor LLC) — Blue Owl 80% / Meta 20%; $27.3bn A+ private bond led by PIMCO (~$18bn) &amp; BlackRock; off-B/S SPV w/ residual-value guarantee</t>
-        </is>
-      </c>
-      <c r="C5" s="93" t="inlineStr">
+      <c r="C33" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D33" s="70" t="inlineStr"/>
+      <c r="E33" s="92" t="inlineStr">
+        <is>
+          <t>$30bn</t>
+        </is>
+      </c>
+      <c r="F33" s="70" t="inlineStr">
+        <is>
+          <t>Corporate bonds</t>
+        </is>
+      </c>
+      <c r="G33" s="70" t="inlineStr"/>
+      <c r="H33" s="70" t="inlineStr"/>
+      <c r="I33" s="70" t="inlineStr">
+        <is>
+          <t>$30bn multi-tranche IG corporate bond (largest 2025 IG deal), maturities to 2063</t>
+        </is>
+      </c>
+      <c r="J33" s="74" t="inlineStr">
+        <is>
+          <t>BofA; MUFG</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="70" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B34" s="70" t="inlineStr">
+        <is>
+          <t>Amazon (AWS)</t>
+        </is>
+      </c>
+      <c r="C34" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D34" s="70" t="inlineStr"/>
+      <c r="E34" s="92" t="inlineStr">
+        <is>
+          <t>~$71bn</t>
+        </is>
+      </c>
+      <c r="F34" s="70" t="inlineStr">
+        <is>
+          <t>Corporate bonds</t>
+        </is>
+      </c>
+      <c r="G34" s="70" t="inlineStr"/>
+      <c r="H34" s="70" t="inlineStr"/>
+      <c r="I34" s="70" t="inlineStr">
+        <is>
+          <t>~$54bn USD + €14.5bn (~$16.8bn) IG bonds (near-record), ~4x oversubscribed</t>
+        </is>
+      </c>
+      <c r="J34" s="74" t="inlineStr">
+        <is>
+          <t>CNA; Reuters</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="70" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D5" s="93" t="inlineStr">
-        <is>
-          <t>$27.3bn debt</t>
-        </is>
-      </c>
-      <c r="E5" s="93" t="inlineStr">
-        <is>
-          <t>SPV / private credit / insurance</t>
-        </is>
-      </c>
-      <c r="F5" s="94" t="inlineStr">
-        <is>
-          <t>Meta IR; FT; S&amp;P</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="95" t="inlineStr">
-        <is>
-          <t>Meta Platforms</t>
-        </is>
-      </c>
-      <c r="B6" s="96" t="inlineStr">
-        <is>
-          <t>$30bn multi-tranche IG corporate bond (largest 2025 IG deal), maturities to 2063</t>
-        </is>
-      </c>
-      <c r="C6" s="96" t="inlineStr">
+      <c r="B35" s="70" t="inlineStr">
+        <is>
+          <t>Amazon (AWS)</t>
+        </is>
+      </c>
+      <c r="C35" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D35" s="70" t="inlineStr"/>
+      <c r="E35" s="92" t="inlineStr">
+        <is>
+          <t>$15bn</t>
+        </is>
+      </c>
+      <c r="F35" s="70" t="inlineStr">
+        <is>
+          <t>Corporate bonds</t>
+        </is>
+      </c>
+      <c r="G35" s="70" t="inlineStr"/>
+      <c r="H35" s="70" t="inlineStr"/>
+      <c r="I35" s="70" t="inlineStr">
+        <is>
+          <t>$15bn IG bond</t>
+        </is>
+      </c>
+      <c r="J35" s="74" t="inlineStr">
+        <is>
+          <t>CNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="70" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B36" s="70" t="inlineStr">
+        <is>
+          <t>Alphabet (Google)</t>
+        </is>
+      </c>
+      <c r="C36" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D36" s="70" t="inlineStr"/>
+      <c r="E36" s="92" t="inlineStr">
+        <is>
+          <t>~$50bn</t>
+        </is>
+      </c>
+      <c r="F36" s="70" t="inlineStr">
+        <is>
+          <t>Corporate bonds</t>
+        </is>
+      </c>
+      <c r="G36" s="70" t="inlineStr"/>
+      <c r="H36" s="70" t="inlineStr"/>
+      <c r="I36" s="70" t="inlineStr">
+        <is>
+          <t>~$32bn multi-currency bond incl. rare 100-yr tranche; plus $17.5bn Nov 2025</t>
+        </is>
+      </c>
+      <c r="J36" s="74" t="inlineStr">
+        <is>
+          <t>ConstructConnect; CNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="70" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B37" s="70" t="inlineStr">
+        <is>
+          <t>Oracle (OCI)</t>
+        </is>
+      </c>
+      <c r="C37" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D37" s="70" t="inlineStr"/>
+      <c r="E37" s="92" t="inlineStr">
+        <is>
+          <t>$25bn debt</t>
+        </is>
+      </c>
+      <c r="F37" s="70" t="inlineStr">
+        <is>
+          <t>Corporate bonds + equity</t>
+        </is>
+      </c>
+      <c r="G37" s="70" t="inlineStr"/>
+      <c r="H37" s="70" t="inlineStr"/>
+      <c r="I37" s="70" t="inlineStr">
+        <is>
+          <t>$25bn 8-part IG bond (Feb 2026) within $45-50bn CY26 debt+equity plan; $20bn ATM + mandatory convertible preferred (equity)</t>
+        </is>
+      </c>
+      <c r="J37" s="74" t="inlineStr">
+        <is>
+          <t>Oracle IR; IFR</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="70" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D6" s="96" t="inlineStr">
-        <is>
-          <t>$30bn</t>
-        </is>
-      </c>
-      <c r="E6" s="96" t="inlineStr">
+      <c r="B38" s="70" t="inlineStr">
+        <is>
+          <t>Oracle (OCI)</t>
+        </is>
+      </c>
+      <c r="C38" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D38" s="70" t="inlineStr"/>
+      <c r="E38" s="92" t="inlineStr">
+        <is>
+          <t>$18bn</t>
+        </is>
+      </c>
+      <c r="F38" s="70" t="inlineStr">
         <is>
           <t>Corporate bonds</t>
         </is>
       </c>
-      <c r="F6" s="97" t="inlineStr">
-        <is>
-          <t>BofA; MUFG</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="92" t="inlineStr">
-        <is>
-          <t>Amazon (AWS)</t>
-        </is>
-      </c>
-      <c r="B7" s="93" t="inlineStr">
-        <is>
-          <t>~$54bn USD + €14.5bn (~$16.8bn) IG bonds (near-record), ~4x oversubscribed</t>
-        </is>
-      </c>
-      <c r="C7" s="93" t="inlineStr">
+      <c r="G38" s="70" t="inlineStr"/>
+      <c r="H38" s="70" t="inlineStr"/>
+      <c r="I38" s="70" t="inlineStr">
+        <is>
+          <t>$18bn 6-part IG bond (Sep 2025)</t>
+        </is>
+      </c>
+      <c r="J38" s="74" t="inlineStr">
+        <is>
+          <t>Reuters/CNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="70" t="inlineStr">
+        <is>
+          <t>2024-30</t>
+        </is>
+      </c>
+      <c r="B39" s="70" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="C39" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D39" s="70" t="inlineStr"/>
+      <c r="E39" s="92" t="inlineStr">
+        <is>
+          <t>$100bn+ leases</t>
+        </is>
+      </c>
+      <c r="F39" s="70" t="inlineStr">
+        <is>
+          <t>Vendor / lease / SPV</t>
+        </is>
+      </c>
+      <c r="G39" s="70" t="inlineStr"/>
+      <c r="H39" s="70" t="inlineStr"/>
+      <c r="I39" s="70" t="inlineStr">
+        <is>
+          <t>Finance-lease driven build (~$108bn uncommenced finance leases as of 9/30/24; commence FY25-FY30)</t>
+        </is>
+      </c>
+      <c r="J39" s="74" t="inlineStr">
+        <is>
+          <t>MSFT 10-Q; CNBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="75" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B40" s="75" t="inlineStr">
+        <is>
+          <t>CoreWeave</t>
+        </is>
+      </c>
+      <c r="C40" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D40" s="75" t="inlineStr"/>
+      <c r="E40" s="93" t="inlineStr">
+        <is>
+          <t>$2.7bn conv.</t>
+        </is>
+      </c>
+      <c r="F40" s="75" t="inlineStr">
+        <is>
+          <t>Convertibles</t>
+        </is>
+      </c>
+      <c r="G40" s="75" t="inlineStr"/>
+      <c r="H40" s="75" t="inlineStr"/>
+      <c r="I40" s="75" t="inlineStr">
+        <is>
+          <t>$2.7bn 1.75% convertible notes; ~$30bn total debt by early 2026; ~$28bn debt+equity raised in 12 mos</t>
+        </is>
+      </c>
+      <c r="J40" s="79" t="inlineStr">
+        <is>
+          <t>thedig; CoreWeave</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="75" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B41" s="75" t="inlineStr">
+        <is>
+          <t>CoreWeave</t>
+        </is>
+      </c>
+      <c r="C41" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D41" s="75" t="inlineStr"/>
+      <c r="E41" s="93" t="inlineStr">
+        <is>
+          <t>$3.5bn equity</t>
+        </is>
+      </c>
+      <c r="F41" s="75" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="G41" s="75" t="inlineStr"/>
+      <c r="H41" s="75" t="inlineStr"/>
+      <c r="I41" s="75" t="inlineStr">
+        <is>
+          <t>$2bn strategic equity from NVIDIA; IPO Mar 2025 raised ~$1.5bn</t>
+        </is>
+      </c>
+      <c r="J41" s="79" t="inlineStr">
+        <is>
+          <t>CNBC; CoreWeave</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="75" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D7" s="93" t="inlineStr">
-        <is>
-          <t>~$71bn</t>
-        </is>
-      </c>
-      <c r="E7" s="93" t="inlineStr">
-        <is>
-          <t>Corporate bonds</t>
-        </is>
-      </c>
-      <c r="F7" s="94" t="inlineStr">
-        <is>
-          <t>CNA; Reuters</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="95" t="inlineStr">
-        <is>
-          <t>Amazon (AWS)</t>
-        </is>
-      </c>
-      <c r="B8" s="96" t="inlineStr">
-        <is>
-          <t>$15bn IG bond</t>
-        </is>
-      </c>
-      <c r="C8" s="96" t="inlineStr">
+      <c r="B42" s="75" t="inlineStr">
+        <is>
+          <t>SpaceX / xAI</t>
+        </is>
+      </c>
+      <c r="C42" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D42" s="75" t="inlineStr"/>
+      <c r="E42" s="93" t="inlineStr">
+        <is>
+          <t>merger</t>
+        </is>
+      </c>
+      <c r="F42" s="75" t="inlineStr">
+        <is>
+          <t>Equity / M&amp;A</t>
+        </is>
+      </c>
+      <c r="G42" s="75" t="inlineStr"/>
+      <c r="H42" s="75" t="inlineStr"/>
+      <c r="I42" s="75" t="inlineStr">
+        <is>
+          <t>SpaceX acquired xAI effective Feb 2, 2026; Colossus I &amp; II now SpaceX-owned (vertically-integrated AI platform; Terafab chip JV w/ Tesla &amp; Intel)</t>
+        </is>
+      </c>
+      <c r="J42" s="79" t="inlineStr">
+        <is>
+          <t>SpaceX S-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="75" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B43" s="75" t="inlineStr">
+        <is>
+          <t>SpaceX / xAI</t>
+        </is>
+      </c>
+      <c r="C43" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D43" s="75" t="inlineStr"/>
+      <c r="E43" s="93" t="inlineStr">
+        <is>
+          <t>$20bn+ capex</t>
+        </is>
+      </c>
+      <c r="F43" s="75" t="inlineStr">
+        <is>
+          <t>Internal / equity</t>
+        </is>
+      </c>
+      <c r="G43" s="75" t="inlineStr"/>
+      <c r="H43" s="75" t="inlineStr"/>
+      <c r="I43" s="75" t="inlineStr">
+        <is>
+          <t>SpaceX AI capex $12.7bn in 2025 (~61% of total) + $7.7bn in Q1 2026; AI buildout funded by Starlink FCF, private raises, planned IPO</t>
+        </is>
+      </c>
+      <c r="J43" s="79" t="inlineStr">
+        <is>
+          <t>SpaceX S-1; The Verge</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="75" t="inlineStr">
+        <is>
+          <t>2026-29</t>
+        </is>
+      </c>
+      <c r="B44" s="75" t="inlineStr">
+        <is>
+          <t>SpaceX / xAI</t>
+        </is>
+      </c>
+      <c r="C44" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D44" s="75" t="inlineStr"/>
+      <c r="E44" s="93" t="inlineStr">
+        <is>
+          <t>~$45bn</t>
+        </is>
+      </c>
+      <c r="F44" s="75" t="inlineStr">
+        <is>
+          <t>Take-or-pay (demand)</t>
+        </is>
+      </c>
+      <c r="G44" s="75" t="inlineStr"/>
+      <c r="H44" s="75" t="inlineStr"/>
+      <c r="I44" s="75" t="inlineStr">
+        <is>
+          <t>Anthropic compute contract: $1.25bn/month (~$45bn) through May 2029 for Colossus I &amp; II — anchor revenue underwriting infra financing</t>
+        </is>
+      </c>
+      <c r="J44" s="79" t="inlineStr">
+        <is>
+          <t>SpaceX S-1; The Verge</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="75" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D8" s="96" t="inlineStr">
-        <is>
-          <t>$15bn</t>
-        </is>
-      </c>
-      <c r="E8" s="96" t="inlineStr">
-        <is>
-          <t>Corporate bonds</t>
-        </is>
-      </c>
-      <c r="F8" s="97" t="inlineStr">
-        <is>
-          <t>CNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="92" t="inlineStr">
-        <is>
-          <t>Alphabet (Google)</t>
-        </is>
-      </c>
-      <c r="B9" s="93" t="inlineStr">
-        <is>
-          <t>~$32bn multi-currency bond incl. rare 100-yr tranche; plus $17.5bn Nov 2025</t>
-        </is>
-      </c>
-      <c r="C9" s="93" t="inlineStr">
+      <c r="B45" s="75" t="inlineStr">
+        <is>
+          <t>SpaceX / xAI</t>
+        </is>
+      </c>
+      <c r="C45" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D45" s="75" t="inlineStr"/>
+      <c r="E45" s="93" t="inlineStr">
+        <is>
+          <t>$10bn</t>
+        </is>
+      </c>
+      <c r="F45" s="75" t="inlineStr">
+        <is>
+          <t>Loans + equity</t>
+        </is>
+      </c>
+      <c r="G45" s="75" t="inlineStr"/>
+      <c r="H45" s="75" t="inlineStr"/>
+      <c r="I45" s="75" t="inlineStr">
+        <is>
+          <t>xAI $10bn raise ($5bn secured notes/term loans incl. Apollo $5bn facility + $5bn equity) via Morgan Stanley</t>
+        </is>
+      </c>
+      <c r="J45" s="79" t="inlineStr">
+        <is>
+          <t>CNBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="75" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D9" s="93" t="inlineStr">
-        <is>
-          <t>~$50bn</t>
-        </is>
-      </c>
-      <c r="E9" s="93" t="inlineStr">
-        <is>
-          <t>Corporate bonds</t>
-        </is>
-      </c>
-      <c r="F9" s="94" t="inlineStr">
-        <is>
-          <t>ConstructConnect; CNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="95" t="inlineStr">
-        <is>
-          <t>Oracle (OCI)</t>
-        </is>
-      </c>
-      <c r="B10" s="96" t="inlineStr">
-        <is>
-          <t>$25bn 8-part IG bond (Feb 2026) within $45-50bn CY26 debt+equity plan; $20bn ATM + mandatory convertible preferred (equity)</t>
-        </is>
-      </c>
-      <c r="C10" s="96" t="inlineStr">
+      <c r="B46" s="75" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="C46" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D46" s="75" t="inlineStr"/>
+      <c r="E46" s="93" t="inlineStr">
+        <is>
+          <t>$3bn+</t>
+        </is>
+      </c>
+      <c r="F46" s="75" t="inlineStr">
+        <is>
+          <t>Convertibles</t>
+        </is>
+      </c>
+      <c r="G46" s="75" t="inlineStr"/>
+      <c r="H46" s="75" t="inlineStr"/>
+      <c r="I46" s="75" t="inlineStr">
+        <is>
+          <t>$3bn+ convertibles + bank lines; lighter balance sheet; Yandex spin-off cash ~$2.5bn; NVIDIA ~$2bn equity; Microsoft ~$7bn prepay</t>
+        </is>
+      </c>
+      <c r="J46" s="79" t="inlineStr">
+        <is>
+          <t>frankk research</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="80" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D10" s="96" t="inlineStr">
-        <is>
-          <t>$25bn debt</t>
-        </is>
-      </c>
-      <c r="E10" s="96" t="inlineStr">
-        <is>
-          <t>Corporate bonds + equity</t>
-        </is>
-      </c>
-      <c r="F10" s="97" t="inlineStr">
-        <is>
-          <t>Oracle IR; IFR</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="92" t="inlineStr">
-        <is>
-          <t>Oracle (OCI)</t>
-        </is>
-      </c>
-      <c r="B11" s="93" t="inlineStr">
-        <is>
-          <t>$18bn 6-part IG bond (Sep 2025)</t>
-        </is>
-      </c>
-      <c r="C11" s="93" t="inlineStr">
+      <c r="B47" s="80" t="inlineStr">
+        <is>
+          <t>Applied Digital</t>
+        </is>
+      </c>
+      <c r="C47" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D47" s="80" t="inlineStr"/>
+      <c r="E47" s="94" t="inlineStr">
+        <is>
+          <t>$1.59bn</t>
+        </is>
+      </c>
+      <c r="F47" s="80" t="inlineStr">
+        <is>
+          <t>Securitization / HY bond</t>
+        </is>
+      </c>
+      <c r="G47" s="80" t="inlineStr"/>
+      <c r="H47" s="80" t="inlineStr"/>
+      <c r="I47" s="80" t="inlineStr">
+        <is>
+          <t>$1.59bn high-yield bond (7%) for CoreWeave-leased campus (Polaris Forge 1)</t>
+        </is>
+      </c>
+      <c r="J47" s="84" t="inlineStr">
+        <is>
+          <t>TNW</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="80" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D11" s="93" t="inlineStr">
-        <is>
-          <t>$18bn</t>
-        </is>
-      </c>
-      <c r="E11" s="93" t="inlineStr">
-        <is>
-          <t>Corporate bonds</t>
-        </is>
-      </c>
-      <c r="F11" s="94" t="inlineStr">
-        <is>
-          <t>Reuters/CNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="95" t="inlineStr">
-        <is>
-          <t>Oracle (OCI)</t>
-        </is>
-      </c>
-      <c r="B12" s="96" t="inlineStr">
-        <is>
-          <t>Project-level SPV financing: ~$16.3bn Michigan campus; further Texas / Wisconsin deals</t>
-        </is>
-      </c>
-      <c r="C12" s="96" t="inlineStr">
+      <c r="B48" s="80" t="inlineStr">
+        <is>
+          <t>Aligned Data Centers</t>
+        </is>
+      </c>
+      <c r="C48" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D48" s="80" t="inlineStr"/>
+      <c r="E48" s="94" t="inlineStr">
+        <is>
+          <t>$12bn / $40bn</t>
+        </is>
+      </c>
+      <c r="F48" s="80" t="inlineStr">
+        <is>
+          <t>Infra equity + debt</t>
+        </is>
+      </c>
+      <c r="G48" s="80" t="inlineStr"/>
+      <c r="H48" s="80" t="inlineStr"/>
+      <c r="I48" s="80" t="inlineStr">
+        <is>
+          <t>$12bn capital raise ($5bn+ new equity + $7bn debt commitments) led by Macquarie (early 2025); later acquired by MGX/BlackRock consortium (~$40bn)</t>
+        </is>
+      </c>
+      <c r="J48" s="84" t="inlineStr">
+        <is>
+          <t>SFA; NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="80" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B49" s="80" t="inlineStr">
+        <is>
+          <t>QTS (Blackstone)</t>
+        </is>
+      </c>
+      <c r="C49" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D49" s="80" t="inlineStr"/>
+      <c r="E49" s="94" t="inlineStr">
+        <is>
+          <t>$3.5bn+</t>
+        </is>
+      </c>
+      <c r="F49" s="80" t="inlineStr">
+        <is>
+          <t>Securitization (CMBS/ABS)</t>
+        </is>
+      </c>
+      <c r="G49" s="80" t="inlineStr"/>
+      <c r="H49" s="80" t="inlineStr"/>
+      <c r="I49" s="80" t="inlineStr">
+        <is>
+          <t>BX 2025-VOLT SASB CMBS $3.5bn (~10 QTS DCs); + Phoenix ABS (QTS Issuer 2025-1)</t>
+        </is>
+      </c>
+      <c r="J49" s="84" t="inlineStr">
+        <is>
+          <t>CREFC; SFA</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="80" t="inlineStr">
+        <is>
+          <t>2024-25</t>
+        </is>
+      </c>
+      <c r="B50" s="80" t="inlineStr">
+        <is>
+          <t>Switch (DigitalBridge)</t>
+        </is>
+      </c>
+      <c r="C50" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D50" s="80" t="inlineStr"/>
+      <c r="E50" s="94" t="inlineStr">
+        <is>
+          <t>$3.5bn</t>
+        </is>
+      </c>
+      <c r="F50" s="80" t="inlineStr">
+        <is>
+          <t>Securitization (CMBS/ABS)</t>
+        </is>
+      </c>
+      <c r="G50" s="80" t="inlineStr"/>
+      <c r="H50" s="80" t="inlineStr"/>
+      <c r="I50" s="80" t="inlineStr">
+        <is>
+          <t>$2.4bn SASB CMBS (SWCH 2025-DATA) + $1.1bn ABS — green bonds</t>
+        </is>
+      </c>
+      <c r="J50" s="84" t="inlineStr">
+        <is>
+          <t>SFA; CREFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="80" t="inlineStr">
+        <is>
+          <t>2024-26</t>
+        </is>
+      </c>
+      <c r="B51" s="80" t="inlineStr">
+        <is>
+          <t>Vantage Data Centers</t>
+        </is>
+      </c>
+      <c r="C51" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D51" s="80" t="inlineStr"/>
+      <c r="E51" s="94" t="inlineStr">
+        <is>
+          <t>multi-$bn</t>
+        </is>
+      </c>
+      <c r="F51" s="80" t="inlineStr">
+        <is>
+          <t>Securitization / equity</t>
+        </is>
+      </c>
+      <c r="G51" s="80" t="inlineStr"/>
+      <c r="H51" s="80" t="inlineStr"/>
+      <c r="I51" s="80" t="inlineStr">
+        <is>
+          <t>First public data-center ABS (2024); ongoing multi-billion securitization &amp; infra-equity program</t>
+        </is>
+      </c>
+      <c r="J51" s="84" t="inlineStr">
+        <is>
+          <t>Dentons</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="88" t="inlineStr">
+        <is>
+          <t>2025-28</t>
+        </is>
+      </c>
+      <c r="B52" s="88" t="inlineStr">
+        <is>
+          <t>Colocation sector</t>
+        </is>
+      </c>
+      <c r="C52" s="89" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D52" s="88" t="inlineStr"/>
+      <c r="E52" s="95" t="inlineStr">
+        <is>
+          <t>~$130bn</t>
+        </is>
+      </c>
+      <c r="F52" s="88" t="inlineStr">
+        <is>
+          <t>Securitization (ABS/CMBS)</t>
+        </is>
+      </c>
+      <c r="G52" s="88" t="inlineStr"/>
+      <c r="H52" s="88" t="inlineStr"/>
+      <c r="I52" s="88" t="inlineStr">
+        <is>
+          <t>US data-center ABS+CMBS issuance ~$26bn in 2025 (~10x 2020); ~$57bn since 2021; Morgan Stanley ~$130bn securitized net issuance 2026-28; ~$150bn permanent financing need 2026-27</t>
+        </is>
+      </c>
+      <c r="J52" s="91" t="inlineStr">
+        <is>
+          <t>Impax; CREFC; Morgan Stanley</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="96" t="inlineStr">
+        <is>
+          <t>2025-30</t>
+        </is>
+      </c>
+      <c r="B53" s="96" t="inlineStr">
+        <is>
+          <t>HUMAIN (Saudi PIF)</t>
+        </is>
+      </c>
+      <c r="C53" s="97" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="D53" s="96" t="inlineStr"/>
+      <c r="E53" s="98" t="inlineStr">
+        <is>
+          <t>~$100bn</t>
+        </is>
+      </c>
+      <c r="F53" s="96" t="inlineStr">
+        <is>
+          <t>Sovereign equity</t>
+        </is>
+      </c>
+      <c r="G53" s="96" t="inlineStr"/>
+      <c r="H53" s="96" t="inlineStr"/>
+      <c r="I53" s="96" t="inlineStr">
+        <is>
+          <t>PIF national AI champion (announced 13 May 2025): ~$100bn across 11 data centers / 2.2 GW; ~600k NVIDIA GPUs; ALLAM Arabic LLM</t>
+        </is>
+      </c>
+      <c r="J53" s="99" t="inlineStr">
+        <is>
+          <t>Presenc AI; NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="96" t="inlineStr">
+        <is>
+          <t>2025-30</t>
+        </is>
+      </c>
+      <c r="B54" s="96" t="inlineStr">
+        <is>
+          <t>Stargate UAE / G42</t>
+        </is>
+      </c>
+      <c r="C54" s="97" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="D54" s="96" t="inlineStr"/>
+      <c r="E54" s="98" t="inlineStr">
+        <is>
+          <t>~$30bn+</t>
+        </is>
+      </c>
+      <c r="F54" s="96" t="inlineStr">
+        <is>
+          <t>Sovereign equity + JV</t>
+        </is>
+      </c>
+      <c r="G54" s="96" t="inlineStr"/>
+      <c r="H54" s="96" t="inlineStr"/>
+      <c r="I54" s="96" t="inlineStr">
+        <is>
+          <t>$30bn+ 5GW Abu Dhabi campus (Khazna/G42 w/ OpenAI, Oracle, NVIDIA, Cisco, SoftBank); Phase 1 200MW Q3 2026; Microsoft ~$1.5bn equity</t>
+        </is>
+      </c>
+      <c r="J54" s="99" t="inlineStr">
+        <is>
+          <t>Khaleej Times; dcpulse</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="96" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="D12" s="96" t="inlineStr">
-        <is>
-          <t>~$25bn+</t>
-        </is>
-      </c>
-      <c r="E12" s="96" t="inlineStr">
-        <is>
-          <t>SPV / project finance</t>
-        </is>
-      </c>
-      <c r="F12" s="97" t="inlineStr">
-        <is>
-          <t>Press reports</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="92" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="B13" s="93" t="inlineStr">
-        <is>
-          <t>Finance-lease driven build (~$108bn uncommenced finance leases as of 9/30/24; commence FY25-FY30)</t>
-        </is>
-      </c>
-      <c r="C13" s="93" t="inlineStr">
-        <is>
-          <t>2024-30</t>
-        </is>
-      </c>
-      <c r="D13" s="93" t="inlineStr">
-        <is>
-          <t>$100bn+ leases</t>
-        </is>
-      </c>
-      <c r="E13" s="93" t="inlineStr">
-        <is>
-          <t>Vendor / lease / SPV</t>
-        </is>
-      </c>
-      <c r="F13" s="94" t="inlineStr">
-        <is>
-          <t>MSFT 10-Q; CNBC</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="95" t="inlineStr">
-        <is>
-          <t>CoreWeave</t>
-        </is>
-      </c>
-      <c r="B14" s="96" t="inlineStr">
-        <is>
-          <t>DDTL 4.0 — $8.5bn delayed-draw term loan; first IG-rated (Moody's A3 / DBRS A-low) GPU-backed financing; SOFR+225 / ~5.9%</t>
-        </is>
-      </c>
-      <c r="C14" s="96" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="D14" s="96" t="inlineStr">
-        <is>
-          <t>$8.5bn</t>
-        </is>
-      </c>
-      <c r="E14" s="96" t="inlineStr">
-        <is>
-          <t>Bank / GPU-backed loan</t>
-        </is>
-      </c>
-      <c r="F14" s="97" t="inlineStr">
-        <is>
-          <t>CoreWeave IR</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="92" t="inlineStr">
-        <is>
-          <t>CoreWeave</t>
-        </is>
-      </c>
-      <c r="B15" s="93" t="inlineStr">
-        <is>
-          <t>$7.5bn debt facility led by Blackstone &amp; Magnetar (largest private debt deal at the time)</t>
-        </is>
-      </c>
-      <c r="C15" s="93" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="D15" s="93" t="inlineStr">
-        <is>
-          <t>$7.5bn</t>
-        </is>
-      </c>
-      <c r="E15" s="93" t="inlineStr">
-        <is>
-          <t>Private credit / loan</t>
-        </is>
-      </c>
-      <c r="F15" s="94" t="inlineStr">
-        <is>
-          <t>Blackstone</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="95" t="inlineStr">
-        <is>
-          <t>CoreWeave</t>
-        </is>
-      </c>
-      <c r="B16" s="96" t="inlineStr">
-        <is>
-          <t>$2.7bn 1.75% convertible notes; ~$30bn total debt by early 2026; ~$28bn debt+equity raised in 12 mos</t>
-        </is>
-      </c>
-      <c r="C16" s="96" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="D16" s="96" t="inlineStr">
-        <is>
-          <t>$2.7bn conv.</t>
-        </is>
-      </c>
-      <c r="E16" s="96" t="inlineStr">
-        <is>
-          <t>Convertibles</t>
-        </is>
-      </c>
-      <c r="F16" s="97" t="inlineStr">
-        <is>
-          <t>thedig; CoreWeave</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="92" t="inlineStr">
-        <is>
-          <t>CoreWeave</t>
-        </is>
-      </c>
-      <c r="B17" s="93" t="inlineStr">
-        <is>
-          <t>$2bn strategic equity from NVIDIA; IPO Mar 2025 raised ~$1.5bn</t>
-        </is>
-      </c>
-      <c r="C17" s="93" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="D17" s="93" t="inlineStr">
-        <is>
-          <t>$3.5bn equity</t>
-        </is>
-      </c>
-      <c r="E17" s="93" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="F17" s="94" t="inlineStr">
-        <is>
-          <t>CNBC; CoreWeave</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="95" t="inlineStr">
-        <is>
-          <t>SpaceX / xAI</t>
-        </is>
-      </c>
-      <c r="B18" s="96" t="inlineStr">
-        <is>
-          <t>SpaceX acquired xAI effective Feb 2, 2026; Colossus I &amp; II now SpaceX-owned (vertically-integrated AI platform; Terafab chip JV w/ Tesla &amp; Intel)</t>
-        </is>
-      </c>
-      <c r="C18" s="96" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="D18" s="96" t="inlineStr">
-        <is>
-          <t>merger</t>
-        </is>
-      </c>
-      <c r="E18" s="96" t="inlineStr">
-        <is>
-          <t>Equity / M&amp;A</t>
-        </is>
-      </c>
-      <c r="F18" s="97" t="inlineStr">
-        <is>
-          <t>SpaceX S-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="92" t="inlineStr">
-        <is>
-          <t>SpaceX / xAI</t>
-        </is>
-      </c>
-      <c r="B19" s="93" t="inlineStr">
-        <is>
-          <t>SpaceX AI capex $12.7bn in 2025 (~61% of total) + $7.7bn in Q1 2026; AI buildout funded by Starlink FCF, private raises, planned IPO</t>
-        </is>
-      </c>
-      <c r="C19" s="93" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="D19" s="93" t="inlineStr">
-        <is>
-          <t>$20bn+ capex</t>
-        </is>
-      </c>
-      <c r="E19" s="93" t="inlineStr">
-        <is>
-          <t>Internal / equity</t>
-        </is>
-      </c>
-      <c r="F19" s="94" t="inlineStr">
-        <is>
-          <t>SpaceX S-1; The Verge</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="95" t="inlineStr">
-        <is>
-          <t>SpaceX / xAI</t>
-        </is>
-      </c>
-      <c r="B20" s="96" t="inlineStr">
-        <is>
-          <t>Anthropic compute contract: $1.25bn/month (~$45bn) through May 2029 for Colossus I &amp; II — anchor revenue underwriting infra financing</t>
-        </is>
-      </c>
-      <c r="C20" s="96" t="inlineStr">
-        <is>
-          <t>2026-29</t>
-        </is>
-      </c>
-      <c r="D20" s="96" t="inlineStr">
-        <is>
-          <t>~$45bn</t>
-        </is>
-      </c>
-      <c r="E20" s="96" t="inlineStr">
-        <is>
-          <t>Take-or-pay (demand)</t>
-        </is>
-      </c>
-      <c r="F20" s="97" t="inlineStr">
-        <is>
-          <t>SpaceX S-1; The Verge</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="92" t="inlineStr">
-        <is>
-          <t>SpaceX / xAI</t>
-        </is>
-      </c>
-      <c r="B21" s="93" t="inlineStr">
-        <is>
-          <t>xAI $10bn raise ($5bn secured notes/term loans incl. Apollo $5bn facility + $5bn equity) via Morgan Stanley</t>
-        </is>
-      </c>
-      <c r="C21" s="93" t="inlineStr">
+      <c r="B55" s="96" t="inlineStr">
+        <is>
+          <t>MGX / Mubadala (UAE)</t>
+        </is>
+      </c>
+      <c r="C55" s="97" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="D55" s="96" t="inlineStr"/>
+      <c r="E55" s="98" t="inlineStr">
+        <is>
+          <t>~$40bn+</t>
+        </is>
+      </c>
+      <c r="F55" s="96" t="inlineStr">
+        <is>
+          <t>Sovereign equity / infra</t>
+        </is>
+      </c>
+      <c r="G55" s="96" t="inlineStr"/>
+      <c r="H55" s="96" t="inlineStr"/>
+      <c r="I55" s="96" t="inlineStr">
+        <is>
+          <t>Anchored Stargate; co-led ~$40bn Aligned Data Centers acquisition w/ BlackRock; AIP (BlackRock-Microsoft) targets up to $100bn global AI infra</t>
+        </is>
+      </c>
+      <c r="J55" s="99" t="inlineStr">
+        <is>
+          <t>NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="88" t="inlineStr">
+        <is>
+          <t>to 2026</t>
+        </is>
+      </c>
+      <c r="B56" s="88" t="inlineStr">
+        <is>
+          <t>Sector-wide</t>
+        </is>
+      </c>
+      <c r="C56" s="89" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D56" s="88" t="inlineStr"/>
+      <c r="E56" s="95" t="inlineStr">
+        <is>
+          <t>~$107bn</t>
+        </is>
+      </c>
+      <c r="F56" s="88" t="inlineStr">
+        <is>
+          <t>All debt</t>
+        </is>
+      </c>
+      <c r="G56" s="88" t="inlineStr"/>
+      <c r="H56" s="88" t="inlineStr"/>
+      <c r="I56" s="88" t="inlineStr">
+        <is>
+          <t>HY/unrated AI-infra issuers raised ~$107bn funded+committed debt by ~May 2026 ($68.7bn neoclouds / $38.7bn AI-native DCs)</t>
+        </is>
+      </c>
+      <c r="J56" s="91" t="inlineStr">
+        <is>
+          <t>Octus</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="88" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D21" s="93" t="inlineStr">
-        <is>
-          <t>$10bn</t>
-        </is>
-      </c>
-      <c r="E21" s="93" t="inlineStr">
-        <is>
-          <t>Loans + equity</t>
-        </is>
-      </c>
-      <c r="F21" s="94" t="inlineStr">
-        <is>
-          <t>CNBC</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="95" t="inlineStr">
-        <is>
-          <t>SpaceX / xAI</t>
-        </is>
-      </c>
-      <c r="B22" s="96" t="inlineStr">
-        <is>
-          <t>Colossus 2 SPV (Valor Equity): ~$12.5bn debt + ~$7.5bn equity (NVIDIA up to $2bn) to buy &amp; lease GPUs</t>
-        </is>
-      </c>
-      <c r="C22" s="96" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="D22" s="96" t="inlineStr">
-        <is>
-          <t>~$20bn</t>
-        </is>
-      </c>
-      <c r="E22" s="96" t="inlineStr">
-        <is>
-          <t>SPV / vendor lease</t>
-        </is>
-      </c>
-      <c r="F22" s="97" t="inlineStr">
-        <is>
-          <t>The Information; Yahoo</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="92" t="inlineStr">
-        <is>
-          <t>Nebius</t>
-        </is>
-      </c>
-      <c r="B23" s="93" t="inlineStr">
-        <is>
-          <t>$3bn+ convertibles + bank lines; lighter balance sheet; Yandex spin-off cash ~$2.5bn; NVIDIA ~$2bn equity; Microsoft ~$7bn prepay</t>
-        </is>
-      </c>
-      <c r="C23" s="93" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="D23" s="93" t="inlineStr">
-        <is>
-          <t>$3bn+</t>
-        </is>
-      </c>
-      <c r="E23" s="93" t="inlineStr">
-        <is>
-          <t>Convertibles</t>
-        </is>
-      </c>
-      <c r="F23" s="94" t="inlineStr">
-        <is>
-          <t>frankk research</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="95" t="inlineStr">
-        <is>
-          <t>Lambda</t>
-        </is>
-      </c>
-      <c r="B24" s="96" t="inlineStr">
-        <is>
-          <t>$500m GPU-backed facility from Macquarie</t>
-        </is>
-      </c>
-      <c r="C24" s="96" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="D24" s="96" t="inlineStr">
-        <is>
-          <t>$0.5bn</t>
-        </is>
-      </c>
-      <c r="E24" s="96" t="inlineStr">
-        <is>
-          <t>Bank / GPU-backed loan</t>
-        </is>
-      </c>
-      <c r="F24" s="97" t="inlineStr">
-        <is>
-          <t>theaiinsider</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="92" t="inlineStr">
-        <is>
-          <t>Nscale</t>
-        </is>
-      </c>
-      <c r="B25" s="93" t="inlineStr">
-        <is>
-          <t>$1.4bn term loan</t>
-        </is>
-      </c>
-      <c r="C25" s="93" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="D25" s="93" t="inlineStr">
-        <is>
-          <t>$1.4bn</t>
-        </is>
-      </c>
-      <c r="E25" s="93" t="inlineStr">
-        <is>
-          <t>Bank loan</t>
-        </is>
-      </c>
-      <c r="F25" s="94" t="inlineStr">
-        <is>
-          <t>theaiinsider</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="95" t="inlineStr">
-        <is>
-          <t>Fluidstack</t>
-        </is>
-      </c>
-      <c r="B26" s="96" t="inlineStr">
-        <is>
-          <t>Facility backed by ~$6.7bn Google-contracted revenue (Google lease backstop)</t>
-        </is>
-      </c>
-      <c r="C26" s="96" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="D26" s="96" t="inlineStr">
-        <is>
-          <t>~$6.7bn</t>
-        </is>
-      </c>
-      <c r="E26" s="96" t="inlineStr">
-        <is>
-          <t>SPV / private credit</t>
-        </is>
-      </c>
-      <c r="F26" s="97" t="inlineStr">
-        <is>
-          <t>theaiinsider</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="92" t="inlineStr">
-        <is>
-          <t>Applied Digital</t>
-        </is>
-      </c>
-      <c r="B27" s="93" t="inlineStr">
-        <is>
-          <t>$1.59bn high-yield bond (7%) for CoreWeave-leased campus (Polaris Forge 1)</t>
-        </is>
-      </c>
-      <c r="C27" s="93" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="D27" s="93" t="inlineStr">
-        <is>
-          <t>$1.59bn</t>
-        </is>
-      </c>
-      <c r="E27" s="93" t="inlineStr">
-        <is>
-          <t>Securitization / HY bond</t>
-        </is>
-      </c>
-      <c r="F27" s="94" t="inlineStr">
-        <is>
-          <t>TNW</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="95" t="inlineStr">
-        <is>
-          <t>Aligned Data Centers</t>
-        </is>
-      </c>
-      <c r="B28" s="96" t="inlineStr">
-        <is>
-          <t>$12bn capital raise ($5bn+ new equity + $7bn debt commitments) led by Macquarie (early 2025); later acquired by MGX/BlackRock consortium (~$40bn)</t>
-        </is>
-      </c>
-      <c r="C28" s="96" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="D28" s="96" t="inlineStr">
-        <is>
-          <t>$12bn / $40bn</t>
-        </is>
-      </c>
-      <c r="E28" s="96" t="inlineStr">
-        <is>
-          <t>Infra equity + debt</t>
-        </is>
-      </c>
-      <c r="F28" s="97" t="inlineStr">
-        <is>
-          <t>SFA; NYU DRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="92" t="inlineStr">
-        <is>
-          <t>QTS (Blackstone)</t>
-        </is>
-      </c>
-      <c r="B29" s="93" t="inlineStr">
-        <is>
-          <t>BX 2025-VOLT SASB CMBS $3.5bn (~10 QTS DCs); + Phoenix ABS (QTS Issuer 2025-1)</t>
-        </is>
-      </c>
-      <c r="C29" s="93" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="D29" s="93" t="inlineStr">
-        <is>
-          <t>$3.5bn+</t>
-        </is>
-      </c>
-      <c r="E29" s="93" t="inlineStr">
-        <is>
-          <t>Securitization (CMBS/ABS)</t>
-        </is>
-      </c>
-      <c r="F29" s="94" t="inlineStr">
-        <is>
-          <t>CREFC; SFA</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="95" t="inlineStr">
-        <is>
-          <t>Switch (DigitalBridge)</t>
-        </is>
-      </c>
-      <c r="B30" s="96" t="inlineStr">
-        <is>
-          <t>$2.4bn SASB CMBS (SWCH 2025-DATA) + $1.1bn ABS — green bonds</t>
-        </is>
-      </c>
-      <c r="C30" s="96" t="inlineStr">
-        <is>
-          <t>2024-25</t>
-        </is>
-      </c>
-      <c r="D30" s="96" t="inlineStr">
-        <is>
-          <t>$3.5bn</t>
-        </is>
-      </c>
-      <c r="E30" s="96" t="inlineStr">
-        <is>
-          <t>Securitization (CMBS/ABS)</t>
-        </is>
-      </c>
-      <c r="F30" s="97" t="inlineStr">
-        <is>
-          <t>SFA; CREFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="92" t="inlineStr">
-        <is>
-          <t>Vantage Data Centers</t>
-        </is>
-      </c>
-      <c r="B31" s="93" t="inlineStr">
-        <is>
-          <t>First public data-center ABS (2024); ongoing multi-billion securitization &amp; infra-equity program</t>
-        </is>
-      </c>
-      <c r="C31" s="93" t="inlineStr">
-        <is>
-          <t>2024-26</t>
-        </is>
-      </c>
-      <c r="D31" s="93" t="inlineStr">
-        <is>
-          <t>multi-$bn</t>
-        </is>
-      </c>
-      <c r="E31" s="93" t="inlineStr">
-        <is>
-          <t>Securitization / equity</t>
-        </is>
-      </c>
-      <c r="F31" s="94" t="inlineStr">
-        <is>
-          <t>Dentons</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="95" t="inlineStr">
-        <is>
-          <t>Colocation sector</t>
-        </is>
-      </c>
-      <c r="B32" s="96" t="inlineStr">
-        <is>
-          <t>US data-center ABS+CMBS issuance ~$26bn in 2025 (~10x 2020); ~$57bn since 2021; Morgan Stanley ~$130bn securitized net issuance 2026-28; ~$150bn permanent financing need 2026-27</t>
-        </is>
-      </c>
-      <c r="C32" s="96" t="inlineStr">
-        <is>
-          <t>2025-28</t>
-        </is>
-      </c>
-      <c r="D32" s="96" t="inlineStr">
-        <is>
-          <t>~$130bn</t>
-        </is>
-      </c>
-      <c r="E32" s="96" t="inlineStr">
-        <is>
-          <t>Securitization (ABS/CMBS)</t>
-        </is>
-      </c>
-      <c r="F32" s="97" t="inlineStr">
-        <is>
-          <t>Impax; CREFC; Morgan Stanley</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="92" t="inlineStr">
-        <is>
-          <t>HUMAIN (Saudi PIF)</t>
-        </is>
-      </c>
-      <c r="B33" s="93" t="inlineStr">
-        <is>
-          <t>PIF national AI champion (announced 13 May 2025): ~$100bn across 11 data centers / 2.2 GW; ~600k NVIDIA GPUs; ALLAM Arabic LLM</t>
-        </is>
-      </c>
-      <c r="C33" s="93" t="inlineStr">
+      <c r="B57" s="88" t="inlineStr">
+        <is>
+          <t>Sector-wide</t>
+        </is>
+      </c>
+      <c r="C57" s="89" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D57" s="88" t="inlineStr"/>
+      <c r="E57" s="95" t="inlineStr">
+        <is>
+          <t>~$180bn</t>
+        </is>
+      </c>
+      <c r="F57" s="88" t="inlineStr">
+        <is>
+          <t>Insurance / private credit</t>
+        </is>
+      </c>
+      <c r="G57" s="88" t="inlineStr"/>
+      <c r="H57" s="88" t="inlineStr"/>
+      <c r="I57" s="88" t="inlineStr">
+        <is>
+          <t>Insurance-linked platforms deployed ~$180bn into private credit in 2025 (~25% of global private credit AUM)</t>
+        </is>
+      </c>
+      <c r="J57" s="91" t="inlineStr">
+        <is>
+          <t>McKinsey; ABF Journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="88" t="inlineStr">
         <is>
           <t>2025-30</t>
         </is>
       </c>
-      <c r="D33" s="93" t="inlineStr">
-        <is>
-          <t>~$100bn</t>
-        </is>
-      </c>
-      <c r="E33" s="93" t="inlineStr">
-        <is>
-          <t>Sovereign equity</t>
-        </is>
-      </c>
-      <c r="F33" s="94" t="inlineStr">
-        <is>
-          <t>Presenc AI; NYU DRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="95" t="inlineStr">
-        <is>
-          <t>Stargate UAE / G42</t>
-        </is>
-      </c>
-      <c r="B34" s="96" t="inlineStr">
-        <is>
-          <t>$30bn+ 5GW Abu Dhabi campus (Khazna/G42 w/ OpenAI, Oracle, NVIDIA, Cisco, SoftBank); Phase 1 200MW Q3 2026; Microsoft ~$1.5bn equity</t>
-        </is>
-      </c>
-      <c r="C34" s="96" t="inlineStr">
-        <is>
-          <t>2025-30</t>
-        </is>
-      </c>
-      <c r="D34" s="96" t="inlineStr">
-        <is>
-          <t>~$30bn+</t>
-        </is>
-      </c>
-      <c r="E34" s="96" t="inlineStr">
-        <is>
-          <t>Sovereign equity + JV</t>
-        </is>
-      </c>
-      <c r="F34" s="97" t="inlineStr">
-        <is>
-          <t>Khaleej Times; dcpulse</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="92" t="inlineStr">
-        <is>
-          <t>MGX / Mubadala (UAE)</t>
-        </is>
-      </c>
-      <c r="B35" s="93" t="inlineStr">
-        <is>
-          <t>Anchored Stargate; co-led ~$40bn Aligned Data Centers acquisition w/ BlackRock; AIP (BlackRock-Microsoft) targets up to $100bn global AI infra</t>
-        </is>
-      </c>
-      <c r="C35" s="93" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="D35" s="93" t="inlineStr">
-        <is>
-          <t>~$40bn+</t>
-        </is>
-      </c>
-      <c r="E35" s="93" t="inlineStr">
-        <is>
-          <t>Sovereign equity / infra</t>
-        </is>
-      </c>
-      <c r="F35" s="94" t="inlineStr">
-        <is>
-          <t>NYU DRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="95" t="inlineStr">
-        <is>
-          <t>Qatar (QIA / Qai)</t>
-        </is>
-      </c>
-      <c r="B36" s="96" t="inlineStr">
-        <is>
-          <t>~$20bn AI-infrastructure JV with Brookfield (late 2025); earlier positions in xAI &amp; Databricks</t>
-        </is>
-      </c>
-      <c r="C36" s="96" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="D36" s="96" t="inlineStr">
-        <is>
-          <t>~$20bn</t>
-        </is>
-      </c>
-      <c r="E36" s="96" t="inlineStr">
-        <is>
-          <t>Sovereign equity + JV</t>
-        </is>
-      </c>
-      <c r="F36" s="97" t="inlineStr">
-        <is>
-          <t>NYU DRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="92" t="inlineStr">
+      <c r="B58" s="88" t="inlineStr">
         <is>
           <t>Sector-wide</t>
         </is>
       </c>
-      <c r="B37" s="93" t="inlineStr">
-        <is>
-          <t>HY/unrated AI-infra issuers raised ~$107bn funded+committed debt by ~May 2026 ($68.7bn neoclouds / $38.7bn AI-native DCs)</t>
-        </is>
-      </c>
-      <c r="C37" s="93" t="inlineStr">
-        <is>
-          <t>to 2026</t>
-        </is>
-      </c>
-      <c r="D37" s="93" t="inlineStr">
-        <is>
-          <t>~$107bn</t>
-        </is>
-      </c>
-      <c r="E37" s="93" t="inlineStr">
-        <is>
-          <t>All debt</t>
-        </is>
-      </c>
-      <c r="F37" s="94" t="inlineStr">
-        <is>
-          <t>Octus</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="95" t="inlineStr">
-        <is>
-          <t>Sector-wide</t>
-        </is>
-      </c>
-      <c r="B38" s="96" t="inlineStr">
-        <is>
-          <t>Insurance-linked platforms deployed ~$180bn into private credit in 2025 (~25% of global private credit AUM)</t>
-        </is>
-      </c>
-      <c r="C38" s="96" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="D38" s="96" t="inlineStr">
-        <is>
-          <t>~$180bn</t>
-        </is>
-      </c>
-      <c r="E38" s="96" t="inlineStr">
-        <is>
-          <t>Insurance / private credit</t>
-        </is>
-      </c>
-      <c r="F38" s="97" t="inlineStr">
-        <is>
-          <t>McKinsey; ABF Journal</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="92" t="inlineStr">
-        <is>
-          <t>Sector-wide</t>
-        </is>
-      </c>
-      <c r="B39" s="93" t="inlineStr">
+      <c r="C58" s="89" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D58" s="88" t="inlineStr"/>
+      <c r="E58" s="95" t="inlineStr">
+        <is>
+          <t>$5.3tn capex</t>
+        </is>
+      </c>
+      <c r="F58" s="88" t="inlineStr">
+        <is>
+          <t>Context</t>
+        </is>
+      </c>
+      <c r="G58" s="88" t="inlineStr"/>
+      <c r="H58" s="88" t="inlineStr"/>
+      <c r="I58" s="88" t="inlineStr">
         <is>
           <t>Goldman Sachs: ~$5.3tn AI + data-center capex 2025-2030; Morgan Stanley: ~$800bn private credit for AI DCs 2025-28</t>
         </is>
       </c>
-      <c r="C39" s="93" t="inlineStr">
-        <is>
-          <t>2025-30</t>
-        </is>
-      </c>
-      <c r="D39" s="93" t="inlineStr">
-        <is>
-          <t>$5.3tn capex</t>
-        </is>
-      </c>
-      <c r="E39" s="93" t="inlineStr">
-        <is>
-          <t>Context</t>
-        </is>
-      </c>
-      <c r="F39" s="94" t="inlineStr">
+      <c r="J58" s="91" t="inlineStr">
         <is>
           <t>Goldman; Morgan Stanley</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="98" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="100" t="inlineStr">
         <is>
           <t>Selected sources:</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="99" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="101" t="inlineStr">
         <is>
           <t>Goldman Sachs Research — ~$5.3tn AI + data-center capex 2025-2030; private markets in DC financing.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="99" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="101" t="inlineStr">
         <is>
           <t>Morgan Stanley — ~$2tn capex 2025-28 with &gt;$1tn debt; ~$800bn private credit for AI DCs.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="99" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="101" t="inlineStr">
         <is>
           <t>Bank of America / BofA Securities — hyperscaler bond issuance ($121bn 2025; ~$175bn 2026E).</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="99" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="101" t="inlineStr">
         <is>
           <t>Moody's Ratings — hyperscaler capex (~$785bn 2026, ~$1tn 2027); $662bn off-B/S DC leases.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="99" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="101" t="inlineStr">
         <is>
           <t>McKinsey — ~$2.7tn US (5.2tn global) data-center capex by 2030; insurance-linked private credit.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="99" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="101" t="inlineStr">
         <is>
           <t>Octus — HY/unrated AI-infra debt (~$107bn to ~May 2026); ~14GW unfunded ≈ $344bn need.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="99" t="inlineStr">
-        <is>
-          <t>Company disclosures &amp; press: Meta IR / FT / S&amp;P (Hyperion); Oracle IR / IFR / Reuters; CoreWeave IR;</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CNBC / WSJ / The Information (xAI); Blackstone; Apollo Academy; MUFG; CreditSights; CNA.</t>
+    <row r="67">
+      <c r="A67" s="101" t="inlineStr">
+        <is>
+          <t>Company / press: Meta IR, FT, S&amp;P, IFR (Hyperion); Oracle IR, IFR, Reuters; CoreWeave IR; Blackstone;</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Apollo Academy; privatedebtnews; Bisnow; Quinn Emanuel; Build.inc; CNBC / WSJ / The Information (xAI).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make Deals tab debt-amount column numeric-only; group by instrument incl. loans, private credit, insurance-linked
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AI_Infrastructure_Financing_2025-2030.xlsx
+++ b/AI_Infrastructure_Financing_2025-2030.xlsx
@@ -214,12 +214,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCEFC7"/>
+        <fgColor rgb="00F0F0F0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0F0F0"/>
+        <fgColor rgb="00FCEFC7"/>
       </patternFill>
     </fill>
   </fills>
@@ -249,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -455,46 +455,49 @@
     <xf numFmtId="0" fontId="28" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="26" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="26" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -8143,7 +8146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8161,14 +8164,14 @@
     <row r="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>AI-Infrastructure Deals — Private Credit &amp; Other Key Transactions (US$bn)</t>
+          <t>AI-Infrastructure Debt Transactions &amp; Sources (US$bn)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Unified transaction log. Section 1: private-credit / SPV / 144A debt (itemized deals summed). Section 2: context/frameworks. Section 3: other key deals (bonds, equity, securitization, sovereign, leases). Amounts '~' = approximate.</t>
+          <t>Transaction log grouped by debt instrument (bonds, loans, alternate private credit, insurance-linked, securitization, convertibles). Groups 1,2,3,5,6 are summed; insurance-linked (4), vendor (7), equity/sovereign (8) and context (9) are memos. 'Debt amount ($bn)' is numeric only.</t>
         </is>
       </c>
     </row>
@@ -8229,7 +8232,7 @@
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>1) PRIVATE CREDIT TRANSACTIONS (itemized — summed below)</t>
+          <t>1) CORPORATE BONDS (public IG/HY)</t>
         </is>
       </c>
       <c r="B5" s="15" t="n"/>
@@ -8245,112 +8248,112 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="70" t="inlineStr">
         <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B6" s="71" t="inlineStr">
+        <is>
+          <t>Amazon (AWS)</t>
+        </is>
+      </c>
+      <c r="C6" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D6" s="70" t="inlineStr">
+        <is>
+          <t>Bank syndicate</t>
+        </is>
+      </c>
+      <c r="E6" s="73" t="n">
+        <v>71</v>
+      </c>
+      <c r="F6" s="70" t="inlineStr">
+        <is>
+          <t>Public IG bonds ($54bn + EUR14.5bn)</t>
+        </is>
+      </c>
+      <c r="G6" s="70" t="inlineStr">
+        <is>
+          <t>IG</t>
+        </is>
+      </c>
+      <c r="H6" s="70" t="inlineStr">
+        <is>
+          <t>3-40y</t>
+        </is>
+      </c>
+      <c r="I6" s="70" t="inlineStr">
+        <is>
+          <t>~4x oversubscribed</t>
+        </is>
+      </c>
+      <c r="J6" s="74" t="inlineStr">
+        <is>
+          <t>CNA; Reuters</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="70" t="inlineStr">
+        <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="B6" s="71" t="inlineStr">
-        <is>
-          <t>Oracle — Texas + Wisconsin data centers</t>
-        </is>
-      </c>
-      <c r="C6" s="72" t="inlineStr">
+      <c r="B7" s="71" t="inlineStr">
+        <is>
+          <t>Alphabet (Google)</t>
+        </is>
+      </c>
+      <c r="C7" s="72" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="D6" s="70" t="inlineStr">
-        <is>
-          <t>Private credit consortium</t>
-        </is>
-      </c>
-      <c r="E6" s="73" t="n">
-        <v>38</v>
-      </c>
-      <c r="F6" s="70" t="inlineStr">
-        <is>
-          <t>SPV debt package</t>
-        </is>
-      </c>
-      <c r="G6" s="70" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H6" s="70" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I6" s="70" t="inlineStr">
-        <is>
-          <t>Two-site off-B/S financing</t>
-        </is>
-      </c>
-      <c r="J6" s="74" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="75" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B7" s="76" t="inlineStr">
-        <is>
-          <t>Anthropic — Google TPU chip SPV</t>
-        </is>
-      </c>
-      <c r="C7" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D7" s="75" t="inlineStr">
-        <is>
-          <t>Apollo (Atlas SP $0.8bn equity; Athene), Blackstone; Broadcom RVG</t>
-        </is>
-      </c>
-      <c r="E7" s="78" t="n">
-        <v>35</v>
-      </c>
-      <c r="F7" s="75" t="inlineStr">
-        <is>
-          <t>Chip-leasing SPV; 3 tranches; ~half syndicated</t>
-        </is>
-      </c>
-      <c r="G7" s="75" t="inlineStr">
-        <is>
-          <t>A1 T+100bp; A2 5.75%; B 8.5%</t>
-        </is>
-      </c>
-      <c r="H7" s="75" t="inlineStr">
-        <is>
-          <t>~5y</t>
-        </is>
-      </c>
-      <c r="I7" s="75" t="inlineStr">
-        <is>
-          <t>Buys Google TPUs leased to Anthropic; Broadcom residual-value support</t>
-        </is>
-      </c>
-      <c r="J7" s="79" t="inlineStr">
-        <is>
-          <t>privatedebtnews; Build.inc</t>
+      <c r="D7" s="70" t="inlineStr">
+        <is>
+          <t>Bank syndicate</t>
+        </is>
+      </c>
+      <c r="E7" s="73" t="n">
+        <v>50</v>
+      </c>
+      <c r="F7" s="70" t="inlineStr">
+        <is>
+          <t>Public bonds ($32bn incl 100-yr + $17.5bn)</t>
+        </is>
+      </c>
+      <c r="G7" s="70" t="inlineStr">
+        <is>
+          <t>IG</t>
+        </is>
+      </c>
+      <c r="H7" s="70" t="inlineStr">
+        <is>
+          <t>to 100y</t>
+        </is>
+      </c>
+      <c r="I7" s="70" t="inlineStr">
+        <is>
+          <t>Rare 100-year tranche</t>
+        </is>
+      </c>
+      <c r="J7" s="74" t="inlineStr">
+        <is>
+          <t>ConstructConnect; CNA</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="70" t="inlineStr">
         <is>
-          <t>Oct 2025</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="B8" s="71" t="inlineStr">
         <is>
-          <t>Meta — Hyperion (Beignet Investor LLC), Louisiana</t>
+          <t>Meta Platforms</t>
         </is>
       </c>
       <c r="C8" s="72" t="inlineStr">
@@ -8360,47 +8363,47 @@
       </c>
       <c r="D8" s="70" t="inlineStr">
         <is>
-          <t>PIMCO (~$18bn), BlackRock, Apollo (debt); Blue Owl (equity); MS adviser</t>
+          <t>Bank syndicate (BofA et al.)</t>
         </is>
       </c>
       <c r="E8" s="73" t="n">
-        <v>27.3</v>
+        <v>30</v>
       </c>
       <c r="F8" s="70" t="inlineStr">
         <is>
-          <t>Off-B/S SPV; 144A senior secured bond</t>
+          <t>Public IG corporate bond</t>
         </is>
       </c>
       <c r="G8" s="70" t="inlineStr">
         <is>
-          <t>6.581% / T+225bp</t>
+          <t>~5-6%</t>
         </is>
       </c>
       <c r="H8" s="70" t="inlineStr">
         <is>
-          <t>Due May 2049 (~23.6y)</t>
+          <t>to 2063</t>
         </is>
       </c>
       <c r="I8" s="70" t="inlineStr">
         <is>
-          <t>2.1GW campus; Meta lease + residual-value guarantee (up to ~$28bn); A+ (S&amp;P)</t>
+          <t>Largest IG deal of 2025</t>
         </is>
       </c>
       <c r="J8" s="74" t="inlineStr">
         <is>
-          <t>IFR; FT; Quinn Emanuel</t>
+          <t>BofA; MUFG</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="70" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="B9" s="71" t="inlineStr">
         <is>
-          <t>Oracle — New Mexico site</t>
+          <t>Oracle (OCI)</t>
         </is>
       </c>
       <c r="C9" s="72" t="inlineStr">
@@ -8410,35 +8413,35 @@
       </c>
       <c r="D9" s="70" t="inlineStr">
         <is>
-          <t>Private credit lenders</t>
+          <t>Goldman Sachs</t>
         </is>
       </c>
       <c r="E9" s="73" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F9" s="70" t="inlineStr">
         <is>
-          <t>SPV / project loan</t>
+          <t>Public IG bond (8-part)</t>
         </is>
       </c>
       <c r="G9" s="70" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="H9" s="70" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>3-40y</t>
         </is>
       </c>
       <c r="I9" s="70" t="inlineStr">
         <is>
-          <t>Single-site project loan</t>
+          <t>Within $45-50bn CY26 plan</t>
         </is>
       </c>
       <c r="J9" s="74" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>Oracle IR; IFR</t>
         </is>
       </c>
     </row>
@@ -8450,7 +8453,7 @@
       </c>
       <c r="B10" s="71" t="inlineStr">
         <is>
-          <t>Oracle — Michigan campus</t>
+          <t>Oracle (OCI)</t>
         </is>
       </c>
       <c r="C10" s="72" t="inlineStr">
@@ -8460,137 +8463,95 @@
       </c>
       <c r="D10" s="70" t="inlineStr">
         <is>
-          <t>Project-finance lenders</t>
+          <t>Bank syndicate</t>
         </is>
       </c>
       <c r="E10" s="73" t="n">
-        <v>16.3</v>
+        <v>18</v>
       </c>
       <c r="F10" s="70" t="inlineStr">
         <is>
-          <t>Project-level SPV financing</t>
+          <t>Public IG bond (6-part)</t>
         </is>
       </c>
       <c r="G10" s="70" t="inlineStr">
         <is>
+          <t>IG</t>
+        </is>
+      </c>
+      <c r="H10" s="70" t="inlineStr">
+        <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H10" s="70" t="inlineStr">
+      <c r="I10" s="70" t="inlineStr"/>
+      <c r="J10" s="74" t="inlineStr">
+        <is>
+          <t>Reuters; CNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B11" s="71" t="inlineStr">
+        <is>
+          <t>Amazon (AWS)</t>
+        </is>
+      </c>
+      <c r="C11" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D11" s="70" t="inlineStr">
+        <is>
+          <t>Bank syndicate</t>
+        </is>
+      </c>
+      <c r="E11" s="73" t="n">
+        <v>15</v>
+      </c>
+      <c r="F11" s="70" t="inlineStr">
+        <is>
+          <t>Public IG bond</t>
+        </is>
+      </c>
+      <c r="G11" s="70" t="inlineStr">
+        <is>
+          <t>IG</t>
+        </is>
+      </c>
+      <c r="H11" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I10" s="70" t="inlineStr">
-        <is>
-          <t>OCI capacity build</t>
-        </is>
-      </c>
-      <c r="J10" s="74" t="inlineStr">
-        <is>
-          <t>Press reports</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="75" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="B11" s="76" t="inlineStr">
-        <is>
-          <t>xAI — Colossus 2 chip SPV (Memphis/Southaven)</t>
-        </is>
-      </c>
-      <c r="C11" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D11" s="75" t="inlineStr">
-        <is>
-          <t>Valor Equity (lead), Apollo, Diameter (debt); NVIDIA up to $2bn equity</t>
-        </is>
-      </c>
-      <c r="E11" s="78" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="F11" s="75" t="inlineStr">
-        <is>
-          <t>SPV; debt + ~$7.5bn equity to buy &amp; lease GPUs</t>
-        </is>
-      </c>
-      <c r="G11" s="75" t="inlineStr">
-        <is>
-          <t>~10.5%</t>
-        </is>
-      </c>
-      <c r="H11" s="75" t="inlineStr">
-        <is>
-          <t>5y (~2.5y avg life)</t>
-        </is>
-      </c>
-      <c r="I11" s="75" t="inlineStr">
-        <is>
-          <t>Buys NVIDIA GPUs leased to xAI; chips as collateral</t>
-        </is>
-      </c>
-      <c r="J11" s="79" t="inlineStr">
-        <is>
-          <t>FT; WSJ; AAE filing</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="70" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B12" s="71" t="inlineStr">
-        <is>
-          <t>Oracle/OpenAI — Abilene, TX (Stargate; Crusoe developer)</t>
-        </is>
-      </c>
-      <c r="C12" s="72" t="inlineStr">
-        <is>
-          <t>Hyperscaler</t>
-        </is>
-      </c>
-      <c r="D12" s="70" t="inlineStr">
-        <is>
-          <t>Blue Owl + JPMorgan (incl. Crusoe, Primary Digital Infrastructure)</t>
-        </is>
-      </c>
-      <c r="E12" s="73" t="n">
-        <v>10</v>
-      </c>
-      <c r="F12" s="70" t="inlineStr">
-        <is>
-          <t>Off-B/S SPV (~$13bn incl. equity)</t>
-        </is>
-      </c>
-      <c r="G12" s="70" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H12" s="70" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I12" s="70" t="inlineStr">
-        <is>
-          <t>SPV owns OpenAI Abilene facility</t>
-        </is>
-      </c>
-      <c r="J12" s="74" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
+      <c r="I11" s="70" t="inlineStr"/>
+      <c r="J11" s="74" t="inlineStr">
+        <is>
+          <t>CNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>2) BANK &amp; SYNDICATED LOANS (incl. GPU-backed term loans)</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="15" t="n"/>
+      <c r="I12" s="15" t="n"/>
+      <c r="J12" s="15" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="75" t="inlineStr">
@@ -8600,7 +8561,7 @@
       </c>
       <c r="B13" s="76" t="inlineStr">
         <is>
-          <t>CoreWeave — DDTL 4.0 (Compute Acq. Co. VIII)</t>
+          <t>CoreWeave — DDTL 4.0</t>
         </is>
       </c>
       <c r="C13" s="77" t="inlineStr">
@@ -8618,12 +8579,12 @@
       </c>
       <c r="F13" s="75" t="inlineStr">
         <is>
-          <t>Non-recourse GPU-backed delayed-draw term loan</t>
+          <t>GPU-backed delayed-draw term loan</t>
         </is>
       </c>
       <c r="G13" s="75" t="inlineStr">
         <is>
-          <t>SOFR+225 / ~5.9% fixed</t>
+          <t>SOFR+225 / ~5.9%</t>
         </is>
       </c>
       <c r="H13" s="75" t="inlineStr">
@@ -8633,7 +8594,7 @@
       </c>
       <c r="I13" s="75" t="inlineStr">
         <is>
-          <t>First IG-rated (A3 / A low) HPC-collateralized loan</t>
+          <t>First IG-rated (A3 / A low) HPC loan; non-recourse</t>
         </is>
       </c>
       <c r="J13" s="79" t="inlineStr">
@@ -8643,102 +8604,102 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="75" t="inlineStr">
-        <is>
-          <t>May 2024</t>
-        </is>
-      </c>
-      <c r="B14" s="76" t="inlineStr">
-        <is>
-          <t>CoreWeave — $7.5bn debt facility</t>
-        </is>
-      </c>
-      <c r="C14" s="77" t="inlineStr">
+      <c r="A14" s="80" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="B14" s="81" t="inlineStr">
+        <is>
+          <t>Applied Digital</t>
+        </is>
+      </c>
+      <c r="C14" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D14" s="80" t="inlineStr">
+        <is>
+          <t>Macquarie</t>
+        </is>
+      </c>
+      <c r="E14" s="83" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" s="80" t="inlineStr">
+        <is>
+          <t>Structured HPC financing</t>
+        </is>
+      </c>
+      <c r="G14" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H14" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I14" s="80" t="inlineStr">
+        <is>
+          <t>Powered-shell build for CoreWeave</t>
+        </is>
+      </c>
+      <c r="J14" s="84" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="75" t="inlineStr">
+        <is>
+          <t>May 2025</t>
+        </is>
+      </c>
+      <c r="B15" s="76" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C15" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D14" s="75" t="inlineStr">
-        <is>
-          <t>Blackstone, Magnetar (co-leads), Coatue, Carlyle, CDPQ, BlackRock, Eldridge</t>
-        </is>
-      </c>
-      <c r="E14" s="78" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="F14" s="75" t="inlineStr">
-        <is>
-          <t>GPU + customer-contract secured facility</t>
-        </is>
-      </c>
-      <c r="G14" s="75" t="inlineStr">
-        <is>
-          <t>~10%+ (at issue)</t>
-        </is>
-      </c>
-      <c r="H14" s="75" t="inlineStr">
+      <c r="D15" s="75" t="inlineStr">
+        <is>
+          <t>Bank syndicate</t>
+        </is>
+      </c>
+      <c r="E15" s="78" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F15" s="75" t="inlineStr">
+        <is>
+          <t>Revolving credit line</t>
+        </is>
+      </c>
+      <c r="G15" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I14" s="75" t="inlineStr">
-        <is>
-          <t>Largest private debt deal at the time</t>
-        </is>
-      </c>
-      <c r="J14" s="79" t="inlineStr">
-        <is>
-          <t>Blackstone</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="80" t="inlineStr">
-        <is>
-          <t>Early 2025</t>
-        </is>
-      </c>
-      <c r="B15" s="81" t="inlineStr">
-        <is>
-          <t>Aligned Data Centers — debt commitments</t>
-        </is>
-      </c>
-      <c r="C15" s="82" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REIT</t>
-        </is>
-      </c>
-      <c r="D15" s="80" t="inlineStr">
-        <is>
-          <t>Macquarie + global investors</t>
-        </is>
-      </c>
-      <c r="E15" s="83" t="n">
-        <v>7</v>
-      </c>
-      <c r="F15" s="80" t="inlineStr">
-        <is>
-          <t>Debt within $12bn raise (+$5bn equity)</t>
-        </is>
-      </c>
-      <c r="G15" s="80" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H15" s="80" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I15" s="80" t="inlineStr">
-        <is>
-          <t>Later acquired by MGX/BlackRock (~$40bn)</t>
-        </is>
-      </c>
-      <c r="J15" s="84" t="inlineStr">
-        <is>
-          <t>SFA; NYU DRI</t>
+      <c r="H15" s="75" t="inlineStr">
+        <is>
+          <t>5y</t>
+        </is>
+      </c>
+      <c r="I15" s="75" t="inlineStr">
+        <is>
+          <t>Liquidity backstop</t>
+        </is>
+      </c>
+      <c r="J15" s="79" t="inlineStr">
+        <is>
+          <t>CNBC</t>
         </is>
       </c>
     </row>
@@ -8750,7 +8711,7 @@
       </c>
       <c r="B16" s="76" t="inlineStr">
         <is>
-          <t>Fluidstack — Google-backed facility</t>
+          <t>Nscale</t>
         </is>
       </c>
       <c r="C16" s="77" t="inlineStr">
@@ -8760,15 +8721,15 @@
       </c>
       <c r="D16" s="75" t="inlineStr">
         <is>
-          <t>Private credit (Google lease backstop)</t>
+          <t>Private credit / banks</t>
         </is>
       </c>
       <c r="E16" s="78" t="n">
-        <v>6.7</v>
+        <v>1.4</v>
       </c>
       <c r="F16" s="75" t="inlineStr">
         <is>
-          <t>SPV backed by contracted revenue</t>
+          <t>Term loan</t>
         </is>
       </c>
       <c r="G16" s="75" t="inlineStr">
@@ -8783,7 +8744,7 @@
       </c>
       <c r="I16" s="75" t="inlineStr">
         <is>
-          <t>~$6.7bn Google-contracted revenue backstop</t>
+          <t>GPU-cloud build</t>
         </is>
       </c>
       <c r="J16" s="79" t="inlineStr">
@@ -8795,12 +8756,12 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="75" t="inlineStr">
         <is>
-          <t>Jun-Jul 2025</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="B17" s="76" t="inlineStr">
         <is>
-          <t>xAI — secured notes / term loan (part of $10bn raise)</t>
+          <t>Lambda</t>
         </is>
       </c>
       <c r="C17" s="77" t="inlineStr">
@@ -8810,133 +8771,99 @@
       </c>
       <c r="D17" s="75" t="inlineStr">
         <is>
-          <t>Apollo, Diameter; Morgan Stanley arranger</t>
+          <t>Macquarie</t>
         </is>
       </c>
       <c r="E17" s="78" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="F17" s="75" t="inlineStr">
         <is>
-          <t>Secured notes + term loan</t>
+          <t>GPU-backed facility</t>
         </is>
       </c>
       <c r="G17" s="75" t="inlineStr">
         <is>
-          <t>up to ~12.5%</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H17" s="75" t="inlineStr">
         <is>
-          <t>~3-5y</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I17" s="75" t="inlineStr">
         <is>
-          <t>Lenders can seize/operate Colossus on default</t>
+          <t>GPU-cloud build</t>
         </is>
       </c>
       <c r="J17" s="79" t="inlineStr">
         <is>
-          <t>CNBC; ciphertalk</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="80" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B18" s="81" t="inlineStr">
-        <is>
-          <t>Applied Digital — Macquarie financing</t>
-        </is>
-      </c>
-      <c r="C18" s="82" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REIT</t>
-        </is>
-      </c>
-      <c r="D18" s="80" t="inlineStr">
-        <is>
-          <t>Macquarie</t>
-        </is>
-      </c>
-      <c r="E18" s="83" t="n">
-        <v>5</v>
-      </c>
-      <c r="F18" s="80" t="inlineStr">
-        <is>
-          <t>Perpetual/structured HPC financing</t>
-        </is>
-      </c>
-      <c r="G18" s="80" t="inlineStr">
+          <t>theaiinsider</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>3) ALTERNATE PRIVATE CREDIT / SPV / 144A</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="15" t="n"/>
+      <c r="I18" s="15" t="n"/>
+      <c r="J18" s="15" t="n"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="70" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B19" s="71" t="inlineStr">
+        <is>
+          <t>Oracle — Texas + Wisconsin DCs</t>
+        </is>
+      </c>
+      <c r="C19" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D19" s="70" t="inlineStr">
+        <is>
+          <t>Private credit consortium</t>
+        </is>
+      </c>
+      <c r="E19" s="73" t="n">
+        <v>38</v>
+      </c>
+      <c r="F19" s="70" t="inlineStr">
+        <is>
+          <t>SPV debt package</t>
+        </is>
+      </c>
+      <c r="G19" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H18" s="80" t="inlineStr">
+      <c r="H19" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I18" s="80" t="inlineStr">
-        <is>
-          <t>Powered-shell build for CoreWeave (Polaris Forge)</t>
-        </is>
-      </c>
-      <c r="J18" s="84" t="inlineStr">
-        <is>
-          <t>press</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="75" t="inlineStr">
-        <is>
-          <t>Jul 2025</t>
-        </is>
-      </c>
-      <c r="B19" s="76" t="inlineStr">
-        <is>
-          <t>CoreWeave — OpenAI contract financing</t>
-        </is>
-      </c>
-      <c r="C19" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D19" s="75" t="inlineStr">
-        <is>
-          <t>Private lenders (SPV)</t>
-        </is>
-      </c>
-      <c r="E19" s="78" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="F19" s="75" t="inlineStr">
-        <is>
-          <t>SPV debt vs. $11.9bn OpenAI contract</t>
-        </is>
-      </c>
-      <c r="G19" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H19" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I19" s="75" t="inlineStr">
-        <is>
-          <t>Funds CoreWeave's OpenAI compute obligations</t>
-        </is>
-      </c>
-      <c r="J19" s="79" t="inlineStr">
+      <c r="I19" s="70" t="inlineStr">
+        <is>
+          <t>Two-site off-B/S financing</t>
+        </is>
+      </c>
+      <c r="J19" s="74" t="inlineStr">
         <is>
           <t>FT</t>
         </is>
@@ -8945,452 +8872,607 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="75" t="inlineStr">
         <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B20" s="76" t="inlineStr">
+        <is>
+          <t>Anthropic — Google TPU chip SPV</t>
+        </is>
+      </c>
+      <c r="C20" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D20" s="75" t="inlineStr">
+        <is>
+          <t>Apollo, Blackstone; Broadcom RVG</t>
+        </is>
+      </c>
+      <c r="E20" s="78" t="n">
+        <v>35</v>
+      </c>
+      <c r="F20" s="75" t="inlineStr">
+        <is>
+          <t>Chip-leasing SPV; 3 tranches; ~half syndicated</t>
+        </is>
+      </c>
+      <c r="G20" s="75" t="inlineStr">
+        <is>
+          <t>A1 T+100bp; A2 5.75%; B 8.5%</t>
+        </is>
+      </c>
+      <c r="H20" s="75" t="inlineStr">
+        <is>
+          <t>~5y</t>
+        </is>
+      </c>
+      <c r="I20" s="75" t="inlineStr">
+        <is>
+          <t>Buys Google TPUs leased to Anthropic</t>
+        </is>
+      </c>
+      <c r="J20" s="79" t="inlineStr">
+        <is>
+          <t>privatedebtnews; Build.inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="70" t="inlineStr">
+        <is>
+          <t>Oct 2025</t>
+        </is>
+      </c>
+      <c r="B21" s="71" t="inlineStr">
+        <is>
+          <t>Meta — Hyperion (Beignet Investor LLC)</t>
+        </is>
+      </c>
+      <c r="C21" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D21" s="70" t="inlineStr">
+        <is>
+          <t>PIMCO (~$18bn), BlackRock, Apollo; Blue Owl equity</t>
+        </is>
+      </c>
+      <c r="E21" s="73" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="F21" s="70" t="inlineStr">
+        <is>
+          <t>Off-B/S SPV; 144A senior secured bond</t>
+        </is>
+      </c>
+      <c r="G21" s="70" t="inlineStr">
+        <is>
+          <t>6.581% / T+225bp</t>
+        </is>
+      </c>
+      <c r="H21" s="70" t="inlineStr">
+        <is>
+          <t>Due May 2049</t>
+        </is>
+      </c>
+      <c r="I21" s="70" t="inlineStr">
+        <is>
+          <t>2.1GW; Meta lease + residual-value guarantee; A+ (S&amp;P)</t>
+        </is>
+      </c>
+      <c r="J21" s="74" t="inlineStr">
+        <is>
+          <t>IFR; FT; Quinn Emanuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="70" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B22" s="71" t="inlineStr">
+        <is>
+          <t>Oracle — New Mexico site</t>
+        </is>
+      </c>
+      <c r="C22" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D22" s="70" t="inlineStr">
+        <is>
+          <t>Private credit lenders</t>
+        </is>
+      </c>
+      <c r="E22" s="73" t="n">
+        <v>18</v>
+      </c>
+      <c r="F22" s="70" t="inlineStr">
+        <is>
+          <t>SPV / project loan</t>
+        </is>
+      </c>
+      <c r="G22" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H22" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I22" s="70" t="inlineStr">
+        <is>
+          <t>Single-site project loan</t>
+        </is>
+      </c>
+      <c r="J22" s="74" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B23" s="71" t="inlineStr">
+        <is>
+          <t>Oracle — Michigan campus</t>
+        </is>
+      </c>
+      <c r="C23" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D23" s="70" t="inlineStr">
+        <is>
+          <t>Project-finance lenders</t>
+        </is>
+      </c>
+      <c r="E23" s="73" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="F23" s="70" t="inlineStr">
+        <is>
+          <t>Project-level SPV financing</t>
+        </is>
+      </c>
+      <c r="G23" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H23" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I23" s="70" t="inlineStr">
+        <is>
+          <t>OCI capacity build</t>
+        </is>
+      </c>
+      <c r="J23" s="74" t="inlineStr">
+        <is>
+          <t>Press reports</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="75" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B24" s="76" t="inlineStr">
+        <is>
+          <t>xAI — Colossus 2 chip SPV</t>
+        </is>
+      </c>
+      <c r="C24" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D24" s="75" t="inlineStr">
+        <is>
+          <t>Valor Equity, Apollo, Diameter; NVIDIA equity</t>
+        </is>
+      </c>
+      <c r="E24" s="78" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F24" s="75" t="inlineStr">
+        <is>
+          <t>SPV; debt + ~$7.5bn equity</t>
+        </is>
+      </c>
+      <c r="G24" s="75" t="inlineStr">
+        <is>
+          <t>~10.5%</t>
+        </is>
+      </c>
+      <c r="H24" s="75" t="inlineStr">
+        <is>
+          <t>5y (~2.5y avg)</t>
+        </is>
+      </c>
+      <c r="I24" s="75" t="inlineStr">
+        <is>
+          <t>Buys NVIDIA GPUs leased to xAI</t>
+        </is>
+      </c>
+      <c r="J24" s="79" t="inlineStr">
+        <is>
+          <t>FT; WSJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B25" s="71" t="inlineStr">
+        <is>
+          <t>Oracle/OpenAI — Abilene, TX (Stargate)</t>
+        </is>
+      </c>
+      <c r="C25" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D25" s="70" t="inlineStr">
+        <is>
+          <t>Blue Owl + JPMorgan (Crusoe, Primary Digital)</t>
+        </is>
+      </c>
+      <c r="E25" s="73" t="n">
+        <v>10</v>
+      </c>
+      <c r="F25" s="70" t="inlineStr">
+        <is>
+          <t>Off-B/S SPV (~$13bn incl equity)</t>
+        </is>
+      </c>
+      <c r="G25" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H25" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I25" s="70" t="inlineStr">
+        <is>
+          <t>SPV owns OpenAI Abilene facility</t>
+        </is>
+      </c>
+      <c r="J25" s="74" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="75" t="inlineStr">
+        <is>
+          <t>May 2024</t>
+        </is>
+      </c>
+      <c r="B26" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — $7.5bn facility</t>
+        </is>
+      </c>
+      <c r="C26" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D26" s="75" t="inlineStr">
+        <is>
+          <t>Blackstone, Magnetar, Coatue, Carlyle, CDPQ, BlackRock</t>
+        </is>
+      </c>
+      <c r="E26" s="78" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F26" s="75" t="inlineStr">
+        <is>
+          <t>GPU + customer-contract secured facility</t>
+        </is>
+      </c>
+      <c r="G26" s="75" t="inlineStr">
+        <is>
+          <t>~10%+</t>
+        </is>
+      </c>
+      <c r="H26" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I26" s="75" t="inlineStr">
+        <is>
+          <t>Largest private debt deal at the time</t>
+        </is>
+      </c>
+      <c r="J26" s="79" t="inlineStr">
+        <is>
+          <t>Blackstone</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="80" t="inlineStr">
+        <is>
+          <t>Early 2025</t>
+        </is>
+      </c>
+      <c r="B27" s="81" t="inlineStr">
+        <is>
+          <t>Aligned Data Centers — debt</t>
+        </is>
+      </c>
+      <c r="C27" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D27" s="80" t="inlineStr">
+        <is>
+          <t>Macquarie + global investors</t>
+        </is>
+      </c>
+      <c r="E27" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="F27" s="80" t="inlineStr">
+        <is>
+          <t>Debt within $12bn raise (+$5bn equity)</t>
+        </is>
+      </c>
+      <c r="G27" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H27" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I27" s="80" t="inlineStr">
+        <is>
+          <t>Later acquired by MGX/BlackRock (~$40bn)</t>
+        </is>
+      </c>
+      <c r="J27" s="84" t="inlineStr">
+        <is>
+          <t>SFA; NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="75" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B28" s="76" t="inlineStr">
+        <is>
+          <t>Fluidstack — Google-backed facility</t>
+        </is>
+      </c>
+      <c r="C28" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D28" s="75" t="inlineStr">
+        <is>
+          <t>Private credit (Google lease backstop)</t>
+        </is>
+      </c>
+      <c r="E28" s="78" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="F28" s="75" t="inlineStr">
+        <is>
+          <t>SPV backed by contracted revenue</t>
+        </is>
+      </c>
+      <c r="G28" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H28" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I28" s="75" t="inlineStr">
+        <is>
+          <t>~$6.7bn Google-contracted revenue</t>
+        </is>
+      </c>
+      <c r="J28" s="79" t="inlineStr">
+        <is>
+          <t>theaiinsider</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="75" t="inlineStr">
+        <is>
+          <t>Jun-Jul 2025</t>
+        </is>
+      </c>
+      <c r="B29" s="76" t="inlineStr">
+        <is>
+          <t>xAI — secured notes / term loan</t>
+        </is>
+      </c>
+      <c r="C29" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D29" s="75" t="inlineStr">
+        <is>
+          <t>Apollo, Diameter; Morgan Stanley</t>
+        </is>
+      </c>
+      <c r="E29" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="F29" s="75" t="inlineStr">
+        <is>
+          <t>Secured notes + term loan (part of $10bn raise)</t>
+        </is>
+      </c>
+      <c r="G29" s="75" t="inlineStr">
+        <is>
+          <t>up to ~12.5%</t>
+        </is>
+      </c>
+      <c r="H29" s="75" t="inlineStr">
+        <is>
+          <t>~3-5y</t>
+        </is>
+      </c>
+      <c r="I29" s="75" t="inlineStr">
+        <is>
+          <t>Lenders can operate Colossus on default</t>
+        </is>
+      </c>
+      <c r="J29" s="79" t="inlineStr">
+        <is>
+          <t>CNBC; ciphertalk</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="75" t="inlineStr">
+        <is>
+          <t>Jul 2025</t>
+        </is>
+      </c>
+      <c r="B30" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — OpenAI contract financing</t>
+        </is>
+      </c>
+      <c r="C30" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D30" s="75" t="inlineStr">
+        <is>
+          <t>Private lenders (SPV)</t>
+        </is>
+      </c>
+      <c r="E30" s="78" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F30" s="75" t="inlineStr">
+        <is>
+          <t>SPV debt vs $11.9bn OpenAI contract</t>
+        </is>
+      </c>
+      <c r="G30" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H30" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I30" s="75" t="inlineStr">
+        <is>
+          <t>Funds OpenAI compute obligations</t>
+        </is>
+      </c>
+      <c r="J30" s="79" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="75" t="inlineStr">
+        <is>
           <t>Aug 2023</t>
         </is>
       </c>
-      <c r="B20" s="76" t="inlineStr">
-        <is>
-          <t>CoreWeave — $2.3bn debt facility</t>
-        </is>
-      </c>
-      <c r="C20" s="77" t="inlineStr">
+      <c r="B31" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — $2.3bn facility</t>
+        </is>
+      </c>
+      <c r="C31" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D20" s="75" t="inlineStr">
+      <c r="D31" s="75" t="inlineStr">
         <is>
           <t>Blackstone, Magnetar</t>
         </is>
       </c>
-      <c r="E20" s="78" t="n">
+      <c r="E31" s="78" t="n">
         <v>2.3</v>
       </c>
-      <c r="F20" s="75" t="inlineStr">
+      <c r="F31" s="75" t="inlineStr">
         <is>
           <t>GPU-backed facility</t>
         </is>
       </c>
-      <c r="G20" s="75" t="inlineStr">
+      <c r="G31" s="75" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="H20" s="75" t="inlineStr">
+      <c r="H31" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I20" s="75" t="inlineStr">
-        <is>
-          <t>Early template for GPU-collateralized debt</t>
-        </is>
-      </c>
-      <c r="J20" s="79" t="inlineStr">
+      <c r="I31" s="75" t="inlineStr">
+        <is>
+          <t>Early GPU-collateralized template</t>
+        </is>
+      </c>
+      <c r="J31" s="79" t="inlineStr">
         <is>
           <t>Blackstone</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="75" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B21" s="76" t="inlineStr">
-        <is>
-          <t>Nscale — term loan</t>
-        </is>
-      </c>
-      <c r="C21" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D21" s="75" t="inlineStr">
-        <is>
-          <t>Private credit</t>
-        </is>
-      </c>
-      <c r="E21" s="78" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="F21" s="75" t="inlineStr">
-        <is>
-          <t>Term loan</t>
-        </is>
-      </c>
-      <c r="G21" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H21" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I21" s="75" t="inlineStr">
-        <is>
-          <t>GPU-cloud build</t>
-        </is>
-      </c>
-      <c r="J21" s="79" t="inlineStr">
-        <is>
-          <t>theaiinsider</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="75" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B22" s="76" t="inlineStr">
-        <is>
-          <t>Lambda — GPU-backed facility</t>
-        </is>
-      </c>
-      <c r="C22" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D22" s="75" t="inlineStr">
-        <is>
-          <t>Macquarie</t>
-        </is>
-      </c>
-      <c r="E22" s="78" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F22" s="75" t="inlineStr">
-        <is>
-          <t>GPU-backed facility</t>
-        </is>
-      </c>
-      <c r="G22" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H22" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I22" s="75" t="inlineStr">
-        <is>
-          <t>GPU-cloud build</t>
-        </is>
-      </c>
-      <c r="J22" s="79" t="inlineStr">
-        <is>
-          <t>theaiinsider</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="85" t="n"/>
-      <c r="B23" s="86" t="inlineStr">
-        <is>
-          <t>Total — itemized private credit deals</t>
-        </is>
-      </c>
-      <c r="C23" s="85" t="n"/>
-      <c r="D23" s="85" t="n"/>
-      <c r="E23" s="87">
-        <f>SUM(E6:E22)</f>
-        <v/>
-      </c>
-      <c r="F23" s="85" t="n"/>
-      <c r="G23" s="85" t="n"/>
-      <c r="H23" s="85" t="n"/>
-      <c r="I23" s="85" t="n"/>
-      <c r="J23" s="85" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="14" t="inlineStr">
-        <is>
-          <t>2) CONTEXT / FRAMEWORKS / PROJECTIONS (not summed)</t>
-        </is>
-      </c>
-      <c r="B25" s="15" t="n"/>
-      <c r="C25" s="15" t="n"/>
-      <c r="D25" s="15" t="n"/>
-      <c r="E25" s="15" t="n"/>
-      <c r="F25" s="15" t="n"/>
-      <c r="G25" s="15" t="n"/>
-      <c r="H25" s="15" t="n"/>
-      <c r="I25" s="15" t="n"/>
-      <c r="J25" s="15" t="n"/>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="88" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B26" s="88" t="inlineStr">
-        <is>
-          <t>KKR + Energy Capital Partners — AI infrastructure partnership</t>
-        </is>
-      </c>
-      <c r="C26" s="89" t="inlineStr">
-        <is>
-          <t>Context / market</t>
-        </is>
-      </c>
-      <c r="D26" s="88" t="inlineStr">
-        <is>
-          <t>KKR, Energy Capital Partners</t>
-        </is>
-      </c>
-      <c r="E26" s="90" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F26" s="88" t="inlineStr">
-        <is>
-          <t>Strategic partnership/commitment</t>
-        </is>
-      </c>
-      <c r="G26" s="88" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H26" s="88" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I26" s="88" t="inlineStr">
-        <is>
-          <t>~$50bn to accelerate AI infrastructure</t>
-        </is>
-      </c>
-      <c r="J26" s="91" t="inlineStr">
-        <is>
-          <t>Business Times</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="88" t="inlineStr">
-        <is>
-          <t>Late 2025</t>
-        </is>
-      </c>
-      <c r="B27" s="88" t="inlineStr">
-        <is>
-          <t>Qatar (QIA / Qai) + Brookfield — AI infrastructure JV</t>
-        </is>
-      </c>
-      <c r="C27" s="89" t="inlineStr">
-        <is>
-          <t>Context / market</t>
-        </is>
-      </c>
-      <c r="D27" s="88" t="inlineStr">
-        <is>
-          <t>QIA / Qai, Brookfield</t>
-        </is>
-      </c>
-      <c r="E27" s="90" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F27" s="88" t="inlineStr">
-        <is>
-          <t>Joint venture / infra credit</t>
-        </is>
-      </c>
-      <c r="G27" s="88" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H27" s="88" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I27" s="88" t="inlineStr">
-        <is>
-          <t>~$20bn JV</t>
-        </is>
-      </c>
-      <c r="J27" s="91" t="inlineStr">
-        <is>
-          <t>NYU DRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="88" t="inlineStr">
-        <is>
-          <t>2025-28</t>
-        </is>
-      </c>
-      <c r="B28" s="88" t="inlineStr">
-        <is>
-          <t>Broadcom + Apollo + Blackstone — AI compute platform</t>
-        </is>
-      </c>
-      <c r="C28" s="89" t="inlineStr">
-        <is>
-          <t>Context / market</t>
-        </is>
-      </c>
-      <c r="D28" s="88" t="inlineStr">
-        <is>
-          <t>Apollo, Blackstone, Broadcom</t>
-        </is>
-      </c>
-      <c r="E28" s="90" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F28" s="88" t="inlineStr">
-        <is>
-          <t>Platform framework</t>
-        </is>
-      </c>
-      <c r="G28" s="88" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H28" s="88" t="inlineStr">
-        <is>
-          <t>through 2028</t>
-        </is>
-      </c>
-      <c r="I28" s="88" t="inlineStr">
-        <is>
-          <t>&gt;20 GW of compute to be deployed</t>
-        </is>
-      </c>
-      <c r="J28" s="91" t="inlineStr">
-        <is>
-          <t>privatedebtnews</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="88" t="inlineStr">
-        <is>
-          <t>from Nov 2025</t>
-        </is>
-      </c>
-      <c r="B29" s="88" t="inlineStr">
-        <is>
-          <t>Sector — 144A private placements (data centers)</t>
-        </is>
-      </c>
-      <c r="C29" s="89" t="inlineStr">
-        <is>
-          <t>Context / market</t>
-        </is>
-      </c>
-      <c r="D29" s="88" t="inlineStr">
-        <is>
-          <t>Multiple (Blue Owl, PIMCO, etc.)</t>
-        </is>
-      </c>
-      <c r="E29" s="90" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F29" s="88" t="inlineStr">
-        <is>
-          <t>144A private placement bonds</t>
-        </is>
-      </c>
-      <c r="G29" s="88" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H29" s="88" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I29" s="88" t="inlineStr">
-        <is>
-          <t>&gt;$40bn by Applied Digital, CoreWeave, Hut 8, Related since Nov 2025</t>
-        </is>
-      </c>
-      <c r="J29" s="91" t="inlineStr">
-        <is>
-          <t>Bisnow</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="88" t="inlineStr">
-        <is>
-          <t>2025-28</t>
-        </is>
-      </c>
-      <c r="B30" s="88" t="inlineStr">
-        <is>
-          <t>Market — projected private credit for AI data centers</t>
-        </is>
-      </c>
-      <c r="C30" s="89" t="inlineStr">
-        <is>
-          <t>Context / market</t>
-        </is>
-      </c>
-      <c r="D30" s="88" t="inlineStr">
-        <is>
-          <t>Industry-wide</t>
-        </is>
-      </c>
-      <c r="E30" s="90" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F30" s="88" t="inlineStr">
-        <is>
-          <t>Projection</t>
-        </is>
-      </c>
-      <c r="G30" s="88" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H30" s="88" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I30" s="88" t="inlineStr">
-        <is>
-          <t>Morgan Stanley: ~$800bn over next 2 years; &gt;$200bn already outstanding</t>
-        </is>
-      </c>
-      <c r="J30" s="91" t="inlineStr">
-        <is>
-          <t>Morgan Stanley; Quinn Emanuel</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>3) OTHER KEY DEALS — bonds · equity · securitization · sovereign · leases</t>
+          <t>4) INSURANCE-LINKED LENDING (memo — overlaps groups 1-3)</t>
         </is>
       </c>
       <c r="B32" s="15" t="n"/>
@@ -9404,94 +9486,114 @@
       <c r="J32" s="15" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="70" t="inlineStr">
+      <c r="A33" s="75" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B33" s="76" t="inlineStr">
+        <is>
+          <t>Anthropic — A2 notes (insurer tranche)</t>
+        </is>
+      </c>
+      <c r="C33" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D33" s="75" t="inlineStr">
+        <is>
+          <t>Apollo / Athene + insurers</t>
+        </is>
+      </c>
+      <c r="E33" s="78" t="n">
+        <v>24</v>
+      </c>
+      <c r="F33" s="75" t="inlineStr">
+        <is>
+          <t>Insurance-bought A2 tranche of TPU SPV</t>
+        </is>
+      </c>
+      <c r="G33" s="75" t="inlineStr">
+        <is>
+          <t>5.75%</t>
+        </is>
+      </c>
+      <c r="H33" s="75" t="inlineStr">
+        <is>
+          <t>~5y</t>
+        </is>
+      </c>
+      <c r="I33" s="75" t="inlineStr">
+        <is>
+          <t>Within the $35bn Anthropic deal (group 3)</t>
+        </is>
+      </c>
+      <c r="J33" s="79" t="inlineStr">
+        <is>
+          <t>privatedebtnews</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="85" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B33" s="70" t="inlineStr">
-        <is>
-          <t>Meta Platforms</t>
-        </is>
-      </c>
-      <c r="C33" s="72" t="inlineStr">
-        <is>
-          <t>Hyperscaler</t>
-        </is>
-      </c>
-      <c r="D33" s="70" t="inlineStr"/>
-      <c r="E33" s="92" t="inlineStr">
-        <is>
-          <t>$30bn</t>
-        </is>
-      </c>
-      <c r="F33" s="70" t="inlineStr">
-        <is>
-          <t>Corporate bonds</t>
-        </is>
-      </c>
-      <c r="G33" s="70" t="inlineStr"/>
-      <c r="H33" s="70" t="inlineStr"/>
-      <c r="I33" s="70" t="inlineStr">
-        <is>
-          <t>$30bn multi-tranche IG corporate bond (largest 2025 IG deal), maturities to 2063</t>
-        </is>
-      </c>
-      <c r="J33" s="74" t="inlineStr">
-        <is>
-          <t>BofA; MUFG</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="70" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B34" s="70" t="inlineStr">
-        <is>
-          <t>Amazon (AWS)</t>
-        </is>
-      </c>
-      <c r="C34" s="72" t="inlineStr">
-        <is>
-          <t>Hyperscaler</t>
-        </is>
-      </c>
-      <c r="D34" s="70" t="inlineStr"/>
-      <c r="E34" s="92" t="inlineStr">
-        <is>
-          <t>~$71bn</t>
-        </is>
-      </c>
-      <c r="F34" s="70" t="inlineStr">
-        <is>
-          <t>Corporate bonds</t>
-        </is>
-      </c>
-      <c r="G34" s="70" t="inlineStr"/>
-      <c r="H34" s="70" t="inlineStr"/>
-      <c r="I34" s="70" t="inlineStr">
-        <is>
-          <t>~$54bn USD + €14.5bn (~$16.8bn) IG bonds (near-record), ~4x oversubscribed</t>
-        </is>
-      </c>
-      <c r="J34" s="74" t="inlineStr">
-        <is>
-          <t>CNA; Reuters</t>
+      <c r="B34" s="86" t="inlineStr">
+        <is>
+          <t>Athene (Apollo) — AP Grange</t>
+        </is>
+      </c>
+      <c r="C34" s="87" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D34" s="85" t="inlineStr">
+        <is>
+          <t>Athene / Apollo (+ Intel equity)</t>
+        </is>
+      </c>
+      <c r="E34" s="88" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F34" s="85" t="inlineStr">
+        <is>
+          <t>Insurer JV investment (semis-adjacent)</t>
+        </is>
+      </c>
+      <c r="G34" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H34" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I34" s="85" t="inlineStr">
+        <is>
+          <t>Largest single-issuer insurer credit exposure</t>
+        </is>
+      </c>
+      <c r="J34" s="89" t="inlineStr">
+        <is>
+          <t>Moody's</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="70" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B35" s="70" t="inlineStr">
-        <is>
-          <t>Amazon (AWS)</t>
+          <t>Oct 2025</t>
+        </is>
+      </c>
+      <c r="B35" s="71" t="inlineStr">
+        <is>
+          <t>Meta — Hyperion insurance allocation</t>
         </is>
       </c>
       <c r="C35" s="72" t="inlineStr">
@@ -9499,279 +9601,277 @@
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="D35" s="70" t="inlineStr"/>
-      <c r="E35" s="92" t="inlineStr">
-        <is>
-          <t>$15bn</t>
-        </is>
-      </c>
+      <c r="D35" s="70" t="inlineStr">
+        <is>
+          <t>Insurers via PIMCO / BlackRock</t>
+        </is>
+      </c>
+      <c r="E35" s="90" t="n"/>
       <c r="F35" s="70" t="inlineStr">
         <is>
-          <t>Corporate bonds</t>
-        </is>
-      </c>
-      <c r="G35" s="70" t="inlineStr"/>
-      <c r="H35" s="70" t="inlineStr"/>
+          <t>Insurance allocation of 144A bond</t>
+        </is>
+      </c>
+      <c r="G35" s="70" t="inlineStr">
+        <is>
+          <t>6.581%</t>
+        </is>
+      </c>
+      <c r="H35" s="70" t="inlineStr">
+        <is>
+          <t>2049</t>
+        </is>
+      </c>
       <c r="I35" s="70" t="inlineStr">
         <is>
-          <t>$15bn IG bond</t>
+          <t>Subset of the $27.3bn Hyperion bond (group 3)</t>
         </is>
       </c>
       <c r="J35" s="74" t="inlineStr">
         <is>
-          <t>CNA</t>
+          <t>FT; S&amp;P</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="70" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="B36" s="70" t="inlineStr">
-        <is>
-          <t>Alphabet (Google)</t>
-        </is>
-      </c>
-      <c r="C36" s="72" t="inlineStr">
-        <is>
-          <t>Hyperscaler</t>
-        </is>
-      </c>
-      <c r="D36" s="70" t="inlineStr"/>
-      <c r="E36" s="92" t="inlineStr">
-        <is>
-          <t>~$50bn</t>
-        </is>
-      </c>
-      <c r="F36" s="70" t="inlineStr">
-        <is>
-          <t>Corporate bonds</t>
-        </is>
-      </c>
-      <c r="G36" s="70" t="inlineStr"/>
-      <c r="H36" s="70" t="inlineStr"/>
-      <c r="I36" s="70" t="inlineStr">
-        <is>
-          <t>~$32bn multi-currency bond incl. rare 100-yr tranche; plus $17.5bn Nov 2025</t>
-        </is>
-      </c>
-      <c r="J36" s="74" t="inlineStr">
-        <is>
-          <t>ConstructConnect; CNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="70" t="inlineStr">
+      <c r="A36" s="75" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B36" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — DDTL 4.0 insurance anchor</t>
+        </is>
+      </c>
+      <c r="C36" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D36" s="75" t="inlineStr">
+        <is>
+          <t>Blackstone Credit &amp; Insurance + insurers</t>
+        </is>
+      </c>
+      <c r="E36" s="91" t="n"/>
+      <c r="F36" s="75" t="inlineStr">
+        <is>
+          <t>Insurance anchor of GPU-backed loan</t>
+        </is>
+      </c>
+      <c r="G36" s="75" t="inlineStr">
+        <is>
+          <t>SOFR+225 / 5.9%</t>
+        </is>
+      </c>
+      <c r="H36" s="75" t="inlineStr">
+        <is>
+          <t>2032</t>
+        </is>
+      </c>
+      <c r="I36" s="75" t="inlineStr">
+        <is>
+          <t>Subset of the $8.5bn DDTL (group 2)</t>
+        </is>
+      </c>
+      <c r="J36" s="79" t="inlineStr">
+        <is>
+          <t>CoreWeave IR</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>5) SECURITIZATION / ABS / CMBS</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="n"/>
+      <c r="C37" s="15" t="n"/>
+      <c r="D37" s="15" t="n"/>
+      <c r="E37" s="15" t="n"/>
+      <c r="F37" s="15" t="n"/>
+      <c r="G37" s="15" t="n"/>
+      <c r="H37" s="15" t="n"/>
+      <c r="I37" s="15" t="n"/>
+      <c r="J37" s="15" t="n"/>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="80" t="inlineStr">
+        <is>
+          <t>Nov 2025</t>
+        </is>
+      </c>
+      <c r="B38" s="81" t="inlineStr">
+        <is>
+          <t>QTS (Blackstone) — BX 2025-VOLT</t>
+        </is>
+      </c>
+      <c r="C38" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D38" s="80" t="inlineStr">
+        <is>
+          <t>Blackstone</t>
+        </is>
+      </c>
+      <c r="E38" s="83" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F38" s="80" t="inlineStr">
+        <is>
+          <t>SASB CMBS (~10 QTS DCs)</t>
+        </is>
+      </c>
+      <c r="G38" s="80" t="inlineStr">
+        <is>
+          <t>floating</t>
+        </is>
+      </c>
+      <c r="H38" s="80" t="inlineStr">
+        <is>
+          <t>2y + ext</t>
+        </is>
+      </c>
+      <c r="I38" s="80" t="inlineStr">
+        <is>
+          <t>Year's largest data-center CMBS</t>
+        </is>
+      </c>
+      <c r="J38" s="84" t="inlineStr">
+        <is>
+          <t>CREFC; SFA</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="80" t="inlineStr">
+        <is>
+          <t>2024-25</t>
+        </is>
+      </c>
+      <c r="B39" s="81" t="inlineStr">
+        <is>
+          <t>Switch (DigitalBridge) — SWCH 2025-DATA</t>
+        </is>
+      </c>
+      <c r="C39" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D39" s="80" t="inlineStr">
+        <is>
+          <t>DigitalBridge</t>
+        </is>
+      </c>
+      <c r="E39" s="83" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F39" s="80" t="inlineStr">
+        <is>
+          <t>$2.4bn SASB CMBS + $1.1bn ABS (green)</t>
+        </is>
+      </c>
+      <c r="G39" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H39" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I39" s="80" t="inlineStr">
+        <is>
+          <t>Green-bond framework</t>
+        </is>
+      </c>
+      <c r="J39" s="84" t="inlineStr">
+        <is>
+          <t>SFA; CREFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="80" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="B37" s="70" t="inlineStr">
-        <is>
-          <t>Oracle (OCI)</t>
-        </is>
-      </c>
-      <c r="C37" s="72" t="inlineStr">
-        <is>
-          <t>Hyperscaler</t>
-        </is>
-      </c>
-      <c r="D37" s="70" t="inlineStr"/>
-      <c r="E37" s="92" t="inlineStr">
-        <is>
-          <t>$25bn debt</t>
-        </is>
-      </c>
-      <c r="F37" s="70" t="inlineStr">
-        <is>
-          <t>Corporate bonds + equity</t>
-        </is>
-      </c>
-      <c r="G37" s="70" t="inlineStr"/>
-      <c r="H37" s="70" t="inlineStr"/>
-      <c r="I37" s="70" t="inlineStr">
-        <is>
-          <t>$25bn 8-part IG bond (Feb 2026) within $45-50bn CY26 debt+equity plan; $20bn ATM + mandatory convertible preferred (equity)</t>
-        </is>
-      </c>
-      <c r="J37" s="74" t="inlineStr">
-        <is>
-          <t>Oracle IR; IFR</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="70" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B38" s="70" t="inlineStr">
-        <is>
-          <t>Oracle (OCI)</t>
-        </is>
-      </c>
-      <c r="C38" s="72" t="inlineStr">
-        <is>
-          <t>Hyperscaler</t>
-        </is>
-      </c>
-      <c r="D38" s="70" t="inlineStr"/>
-      <c r="E38" s="92" t="inlineStr">
-        <is>
-          <t>$18bn</t>
-        </is>
-      </c>
-      <c r="F38" s="70" t="inlineStr">
-        <is>
-          <t>Corporate bonds</t>
-        </is>
-      </c>
-      <c r="G38" s="70" t="inlineStr"/>
-      <c r="H38" s="70" t="inlineStr"/>
-      <c r="I38" s="70" t="inlineStr">
-        <is>
-          <t>$18bn 6-part IG bond (Sep 2025)</t>
-        </is>
-      </c>
-      <c r="J38" s="74" t="inlineStr">
-        <is>
-          <t>Reuters/CNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="70" t="inlineStr">
-        <is>
-          <t>2024-30</t>
-        </is>
-      </c>
-      <c r="B39" s="70" t="inlineStr">
-        <is>
-          <t>Microsoft</t>
-        </is>
-      </c>
-      <c r="C39" s="72" t="inlineStr">
-        <is>
-          <t>Hyperscaler</t>
-        </is>
-      </c>
-      <c r="D39" s="70" t="inlineStr"/>
-      <c r="E39" s="92" t="inlineStr">
-        <is>
-          <t>$100bn+ leases</t>
-        </is>
-      </c>
-      <c r="F39" s="70" t="inlineStr">
-        <is>
-          <t>Vendor / lease / SPV</t>
-        </is>
-      </c>
-      <c r="G39" s="70" t="inlineStr"/>
-      <c r="H39" s="70" t="inlineStr"/>
-      <c r="I39" s="70" t="inlineStr">
-        <is>
-          <t>Finance-lease driven build (~$108bn uncommenced finance leases as of 9/30/24; commence FY25-FY30)</t>
-        </is>
-      </c>
-      <c r="J39" s="74" t="inlineStr">
-        <is>
-          <t>MSFT 10-Q; CNBC</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="75" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="B40" s="75" t="inlineStr">
-        <is>
-          <t>CoreWeave</t>
-        </is>
-      </c>
-      <c r="C40" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D40" s="75" t="inlineStr"/>
-      <c r="E40" s="93" t="inlineStr">
-        <is>
-          <t>$2.7bn conv.</t>
-        </is>
-      </c>
-      <c r="F40" s="75" t="inlineStr">
-        <is>
-          <t>Convertibles</t>
-        </is>
-      </c>
-      <c r="G40" s="75" t="inlineStr"/>
-      <c r="H40" s="75" t="inlineStr"/>
-      <c r="I40" s="75" t="inlineStr">
-        <is>
-          <t>$2.7bn 1.75% convertible notes; ~$30bn total debt by early 2026; ~$28bn debt+equity raised in 12 mos</t>
-        </is>
-      </c>
-      <c r="J40" s="79" t="inlineStr">
-        <is>
-          <t>thedig; CoreWeave</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="75" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="B41" s="75" t="inlineStr">
-        <is>
-          <t>CoreWeave</t>
-        </is>
-      </c>
-      <c r="C41" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D41" s="75" t="inlineStr"/>
-      <c r="E41" s="93" t="inlineStr">
-        <is>
-          <t>$3.5bn equity</t>
-        </is>
-      </c>
-      <c r="F41" s="75" t="inlineStr">
-        <is>
-          <t>Equity</t>
-        </is>
-      </c>
-      <c r="G41" s="75" t="inlineStr"/>
-      <c r="H41" s="75" t="inlineStr"/>
-      <c r="I41" s="75" t="inlineStr">
-        <is>
-          <t>$2bn strategic equity from NVIDIA; IPO Mar 2025 raised ~$1.5bn</t>
-        </is>
-      </c>
-      <c r="J41" s="79" t="inlineStr">
-        <is>
-          <t>CNBC; CoreWeave</t>
-        </is>
-      </c>
+      <c r="B40" s="81" t="inlineStr">
+        <is>
+          <t>Applied Digital — Polaris Forge HY bond</t>
+        </is>
+      </c>
+      <c r="C40" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D40" s="80" t="inlineStr">
+        <is>
+          <t>HY market</t>
+        </is>
+      </c>
+      <c r="E40" s="83" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="F40" s="80" t="inlineStr">
+        <is>
+          <t>HY / securitized bond (CoreWeave campus)</t>
+        </is>
+      </c>
+      <c r="G40" s="80" t="inlineStr">
+        <is>
+          <t>7%</t>
+        </is>
+      </c>
+      <c r="H40" s="80" t="inlineStr">
+        <is>
+          <t>15y contract</t>
+        </is>
+      </c>
+      <c r="I40" s="80" t="inlineStr">
+        <is>
+          <t>150MW for CoreWeave</t>
+        </is>
+      </c>
+      <c r="J40" s="84" t="inlineStr">
+        <is>
+          <t>TNW</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>6) CONVERTIBLES / EQUITY-LINKED</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="n"/>
+      <c r="C41" s="15" t="n"/>
+      <c r="D41" s="15" t="n"/>
+      <c r="E41" s="15" t="n"/>
+      <c r="F41" s="15" t="n"/>
+      <c r="G41" s="15" t="n"/>
+      <c r="H41" s="15" t="n"/>
+      <c r="I41" s="15" t="n"/>
+      <c r="J41" s="15" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="75" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B42" s="75" t="inlineStr">
-        <is>
-          <t>SpaceX / xAI</t>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B42" s="76" t="inlineStr">
+        <is>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="C42" s="77" t="inlineStr">
@@ -9779,728 +9879,913 @@
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D42" s="75" t="inlineStr"/>
-      <c r="E42" s="93" t="inlineStr">
-        <is>
-          <t>merger</t>
-        </is>
+      <c r="D42" s="75" t="inlineStr">
+        <is>
+          <t>Convertible market</t>
+        </is>
+      </c>
+      <c r="E42" s="78" t="n">
+        <v>3</v>
       </c>
       <c r="F42" s="75" t="inlineStr">
         <is>
-          <t>Equity / M&amp;A</t>
-        </is>
-      </c>
-      <c r="G42" s="75" t="inlineStr"/>
-      <c r="H42" s="75" t="inlineStr"/>
+          <t>Convertible notes</t>
+        </is>
+      </c>
+      <c r="G42" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H42" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
       <c r="I42" s="75" t="inlineStr">
         <is>
-          <t>SpaceX acquired xAI effective Feb 2, 2026; Colossus I &amp; II now SpaceX-owned (vertically-integrated AI platform; Terafab chip JV w/ Tesla &amp; Intel)</t>
+          <t>Lighter-balance-sheet strategy</t>
         </is>
       </c>
       <c r="J42" s="79" t="inlineStr">
         <is>
-          <t>SpaceX S-1</t>
+          <t>frankk research</t>
         </is>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="75" t="inlineStr">
         <is>
+          <t>Dec 2025</t>
+        </is>
+      </c>
+      <c r="B43" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave</t>
+        </is>
+      </c>
+      <c r="C43" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D43" s="75" t="inlineStr">
+        <is>
+          <t>Convertible market</t>
+        </is>
+      </c>
+      <c r="E43" s="78" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F43" s="75" t="inlineStr">
+        <is>
+          <t>Convertible notes</t>
+        </is>
+      </c>
+      <c r="G43" s="75" t="inlineStr">
+        <is>
+          <t>1.75%</t>
+        </is>
+      </c>
+      <c r="H43" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I43" s="75" t="inlineStr">
+        <is>
+          <t>Shift toward hybrid instruments</t>
+        </is>
+      </c>
+      <c r="J43" s="79" t="inlineStr">
+        <is>
+          <t>thedig; CoreWeave</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="92" t="n"/>
+      <c r="B44" s="93" t="inlineStr">
+        <is>
+          <t>TOTAL — itemized debt transactions (bonds + loans + private credit + ABS + converts)</t>
+        </is>
+      </c>
+      <c r="C44" s="92" t="n"/>
+      <c r="D44" s="92" t="n"/>
+      <c r="E44" s="94">
+        <f>SUM(E6,E7,E8,E9,E10,E11,E13,E14,E15,E16,E17,E19,E20,E21,E22,E23,E24,E25,E26,E27,E28,E29,E30,E31,E38,E39,E40,E42,E43)</f>
+        <v/>
+      </c>
+      <c r="F44" s="92" t="n"/>
+      <c r="G44" s="92" t="n"/>
+      <c r="H44" s="92" t="n"/>
+      <c r="I44" s="92" t="n"/>
+      <c r="J44" s="92" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>7) VENDOR / EQUIPMENT-LEASE FINANCING &amp; BACKSTOPS (memo)</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="n"/>
+      <c r="C46" s="15" t="n"/>
+      <c r="D46" s="15" t="n"/>
+      <c r="E46" s="15" t="n"/>
+      <c r="F46" s="15" t="n"/>
+      <c r="G46" s="15" t="n"/>
+      <c r="H46" s="15" t="n"/>
+      <c r="I46" s="15" t="n"/>
+      <c r="J46" s="15" t="n"/>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="70" t="inlineStr">
+        <is>
+          <t>2024-30</t>
+        </is>
+      </c>
+      <c r="B47" s="71" t="inlineStr">
+        <is>
+          <t>Microsoft — finance-lease commitments</t>
+        </is>
+      </c>
+      <c r="C47" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D47" s="70" t="inlineStr">
+        <is>
+          <t>Lessors / developers</t>
+        </is>
+      </c>
+      <c r="E47" s="73" t="n">
+        <v>100</v>
+      </c>
+      <c r="F47" s="70" t="inlineStr">
+        <is>
+          <t>Finance leases (uncommenced ~$108bn at 9/30/24)</t>
+        </is>
+      </c>
+      <c r="G47" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H47" s="70" t="inlineStr">
+        <is>
+          <t>to 20y</t>
+        </is>
+      </c>
+      <c r="I47" s="70" t="inlineStr">
+        <is>
+          <t>Off-B/S; commence FY25-FY30</t>
+        </is>
+      </c>
+      <c r="J47" s="74" t="inlineStr">
+        <is>
+          <t>MSFT 10-Q; CNBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="75" t="inlineStr">
+        <is>
+          <t>through 2032</t>
+        </is>
+      </c>
+      <c r="B48" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — NVIDIA capacity backstop</t>
+        </is>
+      </c>
+      <c r="C48" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D48" s="75" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="E48" s="78" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="F48" s="75" t="inlineStr">
+        <is>
+          <t>Vendor backstop of unsold capacity</t>
+        </is>
+      </c>
+      <c r="G48" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H48" s="75" t="inlineStr">
+        <is>
+          <t>to 2032</t>
+        </is>
+      </c>
+      <c r="I48" s="75" t="inlineStr">
+        <is>
+          <t>De-risks CoreWeave</t>
+        </is>
+      </c>
+      <c r="J48" s="79" t="inlineStr">
+        <is>
+          <t>theaiinsider</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>8) EQUITY &amp; SOVEREIGN COMMITMENTS (memo — not debt)</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="n"/>
+      <c r="C49" s="15" t="n"/>
+      <c r="D49" s="15" t="n"/>
+      <c r="E49" s="15" t="n"/>
+      <c r="F49" s="15" t="n"/>
+      <c r="G49" s="15" t="n"/>
+      <c r="H49" s="15" t="n"/>
+      <c r="I49" s="15" t="n"/>
+      <c r="J49" s="15" t="n"/>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="95" t="inlineStr">
+        <is>
+          <t>2025-30</t>
+        </is>
+      </c>
+      <c r="B50" s="96" t="inlineStr">
+        <is>
+          <t>HUMAIN (Saudi PIF)</t>
+        </is>
+      </c>
+      <c r="C50" s="97" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="D50" s="95" t="inlineStr">
+        <is>
+          <t>Public Investment Fund</t>
+        </is>
+      </c>
+      <c r="E50" s="98" t="n">
+        <v>100</v>
+      </c>
+      <c r="F50" s="95" t="inlineStr">
+        <is>
+          <t>Sovereign equity</t>
+        </is>
+      </c>
+      <c r="G50" s="95" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H50" s="95" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I50" s="95" t="inlineStr">
+        <is>
+          <t>11 DCs / 2.2GW; ~600k GPUs</t>
+        </is>
+      </c>
+      <c r="J50" s="99" t="inlineStr">
+        <is>
+          <t>Presenc AI; NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="95" t="inlineStr">
+        <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="B43" s="75" t="inlineStr">
-        <is>
-          <t>SpaceX / xAI</t>
-        </is>
-      </c>
-      <c r="C43" s="77" t="inlineStr">
+      <c r="B51" s="96" t="inlineStr">
+        <is>
+          <t>MGX / Mubadala (UAE)</t>
+        </is>
+      </c>
+      <c r="C51" s="97" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="D51" s="95" t="inlineStr">
+        <is>
+          <t>Mubadala / MGX</t>
+        </is>
+      </c>
+      <c r="E51" s="98" t="n">
+        <v>40</v>
+      </c>
+      <c r="F51" s="95" t="inlineStr">
+        <is>
+          <t>Sovereign equity / infra</t>
+        </is>
+      </c>
+      <c r="G51" s="95" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H51" s="95" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I51" s="95" t="inlineStr">
+        <is>
+          <t>Anchored Stargate; co-bought Aligned</t>
+        </is>
+      </c>
+      <c r="J51" s="99" t="inlineStr">
+        <is>
+          <t>NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="95" t="inlineStr">
+        <is>
+          <t>2025-30</t>
+        </is>
+      </c>
+      <c r="B52" s="96" t="inlineStr">
+        <is>
+          <t>Stargate UAE / G42 / Khazna</t>
+        </is>
+      </c>
+      <c r="C52" s="97" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="D52" s="95" t="inlineStr">
+        <is>
+          <t>Mubadala, MGX, Microsoft, G42</t>
+        </is>
+      </c>
+      <c r="E52" s="98" t="n">
+        <v>30</v>
+      </c>
+      <c r="F52" s="95" t="inlineStr">
+        <is>
+          <t>Sovereign equity + JV</t>
+        </is>
+      </c>
+      <c r="G52" s="95" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H52" s="95" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I52" s="95" t="inlineStr">
+        <is>
+          <t>5GW Abu Dhabi campus</t>
+        </is>
+      </c>
+      <c r="J52" s="99" t="inlineStr">
+        <is>
+          <t>Khaleej Times; dcpulse</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="95" t="inlineStr">
+        <is>
+          <t>Late 2025</t>
+        </is>
+      </c>
+      <c r="B53" s="96" t="inlineStr">
+        <is>
+          <t>Qatar (QIA / Qai) + Brookfield</t>
+        </is>
+      </c>
+      <c r="C53" s="97" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="D53" s="95" t="inlineStr">
+        <is>
+          <t>QIA / Qai, Brookfield</t>
+        </is>
+      </c>
+      <c r="E53" s="98" t="n">
+        <v>20</v>
+      </c>
+      <c r="F53" s="95" t="inlineStr">
+        <is>
+          <t>JV / infra</t>
+        </is>
+      </c>
+      <c r="G53" s="95" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H53" s="95" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I53" s="95" t="inlineStr">
+        <is>
+          <t>AI-infrastructure JV</t>
+        </is>
+      </c>
+      <c r="J53" s="99" t="inlineStr">
+        <is>
+          <t>NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="75" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B54" s="76" t="inlineStr">
+        <is>
+          <t>SpaceX / xAI — $10bn raise</t>
+        </is>
+      </c>
+      <c r="C54" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D43" s="75" t="inlineStr"/>
-      <c r="E43" s="93" t="inlineStr">
-        <is>
-          <t>$20bn+ capex</t>
-        </is>
-      </c>
-      <c r="F43" s="75" t="inlineStr">
-        <is>
-          <t>Internal / equity</t>
-        </is>
-      </c>
-      <c r="G43" s="75" t="inlineStr"/>
-      <c r="H43" s="75" t="inlineStr"/>
-      <c r="I43" s="75" t="inlineStr">
-        <is>
-          <t>SpaceX AI capex $12.7bn in 2025 (~61% of total) + $7.7bn in Q1 2026; AI buildout funded by Starlink FCF, private raises, planned IPO</t>
-        </is>
-      </c>
-      <c r="J43" s="79" t="inlineStr">
-        <is>
-          <t>SpaceX S-1; The Verge</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="75" t="inlineStr">
-        <is>
-          <t>2026-29</t>
-        </is>
-      </c>
-      <c r="B44" s="75" t="inlineStr">
-        <is>
-          <t>SpaceX / xAI</t>
-        </is>
-      </c>
-      <c r="C44" s="77" t="inlineStr">
+      <c r="D54" s="75" t="inlineStr">
+        <is>
+          <t>Morgan Stanley</t>
+        </is>
+      </c>
+      <c r="E54" s="78" t="n">
+        <v>10</v>
+      </c>
+      <c r="F54" s="75" t="inlineStr">
+        <is>
+          <t>$5bn debt + $5bn equity</t>
+        </is>
+      </c>
+      <c r="G54" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H54" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I54" s="75" t="inlineStr">
+        <is>
+          <t>Debt portion also in group 3</t>
+        </is>
+      </c>
+      <c r="J54" s="79" t="inlineStr">
+        <is>
+          <t>CNBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="75" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B55" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — equity</t>
+        </is>
+      </c>
+      <c r="C55" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D44" s="75" t="inlineStr"/>
-      <c r="E44" s="93" t="inlineStr">
-        <is>
-          <t>~$45bn</t>
-        </is>
-      </c>
-      <c r="F44" s="75" t="inlineStr">
-        <is>
-          <t>Take-or-pay (demand)</t>
-        </is>
-      </c>
-      <c r="G44" s="75" t="inlineStr"/>
-      <c r="H44" s="75" t="inlineStr"/>
-      <c r="I44" s="75" t="inlineStr">
-        <is>
-          <t>Anthropic compute contract: $1.25bn/month (~$45bn) through May 2029 for Colossus I &amp; II — anchor revenue underwriting infra financing</t>
-        </is>
-      </c>
-      <c r="J44" s="79" t="inlineStr">
-        <is>
-          <t>SpaceX S-1; The Verge</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="75" t="inlineStr">
+      <c r="D55" s="75" t="inlineStr">
+        <is>
+          <t>NVIDIA; IPO</t>
+        </is>
+      </c>
+      <c r="E55" s="78" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F55" s="75" t="inlineStr">
+        <is>
+          <t>IPO ($1.5bn) + NVIDIA strategic ($2bn)</t>
+        </is>
+      </c>
+      <c r="G55" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H55" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I55" s="75" t="inlineStr">
+        <is>
+          <t>Equity (not debt)</t>
+        </is>
+      </c>
+      <c r="J55" s="79" t="inlineStr">
+        <is>
+          <t>CNBC; CoreWeave</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>9) CONTEXT / FRAMEWORKS / PROJECTIONS (memo)</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="n"/>
+      <c r="C56" s="15" t="n"/>
+      <c r="D56" s="15" t="n"/>
+      <c r="E56" s="15" t="n"/>
+      <c r="F56" s="15" t="n"/>
+      <c r="G56" s="15" t="n"/>
+      <c r="H56" s="15" t="n"/>
+      <c r="I56" s="15" t="n"/>
+      <c r="J56" s="15" t="n"/>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="85" t="inlineStr">
+        <is>
+          <t>2025-28</t>
+        </is>
+      </c>
+      <c r="B57" s="86" t="inlineStr">
+        <is>
+          <t>Market — private credit for AI data centers</t>
+        </is>
+      </c>
+      <c r="C57" s="87" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D57" s="85" t="inlineStr">
+        <is>
+          <t>Industry-wide</t>
+        </is>
+      </c>
+      <c r="E57" s="88" t="n">
+        <v>800</v>
+      </c>
+      <c r="F57" s="85" t="inlineStr">
+        <is>
+          <t>Projection</t>
+        </is>
+      </c>
+      <c r="G57" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H57" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I57" s="85" t="inlineStr">
+        <is>
+          <t>&gt;$200bn already outstanding</t>
+        </is>
+      </c>
+      <c r="J57" s="89" t="inlineStr">
+        <is>
+          <t>Morgan Stanley; Quinn Emanuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="85" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B45" s="75" t="inlineStr">
-        <is>
-          <t>SpaceX / xAI</t>
-        </is>
-      </c>
-      <c r="C45" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D45" s="75" t="inlineStr"/>
-      <c r="E45" s="93" t="inlineStr">
-        <is>
-          <t>$10bn</t>
-        </is>
-      </c>
-      <c r="F45" s="75" t="inlineStr">
-        <is>
-          <t>Loans + equity</t>
-        </is>
-      </c>
-      <c r="G45" s="75" t="inlineStr"/>
-      <c r="H45" s="75" t="inlineStr"/>
-      <c r="I45" s="75" t="inlineStr">
-        <is>
-          <t>xAI $10bn raise ($5bn secured notes/term loans incl. Apollo $5bn facility + $5bn equity) via Morgan Stanley</t>
-        </is>
-      </c>
-      <c r="J45" s="79" t="inlineStr">
-        <is>
-          <t>CNBC</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="75" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="B46" s="75" t="inlineStr">
-        <is>
-          <t>Nebius</t>
-        </is>
-      </c>
-      <c r="C46" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D46" s="75" t="inlineStr"/>
-      <c r="E46" s="93" t="inlineStr">
-        <is>
-          <t>$3bn+</t>
-        </is>
-      </c>
-      <c r="F46" s="75" t="inlineStr">
-        <is>
-          <t>Convertibles</t>
-        </is>
-      </c>
-      <c r="G46" s="75" t="inlineStr"/>
-      <c r="H46" s="75" t="inlineStr"/>
-      <c r="I46" s="75" t="inlineStr">
-        <is>
-          <t>$3bn+ convertibles + bank lines; lighter balance sheet; Yandex spin-off cash ~$2.5bn; NVIDIA ~$2bn equity; Microsoft ~$7bn prepay</t>
-        </is>
-      </c>
-      <c r="J46" s="79" t="inlineStr">
-        <is>
-          <t>frankk research</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="80" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B47" s="80" t="inlineStr">
-        <is>
-          <t>Applied Digital</t>
-        </is>
-      </c>
-      <c r="C47" s="82" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REIT</t>
-        </is>
-      </c>
-      <c r="D47" s="80" t="inlineStr"/>
-      <c r="E47" s="94" t="inlineStr">
-        <is>
-          <t>$1.59bn</t>
-        </is>
-      </c>
-      <c r="F47" s="80" t="inlineStr">
-        <is>
-          <t>Securitization / HY bond</t>
-        </is>
-      </c>
-      <c r="G47" s="80" t="inlineStr"/>
-      <c r="H47" s="80" t="inlineStr"/>
-      <c r="I47" s="80" t="inlineStr">
-        <is>
-          <t>$1.59bn high-yield bond (7%) for CoreWeave-leased campus (Polaris Forge 1)</t>
-        </is>
-      </c>
-      <c r="J47" s="84" t="inlineStr">
-        <is>
-          <t>TNW</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="80" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B48" s="80" t="inlineStr">
-        <is>
-          <t>Aligned Data Centers</t>
-        </is>
-      </c>
-      <c r="C48" s="82" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REIT</t>
-        </is>
-      </c>
-      <c r="D48" s="80" t="inlineStr"/>
-      <c r="E48" s="94" t="inlineStr">
-        <is>
-          <t>$12bn / $40bn</t>
-        </is>
-      </c>
-      <c r="F48" s="80" t="inlineStr">
-        <is>
-          <t>Infra equity + debt</t>
-        </is>
-      </c>
-      <c r="G48" s="80" t="inlineStr"/>
-      <c r="H48" s="80" t="inlineStr"/>
-      <c r="I48" s="80" t="inlineStr">
-        <is>
-          <t>$12bn capital raise ($5bn+ new equity + $7bn debt commitments) led by Macquarie (early 2025); later acquired by MGX/BlackRock consortium (~$40bn)</t>
-        </is>
-      </c>
-      <c r="J48" s="84" t="inlineStr">
-        <is>
-          <t>SFA; NYU DRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="80" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B49" s="80" t="inlineStr">
-        <is>
-          <t>QTS (Blackstone)</t>
-        </is>
-      </c>
-      <c r="C49" s="82" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REIT</t>
-        </is>
-      </c>
-      <c r="D49" s="80" t="inlineStr"/>
-      <c r="E49" s="94" t="inlineStr">
-        <is>
-          <t>$3.5bn+</t>
-        </is>
-      </c>
-      <c r="F49" s="80" t="inlineStr">
-        <is>
-          <t>Securitization (CMBS/ABS)</t>
-        </is>
-      </c>
-      <c r="G49" s="80" t="inlineStr"/>
-      <c r="H49" s="80" t="inlineStr"/>
-      <c r="I49" s="80" t="inlineStr">
-        <is>
-          <t>BX 2025-VOLT SASB CMBS $3.5bn (~10 QTS DCs); + Phoenix ABS (QTS Issuer 2025-1)</t>
-        </is>
-      </c>
-      <c r="J49" s="84" t="inlineStr">
-        <is>
-          <t>CREFC; SFA</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="80" t="inlineStr">
-        <is>
-          <t>2024-25</t>
-        </is>
-      </c>
-      <c r="B50" s="80" t="inlineStr">
-        <is>
-          <t>Switch (DigitalBridge)</t>
-        </is>
-      </c>
-      <c r="C50" s="82" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REIT</t>
-        </is>
-      </c>
-      <c r="D50" s="80" t="inlineStr"/>
-      <c r="E50" s="94" t="inlineStr">
-        <is>
-          <t>$3.5bn</t>
-        </is>
-      </c>
-      <c r="F50" s="80" t="inlineStr">
-        <is>
-          <t>Securitization (CMBS/ABS)</t>
-        </is>
-      </c>
-      <c r="G50" s="80" t="inlineStr"/>
-      <c r="H50" s="80" t="inlineStr"/>
-      <c r="I50" s="80" t="inlineStr">
-        <is>
-          <t>$2.4bn SASB CMBS (SWCH 2025-DATA) + $1.1bn ABS — green bonds</t>
-        </is>
-      </c>
-      <c r="J50" s="84" t="inlineStr">
-        <is>
-          <t>SFA; CREFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="80" t="inlineStr">
-        <is>
-          <t>2024-26</t>
-        </is>
-      </c>
-      <c r="B51" s="80" t="inlineStr">
-        <is>
-          <t>Vantage Data Centers</t>
-        </is>
-      </c>
-      <c r="C51" s="82" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REIT</t>
-        </is>
-      </c>
-      <c r="D51" s="80" t="inlineStr"/>
-      <c r="E51" s="94" t="inlineStr">
-        <is>
-          <t>multi-$bn</t>
-        </is>
-      </c>
-      <c r="F51" s="80" t="inlineStr">
-        <is>
-          <t>Securitization / equity</t>
-        </is>
-      </c>
-      <c r="G51" s="80" t="inlineStr"/>
-      <c r="H51" s="80" t="inlineStr"/>
-      <c r="I51" s="80" t="inlineStr">
-        <is>
-          <t>First public data-center ABS (2024); ongoing multi-billion securitization &amp; infra-equity program</t>
-        </is>
-      </c>
-      <c r="J51" s="84" t="inlineStr">
-        <is>
-          <t>Dentons</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="88" t="inlineStr">
+      <c r="B58" s="86" t="inlineStr">
+        <is>
+          <t>Insurance-linked platforms — private credit</t>
+        </is>
+      </c>
+      <c r="C58" s="87" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D58" s="85" t="inlineStr">
+        <is>
+          <t>Athene, Global Atlantic, etc.</t>
+        </is>
+      </c>
+      <c r="E58" s="88" t="n">
+        <v>180</v>
+      </c>
+      <c r="F58" s="85" t="inlineStr">
+        <is>
+          <t>Insurance capital into private credit</t>
+        </is>
+      </c>
+      <c r="G58" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H58" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I58" s="85" t="inlineStr">
+        <is>
+          <t>~25% of global private credit AUM</t>
+        </is>
+      </c>
+      <c r="J58" s="89" t="inlineStr">
+        <is>
+          <t>McKinsey; ABF Journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="85" t="inlineStr">
+        <is>
+          <t>2026-28</t>
+        </is>
+      </c>
+      <c r="B59" s="86" t="inlineStr">
+        <is>
+          <t>Colocation — DC securitization supply</t>
+        </is>
+      </c>
+      <c r="C59" s="87" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D59" s="85" t="inlineStr">
+        <is>
+          <t>Industry-wide</t>
+        </is>
+      </c>
+      <c r="E59" s="88" t="n">
+        <v>130</v>
+      </c>
+      <c r="F59" s="85" t="inlineStr">
+        <is>
+          <t>ABS + CMBS net issuance</t>
+        </is>
+      </c>
+      <c r="G59" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H59" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I59" s="85" t="inlineStr">
+        <is>
+          <t>Morgan Stanley estimate</t>
+        </is>
+      </c>
+      <c r="J59" s="89" t="inlineStr">
+        <is>
+          <t>CREFC; Impax</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="85" t="inlineStr">
+        <is>
+          <t>to 2026</t>
+        </is>
+      </c>
+      <c r="B60" s="86" t="inlineStr">
+        <is>
+          <t>Sector — HY/unrated AI-infra debt</t>
+        </is>
+      </c>
+      <c r="C60" s="87" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D60" s="85" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="E60" s="88" t="n">
+        <v>107</v>
+      </c>
+      <c r="F60" s="85" t="inlineStr">
+        <is>
+          <t>Funded + committed debt</t>
+        </is>
+      </c>
+      <c r="G60" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H60" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I60" s="85" t="inlineStr">
+        <is>
+          <t>$68.7bn neoclouds / $38.7bn AI-native DCs</t>
+        </is>
+      </c>
+      <c r="J60" s="89" t="inlineStr">
+        <is>
+          <t>Octus</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="85" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="B61" s="86" t="inlineStr">
+        <is>
+          <t>KKR + Energy Capital Partners — partnership</t>
+        </is>
+      </c>
+      <c r="C61" s="87" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D61" s="85" t="inlineStr">
+        <is>
+          <t>KKR, ECP</t>
+        </is>
+      </c>
+      <c r="E61" s="88" t="n">
+        <v>50</v>
+      </c>
+      <c r="F61" s="85" t="inlineStr">
+        <is>
+          <t>Strategic partnership</t>
+        </is>
+      </c>
+      <c r="G61" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H61" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I61" s="85" t="inlineStr">
+        <is>
+          <t>Accelerate AI infrastructure</t>
+        </is>
+      </c>
+      <c r="J61" s="89" t="inlineStr">
+        <is>
+          <t>Business Times</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="30" customHeight="1">
+      <c r="A62" s="85" t="inlineStr">
         <is>
           <t>2025-28</t>
         </is>
       </c>
-      <c r="B52" s="88" t="inlineStr">
-        <is>
-          <t>Colocation sector</t>
-        </is>
-      </c>
-      <c r="C52" s="89" t="inlineStr">
+      <c r="B62" s="86" t="inlineStr">
+        <is>
+          <t>Broadcom + Apollo + Blackstone — platform</t>
+        </is>
+      </c>
+      <c r="C62" s="87" t="inlineStr">
         <is>
           <t>Context / market</t>
         </is>
       </c>
-      <c r="D52" s="88" t="inlineStr"/>
-      <c r="E52" s="95" t="inlineStr">
-        <is>
-          <t>~$130bn</t>
-        </is>
-      </c>
-      <c r="F52" s="88" t="inlineStr">
-        <is>
-          <t>Securitization (ABS/CMBS)</t>
-        </is>
-      </c>
-      <c r="G52" s="88" t="inlineStr"/>
-      <c r="H52" s="88" t="inlineStr"/>
-      <c r="I52" s="88" t="inlineStr">
-        <is>
-          <t>US data-center ABS+CMBS issuance ~$26bn in 2025 (~10x 2020); ~$57bn since 2021; Morgan Stanley ~$130bn securitized net issuance 2026-28; ~$150bn permanent financing need 2026-27</t>
-        </is>
-      </c>
-      <c r="J52" s="91" t="inlineStr">
-        <is>
-          <t>Impax; CREFC; Morgan Stanley</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="96" t="inlineStr">
-        <is>
-          <t>2025-30</t>
-        </is>
-      </c>
-      <c r="B53" s="96" t="inlineStr">
-        <is>
-          <t>HUMAIN (Saudi PIF)</t>
-        </is>
-      </c>
-      <c r="C53" s="97" t="inlineStr">
-        <is>
-          <t>Sovereign cloud</t>
-        </is>
-      </c>
-      <c r="D53" s="96" t="inlineStr"/>
-      <c r="E53" s="98" t="inlineStr">
-        <is>
-          <t>~$100bn</t>
-        </is>
-      </c>
-      <c r="F53" s="96" t="inlineStr">
-        <is>
-          <t>Sovereign equity</t>
-        </is>
-      </c>
-      <c r="G53" s="96" t="inlineStr"/>
-      <c r="H53" s="96" t="inlineStr"/>
-      <c r="I53" s="96" t="inlineStr">
-        <is>
-          <t>PIF national AI champion (announced 13 May 2025): ~$100bn across 11 data centers / 2.2 GW; ~600k NVIDIA GPUs; ALLAM Arabic LLM</t>
-        </is>
-      </c>
-      <c r="J53" s="99" t="inlineStr">
-        <is>
-          <t>Presenc AI; NYU DRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="96" t="inlineStr">
-        <is>
-          <t>2025-30</t>
-        </is>
-      </c>
-      <c r="B54" s="96" t="inlineStr">
-        <is>
-          <t>Stargate UAE / G42</t>
-        </is>
-      </c>
-      <c r="C54" s="97" t="inlineStr">
-        <is>
-          <t>Sovereign cloud</t>
-        </is>
-      </c>
-      <c r="D54" s="96" t="inlineStr"/>
-      <c r="E54" s="98" t="inlineStr">
-        <is>
-          <t>~$30bn+</t>
-        </is>
-      </c>
-      <c r="F54" s="96" t="inlineStr">
-        <is>
-          <t>Sovereign equity + JV</t>
-        </is>
-      </c>
-      <c r="G54" s="96" t="inlineStr"/>
-      <c r="H54" s="96" t="inlineStr"/>
-      <c r="I54" s="96" t="inlineStr">
-        <is>
-          <t>$30bn+ 5GW Abu Dhabi campus (Khazna/G42 w/ OpenAI, Oracle, NVIDIA, Cisco, SoftBank); Phase 1 200MW Q3 2026; Microsoft ~$1.5bn equity</t>
-        </is>
-      </c>
-      <c r="J54" s="99" t="inlineStr">
-        <is>
-          <t>Khaleej Times; dcpulse</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="96" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="B55" s="96" t="inlineStr">
-        <is>
-          <t>MGX / Mubadala (UAE)</t>
-        </is>
-      </c>
-      <c r="C55" s="97" t="inlineStr">
-        <is>
-          <t>Sovereign cloud</t>
-        </is>
-      </c>
-      <c r="D55" s="96" t="inlineStr"/>
-      <c r="E55" s="98" t="inlineStr">
-        <is>
-          <t>~$40bn+</t>
-        </is>
-      </c>
-      <c r="F55" s="96" t="inlineStr">
-        <is>
-          <t>Sovereign equity / infra</t>
-        </is>
-      </c>
-      <c r="G55" s="96" t="inlineStr"/>
-      <c r="H55" s="96" t="inlineStr"/>
-      <c r="I55" s="96" t="inlineStr">
-        <is>
-          <t>Anchored Stargate; co-led ~$40bn Aligned Data Centers acquisition w/ BlackRock; AIP (BlackRock-Microsoft) targets up to $100bn global AI infra</t>
-        </is>
-      </c>
-      <c r="J55" s="99" t="inlineStr">
-        <is>
-          <t>NYU DRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="88" t="inlineStr">
-        <is>
-          <t>to 2026</t>
-        </is>
-      </c>
-      <c r="B56" s="88" t="inlineStr">
-        <is>
-          <t>Sector-wide</t>
-        </is>
-      </c>
-      <c r="C56" s="89" t="inlineStr">
-        <is>
-          <t>Context / market</t>
-        </is>
-      </c>
-      <c r="D56" s="88" t="inlineStr"/>
-      <c r="E56" s="95" t="inlineStr">
-        <is>
-          <t>~$107bn</t>
-        </is>
-      </c>
-      <c r="F56" s="88" t="inlineStr">
-        <is>
-          <t>All debt</t>
-        </is>
-      </c>
-      <c r="G56" s="88" t="inlineStr"/>
-      <c r="H56" s="88" t="inlineStr"/>
-      <c r="I56" s="88" t="inlineStr">
-        <is>
-          <t>HY/unrated AI-infra issuers raised ~$107bn funded+committed debt by ~May 2026 ($68.7bn neoclouds / $38.7bn AI-native DCs)</t>
-        </is>
-      </c>
-      <c r="J56" s="91" t="inlineStr">
-        <is>
-          <t>Octus</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="88" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B57" s="88" t="inlineStr">
-        <is>
-          <t>Sector-wide</t>
-        </is>
-      </c>
-      <c r="C57" s="89" t="inlineStr">
-        <is>
-          <t>Context / market</t>
-        </is>
-      </c>
-      <c r="D57" s="88" t="inlineStr"/>
-      <c r="E57" s="95" t="inlineStr">
-        <is>
-          <t>~$180bn</t>
-        </is>
-      </c>
-      <c r="F57" s="88" t="inlineStr">
-        <is>
-          <t>Insurance / private credit</t>
-        </is>
-      </c>
-      <c r="G57" s="88" t="inlineStr"/>
-      <c r="H57" s="88" t="inlineStr"/>
-      <c r="I57" s="88" t="inlineStr">
-        <is>
-          <t>Insurance-linked platforms deployed ~$180bn into private credit in 2025 (~25% of global private credit AUM)</t>
-        </is>
-      </c>
-      <c r="J57" s="91" t="inlineStr">
-        <is>
-          <t>McKinsey; ABF Journal</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="88" t="inlineStr">
-        <is>
-          <t>2025-30</t>
-        </is>
-      </c>
-      <c r="B58" s="88" t="inlineStr">
-        <is>
-          <t>Sector-wide</t>
-        </is>
-      </c>
-      <c r="C58" s="89" t="inlineStr">
-        <is>
-          <t>Context / market</t>
-        </is>
-      </c>
-      <c r="D58" s="88" t="inlineStr"/>
-      <c r="E58" s="95" t="inlineStr">
-        <is>
-          <t>$5.3tn capex</t>
-        </is>
-      </c>
-      <c r="F58" s="88" t="inlineStr">
-        <is>
-          <t>Context</t>
-        </is>
-      </c>
-      <c r="G58" s="88" t="inlineStr"/>
-      <c r="H58" s="88" t="inlineStr"/>
-      <c r="I58" s="88" t="inlineStr">
-        <is>
-          <t>Goldman Sachs: ~$5.3tn AI + data-center capex 2025-2030; Morgan Stanley: ~$800bn private credit for AI DCs 2025-28</t>
-        </is>
-      </c>
-      <c r="J58" s="91" t="inlineStr">
-        <is>
-          <t>Goldman; Morgan Stanley</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="100" t="inlineStr">
-        <is>
-          <t>Selected sources:</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="101" t="inlineStr">
-        <is>
-          <t>Goldman Sachs Research — ~$5.3tn AI + data-center capex 2025-2030; private markets in DC financing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="101" t="inlineStr">
-        <is>
-          <t>Morgan Stanley — ~$2tn capex 2025-28 with &gt;$1tn debt; ~$800bn private credit for AI DCs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="101" t="inlineStr">
-        <is>
-          <t>Bank of America / BofA Securities — hyperscaler bond issuance ($121bn 2025; ~$175bn 2026E).</t>
+      <c r="D62" s="85" t="inlineStr">
+        <is>
+          <t>Apollo, Blackstone, Broadcom</t>
+        </is>
+      </c>
+      <c r="E62" s="100" t="n"/>
+      <c r="F62" s="85" t="inlineStr">
+        <is>
+          <t>Platform framework</t>
+        </is>
+      </c>
+      <c r="G62" s="85" t="inlineStr">
+        <is>
+          <t>&gt;20 GW</t>
+        </is>
+      </c>
+      <c r="H62" s="85" t="inlineStr">
+        <is>
+          <t>to 2028</t>
+        </is>
+      </c>
+      <c r="I62" s="85" t="inlineStr">
+        <is>
+          <t>Deploy &gt;20GW compute</t>
+        </is>
+      </c>
+      <c r="J62" s="89" t="inlineStr">
+        <is>
+          <t>privatedebtnews</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="101" t="inlineStr">
         <is>
+          <t>Selected sources:</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="102" t="inlineStr">
+        <is>
+          <t>Goldman Sachs Research — ~$5.3tn AI + data-center capex 2025-2030; private markets in DC financing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="102" t="inlineStr">
+        <is>
+          <t>Morgan Stanley — ~$2tn capex 2025-28 with &gt;$1tn debt; ~$800bn private credit for AI DCs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="102" t="inlineStr">
+        <is>
+          <t>Bank of America / BofA Securities — hyperscaler bond issuance ($121bn 2025; ~$175bn 2026E).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="102" t="inlineStr">
+        <is>
           <t>Moody's Ratings — hyperscaler capex (~$785bn 2026, ~$1tn 2027); $662bn off-B/S DC leases.</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="101" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="102" t="inlineStr">
         <is>
           <t>McKinsey — ~$2.7tn US (5.2tn global) data-center capex by 2030; insurance-linked private credit.</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="101" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="102" t="inlineStr">
         <is>
           <t>Octus — HY/unrated AI-infra debt (~$107bn to ~May 2026); ~14GW unfunded ≈ $344bn need.</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="101" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="102" t="inlineStr">
         <is>
           <t>Company / press: Meta IR, FT, S&amp;P, IFR (Hyperion); Oracle IR, IFR, Reuters; CoreWeave IR; Blackstone;</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="101" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="102" t="inlineStr">
         <is>
           <t xml:space="preserve">  Apollo Academy; privatedebtnews; Bisnow; Quinn Emanuel; Build.inc; CNBC / WSJ / The Information (xAI).</t>
         </is>

</xml_diff>

<commit_message>
Add Microsoft (finance leases, AIP) and SpaceX ($25bn bond) to deals tab
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AI_Infrastructure_Financing_2025-2030.xlsx
+++ b/AI_Infrastructure_Financing_2025-2030.xlsx
@@ -8146,7 +8146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8446,48 +8446,52 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="70" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B10" s="71" t="inlineStr">
-        <is>
-          <t>Oracle (OCI)</t>
-        </is>
-      </c>
-      <c r="C10" s="72" t="inlineStr">
-        <is>
-          <t>Hyperscaler</t>
-        </is>
-      </c>
-      <c r="D10" s="70" t="inlineStr">
+      <c r="A10" s="75" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B10" s="76" t="inlineStr">
+        <is>
+          <t>SpaceX / xAI</t>
+        </is>
+      </c>
+      <c r="C10" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D10" s="75" t="inlineStr">
         <is>
           <t>Bank syndicate</t>
         </is>
       </c>
-      <c r="E10" s="73" t="n">
-        <v>18</v>
-      </c>
-      <c r="F10" s="70" t="inlineStr">
-        <is>
-          <t>Public IG bond (6-part)</t>
-        </is>
-      </c>
-      <c r="G10" s="70" t="inlineStr">
-        <is>
-          <t>IG</t>
-        </is>
-      </c>
-      <c r="H10" s="70" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I10" s="70" t="inlineStr"/>
-      <c r="J10" s="74" t="inlineStr">
-        <is>
-          <t>Reuters; CNA</t>
+      <c r="E10" s="78" t="n">
+        <v>25</v>
+      </c>
+      <c r="F10" s="75" t="inlineStr">
+        <is>
+          <t>Inaugural senior unsecured bond (5 tranches)</t>
+        </is>
+      </c>
+      <c r="G10" s="75" t="inlineStr">
+        <is>
+          <t>5.35-6.65%</t>
+        </is>
+      </c>
+      <c r="H10" s="75" t="inlineStr">
+        <is>
+          <t>2031-2056</t>
+        </is>
+      </c>
+      <c r="I10" s="75" t="inlineStr">
+        <is>
+          <t>Refinanced ~$20bn bridge loan; funds SpaceX/Starlink + xAI compute</t>
+        </is>
+      </c>
+      <c r="J10" s="79" t="inlineStr">
+        <is>
+          <t>SpaceX 8-K; StockTitan</t>
         </is>
       </c>
     </row>
@@ -8499,7 +8503,7 @@
       </c>
       <c r="B11" s="71" t="inlineStr">
         <is>
-          <t>Amazon (AWS)</t>
+          <t>Oracle (OCI)</t>
         </is>
       </c>
       <c r="C11" s="72" t="inlineStr">
@@ -8513,11 +8517,11 @@
         </is>
       </c>
       <c r="E11" s="73" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F11" s="70" t="inlineStr">
         <is>
-          <t>Public IG bond</t>
+          <t>Public IG bond (6-part)</t>
         </is>
       </c>
       <c r="G11" s="70" t="inlineStr">
@@ -8533,185 +8537,181 @@
       <c r="I11" s="70" t="inlineStr"/>
       <c r="J11" s="74" t="inlineStr">
         <is>
+          <t>Reuters; CNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B12" s="71" t="inlineStr">
+        <is>
+          <t>Amazon (AWS)</t>
+        </is>
+      </c>
+      <c r="C12" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D12" s="70" t="inlineStr">
+        <is>
+          <t>Bank syndicate</t>
+        </is>
+      </c>
+      <c r="E12" s="73" t="n">
+        <v>15</v>
+      </c>
+      <c r="F12" s="70" t="inlineStr">
+        <is>
+          <t>Public IG bond</t>
+        </is>
+      </c>
+      <c r="G12" s="70" t="inlineStr">
+        <is>
+          <t>IG</t>
+        </is>
+      </c>
+      <c r="H12" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I12" s="70" t="inlineStr"/>
+      <c r="J12" s="74" t="inlineStr">
+        <is>
           <t>CNA</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>2) BANK &amp; SYNDICATED LOANS (incl. GPU-backed term loans)</t>
         </is>
       </c>
-      <c r="B12" s="15" t="n"/>
-      <c r="C12" s="15" t="n"/>
-      <c r="D12" s="15" t="n"/>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="15" t="n"/>
-      <c r="G12" s="15" t="n"/>
-      <c r="H12" s="15" t="n"/>
-      <c r="I12" s="15" t="n"/>
-      <c r="J12" s="15" t="n"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="75" t="inlineStr">
+      <c r="B13" s="15" t="n"/>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="15" t="n"/>
+      <c r="H13" s="15" t="n"/>
+      <c r="I13" s="15" t="n"/>
+      <c r="J13" s="15" t="n"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="75" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="B13" s="76" t="inlineStr">
+      <c r="B14" s="76" t="inlineStr">
         <is>
           <t>CoreWeave — DDTL 4.0</t>
         </is>
       </c>
-      <c r="C13" s="77" t="inlineStr">
+      <c r="C14" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D13" s="75" t="inlineStr">
+      <c r="D14" s="75" t="inlineStr">
         <is>
           <t>Blackstone Credit &amp; Insurance (anchor); MUFG, MS, GS, JPM</t>
         </is>
       </c>
-      <c r="E13" s="78" t="n">
+      <c r="E14" s="78" t="n">
         <v>8.5</v>
       </c>
-      <c r="F13" s="75" t="inlineStr">
+      <c r="F14" s="75" t="inlineStr">
         <is>
           <t>GPU-backed delayed-draw term loan</t>
         </is>
       </c>
-      <c r="G13" s="75" t="inlineStr">
+      <c r="G14" s="75" t="inlineStr">
         <is>
           <t>SOFR+225 / ~5.9%</t>
         </is>
       </c>
-      <c r="H13" s="75" t="inlineStr">
+      <c r="H14" s="75" t="inlineStr">
         <is>
           <t>Mar 2032</t>
         </is>
       </c>
-      <c r="I13" s="75" t="inlineStr">
+      <c r="I14" s="75" t="inlineStr">
         <is>
           <t>First IG-rated (A3 / A low) HPC loan; non-recourse</t>
         </is>
       </c>
-      <c r="J13" s="79" t="inlineStr">
+      <c r="J14" s="79" t="inlineStr">
         <is>
           <t>CoreWeave IR</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="80" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="80" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="B14" s="81" t="inlineStr">
+      <c r="B15" s="81" t="inlineStr">
         <is>
           <t>Applied Digital</t>
         </is>
       </c>
-      <c r="C14" s="82" t="inlineStr">
+      <c r="C15" s="82" t="inlineStr">
         <is>
           <t>Colocation / data-center REIT</t>
         </is>
       </c>
-      <c r="D14" s="80" t="inlineStr">
+      <c r="D15" s="80" t="inlineStr">
         <is>
           <t>Macquarie</t>
         </is>
       </c>
-      <c r="E14" s="83" t="n">
+      <c r="E15" s="83" t="n">
         <v>5</v>
       </c>
-      <c r="F14" s="80" t="inlineStr">
+      <c r="F15" s="80" t="inlineStr">
         <is>
           <t>Structured HPC financing</t>
         </is>
       </c>
-      <c r="G14" s="80" t="inlineStr">
+      <c r="G15" s="80" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H14" s="80" t="inlineStr">
+      <c r="H15" s="80" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I14" s="80" t="inlineStr">
+      <c r="I15" s="80" t="inlineStr">
         <is>
           <t>Powered-shell build for CoreWeave</t>
         </is>
       </c>
-      <c r="J14" s="84" t="inlineStr">
+      <c r="J15" s="84" t="inlineStr">
         <is>
           <t>press</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="75" t="inlineStr">
-        <is>
-          <t>May 2025</t>
-        </is>
-      </c>
-      <c r="B15" s="76" t="inlineStr">
-        <is>
-          <t>Anthropic</t>
-        </is>
-      </c>
-      <c r="C15" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D15" s="75" t="inlineStr">
-        <is>
-          <t>Bank syndicate</t>
-        </is>
-      </c>
-      <c r="E15" s="78" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F15" s="75" t="inlineStr">
-        <is>
-          <t>Revolving credit line</t>
-        </is>
-      </c>
-      <c r="G15" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H15" s="75" t="inlineStr">
-        <is>
-          <t>5y</t>
-        </is>
-      </c>
-      <c r="I15" s="75" t="inlineStr">
-        <is>
-          <t>Liquidity backstop</t>
-        </is>
-      </c>
-      <c r="J15" s="79" t="inlineStr">
-        <is>
-          <t>CNBC</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="75" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>May 2025</t>
         </is>
       </c>
       <c r="B16" s="76" t="inlineStr">
         <is>
-          <t>Nscale</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C16" s="77" t="inlineStr">
@@ -8721,15 +8721,15 @@
       </c>
       <c r="D16" s="75" t="inlineStr">
         <is>
-          <t>Private credit / banks</t>
+          <t>Bank syndicate</t>
         </is>
       </c>
       <c r="E16" s="78" t="n">
-        <v>1.4</v>
+        <v>2.5</v>
       </c>
       <c r="F16" s="75" t="inlineStr">
         <is>
-          <t>Term loan</t>
+          <t>Revolving credit line</t>
         </is>
       </c>
       <c r="G16" s="75" t="inlineStr">
@@ -8739,245 +8739,245 @@
       </c>
       <c r="H16" s="75" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>5y</t>
         </is>
       </c>
       <c r="I16" s="75" t="inlineStr">
         <is>
-          <t>GPU-cloud build</t>
+          <t>Liquidity backstop</t>
         </is>
       </c>
       <c r="J16" s="79" t="inlineStr">
         <is>
-          <t>theaiinsider</t>
+          <t>CNBC</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="75" t="inlineStr">
         <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B17" s="76" t="inlineStr">
+        <is>
+          <t>Nscale</t>
+        </is>
+      </c>
+      <c r="C17" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D17" s="75" t="inlineStr">
+        <is>
+          <t>Private credit / banks</t>
+        </is>
+      </c>
+      <c r="E17" s="78" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F17" s="75" t="inlineStr">
+        <is>
+          <t>Term loan</t>
+        </is>
+      </c>
+      <c r="G17" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H17" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I17" s="75" t="inlineStr">
+        <is>
+          <t>GPU-cloud build</t>
+        </is>
+      </c>
+      <c r="J17" s="79" t="inlineStr">
+        <is>
+          <t>theaiinsider</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="75" t="inlineStr">
+        <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B17" s="76" t="inlineStr">
+      <c r="B18" s="76" t="inlineStr">
         <is>
           <t>Lambda</t>
         </is>
       </c>
-      <c r="C17" s="77" t="inlineStr">
+      <c r="C18" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D17" s="75" t="inlineStr">
+      <c r="D18" s="75" t="inlineStr">
         <is>
           <t>Macquarie</t>
         </is>
       </c>
-      <c r="E17" s="78" t="n">
+      <c r="E18" s="78" t="n">
         <v>0.5</v>
       </c>
-      <c r="F17" s="75" t="inlineStr">
+      <c r="F18" s="75" t="inlineStr">
         <is>
           <t>GPU-backed facility</t>
         </is>
       </c>
-      <c r="G17" s="75" t="inlineStr">
+      <c r="G18" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H17" s="75" t="inlineStr">
+      <c r="H18" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I17" s="75" t="inlineStr">
+      <c r="I18" s="75" t="inlineStr">
         <is>
           <t>GPU-cloud build</t>
         </is>
       </c>
-      <c r="J17" s="79" t="inlineStr">
+      <c r="J18" s="79" t="inlineStr">
         <is>
           <t>theaiinsider</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>3) ALTERNATE PRIVATE CREDIT / SPV / 144A</t>
         </is>
       </c>
-      <c r="B18" s="15" t="n"/>
-      <c r="C18" s="15" t="n"/>
-      <c r="D18" s="15" t="n"/>
-      <c r="E18" s="15" t="n"/>
-      <c r="F18" s="15" t="n"/>
-      <c r="G18" s="15" t="n"/>
-      <c r="H18" s="15" t="n"/>
-      <c r="I18" s="15" t="n"/>
-      <c r="J18" s="15" t="n"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="70" t="inlineStr">
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="15" t="n"/>
+      <c r="G19" s="15" t="n"/>
+      <c r="H19" s="15" t="n"/>
+      <c r="I19" s="15" t="n"/>
+      <c r="J19" s="15" t="n"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="70" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="B19" s="71" t="inlineStr">
+      <c r="B20" s="71" t="inlineStr">
         <is>
           <t>Oracle — Texas + Wisconsin DCs</t>
         </is>
       </c>
-      <c r="C19" s="72" t="inlineStr">
+      <c r="C20" s="72" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="D19" s="70" t="inlineStr">
+      <c r="D20" s="70" t="inlineStr">
         <is>
           <t>Private credit consortium</t>
         </is>
       </c>
-      <c r="E19" s="73" t="n">
+      <c r="E20" s="73" t="n">
         <v>38</v>
       </c>
-      <c r="F19" s="70" t="inlineStr">
+      <c r="F20" s="70" t="inlineStr">
         <is>
           <t>SPV debt package</t>
         </is>
       </c>
-      <c r="G19" s="70" t="inlineStr">
+      <c r="G20" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H19" s="70" t="inlineStr">
+      <c r="H20" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I19" s="70" t="inlineStr">
+      <c r="I20" s="70" t="inlineStr">
         <is>
           <t>Two-site off-B/S financing</t>
         </is>
       </c>
-      <c r="J19" s="74" t="inlineStr">
+      <c r="J20" s="74" t="inlineStr">
         <is>
           <t>FT</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="75" t="inlineStr">
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="75" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="B20" s="76" t="inlineStr">
+      <c r="B21" s="76" t="inlineStr">
         <is>
           <t>Anthropic — Google TPU chip SPV</t>
         </is>
       </c>
-      <c r="C20" s="77" t="inlineStr">
+      <c r="C21" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D20" s="75" t="inlineStr">
+      <c r="D21" s="75" t="inlineStr">
         <is>
           <t>Apollo, Blackstone; Broadcom RVG</t>
         </is>
       </c>
-      <c r="E20" s="78" t="n">
+      <c r="E21" s="78" t="n">
         <v>35</v>
       </c>
-      <c r="F20" s="75" t="inlineStr">
+      <c r="F21" s="75" t="inlineStr">
         <is>
           <t>Chip-leasing SPV; 3 tranches; ~half syndicated</t>
         </is>
       </c>
-      <c r="G20" s="75" t="inlineStr">
+      <c r="G21" s="75" t="inlineStr">
         <is>
           <t>A1 T+100bp; A2 5.75%; B 8.5%</t>
         </is>
       </c>
-      <c r="H20" s="75" t="inlineStr">
+      <c r="H21" s="75" t="inlineStr">
         <is>
           <t>~5y</t>
         </is>
       </c>
-      <c r="I20" s="75" t="inlineStr">
+      <c r="I21" s="75" t="inlineStr">
         <is>
           <t>Buys Google TPUs leased to Anthropic</t>
         </is>
       </c>
-      <c r="J20" s="79" t="inlineStr">
+      <c r="J21" s="79" t="inlineStr">
         <is>
           <t>privatedebtnews; Build.inc</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="70" t="inlineStr">
-        <is>
-          <t>Oct 2025</t>
-        </is>
-      </c>
-      <c r="B21" s="71" t="inlineStr">
-        <is>
-          <t>Meta — Hyperion (Beignet Investor LLC)</t>
-        </is>
-      </c>
-      <c r="C21" s="72" t="inlineStr">
-        <is>
-          <t>Hyperscaler</t>
-        </is>
-      </c>
-      <c r="D21" s="70" t="inlineStr">
-        <is>
-          <t>PIMCO (~$18bn), BlackRock, Apollo; Blue Owl equity</t>
-        </is>
-      </c>
-      <c r="E21" s="73" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="F21" s="70" t="inlineStr">
-        <is>
-          <t>Off-B/S SPV; 144A senior secured bond</t>
-        </is>
-      </c>
-      <c r="G21" s="70" t="inlineStr">
-        <is>
-          <t>6.581% / T+225bp</t>
-        </is>
-      </c>
-      <c r="H21" s="70" t="inlineStr">
-        <is>
-          <t>Due May 2049</t>
-        </is>
-      </c>
-      <c r="I21" s="70" t="inlineStr">
-        <is>
-          <t>2.1GW; Meta lease + residual-value guarantee; A+ (S&amp;P)</t>
-        </is>
-      </c>
-      <c r="J21" s="74" t="inlineStr">
-        <is>
-          <t>IFR; FT; Quinn Emanuel</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="70" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>Oct 2025</t>
         </is>
       </c>
       <c r="B22" s="71" t="inlineStr">
         <is>
-          <t>Oracle — New Mexico site</t>
+          <t>Meta — Hyperion (Beignet Investor LLC)</t>
         </is>
       </c>
       <c r="C22" s="72" t="inlineStr">
@@ -8987,347 +8987,347 @@
       </c>
       <c r="D22" s="70" t="inlineStr">
         <is>
-          <t>Private credit lenders</t>
+          <t>PIMCO (~$18bn), BlackRock, Apollo; Blue Owl equity</t>
         </is>
       </c>
       <c r="E22" s="73" t="n">
-        <v>18</v>
+        <v>27.3</v>
       </c>
       <c r="F22" s="70" t="inlineStr">
         <is>
-          <t>SPV / project loan</t>
+          <t>Off-B/S SPV; 144A senior secured bond</t>
         </is>
       </c>
       <c r="G22" s="70" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>6.581% / T+225bp</t>
         </is>
       </c>
       <c r="H22" s="70" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Due May 2049</t>
         </is>
       </c>
       <c r="I22" s="70" t="inlineStr">
         <is>
-          <t>Single-site project loan</t>
+          <t>2.1GW; Meta lease + residual-value guarantee; A+ (S&amp;P)</t>
         </is>
       </c>
       <c r="J22" s="74" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>IFR; FT; Quinn Emanuel</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="70" t="inlineStr">
         <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B23" s="71" t="inlineStr">
+        <is>
+          <t>Oracle — New Mexico site</t>
+        </is>
+      </c>
+      <c r="C23" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D23" s="70" t="inlineStr">
+        <is>
+          <t>Private credit lenders</t>
+        </is>
+      </c>
+      <c r="E23" s="73" t="n">
+        <v>18</v>
+      </c>
+      <c r="F23" s="70" t="inlineStr">
+        <is>
+          <t>SPV / project loan</t>
+        </is>
+      </c>
+      <c r="G23" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H23" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I23" s="70" t="inlineStr">
+        <is>
+          <t>Single-site project loan</t>
+        </is>
+      </c>
+      <c r="J23" s="74" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="70" t="inlineStr">
+        <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B23" s="71" t="inlineStr">
+      <c r="B24" s="71" t="inlineStr">
         <is>
           <t>Oracle — Michigan campus</t>
         </is>
       </c>
-      <c r="C23" s="72" t="inlineStr">
+      <c r="C24" s="72" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="D23" s="70" t="inlineStr">
+      <c r="D24" s="70" t="inlineStr">
         <is>
           <t>Project-finance lenders</t>
         </is>
       </c>
-      <c r="E23" s="73" t="n">
+      <c r="E24" s="73" t="n">
         <v>16.3</v>
       </c>
-      <c r="F23" s="70" t="inlineStr">
+      <c r="F24" s="70" t="inlineStr">
         <is>
           <t>Project-level SPV financing</t>
         </is>
       </c>
-      <c r="G23" s="70" t="inlineStr">
+      <c r="G24" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H23" s="70" t="inlineStr">
+      <c r="H24" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I23" s="70" t="inlineStr">
+      <c r="I24" s="70" t="inlineStr">
         <is>
           <t>OCI capacity build</t>
         </is>
       </c>
-      <c r="J23" s="74" t="inlineStr">
+      <c r="J24" s="74" t="inlineStr">
         <is>
           <t>Press reports</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="75" t="inlineStr">
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="75" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="B24" s="76" t="inlineStr">
+      <c r="B25" s="76" t="inlineStr">
         <is>
           <t>xAI — Colossus 2 chip SPV</t>
         </is>
       </c>
-      <c r="C24" s="77" t="inlineStr">
+      <c r="C25" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D24" s="75" t="inlineStr">
+      <c r="D25" s="75" t="inlineStr">
         <is>
           <t>Valor Equity, Apollo, Diameter; NVIDIA equity</t>
         </is>
       </c>
-      <c r="E24" s="78" t="n">
+      <c r="E25" s="78" t="n">
         <v>12.5</v>
       </c>
-      <c r="F24" s="75" t="inlineStr">
+      <c r="F25" s="75" t="inlineStr">
         <is>
           <t>SPV; debt + ~$7.5bn equity</t>
         </is>
       </c>
-      <c r="G24" s="75" t="inlineStr">
+      <c r="G25" s="75" t="inlineStr">
         <is>
           <t>~10.5%</t>
         </is>
       </c>
-      <c r="H24" s="75" t="inlineStr">
+      <c r="H25" s="75" t="inlineStr">
         <is>
           <t>5y (~2.5y avg)</t>
         </is>
       </c>
-      <c r="I24" s="75" t="inlineStr">
+      <c r="I25" s="75" t="inlineStr">
         <is>
           <t>Buys NVIDIA GPUs leased to xAI</t>
         </is>
       </c>
-      <c r="J24" s="79" t="inlineStr">
+      <c r="J25" s="79" t="inlineStr">
         <is>
           <t>FT; WSJ</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="70" t="inlineStr">
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="70" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B25" s="71" t="inlineStr">
+      <c r="B26" s="71" t="inlineStr">
         <is>
           <t>Oracle/OpenAI — Abilene, TX (Stargate)</t>
         </is>
       </c>
-      <c r="C25" s="72" t="inlineStr">
+      <c r="C26" s="72" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="D25" s="70" t="inlineStr">
+      <c r="D26" s="70" t="inlineStr">
         <is>
           <t>Blue Owl + JPMorgan (Crusoe, Primary Digital)</t>
         </is>
       </c>
-      <c r="E25" s="73" t="n">
+      <c r="E26" s="73" t="n">
         <v>10</v>
       </c>
-      <c r="F25" s="70" t="inlineStr">
+      <c r="F26" s="70" t="inlineStr">
         <is>
           <t>Off-B/S SPV (~$13bn incl equity)</t>
         </is>
       </c>
-      <c r="G25" s="70" t="inlineStr">
+      <c r="G26" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H25" s="70" t="inlineStr">
+      <c r="H26" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I25" s="70" t="inlineStr">
+      <c r="I26" s="70" t="inlineStr">
         <is>
           <t>SPV owns OpenAI Abilene facility</t>
         </is>
       </c>
-      <c r="J25" s="74" t="inlineStr">
+      <c r="J26" s="74" t="inlineStr">
         <is>
           <t>FT</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="75" t="inlineStr">
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="75" t="inlineStr">
         <is>
           <t>May 2024</t>
         </is>
       </c>
-      <c r="B26" s="76" t="inlineStr">
+      <c r="B27" s="76" t="inlineStr">
         <is>
           <t>CoreWeave — $7.5bn facility</t>
         </is>
       </c>
-      <c r="C26" s="77" t="inlineStr">
+      <c r="C27" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D26" s="75" t="inlineStr">
+      <c r="D27" s="75" t="inlineStr">
         <is>
           <t>Blackstone, Magnetar, Coatue, Carlyle, CDPQ, BlackRock</t>
         </is>
       </c>
-      <c r="E26" s="78" t="n">
+      <c r="E27" s="78" t="n">
         <v>7.5</v>
       </c>
-      <c r="F26" s="75" t="inlineStr">
+      <c r="F27" s="75" t="inlineStr">
         <is>
           <t>GPU + customer-contract secured facility</t>
         </is>
       </c>
-      <c r="G26" s="75" t="inlineStr">
+      <c r="G27" s="75" t="inlineStr">
         <is>
           <t>~10%+</t>
         </is>
       </c>
-      <c r="H26" s="75" t="inlineStr">
+      <c r="H27" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I26" s="75" t="inlineStr">
+      <c r="I27" s="75" t="inlineStr">
         <is>
           <t>Largest private debt deal at the time</t>
         </is>
       </c>
-      <c r="J26" s="79" t="inlineStr">
+      <c r="J27" s="79" t="inlineStr">
         <is>
           <t>Blackstone</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="80" t="inlineStr">
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="80" t="inlineStr">
         <is>
           <t>Early 2025</t>
         </is>
       </c>
-      <c r="B27" s="81" t="inlineStr">
+      <c r="B28" s="81" t="inlineStr">
         <is>
           <t>Aligned Data Centers — debt</t>
         </is>
       </c>
-      <c r="C27" s="82" t="inlineStr">
+      <c r="C28" s="82" t="inlineStr">
         <is>
           <t>Colocation / data-center REIT</t>
         </is>
       </c>
-      <c r="D27" s="80" t="inlineStr">
+      <c r="D28" s="80" t="inlineStr">
         <is>
           <t>Macquarie + global investors</t>
         </is>
       </c>
-      <c r="E27" s="83" t="n">
+      <c r="E28" s="83" t="n">
         <v>7</v>
       </c>
-      <c r="F27" s="80" t="inlineStr">
+      <c r="F28" s="80" t="inlineStr">
         <is>
           <t>Debt within $12bn raise (+$5bn equity)</t>
         </is>
       </c>
-      <c r="G27" s="80" t="inlineStr">
+      <c r="G28" s="80" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H27" s="80" t="inlineStr">
+      <c r="H28" s="80" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I27" s="80" t="inlineStr">
+      <c r="I28" s="80" t="inlineStr">
         <is>
           <t>Later acquired by MGX/BlackRock (~$40bn)</t>
         </is>
       </c>
-      <c r="J27" s="84" t="inlineStr">
+      <c r="J28" s="84" t="inlineStr">
         <is>
           <t>SFA; NYU DRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="75" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B28" s="76" t="inlineStr">
-        <is>
-          <t>Fluidstack — Google-backed facility</t>
-        </is>
-      </c>
-      <c r="C28" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D28" s="75" t="inlineStr">
-        <is>
-          <t>Private credit (Google lease backstop)</t>
-        </is>
-      </c>
-      <c r="E28" s="78" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="F28" s="75" t="inlineStr">
-        <is>
-          <t>SPV backed by contracted revenue</t>
-        </is>
-      </c>
-      <c r="G28" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H28" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I28" s="75" t="inlineStr">
-        <is>
-          <t>~$6.7bn Google-contracted revenue</t>
-        </is>
-      </c>
-      <c r="J28" s="79" t="inlineStr">
-        <is>
-          <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="75" t="inlineStr">
         <is>
-          <t>Jun-Jul 2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="B29" s="76" t="inlineStr">
         <is>
-          <t>xAI — secured notes / term loan</t>
+          <t>Fluidstack — Google-backed facility</t>
         </is>
       </c>
       <c r="C29" s="77" t="inlineStr">
@@ -9337,47 +9337,47 @@
       </c>
       <c r="D29" s="75" t="inlineStr">
         <is>
-          <t>Apollo, Diameter; Morgan Stanley</t>
+          <t>Private credit (Google lease backstop)</t>
         </is>
       </c>
       <c r="E29" s="78" t="n">
-        <v>5</v>
+        <v>6.7</v>
       </c>
       <c r="F29" s="75" t="inlineStr">
         <is>
-          <t>Secured notes + term loan (part of $10bn raise)</t>
+          <t>SPV backed by contracted revenue</t>
         </is>
       </c>
       <c r="G29" s="75" t="inlineStr">
         <is>
-          <t>up to ~12.5%</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H29" s="75" t="inlineStr">
         <is>
-          <t>~3-5y</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I29" s="75" t="inlineStr">
         <is>
-          <t>Lenders can operate Colossus on default</t>
+          <t>~$6.7bn Google-contracted revenue</t>
         </is>
       </c>
       <c r="J29" s="79" t="inlineStr">
         <is>
-          <t>CNBC; ciphertalk</t>
+          <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="75" t="inlineStr">
         <is>
-          <t>Jul 2025</t>
+          <t>Jun-Jul 2025</t>
         </is>
       </c>
       <c r="B30" s="76" t="inlineStr">
         <is>
-          <t>CoreWeave — OpenAI contract financing</t>
+          <t>xAI — secured notes / term loan</t>
         </is>
       </c>
       <c r="C30" s="77" t="inlineStr">
@@ -9387,375 +9387,375 @@
       </c>
       <c r="D30" s="75" t="inlineStr">
         <is>
-          <t>Private lenders (SPV)</t>
+          <t>Apollo, Diameter; Morgan Stanley</t>
         </is>
       </c>
       <c r="E30" s="78" t="n">
-        <v>2.6</v>
+        <v>5</v>
       </c>
       <c r="F30" s="75" t="inlineStr">
         <is>
-          <t>SPV debt vs $11.9bn OpenAI contract</t>
+          <t>Secured notes + term loan (part of $10bn raise)</t>
         </is>
       </c>
       <c r="G30" s="75" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>up to ~12.5%</t>
         </is>
       </c>
       <c r="H30" s="75" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>~3-5y</t>
         </is>
       </c>
       <c r="I30" s="75" t="inlineStr">
         <is>
-          <t>Funds OpenAI compute obligations</t>
+          <t>Lenders can operate Colossus on default</t>
         </is>
       </c>
       <c r="J30" s="79" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>CNBC; ciphertalk</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="75" t="inlineStr">
         <is>
+          <t>Jul 2025</t>
+        </is>
+      </c>
+      <c r="B31" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — OpenAI contract financing</t>
+        </is>
+      </c>
+      <c r="C31" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D31" s="75" t="inlineStr">
+        <is>
+          <t>Private lenders (SPV)</t>
+        </is>
+      </c>
+      <c r="E31" s="78" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F31" s="75" t="inlineStr">
+        <is>
+          <t>SPV debt vs $11.9bn OpenAI contract</t>
+        </is>
+      </c>
+      <c r="G31" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H31" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I31" s="75" t="inlineStr">
+        <is>
+          <t>Funds OpenAI compute obligations</t>
+        </is>
+      </c>
+      <c r="J31" s="79" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="75" t="inlineStr">
+        <is>
           <t>Aug 2023</t>
         </is>
       </c>
-      <c r="B31" s="76" t="inlineStr">
+      <c r="B32" s="76" t="inlineStr">
         <is>
           <t>CoreWeave — $2.3bn facility</t>
         </is>
       </c>
-      <c r="C31" s="77" t="inlineStr">
+      <c r="C32" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D31" s="75" t="inlineStr">
+      <c r="D32" s="75" t="inlineStr">
         <is>
           <t>Blackstone, Magnetar</t>
         </is>
       </c>
-      <c r="E31" s="78" t="n">
+      <c r="E32" s="78" t="n">
         <v>2.3</v>
       </c>
-      <c r="F31" s="75" t="inlineStr">
+      <c r="F32" s="75" t="inlineStr">
         <is>
           <t>GPU-backed facility</t>
         </is>
       </c>
-      <c r="G31" s="75" t="inlineStr">
+      <c r="G32" s="75" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="H31" s="75" t="inlineStr">
+      <c r="H32" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I31" s="75" t="inlineStr">
+      <c r="I32" s="75" t="inlineStr">
         <is>
           <t>Early GPU-collateralized template</t>
         </is>
       </c>
-      <c r="J31" s="79" t="inlineStr">
+      <c r="J32" s="79" t="inlineStr">
         <is>
           <t>Blackstone</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="14" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>4) INSURANCE-LINKED LENDING (memo — overlaps groups 1-3)</t>
         </is>
       </c>
-      <c r="B32" s="15" t="n"/>
-      <c r="C32" s="15" t="n"/>
-      <c r="D32" s="15" t="n"/>
-      <c r="E32" s="15" t="n"/>
-      <c r="F32" s="15" t="n"/>
-      <c r="G32" s="15" t="n"/>
-      <c r="H32" s="15" t="n"/>
-      <c r="I32" s="15" t="n"/>
-      <c r="J32" s="15" t="n"/>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="75" t="inlineStr">
+      <c r="B33" s="15" t="n"/>
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="15" t="n"/>
+      <c r="E33" s="15" t="n"/>
+      <c r="F33" s="15" t="n"/>
+      <c r="G33" s="15" t="n"/>
+      <c r="H33" s="15" t="n"/>
+      <c r="I33" s="15" t="n"/>
+      <c r="J33" s="15" t="n"/>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="75" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="B33" s="76" t="inlineStr">
+      <c r="B34" s="76" t="inlineStr">
         <is>
           <t>Anthropic — A2 notes (insurer tranche)</t>
         </is>
       </c>
-      <c r="C33" s="77" t="inlineStr">
+      <c r="C34" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D33" s="75" t="inlineStr">
+      <c r="D34" s="75" t="inlineStr">
         <is>
           <t>Apollo / Athene + insurers</t>
         </is>
       </c>
-      <c r="E33" s="78" t="n">
+      <c r="E34" s="78" t="n">
         <v>24</v>
       </c>
-      <c r="F33" s="75" t="inlineStr">
+      <c r="F34" s="75" t="inlineStr">
         <is>
           <t>Insurance-bought A2 tranche of TPU SPV</t>
         </is>
       </c>
-      <c r="G33" s="75" t="inlineStr">
+      <c r="G34" s="75" t="inlineStr">
         <is>
           <t>5.75%</t>
         </is>
       </c>
-      <c r="H33" s="75" t="inlineStr">
+      <c r="H34" s="75" t="inlineStr">
         <is>
           <t>~5y</t>
         </is>
       </c>
-      <c r="I33" s="75" t="inlineStr">
+      <c r="I34" s="75" t="inlineStr">
         <is>
           <t>Within the $35bn Anthropic deal (group 3)</t>
         </is>
       </c>
-      <c r="J33" s="79" t="inlineStr">
+      <c r="J34" s="79" t="inlineStr">
         <is>
           <t>privatedebtnews</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="85" t="inlineStr">
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="85" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B34" s="86" t="inlineStr">
+      <c r="B35" s="86" t="inlineStr">
         <is>
           <t>Athene (Apollo) — AP Grange</t>
         </is>
       </c>
-      <c r="C34" s="87" t="inlineStr">
+      <c r="C35" s="87" t="inlineStr">
         <is>
           <t>Context / market</t>
         </is>
       </c>
-      <c r="D34" s="85" t="inlineStr">
+      <c r="D35" s="85" t="inlineStr">
         <is>
           <t>Athene / Apollo (+ Intel equity)</t>
         </is>
       </c>
-      <c r="E34" s="88" t="n">
+      <c r="E35" s="88" t="n">
         <v>6.5</v>
       </c>
-      <c r="F34" s="85" t="inlineStr">
+      <c r="F35" s="85" t="inlineStr">
         <is>
           <t>Insurer JV investment (semis-adjacent)</t>
         </is>
       </c>
-      <c r="G34" s="85" t="inlineStr">
+      <c r="G35" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H34" s="85" t="inlineStr">
+      <c r="H35" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I34" s="85" t="inlineStr">
+      <c r="I35" s="85" t="inlineStr">
         <is>
           <t>Largest single-issuer insurer credit exposure</t>
         </is>
       </c>
-      <c r="J34" s="89" t="inlineStr">
+      <c r="J35" s="89" t="inlineStr">
         <is>
           <t>Moody's</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="70" t="inlineStr">
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="70" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
       </c>
-      <c r="B35" s="71" t="inlineStr">
+      <c r="B36" s="71" t="inlineStr">
         <is>
           <t>Meta — Hyperion insurance allocation</t>
         </is>
       </c>
-      <c r="C35" s="72" t="inlineStr">
+      <c r="C36" s="72" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="D35" s="70" t="inlineStr">
+      <c r="D36" s="70" t="inlineStr">
         <is>
           <t>Insurers via PIMCO / BlackRock</t>
         </is>
       </c>
-      <c r="E35" s="90" t="n"/>
-      <c r="F35" s="70" t="inlineStr">
+      <c r="E36" s="90" t="n"/>
+      <c r="F36" s="70" t="inlineStr">
         <is>
           <t>Insurance allocation of 144A bond</t>
         </is>
       </c>
-      <c r="G35" s="70" t="inlineStr">
+      <c r="G36" s="70" t="inlineStr">
         <is>
           <t>6.581%</t>
         </is>
       </c>
-      <c r="H35" s="70" t="inlineStr">
+      <c r="H36" s="70" t="inlineStr">
         <is>
           <t>2049</t>
         </is>
       </c>
-      <c r="I35" s="70" t="inlineStr">
+      <c r="I36" s="70" t="inlineStr">
         <is>
           <t>Subset of the $27.3bn Hyperion bond (group 3)</t>
         </is>
       </c>
-      <c r="J35" s="74" t="inlineStr">
+      <c r="J36" s="74" t="inlineStr">
         <is>
           <t>FT; S&amp;P</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="75" t="inlineStr">
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="75" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="B36" s="76" t="inlineStr">
+      <c r="B37" s="76" t="inlineStr">
         <is>
           <t>CoreWeave — DDTL 4.0 insurance anchor</t>
         </is>
       </c>
-      <c r="C36" s="77" t="inlineStr">
+      <c r="C37" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D36" s="75" t="inlineStr">
+      <c r="D37" s="75" t="inlineStr">
         <is>
           <t>Blackstone Credit &amp; Insurance + insurers</t>
         </is>
       </c>
-      <c r="E36" s="91" t="n"/>
-      <c r="F36" s="75" t="inlineStr">
+      <c r="E37" s="91" t="n"/>
+      <c r="F37" s="75" t="inlineStr">
         <is>
           <t>Insurance anchor of GPU-backed loan</t>
         </is>
       </c>
-      <c r="G36" s="75" t="inlineStr">
+      <c r="G37" s="75" t="inlineStr">
         <is>
           <t>SOFR+225 / 5.9%</t>
         </is>
       </c>
-      <c r="H36" s="75" t="inlineStr">
+      <c r="H37" s="75" t="inlineStr">
         <is>
           <t>2032</t>
         </is>
       </c>
-      <c r="I36" s="75" t="inlineStr">
+      <c r="I37" s="75" t="inlineStr">
         <is>
           <t>Subset of the $8.5bn DDTL (group 2)</t>
         </is>
       </c>
-      <c r="J36" s="79" t="inlineStr">
+      <c r="J37" s="79" t="inlineStr">
         <is>
           <t>CoreWeave IR</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="14" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
         <is>
           <t>5) SECURITIZATION / ABS / CMBS</t>
         </is>
       </c>
-      <c r="B37" s="15" t="n"/>
-      <c r="C37" s="15" t="n"/>
-      <c r="D37" s="15" t="n"/>
-      <c r="E37" s="15" t="n"/>
-      <c r="F37" s="15" t="n"/>
-      <c r="G37" s="15" t="n"/>
-      <c r="H37" s="15" t="n"/>
-      <c r="I37" s="15" t="n"/>
-      <c r="J37" s="15" t="n"/>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="80" t="inlineStr">
-        <is>
-          <t>Nov 2025</t>
-        </is>
-      </c>
-      <c r="B38" s="81" t="inlineStr">
-        <is>
-          <t>QTS (Blackstone) — BX 2025-VOLT</t>
-        </is>
-      </c>
-      <c r="C38" s="82" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REIT</t>
-        </is>
-      </c>
-      <c r="D38" s="80" t="inlineStr">
-        <is>
-          <t>Blackstone</t>
-        </is>
-      </c>
-      <c r="E38" s="83" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F38" s="80" t="inlineStr">
-        <is>
-          <t>SASB CMBS (~10 QTS DCs)</t>
-        </is>
-      </c>
-      <c r="G38" s="80" t="inlineStr">
-        <is>
-          <t>floating</t>
-        </is>
-      </c>
-      <c r="H38" s="80" t="inlineStr">
-        <is>
-          <t>2y + ext</t>
-        </is>
-      </c>
-      <c r="I38" s="80" t="inlineStr">
-        <is>
-          <t>Year's largest data-center CMBS</t>
-        </is>
-      </c>
-      <c r="J38" s="84" t="inlineStr">
-        <is>
-          <t>CREFC; SFA</t>
-        </is>
-      </c>
+      <c r="B38" s="15" t="n"/>
+      <c r="C38" s="15" t="n"/>
+      <c r="D38" s="15" t="n"/>
+      <c r="E38" s="15" t="n"/>
+      <c r="F38" s="15" t="n"/>
+      <c r="G38" s="15" t="n"/>
+      <c r="H38" s="15" t="n"/>
+      <c r="I38" s="15" t="n"/>
+      <c r="J38" s="15" t="n"/>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="80" t="inlineStr">
         <is>
-          <t>2024-25</t>
+          <t>Nov 2025</t>
         </is>
       </c>
       <c r="B39" s="81" t="inlineStr">
         <is>
-          <t>Switch (DigitalBridge) — SWCH 2025-DATA</t>
+          <t>QTS (Blackstone) — BX 2025-VOLT</t>
         </is>
       </c>
       <c r="C39" s="82" t="inlineStr">
@@ -9765,7 +9765,7 @@
       </c>
       <c r="D39" s="80" t="inlineStr">
         <is>
-          <t>DigitalBridge</t>
+          <t>Blackstone</t>
         </is>
       </c>
       <c r="E39" s="83" t="n">
@@ -9773,444 +9773,444 @@
       </c>
       <c r="F39" s="80" t="inlineStr">
         <is>
-          <t>$2.4bn SASB CMBS + $1.1bn ABS (green)</t>
+          <t>SASB CMBS (~10 QTS DCs)</t>
         </is>
       </c>
       <c r="G39" s="80" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>floating</t>
         </is>
       </c>
       <c r="H39" s="80" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>2y + ext</t>
         </is>
       </c>
       <c r="I39" s="80" t="inlineStr">
         <is>
-          <t>Green-bond framework</t>
+          <t>Year's largest data-center CMBS</t>
         </is>
       </c>
       <c r="J39" s="84" t="inlineStr">
         <is>
-          <t>SFA; CREFC</t>
+          <t>CREFC; SFA</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="80" t="inlineStr">
         <is>
+          <t>2024-25</t>
+        </is>
+      </c>
+      <c r="B40" s="81" t="inlineStr">
+        <is>
+          <t>Switch (DigitalBridge) — SWCH 2025-DATA</t>
+        </is>
+      </c>
+      <c r="C40" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D40" s="80" t="inlineStr">
+        <is>
+          <t>DigitalBridge</t>
+        </is>
+      </c>
+      <c r="E40" s="83" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F40" s="80" t="inlineStr">
+        <is>
+          <t>$2.4bn SASB CMBS + $1.1bn ABS (green)</t>
+        </is>
+      </c>
+      <c r="G40" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H40" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I40" s="80" t="inlineStr">
+        <is>
+          <t>Green-bond framework</t>
+        </is>
+      </c>
+      <c r="J40" s="84" t="inlineStr">
+        <is>
+          <t>SFA; CREFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="80" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="B40" s="81" t="inlineStr">
+      <c r="B41" s="81" t="inlineStr">
         <is>
           <t>Applied Digital — Polaris Forge HY bond</t>
         </is>
       </c>
-      <c r="C40" s="82" t="inlineStr">
+      <c r="C41" s="82" t="inlineStr">
         <is>
           <t>Colocation / data-center REIT</t>
         </is>
       </c>
-      <c r="D40" s="80" t="inlineStr">
+      <c r="D41" s="80" t="inlineStr">
         <is>
           <t>HY market</t>
         </is>
       </c>
-      <c r="E40" s="83" t="n">
+      <c r="E41" s="83" t="n">
         <v>1.59</v>
       </c>
-      <c r="F40" s="80" t="inlineStr">
+      <c r="F41" s="80" t="inlineStr">
         <is>
           <t>HY / securitized bond (CoreWeave campus)</t>
         </is>
       </c>
-      <c r="G40" s="80" t="inlineStr">
+      <c r="G41" s="80" t="inlineStr">
         <is>
           <t>7%</t>
         </is>
       </c>
-      <c r="H40" s="80" t="inlineStr">
+      <c r="H41" s="80" t="inlineStr">
         <is>
           <t>15y contract</t>
         </is>
       </c>
-      <c r="I40" s="80" t="inlineStr">
+      <c r="I41" s="80" t="inlineStr">
         <is>
           <t>150MW for CoreWeave</t>
         </is>
       </c>
-      <c r="J40" s="84" t="inlineStr">
+      <c r="J41" s="84" t="inlineStr">
         <is>
           <t>TNW</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="14" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
         <is>
           <t>6) CONVERTIBLES / EQUITY-LINKED</t>
         </is>
       </c>
-      <c r="B41" s="15" t="n"/>
-      <c r="C41" s="15" t="n"/>
-      <c r="D41" s="15" t="n"/>
-      <c r="E41" s="15" t="n"/>
-      <c r="F41" s="15" t="n"/>
-      <c r="G41" s="15" t="n"/>
-      <c r="H41" s="15" t="n"/>
-      <c r="I41" s="15" t="n"/>
-      <c r="J41" s="15" t="n"/>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="75" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="B42" s="76" t="inlineStr">
-        <is>
-          <t>Nebius</t>
-        </is>
-      </c>
-      <c r="C42" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D42" s="75" t="inlineStr">
-        <is>
-          <t>Convertible market</t>
-        </is>
-      </c>
-      <c r="E42" s="78" t="n">
-        <v>3</v>
-      </c>
-      <c r="F42" s="75" t="inlineStr">
-        <is>
-          <t>Convertible notes</t>
-        </is>
-      </c>
-      <c r="G42" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H42" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I42" s="75" t="inlineStr">
-        <is>
-          <t>Lighter-balance-sheet strategy</t>
-        </is>
-      </c>
-      <c r="J42" s="79" t="inlineStr">
-        <is>
-          <t>frankk research</t>
-        </is>
-      </c>
+      <c r="B42" s="15" t="n"/>
+      <c r="C42" s="15" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="15" t="n"/>
+      <c r="F42" s="15" t="n"/>
+      <c r="G42" s="15" t="n"/>
+      <c r="H42" s="15" t="n"/>
+      <c r="I42" s="15" t="n"/>
+      <c r="J42" s="15" t="n"/>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="75" t="inlineStr">
         <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B43" s="76" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="C43" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D43" s="75" t="inlineStr">
+        <is>
+          <t>Convertible market</t>
+        </is>
+      </c>
+      <c r="E43" s="78" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" s="75" t="inlineStr">
+        <is>
+          <t>Convertible notes</t>
+        </is>
+      </c>
+      <c r="G43" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H43" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I43" s="75" t="inlineStr">
+        <is>
+          <t>Lighter-balance-sheet strategy</t>
+        </is>
+      </c>
+      <c r="J43" s="79" t="inlineStr">
+        <is>
+          <t>frankk research</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="75" t="inlineStr">
+        <is>
           <t>Dec 2025</t>
         </is>
       </c>
-      <c r="B43" s="76" t="inlineStr">
+      <c r="B44" s="76" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="C43" s="77" t="inlineStr">
+      <c r="C44" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D43" s="75" t="inlineStr">
+      <c r="D44" s="75" t="inlineStr">
         <is>
           <t>Convertible market</t>
         </is>
       </c>
-      <c r="E43" s="78" t="n">
+      <c r="E44" s="78" t="n">
         <v>2.7</v>
       </c>
-      <c r="F43" s="75" t="inlineStr">
+      <c r="F44" s="75" t="inlineStr">
         <is>
           <t>Convertible notes</t>
         </is>
       </c>
-      <c r="G43" s="75" t="inlineStr">
+      <c r="G44" s="75" t="inlineStr">
         <is>
           <t>1.75%</t>
         </is>
       </c>
-      <c r="H43" s="75" t="inlineStr">
+      <c r="H44" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I43" s="75" t="inlineStr">
+      <c r="I44" s="75" t="inlineStr">
         <is>
           <t>Shift toward hybrid instruments</t>
         </is>
       </c>
-      <c r="J43" s="79" t="inlineStr">
+      <c r="J44" s="79" t="inlineStr">
         <is>
           <t>thedig; CoreWeave</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="92" t="n"/>
-      <c r="B44" s="93" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="92" t="n"/>
+      <c r="B45" s="93" t="inlineStr">
         <is>
           <t>TOTAL — itemized debt transactions (bonds + loans + private credit + ABS + converts)</t>
         </is>
       </c>
-      <c r="C44" s="92" t="n"/>
-      <c r="D44" s="92" t="n"/>
-      <c r="E44" s="94">
-        <f>SUM(E6,E7,E8,E9,E10,E11,E13,E14,E15,E16,E17,E19,E20,E21,E22,E23,E24,E25,E26,E27,E28,E29,E30,E31,E38,E39,E40,E42,E43)</f>
-        <v/>
-      </c>
-      <c r="F44" s="92" t="n"/>
-      <c r="G44" s="92" t="n"/>
-      <c r="H44" s="92" t="n"/>
-      <c r="I44" s="92" t="n"/>
-      <c r="J44" s="92" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="14" t="inlineStr">
+      <c r="C45" s="92" t="n"/>
+      <c r="D45" s="92" t="n"/>
+      <c r="E45" s="94">
+        <f>SUM(E6,E7,E8,E9,E10,E11,E12,E14,E15,E16,E17,E18,E20,E21,E22,E23,E24,E25,E26,E27,E28,E29,E30,E31,E32,E39,E40,E41,E43,E44)</f>
+        <v/>
+      </c>
+      <c r="F45" s="92" t="n"/>
+      <c r="G45" s="92" t="n"/>
+      <c r="H45" s="92" t="n"/>
+      <c r="I45" s="92" t="n"/>
+      <c r="J45" s="92" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
         <is>
           <t>7) VENDOR / EQUIPMENT-LEASE FINANCING &amp; BACKSTOPS (memo)</t>
         </is>
       </c>
-      <c r="B46" s="15" t="n"/>
-      <c r="C46" s="15" t="n"/>
-      <c r="D46" s="15" t="n"/>
-      <c r="E46" s="15" t="n"/>
-      <c r="F46" s="15" t="n"/>
-      <c r="G46" s="15" t="n"/>
-      <c r="H46" s="15" t="n"/>
-      <c r="I46" s="15" t="n"/>
-      <c r="J46" s="15" t="n"/>
-    </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="70" t="inlineStr">
-        <is>
-          <t>2024-30</t>
-        </is>
-      </c>
-      <c r="B47" s="71" t="inlineStr">
+      <c r="B47" s="15" t="n"/>
+      <c r="C47" s="15" t="n"/>
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="15" t="n"/>
+      <c r="F47" s="15" t="n"/>
+      <c r="G47" s="15" t="n"/>
+      <c r="H47" s="15" t="n"/>
+      <c r="I47" s="15" t="n"/>
+      <c r="J47" s="15" t="n"/>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="70" t="inlineStr">
+        <is>
+          <t>2024-31</t>
+        </is>
+      </c>
+      <c r="B48" s="71" t="inlineStr">
         <is>
           <t>Microsoft — finance-lease commitments</t>
         </is>
       </c>
-      <c r="C47" s="72" t="inlineStr">
+      <c r="C48" s="72" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="D47" s="70" t="inlineStr">
+      <c r="D48" s="70" t="inlineStr">
         <is>
           <t>Lessors / developers</t>
         </is>
       </c>
-      <c r="E47" s="73" t="n">
+      <c r="E48" s="73" t="n">
+        <v>196.6</v>
+      </c>
+      <c r="F48" s="70" t="inlineStr">
+        <is>
+          <t>Finance leases not yet commenced (as of 31 Mar 2026)</t>
+        </is>
+      </c>
+      <c r="G48" s="70" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H48" s="70" t="inlineStr">
+        <is>
+          <t>to 21y</t>
+        </is>
+      </c>
+      <c r="I48" s="70" t="inlineStr">
+        <is>
+          <t>Off-B/S; commence FY26-FY31; Microsoft funds AI via leases not new bonds</t>
+        </is>
+      </c>
+      <c r="J48" s="74" t="inlineStr">
+        <is>
+          <t>MSFT 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="75" t="inlineStr">
+        <is>
+          <t>through 2032</t>
+        </is>
+      </c>
+      <c r="B49" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — NVIDIA capacity backstop</t>
+        </is>
+      </c>
+      <c r="C49" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D49" s="75" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="E49" s="78" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="F49" s="75" t="inlineStr">
+        <is>
+          <t>Vendor backstop of unsold capacity</t>
+        </is>
+      </c>
+      <c r="G49" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H49" s="75" t="inlineStr">
+        <is>
+          <t>to 2032</t>
+        </is>
+      </c>
+      <c r="I49" s="75" t="inlineStr">
+        <is>
+          <t>De-risks CoreWeave</t>
+        </is>
+      </c>
+      <c r="J49" s="79" t="inlineStr">
+        <is>
+          <t>theaiinsider</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>8) EQUITY &amp; SOVEREIGN COMMITMENTS (memo — not debt)</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="n"/>
+      <c r="C50" s="15" t="n"/>
+      <c r="D50" s="15" t="n"/>
+      <c r="E50" s="15" t="n"/>
+      <c r="F50" s="15" t="n"/>
+      <c r="G50" s="15" t="n"/>
+      <c r="H50" s="15" t="n"/>
+      <c r="I50" s="15" t="n"/>
+      <c r="J50" s="15" t="n"/>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="70" t="inlineStr">
+        <is>
+          <t>2024-25</t>
+        </is>
+      </c>
+      <c r="B51" s="71" t="inlineStr">
+        <is>
+          <t>Microsoft — AI Infrastructure Partnership (AIP)</t>
+        </is>
+      </c>
+      <c r="C51" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D51" s="70" t="inlineStr">
+        <is>
+          <t>Microsoft, BlackRock/GIP, MGX (+ NVIDIA)</t>
+        </is>
+      </c>
+      <c r="E51" s="73" t="n">
         <v>100</v>
       </c>
-      <c r="F47" s="70" t="inlineStr">
-        <is>
-          <t>Finance leases (uncommenced ~$108bn at 9/30/24)</t>
-        </is>
-      </c>
-      <c r="G47" s="70" t="inlineStr">
+      <c r="F51" s="70" t="inlineStr">
+        <is>
+          <t>Co-investment fund (equity sponsor)</t>
+        </is>
+      </c>
+      <c r="G51" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H47" s="70" t="inlineStr">
-        <is>
-          <t>to 20y</t>
-        </is>
-      </c>
-      <c r="I47" s="70" t="inlineStr">
-        <is>
-          <t>Off-B/S; commence FY25-FY30</t>
-        </is>
-      </c>
-      <c r="J47" s="74" t="inlineStr">
-        <is>
-          <t>MSFT 10-Q; CNBC</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="75" t="inlineStr">
-        <is>
-          <t>through 2032</t>
-        </is>
-      </c>
-      <c r="B48" s="76" t="inlineStr">
-        <is>
-          <t>CoreWeave — NVIDIA capacity backstop</t>
-        </is>
-      </c>
-      <c r="C48" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D48" s="75" t="inlineStr">
-        <is>
-          <t>NVIDIA</t>
-        </is>
-      </c>
-      <c r="E48" s="78" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="F48" s="75" t="inlineStr">
-        <is>
-          <t>Vendor backstop of unsold capacity</t>
-        </is>
-      </c>
-      <c r="G48" s="75" t="inlineStr">
+      <c r="H51" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H48" s="75" t="inlineStr">
-        <is>
-          <t>to 2032</t>
-        </is>
-      </c>
-      <c r="I48" s="75" t="inlineStr">
-        <is>
-          <t>De-risks CoreWeave</t>
-        </is>
-      </c>
-      <c r="J48" s="79" t="inlineStr">
-        <is>
-          <t>theaiinsider</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="14" t="inlineStr">
-        <is>
-          <t>8) EQUITY &amp; SOVEREIGN COMMITMENTS (memo — not debt)</t>
-        </is>
-      </c>
-      <c r="B49" s="15" t="n"/>
-      <c r="C49" s="15" t="n"/>
-      <c r="D49" s="15" t="n"/>
-      <c r="E49" s="15" t="n"/>
-      <c r="F49" s="15" t="n"/>
-      <c r="G49" s="15" t="n"/>
-      <c r="H49" s="15" t="n"/>
-      <c r="I49" s="15" t="n"/>
-      <c r="J49" s="15" t="n"/>
-    </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="95" t="inlineStr">
-        <is>
-          <t>2025-30</t>
-        </is>
-      </c>
-      <c r="B50" s="96" t="inlineStr">
-        <is>
-          <t>HUMAIN (Saudi PIF)</t>
-        </is>
-      </c>
-      <c r="C50" s="97" t="inlineStr">
-        <is>
-          <t>Sovereign cloud</t>
-        </is>
-      </c>
-      <c r="D50" s="95" t="inlineStr">
-        <is>
-          <t>Public Investment Fund</t>
-        </is>
-      </c>
-      <c r="E50" s="98" t="n">
-        <v>100</v>
-      </c>
-      <c r="F50" s="95" t="inlineStr">
-        <is>
-          <t>Sovereign equity</t>
-        </is>
-      </c>
-      <c r="G50" s="95" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H50" s="95" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I50" s="95" t="inlineStr">
-        <is>
-          <t>11 DCs / 2.2GW; ~600k GPUs</t>
-        </is>
-      </c>
-      <c r="J50" s="99" t="inlineStr">
-        <is>
-          <t>Presenc AI; NYU DRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="95" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="B51" s="96" t="inlineStr">
-        <is>
-          <t>MGX / Mubadala (UAE)</t>
-        </is>
-      </c>
-      <c r="C51" s="97" t="inlineStr">
-        <is>
-          <t>Sovereign cloud</t>
-        </is>
-      </c>
-      <c r="D51" s="95" t="inlineStr">
-        <is>
-          <t>Mubadala / MGX</t>
-        </is>
-      </c>
-      <c r="E51" s="98" t="n">
-        <v>40</v>
-      </c>
-      <c r="F51" s="95" t="inlineStr">
-        <is>
-          <t>Sovereign equity / infra</t>
-        </is>
-      </c>
-      <c r="G51" s="95" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H51" s="95" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I51" s="95" t="inlineStr">
-        <is>
-          <t>Anchored Stargate; co-bought Aligned</t>
-        </is>
-      </c>
-      <c r="J51" s="99" t="inlineStr">
-        <is>
-          <t>NYU DRI</t>
+      <c r="I51" s="70" t="inlineStr">
+        <is>
+          <t>Up to $100bn incl. debt; first deployment $40bn Aligned (Oct 2025); Microsoft offtake underwrites it</t>
+        </is>
+      </c>
+      <c r="J51" s="74" t="inlineStr">
+        <is>
+          <t>FT; chiragvadhia</t>
         </is>
       </c>
     </row>
@@ -10222,7 +10222,7 @@
       </c>
       <c r="B52" s="96" t="inlineStr">
         <is>
-          <t>Stargate UAE / G42 / Khazna</t>
+          <t>HUMAIN (Saudi PIF)</t>
         </is>
       </c>
       <c r="C52" s="97" t="inlineStr">
@@ -10232,15 +10232,15 @@
       </c>
       <c r="D52" s="95" t="inlineStr">
         <is>
-          <t>Mubadala, MGX, Microsoft, G42</t>
+          <t>Public Investment Fund</t>
         </is>
       </c>
       <c r="E52" s="98" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="F52" s="95" t="inlineStr">
         <is>
-          <t>Sovereign equity + JV</t>
+          <t>Sovereign equity</t>
         </is>
       </c>
       <c r="G52" s="95" t="inlineStr">
@@ -10255,290 +10255,290 @@
       </c>
       <c r="I52" s="95" t="inlineStr">
         <is>
-          <t>5GW Abu Dhabi campus</t>
+          <t>11 DCs / 2.2GW; ~600k GPUs</t>
         </is>
       </c>
       <c r="J52" s="99" t="inlineStr">
         <is>
-          <t>Khaleej Times; dcpulse</t>
+          <t>Presenc AI; NYU DRI</t>
         </is>
       </c>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="95" t="inlineStr">
         <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B53" s="96" t="inlineStr">
+        <is>
+          <t>MGX / Mubadala (UAE)</t>
+        </is>
+      </c>
+      <c r="C53" s="97" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="D53" s="95" t="inlineStr">
+        <is>
+          <t>Mubadala / MGX</t>
+        </is>
+      </c>
+      <c r="E53" s="98" t="n">
+        <v>40</v>
+      </c>
+      <c r="F53" s="95" t="inlineStr">
+        <is>
+          <t>Sovereign equity / infra</t>
+        </is>
+      </c>
+      <c r="G53" s="95" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H53" s="95" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I53" s="95" t="inlineStr">
+        <is>
+          <t>Anchored Stargate; co-bought Aligned</t>
+        </is>
+      </c>
+      <c r="J53" s="99" t="inlineStr">
+        <is>
+          <t>NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="95" t="inlineStr">
+        <is>
+          <t>2025-30</t>
+        </is>
+      </c>
+      <c r="B54" s="96" t="inlineStr">
+        <is>
+          <t>Stargate UAE / G42 / Khazna</t>
+        </is>
+      </c>
+      <c r="C54" s="97" t="inlineStr">
+        <is>
+          <t>Sovereign cloud</t>
+        </is>
+      </c>
+      <c r="D54" s="95" t="inlineStr">
+        <is>
+          <t>Mubadala, MGX, Microsoft, G42</t>
+        </is>
+      </c>
+      <c r="E54" s="98" t="n">
+        <v>30</v>
+      </c>
+      <c r="F54" s="95" t="inlineStr">
+        <is>
+          <t>Sovereign equity + JV</t>
+        </is>
+      </c>
+      <c r="G54" s="95" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H54" s="95" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I54" s="95" t="inlineStr">
+        <is>
+          <t>5GW Abu Dhabi campus</t>
+        </is>
+      </c>
+      <c r="J54" s="99" t="inlineStr">
+        <is>
+          <t>Khaleej Times; dcpulse</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="95" t="inlineStr">
+        <is>
           <t>Late 2025</t>
         </is>
       </c>
-      <c r="B53" s="96" t="inlineStr">
+      <c r="B55" s="96" t="inlineStr">
         <is>
           <t>Qatar (QIA / Qai) + Brookfield</t>
         </is>
       </c>
-      <c r="C53" s="97" t="inlineStr">
+      <c r="C55" s="97" t="inlineStr">
         <is>
           <t>Sovereign cloud</t>
         </is>
       </c>
-      <c r="D53" s="95" t="inlineStr">
+      <c r="D55" s="95" t="inlineStr">
         <is>
           <t>QIA / Qai, Brookfield</t>
         </is>
       </c>
-      <c r="E53" s="98" t="n">
+      <c r="E55" s="98" t="n">
         <v>20</v>
       </c>
-      <c r="F53" s="95" t="inlineStr">
+      <c r="F55" s="95" t="inlineStr">
         <is>
           <t>JV / infra</t>
         </is>
       </c>
-      <c r="G53" s="95" t="inlineStr">
+      <c r="G55" s="95" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H53" s="95" t="inlineStr">
+      <c r="H55" s="95" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I53" s="95" t="inlineStr">
+      <c r="I55" s="95" t="inlineStr">
         <is>
           <t>AI-infrastructure JV</t>
         </is>
       </c>
-      <c r="J53" s="99" t="inlineStr">
+      <c r="J55" s="99" t="inlineStr">
         <is>
           <t>NYU DRI</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="75" t="inlineStr">
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="75" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B54" s="76" t="inlineStr">
+      <c r="B56" s="76" t="inlineStr">
         <is>
           <t>SpaceX / xAI — $10bn raise</t>
         </is>
       </c>
-      <c r="C54" s="77" t="inlineStr">
+      <c r="C56" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D54" s="75" t="inlineStr">
+      <c r="D56" s="75" t="inlineStr">
         <is>
           <t>Morgan Stanley</t>
         </is>
       </c>
-      <c r="E54" s="78" t="n">
+      <c r="E56" s="78" t="n">
         <v>10</v>
       </c>
-      <c r="F54" s="75" t="inlineStr">
+      <c r="F56" s="75" t="inlineStr">
         <is>
           <t>$5bn debt + $5bn equity</t>
         </is>
       </c>
-      <c r="G54" s="75" t="inlineStr">
+      <c r="G56" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H54" s="75" t="inlineStr">
+      <c r="H56" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I54" s="75" t="inlineStr">
+      <c r="I56" s="75" t="inlineStr">
         <is>
           <t>Debt portion also in group 3</t>
         </is>
       </c>
-      <c r="J54" s="79" t="inlineStr">
+      <c r="J56" s="79" t="inlineStr">
         <is>
           <t>CNBC</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="75" t="inlineStr">
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="75" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="B55" s="76" t="inlineStr">
+      <c r="B57" s="76" t="inlineStr">
         <is>
           <t>CoreWeave — equity</t>
         </is>
       </c>
-      <c r="C55" s="77" t="inlineStr">
+      <c r="C57" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D55" s="75" t="inlineStr">
+      <c r="D57" s="75" t="inlineStr">
         <is>
           <t>NVIDIA; IPO</t>
         </is>
       </c>
-      <c r="E55" s="78" t="n">
+      <c r="E57" s="78" t="n">
         <v>3.5</v>
       </c>
-      <c r="F55" s="75" t="inlineStr">
+      <c r="F57" s="75" t="inlineStr">
         <is>
           <t>IPO ($1.5bn) + NVIDIA strategic ($2bn)</t>
         </is>
       </c>
-      <c r="G55" s="75" t="inlineStr">
+      <c r="G57" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H55" s="75" t="inlineStr">
+      <c r="H57" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I55" s="75" t="inlineStr">
+      <c r="I57" s="75" t="inlineStr">
         <is>
           <t>Equity (not debt)</t>
         </is>
       </c>
-      <c r="J55" s="79" t="inlineStr">
+      <c r="J57" s="79" t="inlineStr">
         <is>
           <t>CNBC; CoreWeave</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="14" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
         <is>
           <t>9) CONTEXT / FRAMEWORKS / PROJECTIONS (memo)</t>
         </is>
       </c>
-      <c r="B56" s="15" t="n"/>
-      <c r="C56" s="15" t="n"/>
-      <c r="D56" s="15" t="n"/>
-      <c r="E56" s="15" t="n"/>
-      <c r="F56" s="15" t="n"/>
-      <c r="G56" s="15" t="n"/>
-      <c r="H56" s="15" t="n"/>
-      <c r="I56" s="15" t="n"/>
-      <c r="J56" s="15" t="n"/>
-    </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="85" t="inlineStr">
-        <is>
-          <t>2025-28</t>
-        </is>
-      </c>
-      <c r="B57" s="86" t="inlineStr">
-        <is>
-          <t>Market — private credit for AI data centers</t>
-        </is>
-      </c>
-      <c r="C57" s="87" t="inlineStr">
-        <is>
-          <t>Context / market</t>
-        </is>
-      </c>
-      <c r="D57" s="85" t="inlineStr">
-        <is>
-          <t>Industry-wide</t>
-        </is>
-      </c>
-      <c r="E57" s="88" t="n">
-        <v>800</v>
-      </c>
-      <c r="F57" s="85" t="inlineStr">
-        <is>
-          <t>Projection</t>
-        </is>
-      </c>
-      <c r="G57" s="85" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H57" s="85" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I57" s="85" t="inlineStr">
-        <is>
-          <t>&gt;$200bn already outstanding</t>
-        </is>
-      </c>
-      <c r="J57" s="89" t="inlineStr">
-        <is>
-          <t>Morgan Stanley; Quinn Emanuel</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="85" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B58" s="86" t="inlineStr">
-        <is>
-          <t>Insurance-linked platforms — private credit</t>
-        </is>
-      </c>
-      <c r="C58" s="87" t="inlineStr">
-        <is>
-          <t>Context / market</t>
-        </is>
-      </c>
-      <c r="D58" s="85" t="inlineStr">
-        <is>
-          <t>Athene, Global Atlantic, etc.</t>
-        </is>
-      </c>
-      <c r="E58" s="88" t="n">
-        <v>180</v>
-      </c>
-      <c r="F58" s="85" t="inlineStr">
-        <is>
-          <t>Insurance capital into private credit</t>
-        </is>
-      </c>
-      <c r="G58" s="85" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H58" s="85" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I58" s="85" t="inlineStr">
-        <is>
-          <t>~25% of global private credit AUM</t>
-        </is>
-      </c>
-      <c r="J58" s="89" t="inlineStr">
-        <is>
-          <t>McKinsey; ABF Journal</t>
-        </is>
-      </c>
+      <c r="B58" s="15" t="n"/>
+      <c r="C58" s="15" t="n"/>
+      <c r="D58" s="15" t="n"/>
+      <c r="E58" s="15" t="n"/>
+      <c r="F58" s="15" t="n"/>
+      <c r="G58" s="15" t="n"/>
+      <c r="H58" s="15" t="n"/>
+      <c r="I58" s="15" t="n"/>
+      <c r="J58" s="15" t="n"/>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="85" t="inlineStr">
         <is>
-          <t>2026-28</t>
+          <t>2025-28</t>
         </is>
       </c>
       <c r="B59" s="86" t="inlineStr">
         <is>
-          <t>Colocation — DC securitization supply</t>
+          <t>Market — private credit for AI data centers</t>
         </is>
       </c>
       <c r="C59" s="87" t="inlineStr">
@@ -10552,11 +10552,11 @@
         </is>
       </c>
       <c r="E59" s="88" t="n">
-        <v>130</v>
+        <v>800</v>
       </c>
       <c r="F59" s="85" t="inlineStr">
         <is>
-          <t>ABS + CMBS net issuance</t>
+          <t>Projection</t>
         </is>
       </c>
       <c r="G59" s="85" t="inlineStr">
@@ -10571,24 +10571,24 @@
       </c>
       <c r="I59" s="85" t="inlineStr">
         <is>
-          <t>Morgan Stanley estimate</t>
+          <t>&gt;$200bn already outstanding</t>
         </is>
       </c>
       <c r="J59" s="89" t="inlineStr">
         <is>
-          <t>CREFC; Impax</t>
+          <t>Morgan Stanley; Quinn Emanuel</t>
         </is>
       </c>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="85" t="inlineStr">
         <is>
-          <t>to 2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="B60" s="86" t="inlineStr">
         <is>
-          <t>Sector — HY/unrated AI-infra debt</t>
+          <t>Insurance-linked platforms — private credit</t>
         </is>
       </c>
       <c r="C60" s="87" t="inlineStr">
@@ -10598,15 +10598,15 @@
       </c>
       <c r="D60" s="85" t="inlineStr">
         <is>
-          <t>Multiple</t>
+          <t>Athene, Global Atlantic, etc.</t>
         </is>
       </c>
       <c r="E60" s="88" t="n">
-        <v>107</v>
+        <v>180</v>
       </c>
       <c r="F60" s="85" t="inlineStr">
         <is>
-          <t>Funded + committed debt</t>
+          <t>Insurance capital into private credit</t>
         </is>
       </c>
       <c r="G60" s="85" t="inlineStr">
@@ -10621,24 +10621,24 @@
       </c>
       <c r="I60" s="85" t="inlineStr">
         <is>
-          <t>$68.7bn neoclouds / $38.7bn AI-native DCs</t>
+          <t>~25% of global private credit AUM</t>
         </is>
       </c>
       <c r="J60" s="89" t="inlineStr">
         <is>
-          <t>Octus</t>
+          <t>McKinsey; ABF Journal</t>
         </is>
       </c>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="85" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026-28</t>
         </is>
       </c>
       <c r="B61" s="86" t="inlineStr">
         <is>
-          <t>KKR + Energy Capital Partners — partnership</t>
+          <t>Colocation — DC securitization supply</t>
         </is>
       </c>
       <c r="C61" s="87" t="inlineStr">
@@ -10648,15 +10648,15 @@
       </c>
       <c r="D61" s="85" t="inlineStr">
         <is>
-          <t>KKR, ECP</t>
+          <t>Industry-wide</t>
         </is>
       </c>
       <c r="E61" s="88" t="n">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="F61" s="85" t="inlineStr">
         <is>
-          <t>Strategic partnership</t>
+          <t>ABS + CMBS net issuance</t>
         </is>
       </c>
       <c r="G61" s="85" t="inlineStr">
@@ -10671,121 +10671,221 @@
       </c>
       <c r="I61" s="85" t="inlineStr">
         <is>
-          <t>Accelerate AI infrastructure</t>
+          <t>Morgan Stanley estimate</t>
         </is>
       </c>
       <c r="J61" s="89" t="inlineStr">
         <is>
-          <t>Business Times</t>
+          <t>CREFC; Impax</t>
         </is>
       </c>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="85" t="inlineStr">
         <is>
+          <t>to 2026</t>
+        </is>
+      </c>
+      <c r="B62" s="86" t="inlineStr">
+        <is>
+          <t>Sector — HY/unrated AI-infra debt</t>
+        </is>
+      </c>
+      <c r="C62" s="87" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D62" s="85" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="E62" s="88" t="n">
+        <v>107</v>
+      </c>
+      <c r="F62" s="85" t="inlineStr">
+        <is>
+          <t>Funded + committed debt</t>
+        </is>
+      </c>
+      <c r="G62" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H62" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I62" s="85" t="inlineStr">
+        <is>
+          <t>$68.7bn neoclouds / $38.7bn AI-native DCs</t>
+        </is>
+      </c>
+      <c r="J62" s="89" t="inlineStr">
+        <is>
+          <t>Octus</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="85" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="B63" s="86" t="inlineStr">
+        <is>
+          <t>KKR + Energy Capital Partners — partnership</t>
+        </is>
+      </c>
+      <c r="C63" s="87" t="inlineStr">
+        <is>
+          <t>Context / market</t>
+        </is>
+      </c>
+      <c r="D63" s="85" t="inlineStr">
+        <is>
+          <t>KKR, ECP</t>
+        </is>
+      </c>
+      <c r="E63" s="88" t="n">
+        <v>50</v>
+      </c>
+      <c r="F63" s="85" t="inlineStr">
+        <is>
+          <t>Strategic partnership</t>
+        </is>
+      </c>
+      <c r="G63" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H63" s="85" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I63" s="85" t="inlineStr">
+        <is>
+          <t>Accelerate AI infrastructure</t>
+        </is>
+      </c>
+      <c r="J63" s="89" t="inlineStr">
+        <is>
+          <t>Business Times</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="30" customHeight="1">
+      <c r="A64" s="85" t="inlineStr">
+        <is>
           <t>2025-28</t>
         </is>
       </c>
-      <c r="B62" s="86" t="inlineStr">
+      <c r="B64" s="86" t="inlineStr">
         <is>
           <t>Broadcom + Apollo + Blackstone — platform</t>
         </is>
       </c>
-      <c r="C62" s="87" t="inlineStr">
+      <c r="C64" s="87" t="inlineStr">
         <is>
           <t>Context / market</t>
         </is>
       </c>
-      <c r="D62" s="85" t="inlineStr">
+      <c r="D64" s="85" t="inlineStr">
         <is>
           <t>Apollo, Blackstone, Broadcom</t>
         </is>
       </c>
-      <c r="E62" s="100" t="n"/>
-      <c r="F62" s="85" t="inlineStr">
+      <c r="E64" s="100" t="n"/>
+      <c r="F64" s="85" t="inlineStr">
         <is>
           <t>Platform framework</t>
         </is>
       </c>
-      <c r="G62" s="85" t="inlineStr">
+      <c r="G64" s="85" t="inlineStr">
         <is>
           <t>&gt;20 GW</t>
         </is>
       </c>
-      <c r="H62" s="85" t="inlineStr">
+      <c r="H64" s="85" t="inlineStr">
         <is>
           <t>to 2028</t>
         </is>
       </c>
-      <c r="I62" s="85" t="inlineStr">
+      <c r="I64" s="85" t="inlineStr">
         <is>
           <t>Deploy &gt;20GW compute</t>
         </is>
       </c>
-      <c r="J62" s="89" t="inlineStr">
+      <c r="J64" s="89" t="inlineStr">
         <is>
           <t>privatedebtnews</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="101" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="101" t="inlineStr">
         <is>
           <t>Selected sources:</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="102" t="inlineStr">
-        <is>
-          <t>Goldman Sachs Research — ~$5.3tn AI + data-center capex 2025-2030; private markets in DC financing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="102" t="inlineStr">
-        <is>
-          <t>Morgan Stanley — ~$2tn capex 2025-28 with &gt;$1tn debt; ~$800bn private credit for AI DCs.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="102" t="inlineStr">
         <is>
-          <t>Bank of America / BofA Securities — hyperscaler bond issuance ($121bn 2025; ~$175bn 2026E).</t>
+          <t>Goldman Sachs Research — ~$5.3tn AI + data-center capex 2025-2030; private markets in DC financing.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="102" t="inlineStr">
         <is>
-          <t>Moody's Ratings — hyperscaler capex (~$785bn 2026, ~$1tn 2027); $662bn off-B/S DC leases.</t>
+          <t>Morgan Stanley — ~$2tn capex 2025-28 with &gt;$1tn debt; ~$800bn private credit for AI DCs.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="102" t="inlineStr">
         <is>
-          <t>McKinsey — ~$2.7tn US (5.2tn global) data-center capex by 2030; insurance-linked private credit.</t>
+          <t>Bank of America / BofA Securities — hyperscaler bond issuance ($121bn 2025; ~$175bn 2026E).</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="102" t="inlineStr">
         <is>
-          <t>Octus — HY/unrated AI-infra debt (~$107bn to ~May 2026); ~14GW unfunded ≈ $344bn need.</t>
+          <t>Moody's Ratings — hyperscaler capex (~$785bn 2026, ~$1tn 2027); $662bn off-B/S DC leases.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="102" t="inlineStr">
         <is>
-          <t>Company / press: Meta IR, FT, S&amp;P, IFR (Hyperion); Oracle IR, IFR, Reuters; CoreWeave IR; Blackstone;</t>
+          <t>McKinsey — ~$2.7tn US (5.2tn global) data-center capex by 2030; insurance-linked private credit.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="102" t="inlineStr">
+        <is>
+          <t>Octus — HY/unrated AI-infra debt (~$107bn to ~May 2026); ~14GW unfunded ≈ $344bn need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="102" t="inlineStr">
+        <is>
+          <t>Company / press: Meta IR, FT, S&amp;P, IFR (Hyperion); Oracle IR, IFR, Reuters; CoreWeave IR; Blackstone;</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="102" t="inlineStr">
         <is>
           <t xml:space="preserve">  Apollo Academy; privatedebtnews; Bisnow; Quinn Emanuel; Build.inc; CNBC / WSJ / The Information (xAI).</t>
         </is>

</xml_diff>

<commit_message>
Merge Seaport Global AI data-center bond transactions into Deals tab (categorized by instrument)
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/AI_Infrastructure_Financing_2025-2030.xlsx
+++ b/AI_Infrastructure_Financing_2025-2030.xlsx
@@ -8146,7 +8146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:J97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8587,31 +8587,65 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>2) BANK &amp; SYNDICATED LOANS (incl. GPU-backed term loans)</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="n"/>
-      <c r="C13" s="15" t="n"/>
-      <c r="D13" s="15" t="n"/>
-      <c r="E13" s="15" t="n"/>
-      <c r="F13" s="15" t="n"/>
-      <c r="G13" s="15" t="n"/>
-      <c r="H13" s="15" t="n"/>
-      <c r="I13" s="15" t="n"/>
-      <c r="J13" s="15" t="n"/>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="75" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B13" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave (CRWV)</t>
+        </is>
+      </c>
+      <c r="C13" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D13" s="75" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E13" s="78" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="F13" s="75" t="inlineStr">
+        <is>
+          <t>Senior unsecured HY bond</t>
+        </is>
+      </c>
+      <c r="G13" s="75" t="inlineStr">
+        <is>
+          <t>9.75% cpn; YTW 9.3%; +507</t>
+        </is>
+      </c>
+      <c r="H13" s="75" t="inlineStr">
+        <is>
+          <t>Oct 2031</t>
+        </is>
+      </c>
+      <c r="I13" s="75" t="inlineStr">
+        <is>
+          <t>GCP; B1/B/BB-</t>
+        </is>
+      </c>
+      <c r="J13" s="79" t="inlineStr">
+        <is>
+          <t>Seaport (6/12/26)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="75" t="inlineStr">
         <is>
-          <t>Mar 2026</t>
+          <t>o/s Jun'26</t>
         </is>
       </c>
       <c r="B14" s="76" t="inlineStr">
         <is>
-          <t>CoreWeave — DDTL 4.0</t>
+          <t>CoreWeave (CRWV)</t>
         </is>
       </c>
       <c r="C14" s="77" t="inlineStr">
@@ -8621,97 +8655,97 @@
       </c>
       <c r="D14" s="75" t="inlineStr">
         <is>
-          <t>Blackstone Credit &amp; Insurance (anchor); MUFG, MS, GS, JPM</t>
+          <t>144A bond investors</t>
         </is>
       </c>
       <c r="E14" s="78" t="n">
-        <v>8.5</v>
+        <v>2</v>
       </c>
       <c r="F14" s="75" t="inlineStr">
         <is>
-          <t>GPU-backed delayed-draw term loan</t>
+          <t>Senior unsecured HY bond</t>
         </is>
       </c>
       <c r="G14" s="75" t="inlineStr">
         <is>
-          <t>SOFR+225 / ~5.9%</t>
+          <t>9.25% cpn; YTW 8.6%; +444</t>
         </is>
       </c>
       <c r="H14" s="75" t="inlineStr">
         <is>
-          <t>Mar 2032</t>
+          <t>Jun 2030</t>
         </is>
       </c>
       <c r="I14" s="75" t="inlineStr">
         <is>
-          <t>First IG-rated (A3 / A low) HPC loan; non-recourse</t>
+          <t>GCP; B1/B/BB-</t>
         </is>
       </c>
       <c r="J14" s="79" t="inlineStr">
         <is>
-          <t>CoreWeave IR</t>
+          <t>Seaport (6/12/26)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="80" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B15" s="81" t="inlineStr">
-        <is>
-          <t>Applied Digital</t>
-        </is>
-      </c>
-      <c r="C15" s="82" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REIT</t>
-        </is>
-      </c>
-      <c r="D15" s="80" t="inlineStr">
-        <is>
-          <t>Macquarie</t>
-        </is>
-      </c>
-      <c r="E15" s="83" t="n">
-        <v>5</v>
-      </c>
-      <c r="F15" s="80" t="inlineStr">
-        <is>
-          <t>Structured HPC financing</t>
-        </is>
-      </c>
-      <c r="G15" s="80" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H15" s="80" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I15" s="80" t="inlineStr">
-        <is>
-          <t>Powered-shell build for CoreWeave</t>
-        </is>
-      </c>
-      <c r="J15" s="84" t="inlineStr">
-        <is>
-          <t>press</t>
+      <c r="A15" s="75" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B15" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave (CRWV)</t>
+        </is>
+      </c>
+      <c r="C15" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D15" s="75" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E15" s="78" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F15" s="75" t="inlineStr">
+        <is>
+          <t>Senior unsecured HY bond</t>
+        </is>
+      </c>
+      <c r="G15" s="75" t="inlineStr">
+        <is>
+          <t>9.00% cpn; YTW 9.0%; +478</t>
+        </is>
+      </c>
+      <c r="H15" s="75" t="inlineStr">
+        <is>
+          <t>Feb 2031</t>
+        </is>
+      </c>
+      <c r="I15" s="75" t="inlineStr">
+        <is>
+          <t>GCP; B1/B/BB-</t>
+        </is>
+      </c>
+      <c r="J15" s="79" t="inlineStr">
+        <is>
+          <t>Seaport (6/12/26)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="75" t="inlineStr">
         <is>
-          <t>May 2025</t>
+          <t>o/s Jun'26</t>
         </is>
       </c>
       <c r="B16" s="76" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>CoreWeave (CRWV)</t>
         </is>
       </c>
       <c r="C16" s="77" t="inlineStr">
@@ -8721,97 +8755,63 @@
       </c>
       <c r="D16" s="75" t="inlineStr">
         <is>
-          <t>Bank syndicate</t>
+          <t>144A bond investors</t>
         </is>
       </c>
       <c r="E16" s="78" t="n">
-        <v>2.5</v>
+        <v>1.25</v>
       </c>
       <c r="F16" s="75" t="inlineStr">
         <is>
-          <t>Revolving credit line</t>
+          <t>Senior unsecured HY bond</t>
         </is>
       </c>
       <c r="G16" s="75" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>9.625% cpn; YTW 9.5%; +531</t>
         </is>
       </c>
       <c r="H16" s="75" t="inlineStr">
         <is>
-          <t>5y</t>
+          <t>Jul 2032</t>
         </is>
       </c>
       <c r="I16" s="75" t="inlineStr">
         <is>
-          <t>Liquidity backstop</t>
+          <t>GCP; B1/B/BB-</t>
         </is>
       </c>
       <c r="J16" s="79" t="inlineStr">
         <is>
-          <t>CNBC</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="75" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B17" s="76" t="inlineStr">
-        <is>
-          <t>Nscale</t>
-        </is>
-      </c>
-      <c r="C17" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D17" s="75" t="inlineStr">
-        <is>
-          <t>Private credit / banks</t>
-        </is>
-      </c>
-      <c r="E17" s="78" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="F17" s="75" t="inlineStr">
-        <is>
-          <t>Term loan</t>
-        </is>
-      </c>
-      <c r="G17" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H17" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I17" s="75" t="inlineStr">
-        <is>
-          <t>GPU-cloud build</t>
-        </is>
-      </c>
-      <c r="J17" s="79" t="inlineStr">
-        <is>
-          <t>theaiinsider</t>
-        </is>
-      </c>
+          <t>Seaport (6/12/26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>2) BANK &amp; SYNDICATED LOANS (incl. GPU-backed term loans)</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="n"/>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="n"/>
+      <c r="G17" s="15" t="n"/>
+      <c r="H17" s="15" t="n"/>
+      <c r="I17" s="15" t="n"/>
+      <c r="J17" s="15" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="75" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Mar 2026</t>
         </is>
       </c>
       <c r="B18" s="76" t="inlineStr">
         <is>
-          <t>Lambda</t>
+          <t>CoreWeave — DDTL 4.0</t>
         </is>
       </c>
       <c r="C18" s="77" t="inlineStr">
@@ -8821,101 +8821,135 @@
       </c>
       <c r="D18" s="75" t="inlineStr">
         <is>
+          <t>Blackstone Credit &amp; Insurance (anchor); MUFG, MS, GS, JPM</t>
+        </is>
+      </c>
+      <c r="E18" s="78" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="F18" s="75" t="inlineStr">
+        <is>
+          <t>GPU-backed delayed-draw term loan</t>
+        </is>
+      </c>
+      <c r="G18" s="75" t="inlineStr">
+        <is>
+          <t>SOFR+225 / ~5.9%</t>
+        </is>
+      </c>
+      <c r="H18" s="75" t="inlineStr">
+        <is>
+          <t>Mar 2032</t>
+        </is>
+      </c>
+      <c r="I18" s="75" t="inlineStr">
+        <is>
+          <t>First IG-rated (A3 / A low) HPC loan; non-recourse</t>
+        </is>
+      </c>
+      <c r="J18" s="79" t="inlineStr">
+        <is>
+          <t>CoreWeave IR</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="80" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="B19" s="81" t="inlineStr">
+        <is>
+          <t>Applied Digital</t>
+        </is>
+      </c>
+      <c r="C19" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D19" s="80" t="inlineStr">
+        <is>
           <t>Macquarie</t>
         </is>
       </c>
-      <c r="E18" s="78" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F18" s="75" t="inlineStr">
-        <is>
-          <t>GPU-backed facility</t>
-        </is>
-      </c>
-      <c r="G18" s="75" t="inlineStr">
+      <c r="E19" s="83" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" s="80" t="inlineStr">
+        <is>
+          <t>Structured HPC financing</t>
+        </is>
+      </c>
+      <c r="G19" s="80" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H18" s="75" t="inlineStr">
+      <c r="H19" s="80" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I18" s="75" t="inlineStr">
-        <is>
-          <t>GPU-cloud build</t>
-        </is>
-      </c>
-      <c r="J18" s="79" t="inlineStr">
-        <is>
-          <t>theaiinsider</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>3) ALTERNATE PRIVATE CREDIT / SPV / 144A</t>
-        </is>
-      </c>
-      <c r="B19" s="15" t="n"/>
-      <c r="C19" s="15" t="n"/>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="15" t="n"/>
-      <c r="F19" s="15" t="n"/>
-      <c r="G19" s="15" t="n"/>
-      <c r="H19" s="15" t="n"/>
-      <c r="I19" s="15" t="n"/>
-      <c r="J19" s="15" t="n"/>
+      <c r="I19" s="80" t="inlineStr">
+        <is>
+          <t>Powered-shell build for CoreWeave</t>
+        </is>
+      </c>
+      <c r="J19" s="84" t="inlineStr">
+        <is>
+          <t>press</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="70" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="B20" s="71" t="inlineStr">
-        <is>
-          <t>Oracle — Texas + Wisconsin DCs</t>
-        </is>
-      </c>
-      <c r="C20" s="72" t="inlineStr">
-        <is>
-          <t>Hyperscaler</t>
-        </is>
-      </c>
-      <c r="D20" s="70" t="inlineStr">
-        <is>
-          <t>Private credit consortium</t>
-        </is>
-      </c>
-      <c r="E20" s="73" t="n">
-        <v>38</v>
-      </c>
-      <c r="F20" s="70" t="inlineStr">
-        <is>
-          <t>SPV debt package</t>
-        </is>
-      </c>
-      <c r="G20" s="70" t="inlineStr">
+      <c r="A20" s="75" t="inlineStr">
+        <is>
+          <t>May 2025</t>
+        </is>
+      </c>
+      <c r="B20" s="76" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C20" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D20" s="75" t="inlineStr">
+        <is>
+          <t>Bank syndicate</t>
+        </is>
+      </c>
+      <c r="E20" s="78" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F20" s="75" t="inlineStr">
+        <is>
+          <t>Revolving credit line</t>
+        </is>
+      </c>
+      <c r="G20" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H20" s="70" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I20" s="70" t="inlineStr">
-        <is>
-          <t>Two-site off-B/S financing</t>
-        </is>
-      </c>
-      <c r="J20" s="74" t="inlineStr">
-        <is>
-          <t>FT</t>
+      <c r="H20" s="75" t="inlineStr">
+        <is>
+          <t>5y</t>
+        </is>
+      </c>
+      <c r="I20" s="75" t="inlineStr">
+        <is>
+          <t>Liquidity backstop</t>
+        </is>
+      </c>
+      <c r="J20" s="79" t="inlineStr">
+        <is>
+          <t>CNBC</t>
         </is>
       </c>
     </row>
@@ -8927,7 +8961,7 @@
       </c>
       <c r="B21" s="76" t="inlineStr">
         <is>
-          <t>Anthropic — Google TPU chip SPV</t>
+          <t>Nscale</t>
         </is>
       </c>
       <c r="C21" s="77" t="inlineStr">
@@ -8937,147 +8971,113 @@
       </c>
       <c r="D21" s="75" t="inlineStr">
         <is>
-          <t>Apollo, Blackstone; Broadcom RVG</t>
+          <t>Private credit / banks</t>
         </is>
       </c>
       <c r="E21" s="78" t="n">
-        <v>35</v>
+        <v>1.4</v>
       </c>
       <c r="F21" s="75" t="inlineStr">
         <is>
-          <t>Chip-leasing SPV; 3 tranches; ~half syndicated</t>
+          <t>Term loan</t>
         </is>
       </c>
       <c r="G21" s="75" t="inlineStr">
         <is>
-          <t>A1 T+100bp; A2 5.75%; B 8.5%</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H21" s="75" t="inlineStr">
         <is>
-          <t>~5y</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I21" s="75" t="inlineStr">
         <is>
-          <t>Buys Google TPUs leased to Anthropic</t>
+          <t>GPU-cloud build</t>
         </is>
       </c>
       <c r="J21" s="79" t="inlineStr">
         <is>
-          <t>privatedebtnews; Build.inc</t>
+          <t>theaiinsider</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="70" t="inlineStr">
-        <is>
-          <t>Oct 2025</t>
-        </is>
-      </c>
-      <c r="B22" s="71" t="inlineStr">
-        <is>
-          <t>Meta — Hyperion (Beignet Investor LLC)</t>
-        </is>
-      </c>
-      <c r="C22" s="72" t="inlineStr">
-        <is>
-          <t>Hyperscaler</t>
-        </is>
-      </c>
-      <c r="D22" s="70" t="inlineStr">
-        <is>
-          <t>PIMCO (~$18bn), BlackRock, Apollo; Blue Owl equity</t>
-        </is>
-      </c>
-      <c r="E22" s="73" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="F22" s="70" t="inlineStr">
-        <is>
-          <t>Off-B/S SPV; 144A senior secured bond</t>
-        </is>
-      </c>
-      <c r="G22" s="70" t="inlineStr">
-        <is>
-          <t>6.581% / T+225bp</t>
-        </is>
-      </c>
-      <c r="H22" s="70" t="inlineStr">
-        <is>
-          <t>Due May 2049</t>
-        </is>
-      </c>
-      <c r="I22" s="70" t="inlineStr">
-        <is>
-          <t>2.1GW; Meta lease + residual-value guarantee; A+ (S&amp;P)</t>
-        </is>
-      </c>
-      <c r="J22" s="74" t="inlineStr">
-        <is>
-          <t>IFR; FT; Quinn Emanuel</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="70" t="inlineStr">
-        <is>
-          <t>2025-26</t>
-        </is>
-      </c>
-      <c r="B23" s="71" t="inlineStr">
-        <is>
-          <t>Oracle — New Mexico site</t>
-        </is>
-      </c>
-      <c r="C23" s="72" t="inlineStr">
-        <is>
-          <t>Hyperscaler</t>
-        </is>
-      </c>
-      <c r="D23" s="70" t="inlineStr">
-        <is>
-          <t>Private credit lenders</t>
-        </is>
-      </c>
-      <c r="E23" s="73" t="n">
-        <v>18</v>
-      </c>
-      <c r="F23" s="70" t="inlineStr">
-        <is>
-          <t>SPV / project loan</t>
-        </is>
-      </c>
-      <c r="G23" s="70" t="inlineStr">
+      <c r="A22" s="75" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B22" s="76" t="inlineStr">
+        <is>
+          <t>Lambda</t>
+        </is>
+      </c>
+      <c r="C22" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D22" s="75" t="inlineStr">
+        <is>
+          <t>Macquarie</t>
+        </is>
+      </c>
+      <c r="E22" s="78" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F22" s="75" t="inlineStr">
+        <is>
+          <t>GPU-backed facility</t>
+        </is>
+      </c>
+      <c r="G22" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H23" s="70" t="inlineStr">
+      <c r="H22" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I23" s="70" t="inlineStr">
-        <is>
-          <t>Single-site project loan</t>
-        </is>
-      </c>
-      <c r="J23" s="74" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
+      <c r="I22" s="75" t="inlineStr">
+        <is>
+          <t>GPU-cloud build</t>
+        </is>
+      </c>
+      <c r="J22" s="79" t="inlineStr">
+        <is>
+          <t>theaiinsider</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>3) ALTERNATE PRIVATE CREDIT / SPV / 144A</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
+      <c r="G23" s="15" t="n"/>
+      <c r="H23" s="15" t="n"/>
+      <c r="I23" s="15" t="n"/>
+      <c r="J23" s="15" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="70" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025-26</t>
         </is>
       </c>
       <c r="B24" s="71" t="inlineStr">
         <is>
-          <t>Oracle — Michigan campus</t>
+          <t>Oracle — Texas + Wisconsin DCs</t>
         </is>
       </c>
       <c r="C24" s="72" t="inlineStr">
@@ -9087,15 +9087,15 @@
       </c>
       <c r="D24" s="70" t="inlineStr">
         <is>
-          <t>Project-finance lenders</t>
+          <t>Private credit consortium</t>
         </is>
       </c>
       <c r="E24" s="73" t="n">
-        <v>16.3</v>
+        <v>38</v>
       </c>
       <c r="F24" s="70" t="inlineStr">
         <is>
-          <t>Project-level SPV financing</t>
+          <t>SPV debt package</t>
         </is>
       </c>
       <c r="G24" s="70" t="inlineStr">
@@ -9110,24 +9110,24 @@
       </c>
       <c r="I24" s="70" t="inlineStr">
         <is>
-          <t>OCI capacity build</t>
+          <t>Two-site off-B/S financing</t>
         </is>
       </c>
       <c r="J24" s="74" t="inlineStr">
         <is>
-          <t>Press reports</t>
+          <t>FT</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="75" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="B25" s="76" t="inlineStr">
         <is>
-          <t>xAI — Colossus 2 chip SPV</t>
+          <t>Anthropic — Google TPU chip SPV</t>
         </is>
       </c>
       <c r="C25" s="77" t="inlineStr">
@@ -9137,47 +9137,47 @@
       </c>
       <c r="D25" s="75" t="inlineStr">
         <is>
-          <t>Valor Equity, Apollo, Diameter; NVIDIA equity</t>
+          <t>Apollo, Blackstone; Broadcom RVG</t>
         </is>
       </c>
       <c r="E25" s="78" t="n">
-        <v>12.5</v>
+        <v>35</v>
       </c>
       <c r="F25" s="75" t="inlineStr">
         <is>
-          <t>SPV; debt + ~$7.5bn equity</t>
+          <t>Chip-leasing SPV; 3 tranches; ~half syndicated</t>
         </is>
       </c>
       <c r="G25" s="75" t="inlineStr">
         <is>
-          <t>~10.5%</t>
+          <t>A1 T+100bp; A2 5.75%; B 8.5%</t>
         </is>
       </c>
       <c r="H25" s="75" t="inlineStr">
         <is>
-          <t>5y (~2.5y avg)</t>
+          <t>~5y</t>
         </is>
       </c>
       <c r="I25" s="75" t="inlineStr">
         <is>
-          <t>Buys NVIDIA GPUs leased to xAI</t>
+          <t>Buys Google TPUs leased to Anthropic</t>
         </is>
       </c>
       <c r="J25" s="79" t="inlineStr">
         <is>
-          <t>FT; WSJ</t>
+          <t>privatedebtnews; Build.inc</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="70" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Oct 2025</t>
         </is>
       </c>
       <c r="B26" s="71" t="inlineStr">
         <is>
-          <t>Oracle/OpenAI — Abilene, TX (Stargate)</t>
+          <t>Meta — Hyperion (Beignet Investor LLC, RPLDCI)</t>
         </is>
       </c>
       <c r="C26" s="72" t="inlineStr">
@@ -9187,147 +9187,147 @@
       </c>
       <c r="D26" s="70" t="inlineStr">
         <is>
-          <t>Blue Owl + JPMorgan (Crusoe, Primary Digital)</t>
+          <t>PIMCO (~$18bn), BlackRock, Apollo; Blue Owl equity</t>
         </is>
       </c>
       <c r="E26" s="73" t="n">
-        <v>10</v>
+        <v>27.294</v>
       </c>
       <c r="F26" s="70" t="inlineStr">
         <is>
-          <t>Off-B/S SPV (~$13bn incl equity)</t>
+          <t>Off-B/S SPV; 144A senior secured bond</t>
         </is>
       </c>
       <c r="G26" s="70" t="inlineStr">
         <is>
+          <t>6.581%; YTW 6.4%; +193</t>
+        </is>
+      </c>
+      <c r="H26" s="70" t="inlineStr">
+        <is>
+          <t>May 2049</t>
+        </is>
+      </c>
+      <c r="I26" s="70" t="inlineStr">
+        <is>
+          <t>2.1GW Richland Parish LA; Meta lease + residual-value guarantee; A+ (S&amp;P)</t>
+        </is>
+      </c>
+      <c r="J26" s="74" t="inlineStr">
+        <is>
+          <t>IFR; FT; Seaport</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="70" t="inlineStr">
+        <is>
+          <t>2025-26</t>
+        </is>
+      </c>
+      <c r="B27" s="71" t="inlineStr">
+        <is>
+          <t>Oracle — New Mexico site</t>
+        </is>
+      </c>
+      <c r="C27" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D27" s="70" t="inlineStr">
+        <is>
+          <t>Private credit lenders</t>
+        </is>
+      </c>
+      <c r="E27" s="73" t="n">
+        <v>18</v>
+      </c>
+      <c r="F27" s="70" t="inlineStr">
+        <is>
+          <t>SPV / project loan</t>
+        </is>
+      </c>
+      <c r="G27" s="70" t="inlineStr">
+        <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H26" s="70" t="inlineStr">
+      <c r="H27" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I26" s="70" t="inlineStr">
-        <is>
-          <t>SPV owns OpenAI Abilene facility</t>
-        </is>
-      </c>
-      <c r="J26" s="74" t="inlineStr">
+      <c r="I27" s="70" t="inlineStr">
+        <is>
+          <t>Single-site project loan</t>
+        </is>
+      </c>
+      <c r="J27" s="74" t="inlineStr">
         <is>
           <t>FT</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="75" t="inlineStr">
-        <is>
-          <t>May 2024</t>
-        </is>
-      </c>
-      <c r="B27" s="76" t="inlineStr">
-        <is>
-          <t>CoreWeave — $7.5bn facility</t>
-        </is>
-      </c>
-      <c r="C27" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D27" s="75" t="inlineStr">
-        <is>
-          <t>Blackstone, Magnetar, Coatue, Carlyle, CDPQ, BlackRock</t>
-        </is>
-      </c>
-      <c r="E27" s="78" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="F27" s="75" t="inlineStr">
-        <is>
-          <t>GPU + customer-contract secured facility</t>
-        </is>
-      </c>
-      <c r="G27" s="75" t="inlineStr">
-        <is>
-          <t>~10%+</t>
-        </is>
-      </c>
-      <c r="H27" s="75" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I27" s="75" t="inlineStr">
-        <is>
-          <t>Largest private debt deal at the time</t>
-        </is>
-      </c>
-      <c r="J27" s="79" t="inlineStr">
-        <is>
-          <t>Blackstone</t>
-        </is>
-      </c>
-    </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="80" t="inlineStr">
-        <is>
-          <t>Early 2025</t>
-        </is>
-      </c>
-      <c r="B28" s="81" t="inlineStr">
-        <is>
-          <t>Aligned Data Centers — debt</t>
-        </is>
-      </c>
-      <c r="C28" s="82" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REIT</t>
-        </is>
-      </c>
-      <c r="D28" s="80" t="inlineStr">
-        <is>
-          <t>Macquarie + global investors</t>
-        </is>
-      </c>
-      <c r="E28" s="83" t="n">
-        <v>7</v>
-      </c>
-      <c r="F28" s="80" t="inlineStr">
-        <is>
-          <t>Debt within $12bn raise (+$5bn equity)</t>
-        </is>
-      </c>
-      <c r="G28" s="80" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H28" s="80" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I28" s="80" t="inlineStr">
-        <is>
-          <t>Later acquired by MGX/BlackRock (~$40bn)</t>
-        </is>
-      </c>
-      <c r="J28" s="84" t="inlineStr">
-        <is>
-          <t>SFA; NYU DRI</t>
+      <c r="A28" s="70" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B28" s="71" t="inlineStr">
+        <is>
+          <t>Oracle — Michigan (RD Michigan Property Owner I)</t>
+        </is>
+      </c>
+      <c r="C28" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D28" s="70" t="inlineStr">
+        <is>
+          <t>Blackstone (90%) / Related Digital (10%)</t>
+        </is>
+      </c>
+      <c r="E28" s="73" t="n">
+        <v>14</v>
+      </c>
+      <c r="F28" s="70" t="inlineStr">
+        <is>
+          <t>1st-lien secured DC bond / SPV</t>
+        </is>
+      </c>
+      <c r="G28" s="70" t="inlineStr">
+        <is>
+          <t>7.50%; YTW 7.5%; +301</t>
+        </is>
+      </c>
+      <c r="H28" s="70" t="inlineStr">
+        <is>
+          <t>Mar 2045</t>
+        </is>
+      </c>
+      <c r="I28" s="70" t="inlineStr">
+        <is>
+          <t>974MW Saline MI; Oracle 17.5y lease (guarantee); Baa3/BBB</t>
+        </is>
+      </c>
+      <c r="J28" s="74" t="inlineStr">
+        <is>
+          <t>Seaport (6/13/26); FT</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="75" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025-26</t>
         </is>
       </c>
       <c r="B29" s="76" t="inlineStr">
         <is>
-          <t>Fluidstack — Google-backed facility</t>
+          <t>xAI — Colossus 2 chip SPV</t>
         </is>
       </c>
       <c r="C29" s="77" t="inlineStr">
@@ -9337,97 +9337,97 @@
       </c>
       <c r="D29" s="75" t="inlineStr">
         <is>
-          <t>Private credit (Google lease backstop)</t>
+          <t>Valor Equity, Apollo, Diameter; NVIDIA equity</t>
         </is>
       </c>
       <c r="E29" s="78" t="n">
-        <v>6.7</v>
+        <v>12.5</v>
       </c>
       <c r="F29" s="75" t="inlineStr">
         <is>
-          <t>SPV backed by contracted revenue</t>
+          <t>SPV; debt + ~$7.5bn equity</t>
         </is>
       </c>
       <c r="G29" s="75" t="inlineStr">
         <is>
+          <t>~10.5%</t>
+        </is>
+      </c>
+      <c r="H29" s="75" t="inlineStr">
+        <is>
+          <t>5y (~2.5y avg)</t>
+        </is>
+      </c>
+      <c r="I29" s="75" t="inlineStr">
+        <is>
+          <t>Buys NVIDIA GPUs leased to xAI</t>
+        </is>
+      </c>
+      <c r="J29" s="79" t="inlineStr">
+        <is>
+          <t>FT; WSJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="70" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B30" s="71" t="inlineStr">
+        <is>
+          <t>Oracle/OpenAI — Abilene, TX (Stargate)</t>
+        </is>
+      </c>
+      <c r="C30" s="72" t="inlineStr">
+        <is>
+          <t>Hyperscaler</t>
+        </is>
+      </c>
+      <c r="D30" s="70" t="inlineStr">
+        <is>
+          <t>Blue Owl + JPMorgan (Crusoe, Primary Digital)</t>
+        </is>
+      </c>
+      <c r="E30" s="73" t="n">
+        <v>10</v>
+      </c>
+      <c r="F30" s="70" t="inlineStr">
+        <is>
+          <t>Off-B/S SPV (~$13bn incl equity)</t>
+        </is>
+      </c>
+      <c r="G30" s="70" t="inlineStr">
+        <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H29" s="75" t="inlineStr">
+      <c r="H30" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I29" s="75" t="inlineStr">
-        <is>
-          <t>~$6.7bn Google-contracted revenue</t>
-        </is>
-      </c>
-      <c r="J29" s="79" t="inlineStr">
-        <is>
-          <t>theaiinsider</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="75" t="inlineStr">
-        <is>
-          <t>Jun-Jul 2025</t>
-        </is>
-      </c>
-      <c r="B30" s="76" t="inlineStr">
-        <is>
-          <t>xAI — secured notes / term loan</t>
-        </is>
-      </c>
-      <c r="C30" s="77" t="inlineStr">
-        <is>
-          <t>Neocloud / AI-native</t>
-        </is>
-      </c>
-      <c r="D30" s="75" t="inlineStr">
-        <is>
-          <t>Apollo, Diameter; Morgan Stanley</t>
-        </is>
-      </c>
-      <c r="E30" s="78" t="n">
-        <v>5</v>
-      </c>
-      <c r="F30" s="75" t="inlineStr">
-        <is>
-          <t>Secured notes + term loan (part of $10bn raise)</t>
-        </is>
-      </c>
-      <c r="G30" s="75" t="inlineStr">
-        <is>
-          <t>up to ~12.5%</t>
-        </is>
-      </c>
-      <c r="H30" s="75" t="inlineStr">
-        <is>
-          <t>~3-5y</t>
-        </is>
-      </c>
-      <c r="I30" s="75" t="inlineStr">
-        <is>
-          <t>Lenders can operate Colossus on default</t>
-        </is>
-      </c>
-      <c r="J30" s="79" t="inlineStr">
-        <is>
-          <t>CNBC; ciphertalk</t>
+      <c r="I30" s="70" t="inlineStr">
+        <is>
+          <t>SPV owns OpenAI Abilene facility</t>
+        </is>
+      </c>
+      <c r="J30" s="74" t="inlineStr">
+        <is>
+          <t>FT</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="75" t="inlineStr">
         <is>
-          <t>Jul 2025</t>
+          <t>May 2024</t>
         </is>
       </c>
       <c r="B31" s="76" t="inlineStr">
         <is>
-          <t>CoreWeave — OpenAI contract financing</t>
+          <t>CoreWeave — $7.5bn facility</t>
         </is>
       </c>
       <c r="C31" s="77" t="inlineStr">
@@ -9437,470 +9437,504 @@
       </c>
       <c r="D31" s="75" t="inlineStr">
         <is>
-          <t>Private lenders (SPV)</t>
+          <t>Blackstone, Magnetar, Coatue, Carlyle, CDPQ, BlackRock</t>
         </is>
       </c>
       <c r="E31" s="78" t="n">
-        <v>2.6</v>
+        <v>7.5</v>
       </c>
       <c r="F31" s="75" t="inlineStr">
         <is>
-          <t>SPV debt vs $11.9bn OpenAI contract</t>
+          <t>GPU + customer-contract secured facility</t>
         </is>
       </c>
       <c r="G31" s="75" t="inlineStr">
         <is>
+          <t>~10%+</t>
+        </is>
+      </c>
+      <c r="H31" s="75" t="inlineStr">
+        <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H31" s="75" t="inlineStr">
+      <c r="I31" s="75" t="inlineStr">
+        <is>
+          <t>Largest private debt deal at the time</t>
+        </is>
+      </c>
+      <c r="J31" s="79" t="inlineStr">
+        <is>
+          <t>Blackstone</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="80" t="inlineStr">
+        <is>
+          <t>Early 2025</t>
+        </is>
+      </c>
+      <c r="B32" s="81" t="inlineStr">
+        <is>
+          <t>Aligned Data Centers — debt</t>
+        </is>
+      </c>
+      <c r="C32" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D32" s="80" t="inlineStr">
+        <is>
+          <t>Macquarie + global investors</t>
+        </is>
+      </c>
+      <c r="E32" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="F32" s="80" t="inlineStr">
+        <is>
+          <t>Debt within $12bn raise (+$5bn equity)</t>
+        </is>
+      </c>
+      <c r="G32" s="80" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I31" s="75" t="inlineStr">
-        <is>
-          <t>Funds OpenAI compute obligations</t>
-        </is>
-      </c>
-      <c r="J31" s="79" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="75" t="inlineStr">
-        <is>
-          <t>Aug 2023</t>
-        </is>
-      </c>
-      <c r="B32" s="76" t="inlineStr">
-        <is>
-          <t>CoreWeave — $2.3bn facility</t>
-        </is>
-      </c>
-      <c r="C32" s="77" t="inlineStr">
+      <c r="H32" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I32" s="80" t="inlineStr">
+        <is>
+          <t>Later acquired by MGX/BlackRock (~$40bn)</t>
+        </is>
+      </c>
+      <c r="J32" s="84" t="inlineStr">
+        <is>
+          <t>SFA; NYU DRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="75" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B33" s="76" t="inlineStr">
+        <is>
+          <t>Fluidstack — Google-backed facility</t>
+        </is>
+      </c>
+      <c r="C33" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D32" s="75" t="inlineStr">
-        <is>
-          <t>Blackstone, Magnetar</t>
-        </is>
-      </c>
-      <c r="E32" s="78" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="F32" s="75" t="inlineStr">
-        <is>
-          <t>GPU-backed facility</t>
-        </is>
-      </c>
-      <c r="G32" s="75" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="H32" s="75" t="inlineStr">
+      <c r="D33" s="75" t="inlineStr">
+        <is>
+          <t>Private credit (Google lease backstop)</t>
+        </is>
+      </c>
+      <c r="E33" s="78" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="F33" s="75" t="inlineStr">
+        <is>
+          <t>SPV backed by contracted revenue</t>
+        </is>
+      </c>
+      <c r="G33" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I32" s="75" t="inlineStr">
-        <is>
-          <t>Early GPU-collateralized template</t>
-        </is>
-      </c>
-      <c r="J32" s="79" t="inlineStr">
-        <is>
-          <t>Blackstone</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="14" t="inlineStr">
-        <is>
-          <t>4) INSURANCE-LINKED LENDING (memo — overlaps groups 1-3)</t>
-        </is>
-      </c>
-      <c r="B33" s="15" t="n"/>
-      <c r="C33" s="15" t="n"/>
-      <c r="D33" s="15" t="n"/>
-      <c r="E33" s="15" t="n"/>
-      <c r="F33" s="15" t="n"/>
-      <c r="G33" s="15" t="n"/>
-      <c r="H33" s="15" t="n"/>
-      <c r="I33" s="15" t="n"/>
-      <c r="J33" s="15" t="n"/>
+      <c r="H33" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I33" s="75" t="inlineStr">
+        <is>
+          <t>~$6.7bn Google-contracted revenue</t>
+        </is>
+      </c>
+      <c r="J33" s="79" t="inlineStr">
+        <is>
+          <t>theaiinsider</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="75" t="inlineStr">
         <is>
+          <t>Jun-Jul 2025</t>
+        </is>
+      </c>
+      <c r="B34" s="76" t="inlineStr">
+        <is>
+          <t>xAI — secured notes / term loan</t>
+        </is>
+      </c>
+      <c r="C34" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D34" s="75" t="inlineStr">
+        <is>
+          <t>Apollo, Diameter; Morgan Stanley</t>
+        </is>
+      </c>
+      <c r="E34" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" s="75" t="inlineStr">
+        <is>
+          <t>Secured notes + term loan (part of $10bn raise)</t>
+        </is>
+      </c>
+      <c r="G34" s="75" t="inlineStr">
+        <is>
+          <t>up to ~12.5%</t>
+        </is>
+      </c>
+      <c r="H34" s="75" t="inlineStr">
+        <is>
+          <t>~3-5y</t>
+        </is>
+      </c>
+      <c r="I34" s="75" t="inlineStr">
+        <is>
+          <t>Lenders can operate Colossus on default</t>
+        </is>
+      </c>
+      <c r="J34" s="79" t="inlineStr">
+        <is>
+          <t>CNBC; ciphertalk</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="75" t="inlineStr">
+        <is>
+          <t>Jul 2025</t>
+        </is>
+      </c>
+      <c r="B35" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — OpenAI contract financing</t>
+        </is>
+      </c>
+      <c r="C35" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D35" s="75" t="inlineStr">
+        <is>
+          <t>Private lenders (SPV)</t>
+        </is>
+      </c>
+      <c r="E35" s="78" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F35" s="75" t="inlineStr">
+        <is>
+          <t>SPV debt vs $11.9bn OpenAI contract</t>
+        </is>
+      </c>
+      <c r="G35" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H35" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I35" s="75" t="inlineStr">
+        <is>
+          <t>Funds OpenAI compute obligations</t>
+        </is>
+      </c>
+      <c r="J35" s="79" t="inlineStr">
+        <is>
+          <t>FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="75" t="inlineStr">
+        <is>
+          <t>Aug 2023</t>
+        </is>
+      </c>
+      <c r="B36" s="76" t="inlineStr">
+        <is>
+          <t>CoreWeave — $2.3bn facility</t>
+        </is>
+      </c>
+      <c r="C36" s="77" t="inlineStr">
+        <is>
+          <t>Neocloud / AI-native</t>
+        </is>
+      </c>
+      <c r="D36" s="75" t="inlineStr">
+        <is>
+          <t>Blackstone, Magnetar</t>
+        </is>
+      </c>
+      <c r="E36" s="78" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F36" s="75" t="inlineStr">
+        <is>
+          <t>GPU-backed facility</t>
+        </is>
+      </c>
+      <c r="G36" s="75" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H36" s="75" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I36" s="75" t="inlineStr">
+        <is>
+          <t>Early GPU-collateralized template</t>
+        </is>
+      </c>
+      <c r="J36" s="79" t="inlineStr">
+        <is>
+          <t>Blackstone</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>4) INSURANCE-LINKED LENDING (memo — overlaps groups 1-3)</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="n"/>
+      <c r="C37" s="15" t="n"/>
+      <c r="D37" s="15" t="n"/>
+      <c r="E37" s="15" t="n"/>
+      <c r="F37" s="15" t="n"/>
+      <c r="G37" s="15" t="n"/>
+      <c r="H37" s="15" t="n"/>
+      <c r="I37" s="15" t="n"/>
+      <c r="J37" s="15" t="n"/>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="75" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="B34" s="76" t="inlineStr">
+      <c r="B38" s="76" t="inlineStr">
         <is>
           <t>Anthropic — A2 notes (insurer tranche)</t>
         </is>
       </c>
-      <c r="C34" s="77" t="inlineStr">
+      <c r="C38" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D34" s="75" t="inlineStr">
+      <c r="D38" s="75" t="inlineStr">
         <is>
           <t>Apollo / Athene + insurers</t>
         </is>
       </c>
-      <c r="E34" s="78" t="n">
+      <c r="E38" s="78" t="n">
         <v>24</v>
       </c>
-      <c r="F34" s="75" t="inlineStr">
+      <c r="F38" s="75" t="inlineStr">
         <is>
           <t>Insurance-bought A2 tranche of TPU SPV</t>
         </is>
       </c>
-      <c r="G34" s="75" t="inlineStr">
+      <c r="G38" s="75" t="inlineStr">
         <is>
           <t>5.75%</t>
         </is>
       </c>
-      <c r="H34" s="75" t="inlineStr">
+      <c r="H38" s="75" t="inlineStr">
         <is>
           <t>~5y</t>
         </is>
       </c>
-      <c r="I34" s="75" t="inlineStr">
+      <c r="I38" s="75" t="inlineStr">
         <is>
           <t>Within the $35bn Anthropic deal (group 3)</t>
         </is>
       </c>
-      <c r="J34" s="79" t="inlineStr">
+      <c r="J38" s="79" t="inlineStr">
         <is>
           <t>privatedebtnews</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="85" t="inlineStr">
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="85" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B35" s="86" t="inlineStr">
+      <c r="B39" s="86" t="inlineStr">
         <is>
           <t>Athene (Apollo) — AP Grange</t>
         </is>
       </c>
-      <c r="C35" s="87" t="inlineStr">
+      <c r="C39" s="87" t="inlineStr">
         <is>
           <t>Context / market</t>
         </is>
       </c>
-      <c r="D35" s="85" t="inlineStr">
+      <c r="D39" s="85" t="inlineStr">
         <is>
           <t>Athene / Apollo (+ Intel equity)</t>
         </is>
       </c>
-      <c r="E35" s="88" t="n">
+      <c r="E39" s="88" t="n">
         <v>6.5</v>
       </c>
-      <c r="F35" s="85" t="inlineStr">
+      <c r="F39" s="85" t="inlineStr">
         <is>
           <t>Insurer JV investment (semis-adjacent)</t>
         </is>
       </c>
-      <c r="G35" s="85" t="inlineStr">
+      <c r="G39" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H35" s="85" t="inlineStr">
+      <c r="H39" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I35" s="85" t="inlineStr">
+      <c r="I39" s="85" t="inlineStr">
         <is>
           <t>Largest single-issuer insurer credit exposure</t>
         </is>
       </c>
-      <c r="J35" s="89" t="inlineStr">
+      <c r="J39" s="89" t="inlineStr">
         <is>
           <t>Moody's</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="70" t="inlineStr">
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="70" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
       </c>
-      <c r="B36" s="71" t="inlineStr">
+      <c r="B40" s="71" t="inlineStr">
         <is>
           <t>Meta — Hyperion insurance allocation</t>
         </is>
       </c>
-      <c r="C36" s="72" t="inlineStr">
+      <c r="C40" s="72" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="D36" s="70" t="inlineStr">
+      <c r="D40" s="70" t="inlineStr">
         <is>
           <t>Insurers via PIMCO / BlackRock</t>
         </is>
       </c>
-      <c r="E36" s="90" t="n"/>
-      <c r="F36" s="70" t="inlineStr">
+      <c r="E40" s="90" t="n"/>
+      <c r="F40" s="70" t="inlineStr">
         <is>
           <t>Insurance allocation of 144A bond</t>
         </is>
       </c>
-      <c r="G36" s="70" t="inlineStr">
+      <c r="G40" s="70" t="inlineStr">
         <is>
           <t>6.581%</t>
         </is>
       </c>
-      <c r="H36" s="70" t="inlineStr">
+      <c r="H40" s="70" t="inlineStr">
         <is>
           <t>2049</t>
         </is>
       </c>
-      <c r="I36" s="70" t="inlineStr">
+      <c r="I40" s="70" t="inlineStr">
         <is>
           <t>Subset of the $27.3bn Hyperion bond (group 3)</t>
         </is>
       </c>
-      <c r="J36" s="74" t="inlineStr">
+      <c r="J40" s="74" t="inlineStr">
         <is>
           <t>FT; S&amp;P</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="75" t="inlineStr">
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="75" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="B37" s="76" t="inlineStr">
+      <c r="B41" s="76" t="inlineStr">
         <is>
           <t>CoreWeave — DDTL 4.0 insurance anchor</t>
         </is>
       </c>
-      <c r="C37" s="77" t="inlineStr">
+      <c r="C41" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D37" s="75" t="inlineStr">
+      <c r="D41" s="75" t="inlineStr">
         <is>
           <t>Blackstone Credit &amp; Insurance + insurers</t>
         </is>
       </c>
-      <c r="E37" s="91" t="n"/>
-      <c r="F37" s="75" t="inlineStr">
+      <c r="E41" s="91" t="n"/>
+      <c r="F41" s="75" t="inlineStr">
         <is>
           <t>Insurance anchor of GPU-backed loan</t>
         </is>
       </c>
-      <c r="G37" s="75" t="inlineStr">
+      <c r="G41" s="75" t="inlineStr">
         <is>
           <t>SOFR+225 / 5.9%</t>
         </is>
       </c>
-      <c r="H37" s="75" t="inlineStr">
+      <c r="H41" s="75" t="inlineStr">
         <is>
           <t>2032</t>
         </is>
       </c>
-      <c r="I37" s="75" t="inlineStr">
+      <c r="I41" s="75" t="inlineStr">
         <is>
           <t>Subset of the $8.5bn DDTL (group 2)</t>
         </is>
       </c>
-      <c r="J37" s="79" t="inlineStr">
+      <c r="J41" s="79" t="inlineStr">
         <is>
           <t>CoreWeave IR</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="14" t="inlineStr">
-        <is>
-          <t>5) SECURITIZATION / ABS / CMBS</t>
-        </is>
-      </c>
-      <c r="B38" s="15" t="n"/>
-      <c r="C38" s="15" t="n"/>
-      <c r="D38" s="15" t="n"/>
-      <c r="E38" s="15" t="n"/>
-      <c r="F38" s="15" t="n"/>
-      <c r="G38" s="15" t="n"/>
-      <c r="H38" s="15" t="n"/>
-      <c r="I38" s="15" t="n"/>
-      <c r="J38" s="15" t="n"/>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="80" t="inlineStr">
-        <is>
-          <t>Nov 2025</t>
-        </is>
-      </c>
-      <c r="B39" s="81" t="inlineStr">
-        <is>
-          <t>QTS (Blackstone) — BX 2025-VOLT</t>
-        </is>
-      </c>
-      <c r="C39" s="82" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REIT</t>
-        </is>
-      </c>
-      <c r="D39" s="80" t="inlineStr">
-        <is>
-          <t>Blackstone</t>
-        </is>
-      </c>
-      <c r="E39" s="83" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F39" s="80" t="inlineStr">
-        <is>
-          <t>SASB CMBS (~10 QTS DCs)</t>
-        </is>
-      </c>
-      <c r="G39" s="80" t="inlineStr">
-        <is>
-          <t>floating</t>
-        </is>
-      </c>
-      <c r="H39" s="80" t="inlineStr">
-        <is>
-          <t>2y + ext</t>
-        </is>
-      </c>
-      <c r="I39" s="80" t="inlineStr">
-        <is>
-          <t>Year's largest data-center CMBS</t>
-        </is>
-      </c>
-      <c r="J39" s="84" t="inlineStr">
-        <is>
-          <t>CREFC; SFA</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="80" t="inlineStr">
-        <is>
-          <t>2024-25</t>
-        </is>
-      </c>
-      <c r="B40" s="81" t="inlineStr">
-        <is>
-          <t>Switch (DigitalBridge) — SWCH 2025-DATA</t>
-        </is>
-      </c>
-      <c r="C40" s="82" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REIT</t>
-        </is>
-      </c>
-      <c r="D40" s="80" t="inlineStr">
-        <is>
-          <t>DigitalBridge</t>
-        </is>
-      </c>
-      <c r="E40" s="83" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F40" s="80" t="inlineStr">
-        <is>
-          <t>$2.4bn SASB CMBS + $1.1bn ABS (green)</t>
-        </is>
-      </c>
-      <c r="G40" s="80" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="H40" s="80" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I40" s="80" t="inlineStr">
-        <is>
-          <t>Green-bond framework</t>
-        </is>
-      </c>
-      <c r="J40" s="84" t="inlineStr">
-        <is>
-          <t>SFA; CREFC</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="80" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B41" s="81" t="inlineStr">
-        <is>
-          <t>Applied Digital — Polaris Forge HY bond</t>
-        </is>
-      </c>
-      <c r="C41" s="82" t="inlineStr">
-        <is>
-          <t>Colocation / data-center REIT</t>
-        </is>
-      </c>
-      <c r="D41" s="80" t="inlineStr">
-        <is>
-          <t>HY market</t>
-        </is>
-      </c>
-      <c r="E41" s="83" t="n">
-        <v>1.59</v>
-      </c>
-      <c r="F41" s="80" t="inlineStr">
-        <is>
-          <t>HY / securitized bond (CoreWeave campus)</t>
-        </is>
-      </c>
-      <c r="G41" s="80" t="inlineStr">
-        <is>
-          <t>7%</t>
-        </is>
-      </c>
-      <c r="H41" s="80" t="inlineStr">
-        <is>
-          <t>15y contract</t>
-        </is>
-      </c>
-      <c r="I41" s="80" t="inlineStr">
-        <is>
-          <t>150MW for CoreWeave</t>
-        </is>
-      </c>
-      <c r="J41" s="84" t="inlineStr">
-        <is>
-          <t>TNW</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>6) CONVERTIBLES / EQUITY-LINKED</t>
+          <t>5) SECURITIZATION / ABS / CMBS / SECURED DATA-CENTER BONDS</t>
         </is>
       </c>
       <c r="B42" s="15" t="n"/>
@@ -9914,978 +9948,2008 @@
       <c r="J42" s="15" t="n"/>
     </row>
     <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="75" t="inlineStr">
+      <c r="A43" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B43" s="81" t="inlineStr">
+        <is>
+          <t>Meridian Arc Holdco (MERIDI) — Next Frontier/Fluidstack JV</t>
+        </is>
+      </c>
+      <c r="C43" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D43" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E43" s="83" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="F43" s="80" t="inlineStr">
+        <is>
+          <t>Secured DC bond</t>
+        </is>
+      </c>
+      <c r="G43" s="80" t="inlineStr">
+        <is>
+          <t>6.25%; YTW 6.3%; +207</t>
+        </is>
+      </c>
+      <c r="H43" s="80" t="inlineStr">
+        <is>
+          <t>Apr 2031</t>
+        </is>
+      </c>
+      <c r="I43" s="80" t="inlineStr">
+        <is>
+          <t>Tenant Fluidstack (Google backstop), 15y lease; 245+185MW Sullivan Co. IN; Ba2/BB</t>
+        </is>
+      </c>
+      <c r="J43" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Meridian Compute)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B44" s="81" t="inlineStr">
+        <is>
+          <t>QTS Fayetteville I (QTSQST) — QTS/Blackstone</t>
+        </is>
+      </c>
+      <c r="C44" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D44" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E44" s="83" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F44" s="80" t="inlineStr">
+        <is>
+          <t>Secured DC bond (IG)</t>
+        </is>
+      </c>
+      <c r="G44" s="80" t="inlineStr">
+        <is>
+          <t>5.70%; YTW 6.2%; +171</t>
+        </is>
+      </c>
+      <c r="H44" s="80" t="inlineStr">
+        <is>
+          <t>Apr 2036</t>
+        </is>
+      </c>
+      <c r="I44" s="80" t="inlineStr">
+        <is>
+          <t>Tenant Microsoft (IG), 20y lease; Atlanta GA; Baa2</t>
+        </is>
+      </c>
+      <c r="J44" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (QTS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B45" s="81" t="inlineStr">
+        <is>
+          <t>PR RNO Property Owner 1 (TRACTD) — Tract Capital</t>
+        </is>
+      </c>
+      <c r="C45" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D45" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E45" s="83" t="n">
+        <v>4.585</v>
+      </c>
+      <c r="F45" s="80" t="inlineStr">
+        <is>
+          <t>Secured DC bond</t>
+        </is>
+      </c>
+      <c r="G45" s="80" t="inlineStr">
+        <is>
+          <t>6.50%; YTW 6.6%; +236</t>
+        </is>
+      </c>
+      <c r="H45" s="80" t="inlineStr">
+        <is>
+          <t>May 2031</t>
+        </is>
+      </c>
+      <c r="I45" s="80" t="inlineStr">
+        <is>
+          <t>Tenant Nvidia (IG), 16y lease; 200MW Storey Co. NV; Ba1/(P)BB/BB</t>
+        </is>
+      </c>
+      <c r="J45" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Tract Capital)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B46" s="81" t="inlineStr">
+        <is>
+          <t>Beacon Point DC (HUTBPA) — Hut 8</t>
+        </is>
+      </c>
+      <c r="C46" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D46" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E46" s="83" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="F46" s="80" t="inlineStr">
+        <is>
+          <t>Secured 1st-lien DC bond (IG)</t>
+        </is>
+      </c>
+      <c r="G46" s="80" t="inlineStr">
+        <is>
+          <t>6.129%; YTW 6.0%; +155</t>
+        </is>
+      </c>
+      <c r="H46" s="80" t="inlineStr">
+        <is>
+          <t>Nov 2042</t>
+        </is>
+      </c>
+      <c r="I46" s="80" t="inlineStr">
+        <is>
+          <t>Tenant Nvidia (IG), 15y lease; 352MW Nueces Co. TX; Baa2</t>
+        </is>
+      </c>
+      <c r="J46" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Hut 8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B47" s="81" t="inlineStr">
+        <is>
+          <t>SV RNO Property Owner 1 (TRACTC) — Tract Capital</t>
+        </is>
+      </c>
+      <c r="C47" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D47" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E47" s="83" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F47" s="80" t="inlineStr">
+        <is>
+          <t>Secured DC bond</t>
+        </is>
+      </c>
+      <c r="G47" s="80" t="inlineStr">
+        <is>
+          <t>5.875%; YTW 6.3%; +206</t>
+        </is>
+      </c>
+      <c r="H47" s="80" t="inlineStr">
+        <is>
+          <t>Mar 2031</t>
+        </is>
+      </c>
+      <c r="I47" s="80" t="inlineStr">
+        <is>
+          <t>Tenant Nvidia (IG), 16y lease; 200MW Storey Co. NV; Ba1/(P)BB+/BB</t>
+        </is>
+      </c>
+      <c r="J47" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Tract Capital)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="80" t="inlineStr">
+        <is>
+          <t>Nov 2025</t>
+        </is>
+      </c>
+      <c r="B48" s="81" t="inlineStr">
+        <is>
+          <t>QTS (Blackstone) — BX 2025-VOLT</t>
+        </is>
+      </c>
+      <c r="C48" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D48" s="80" t="inlineStr">
+        <is>
+          <t>Blackstone</t>
+        </is>
+      </c>
+      <c r="E48" s="83" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F48" s="80" t="inlineStr">
+        <is>
+          <t>SASB CMBS (~10 QTS DCs)</t>
+        </is>
+      </c>
+      <c r="G48" s="80" t="inlineStr">
+        <is>
+          <t>floating</t>
+        </is>
+      </c>
+      <c r="H48" s="80" t="inlineStr">
+        <is>
+          <t>2y + ext</t>
+        </is>
+      </c>
+      <c r="I48" s="80" t="inlineStr">
+        <is>
+          <t>Year's largest data-center CMBS</t>
+        </is>
+      </c>
+      <c r="J48" s="84" t="inlineStr">
+        <is>
+          <t>CREFC; SFA</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="80" t="inlineStr">
+        <is>
+          <t>2024-25</t>
+        </is>
+      </c>
+      <c r="B49" s="81" t="inlineStr">
+        <is>
+          <t>Switch (DigitalBridge) — SWCH 2025-DATA</t>
+        </is>
+      </c>
+      <c r="C49" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D49" s="80" t="inlineStr">
+        <is>
+          <t>DigitalBridge</t>
+        </is>
+      </c>
+      <c r="E49" s="83" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F49" s="80" t="inlineStr">
+        <is>
+          <t>$2.4bn SASB CMBS + $1.1bn ABS (green)</t>
+        </is>
+      </c>
+      <c r="G49" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H49" s="80" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I49" s="80" t="inlineStr">
+        <is>
+          <t>Green-bond framework</t>
+        </is>
+      </c>
+      <c r="J49" s="84" t="inlineStr">
+        <is>
+          <t>SFA; CREFC</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B50" s="81" t="inlineStr">
+        <is>
+          <t>Core Scientific Finance I (CORZ)</t>
+        </is>
+      </c>
+      <c r="C50" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D50" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E50" s="83" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F50" s="80" t="inlineStr">
+        <is>
+          <t>Secured DC bond</t>
+        </is>
+      </c>
+      <c r="G50" s="80" t="inlineStr">
+        <is>
+          <t>7.75%; YTW 7.3%; +307</t>
+        </is>
+      </c>
+      <c r="H50" s="80" t="inlineStr">
+        <is>
+          <t>May 2031</t>
+        </is>
+      </c>
+      <c r="I50" s="80" t="inlineStr">
+        <is>
+          <t>Tenant CoreWeave (HY), 12y lease; 6 facilities/5 sites; BB/BB-</t>
+        </is>
+      </c>
+      <c r="J50" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Core Scientific)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B51" s="81" t="inlineStr">
+        <is>
+          <t>HUT 8 DC (HUTRBA) — River Bend</t>
+        </is>
+      </c>
+      <c r="C51" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D51" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E51" s="83" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F51" s="80" t="inlineStr">
+        <is>
+          <t>Secured 1st-lien DC bond (IG)</t>
+        </is>
+      </c>
+      <c r="G51" s="80" t="inlineStr">
+        <is>
+          <t>6.192%; YTW 6.0%; +154</t>
+        </is>
+      </c>
+      <c r="H51" s="80" t="inlineStr">
+        <is>
+          <t>Nov 2042</t>
+        </is>
+      </c>
+      <c r="I51" s="80" t="inlineStr">
+        <is>
+          <t>Tenant Fluidstack (Google backstop), 15y lease; 245MW St. Francisville LA; (P)BBB-/BBB-</t>
+        </is>
+      </c>
+      <c r="J51" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Hut 8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B52" s="81" t="inlineStr">
+        <is>
+          <t>WULF Compute (WULF) — Terawulf</t>
+        </is>
+      </c>
+      <c r="C52" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D52" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E52" s="83" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F52" s="80" t="inlineStr">
+        <is>
+          <t>Secured DC bond</t>
+        </is>
+      </c>
+      <c r="G52" s="80" t="inlineStr">
+        <is>
+          <t>7.75%; YTW 6.0%; +189</t>
+        </is>
+      </c>
+      <c r="H52" s="80" t="inlineStr">
+        <is>
+          <t>Oct 2030</t>
+        </is>
+      </c>
+      <c r="I52" s="80" t="inlineStr">
+        <is>
+          <t>Tenant Fluidstack (Google backstop), 10y lease; 366MW Lake Mariner NY; Ba2/BB/BB</t>
+        </is>
+      </c>
+      <c r="J52" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Terawulf)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B53" s="81" t="inlineStr">
+        <is>
+          <t>APLD ComputeCo (APLD) — Ellendale ND</t>
+        </is>
+      </c>
+      <c r="C53" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D53" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E53" s="83" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="F53" s="80" t="inlineStr">
+        <is>
+          <t>Secured DC bond</t>
+        </is>
+      </c>
+      <c r="G53" s="80" t="inlineStr">
+        <is>
+          <t>9.25%; YTW 6.6%; +254</t>
+        </is>
+      </c>
+      <c r="H53" s="80" t="inlineStr">
+        <is>
+          <t>Dec 2030</t>
+        </is>
+      </c>
+      <c r="I53" s="80" t="inlineStr">
+        <is>
+          <t>Tenant CoreWeave (HY), 15y lease; 100/150MW Polaris Forge 1; BB-/BB-</t>
+        </is>
+      </c>
+      <c r="J53" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Applied Digital)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B54" s="81" t="inlineStr">
+        <is>
+          <t>APLD ComputeCo 2 (PFORGE) — Harwood ND</t>
+        </is>
+      </c>
+      <c r="C54" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D54" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E54" s="83" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="F54" s="80" t="inlineStr">
+        <is>
+          <t>Secured 1st-lien DC bond</t>
+        </is>
+      </c>
+      <c r="G54" s="80" t="inlineStr">
+        <is>
+          <t>6.75%; YTW 6.6%; +244</t>
+        </is>
+      </c>
+      <c r="H54" s="80" t="inlineStr">
+        <is>
+          <t>Mar 2031</t>
+        </is>
+      </c>
+      <c r="I54" s="80" t="inlineStr">
+        <is>
+          <t>Tenant Oracle (IG, guarantee), 15y lease; 150/50MW Polaris Forge 2; Ba3/BB-</t>
+        </is>
+      </c>
+      <c r="J54" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Applied Digital)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B55" s="81" t="inlineStr">
+        <is>
+          <t>Black Pearl Compute (BLKPRL) — Cipher Digital</t>
+        </is>
+      </c>
+      <c r="C55" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D55" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E55" s="83" t="n">
+        <v>2</v>
+      </c>
+      <c r="F55" s="80" t="inlineStr">
+        <is>
+          <t>Secured DC bond</t>
+        </is>
+      </c>
+      <c r="G55" s="80" t="inlineStr">
+        <is>
+          <t>6.125%; YTW 5.8%; +158</t>
+        </is>
+      </c>
+      <c r="H55" s="80" t="inlineStr">
+        <is>
+          <t>Feb 2031</t>
+        </is>
+      </c>
+      <c r="I55" s="80" t="inlineStr">
+        <is>
+          <t>Tenant AWS (IG, guarantee), 15y lease; 300MW TX; Ba2/BB-</t>
+        </is>
+      </c>
+      <c r="J55" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Cipher)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B56" s="81" t="inlineStr">
+        <is>
+          <t>Cipher Compute (CIFR) — Cipher Digital</t>
+        </is>
+      </c>
+      <c r="C56" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D56" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E56" s="83" t="n">
+        <v>1.733</v>
+      </c>
+      <c r="F56" s="80" t="inlineStr">
+        <is>
+          <t>Secured 1st-lien DC bond</t>
+        </is>
+      </c>
+      <c r="G56" s="80" t="inlineStr">
+        <is>
+          <t>7.125%; YTW 6.0%; +184</t>
+        </is>
+      </c>
+      <c r="H56" s="80" t="inlineStr">
+        <is>
+          <t>Nov 2030</t>
+        </is>
+      </c>
+      <c r="I56" s="80" t="inlineStr">
+        <is>
+          <t>Tenant Fluidstack (Google backstop), 10y lease; 300MW Barber Lake TX; Ba3/BB-</t>
+        </is>
+      </c>
+      <c r="J56" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Cipher)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B57" s="81" t="inlineStr">
+        <is>
+          <t>APLD ComputeCo 3 (ELNFOR) — Ellendale ND</t>
+        </is>
+      </c>
+      <c r="C57" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D57" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E57" s="83" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="F57" s="80" t="inlineStr">
+        <is>
+          <t>Secured 1st-lien DC bond</t>
+        </is>
+      </c>
+      <c r="G57" s="80" t="inlineStr">
+        <is>
+          <t>7.00%; YTW 7.0%; +282</t>
+        </is>
+      </c>
+      <c r="H57" s="80" t="inlineStr">
+        <is>
+          <t>Jun 2031</t>
+        </is>
+      </c>
+      <c r="I57" s="80" t="inlineStr">
+        <is>
+          <t>Tenant CoreWeave (HY), 15y lease; 150MW (ELN-4); BB-/BB-</t>
+        </is>
+      </c>
+      <c r="J57" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Applied Digital)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B58" s="81" t="inlineStr">
+        <is>
+          <t>Edged Compute (EDGCOM) — Edged US</t>
+        </is>
+      </c>
+      <c r="C58" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D58" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E58" s="83" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F58" s="80" t="inlineStr">
+        <is>
+          <t>Secured DC bond</t>
+        </is>
+      </c>
+      <c r="G58" s="80" t="inlineStr">
+        <is>
+          <t>7.50%; YTW 7.9%; +369</t>
+        </is>
+      </c>
+      <c r="H58" s="80" t="inlineStr">
+        <is>
+          <t>Apr 2031</t>
+        </is>
+      </c>
+      <c r="I58" s="80" t="inlineStr">
+        <is>
+          <t>Tenants CoreWeave (Chicago 72MW) &amp; Alibaba (Atlanta 42MW); BB+/BB-</t>
+        </is>
+      </c>
+      <c r="J58" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Edged US)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B59" s="81" t="inlineStr">
+        <is>
+          <t>Flash Compute (FLASHC) — Terawulf/Fluidstack JV</t>
+        </is>
+      </c>
+      <c r="C59" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D59" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E59" s="83" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F59" s="80" t="inlineStr">
+        <is>
+          <t>Secured DC bond</t>
+        </is>
+      </c>
+      <c r="G59" s="80" t="inlineStr">
+        <is>
+          <t>7.25%; YTW 6.3%; +213</t>
+        </is>
+      </c>
+      <c r="H59" s="80" t="inlineStr">
+        <is>
+          <t>Dec 2030</t>
+        </is>
+      </c>
+      <c r="I59" s="80" t="inlineStr">
+        <is>
+          <t>Tenant Fluidstack (Google backstop), 10y lease; 240MW Abernathy TX; Ba3</t>
+        </is>
+      </c>
+      <c r="J59" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Terawulf/Fluidstack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B60" s="81" t="inlineStr">
+        <is>
+          <t>SE Cosmos (SECMOS) — SB Energy/SoftBank</t>
+        </is>
+      </c>
+      <c r="C60" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D60" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E60" s="83" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="F60" s="80" t="inlineStr">
+        <is>
+          <t>Secured 1st-lien DC bond</t>
+        </is>
+      </c>
+      <c r="G60" s="80" t="inlineStr">
+        <is>
+          <t>8.875%; YTW 7.8%; +356</t>
+        </is>
+      </c>
+      <c r="H60" s="80" t="inlineStr">
+        <is>
+          <t>May 2031</t>
+        </is>
+      </c>
+      <c r="I60" s="80" t="inlineStr">
+        <is>
+          <t>Tenant SoftBank, 15y lease; 50MW Austin TX; (P)BB+/BB-</t>
+        </is>
+      </c>
+      <c r="J60" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (SB Energy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B61" s="81" t="inlineStr">
+        <is>
+          <t>Elk Grove Village (ELKGVP) — Prime Data Centers</t>
+        </is>
+      </c>
+      <c r="C61" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D61" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E61" s="83" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F61" s="80" t="inlineStr">
+        <is>
+          <t>Secured DC bond</t>
+        </is>
+      </c>
+      <c r="G61" s="80" t="inlineStr">
+        <is>
+          <t>7.50%; YTW 7.2%; +303</t>
+        </is>
+      </c>
+      <c r="H61" s="80" t="inlineStr">
+        <is>
+          <t>Jun 2031</t>
+        </is>
+      </c>
+      <c r="I61" s="80" t="inlineStr">
+        <is>
+          <t>Tenant CoreWeave (HY), 15y lease; 72MW ORD01-01 IL; Ba3/(P)BB-/BB-</t>
+        </is>
+      </c>
+      <c r="J61" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Prime Data Centers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="30" customHeight="1">
+      <c r="A62" s="80" t="inlineStr">
+        <is>
+          <t>o/s Jun'26</t>
+        </is>
+      </c>
+      <c r="B62" s="81" t="inlineStr">
+        <is>
+          <t>Stingray Compute (STNGRY) — Cipher Digital</t>
+        </is>
+      </c>
+      <c r="C62" s="82" t="inlineStr">
+        <is>
+          <t>Colocation / data-center REIT</t>
+        </is>
+      </c>
+      <c r="D62" s="80" t="inlineStr">
+        <is>
+          <t>144A bond investors</t>
+        </is>
+      </c>
+      <c r="E62" s="83" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="F62" s="80" t="inlineStr">
+        <is>
+          <t>Secured DC bond</t>
+        </is>
+      </c>
+      <c r="G62" s="80" t="inlineStr">
+        <is>
+          <t>6.00%; YTW 6.0%; +175</t>
+        </is>
+      </c>
+      <c r="H62" s="80" t="inlineStr">
+        <is>
+          <t>Jun 2031</t>
+        </is>
+      </c>
+      <c r="I62" s="80" t="inlineStr">
+        <is>
+          <t>Tenant AWS (IG), lease; 70MW Andrew TX; Ba2/BB-</t>
+        </is>
+      </c>
+      <c r="J62" s="84" t="inlineStr">
+        <is>
+          <t>Seaport (Cipher)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>6) CONVERTIBLES / EQUITY-LINKED</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="n"/>
+      <c r="C63" s="15" t="n"/>
+      <c r="D63" s="15" t="n"/>
+      <c r="E63" s="15" t="n"/>
+      <c r="F63" s="15" t="n"/>
+      <c r="G63" s="15" t="n"/>
+      <c r="H63" s="15" t="n"/>
+      <c r="I63" s="15" t="n"/>
+      <c r="J63" s="15" t="n"/>
+    </row>
+    <row r="64" ht="30" customHeight="1">
+      <c r="A64" s="75" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="B43" s="76" t="inlineStr">
+      <c r="B64" s="76" t="inlineStr">
         <is>
           <t>Nebius</t>
         </is>
       </c>
-      <c r="C43" s="77" t="inlineStr">
+      <c r="C64" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D43" s="75" t="inlineStr">
+      <c r="D64" s="75" t="inlineStr">
         <is>
           <t>Convertible market</t>
         </is>
       </c>
-      <c r="E43" s="78" t="n">
+      <c r="E64" s="78" t="n">
         <v>3</v>
       </c>
-      <c r="F43" s="75" t="inlineStr">
+      <c r="F64" s="75" t="inlineStr">
         <is>
           <t>Convertible notes</t>
         </is>
       </c>
-      <c r="G43" s="75" t="inlineStr">
+      <c r="G64" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H43" s="75" t="inlineStr">
+      <c r="H64" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I43" s="75" t="inlineStr">
+      <c r="I64" s="75" t="inlineStr">
         <is>
           <t>Lighter-balance-sheet strategy</t>
         </is>
       </c>
-      <c r="J43" s="79" t="inlineStr">
+      <c r="J64" s="79" t="inlineStr">
         <is>
           <t>frankk research</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="75" t="inlineStr">
+    <row r="65" ht="30" customHeight="1">
+      <c r="A65" s="75" t="inlineStr">
         <is>
           <t>Dec 2025</t>
         </is>
       </c>
-      <c r="B44" s="76" t="inlineStr">
+      <c r="B65" s="76" t="inlineStr">
         <is>
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="C44" s="77" t="inlineStr">
+      <c r="C65" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D44" s="75" t="inlineStr">
+      <c r="D65" s="75" t="inlineStr">
         <is>
           <t>Convertible market</t>
         </is>
       </c>
-      <c r="E44" s="78" t="n">
+      <c r="E65" s="78" t="n">
         <v>2.7</v>
       </c>
-      <c r="F44" s="75" t="inlineStr">
+      <c r="F65" s="75" t="inlineStr">
         <is>
           <t>Convertible notes</t>
         </is>
       </c>
-      <c r="G44" s="75" t="inlineStr">
+      <c r="G65" s="75" t="inlineStr">
         <is>
           <t>1.75%</t>
         </is>
       </c>
-      <c r="H44" s="75" t="inlineStr">
+      <c r="H65" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I44" s="75" t="inlineStr">
+      <c r="I65" s="75" t="inlineStr">
         <is>
           <t>Shift toward hybrid instruments</t>
         </is>
       </c>
-      <c r="J44" s="79" t="inlineStr">
+      <c r="J65" s="79" t="inlineStr">
         <is>
           <t>thedig; CoreWeave</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="92" t="n"/>
-      <c r="B45" s="93" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="92" t="n"/>
+      <c r="B66" s="93" t="inlineStr">
         <is>
           <t>TOTAL — itemized debt transactions (bonds + loans + private credit + ABS + converts)</t>
         </is>
       </c>
-      <c r="C45" s="92" t="n"/>
-      <c r="D45" s="92" t="n"/>
-      <c r="E45" s="94">
-        <f>SUM(E6,E7,E8,E9,E10,E11,E12,E14,E15,E16,E17,E18,E20,E21,E22,E23,E24,E25,E26,E27,E28,E29,E30,E31,E32,E39,E40,E41,E43,E44)</f>
-        <v/>
-      </c>
-      <c r="F45" s="92" t="n"/>
-      <c r="G45" s="92" t="n"/>
-      <c r="H45" s="92" t="n"/>
-      <c r="I45" s="92" t="n"/>
-      <c r="J45" s="92" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="14" t="inlineStr">
+      <c r="C66" s="92" t="n"/>
+      <c r="D66" s="92" t="n"/>
+      <c r="E66" s="94">
+        <f>SUM(E6,E7,E8,E9,E10,E11,E12,E13,E14,E15,E16,E18,E19,E20,E21,E22,E24,E25,E26,E27,E28,E29,E30,E31,E32,E33,E34,E35,E36,E43,E44,E45,E46,E47,E48,E49,E50,E51,E52,E53,E54,E55,E56,E57,E58,E59,E60,E61,E62,E64,E65)</f>
+        <v/>
+      </c>
+      <c r="F66" s="92" t="n"/>
+      <c r="G66" s="92" t="n"/>
+      <c r="H66" s="92" t="n"/>
+      <c r="I66" s="92" t="n"/>
+      <c r="J66" s="92" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
         <is>
           <t>7) VENDOR / EQUIPMENT-LEASE FINANCING &amp; BACKSTOPS (memo)</t>
         </is>
       </c>
-      <c r="B47" s="15" t="n"/>
-      <c r="C47" s="15" t="n"/>
-      <c r="D47" s="15" t="n"/>
-      <c r="E47" s="15" t="n"/>
-      <c r="F47" s="15" t="n"/>
-      <c r="G47" s="15" t="n"/>
-      <c r="H47" s="15" t="n"/>
-      <c r="I47" s="15" t="n"/>
-      <c r="J47" s="15" t="n"/>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="70" t="inlineStr">
+      <c r="B68" s="15" t="n"/>
+      <c r="C68" s="15" t="n"/>
+      <c r="D68" s="15" t="n"/>
+      <c r="E68" s="15" t="n"/>
+      <c r="F68" s="15" t="n"/>
+      <c r="G68" s="15" t="n"/>
+      <c r="H68" s="15" t="n"/>
+      <c r="I68" s="15" t="n"/>
+      <c r="J68" s="15" t="n"/>
+    </row>
+    <row r="69" ht="30" customHeight="1">
+      <c r="A69" s="70" t="inlineStr">
         <is>
           <t>2024-31</t>
         </is>
       </c>
-      <c r="B48" s="71" t="inlineStr">
+      <c r="B69" s="71" t="inlineStr">
         <is>
           <t>Microsoft — finance-lease commitments</t>
         </is>
       </c>
-      <c r="C48" s="72" t="inlineStr">
+      <c r="C69" s="72" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="D48" s="70" t="inlineStr">
+      <c r="D69" s="70" t="inlineStr">
         <is>
           <t>Lessors / developers</t>
         </is>
       </c>
-      <c r="E48" s="73" t="n">
+      <c r="E69" s="73" t="n">
         <v>196.6</v>
       </c>
-      <c r="F48" s="70" t="inlineStr">
+      <c r="F69" s="70" t="inlineStr">
         <is>
           <t>Finance leases not yet commenced (as of 31 Mar 2026)</t>
         </is>
       </c>
-      <c r="G48" s="70" t="inlineStr">
+      <c r="G69" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H48" s="70" t="inlineStr">
+      <c r="H69" s="70" t="inlineStr">
         <is>
           <t>to 21y</t>
         </is>
       </c>
-      <c r="I48" s="70" t="inlineStr">
+      <c r="I69" s="70" t="inlineStr">
         <is>
           <t>Off-B/S; commence FY26-FY31; Microsoft funds AI via leases not new bonds</t>
         </is>
       </c>
-      <c r="J48" s="74" t="inlineStr">
+      <c r="J69" s="74" t="inlineStr">
         <is>
           <t>MSFT 10-Q</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="75" t="inlineStr">
+    <row r="70" ht="30" customHeight="1">
+      <c r="A70" s="75" t="inlineStr">
         <is>
           <t>through 2032</t>
         </is>
       </c>
-      <c r="B49" s="76" t="inlineStr">
+      <c r="B70" s="76" t="inlineStr">
         <is>
           <t>CoreWeave — NVIDIA capacity backstop</t>
         </is>
       </c>
-      <c r="C49" s="77" t="inlineStr">
+      <c r="C70" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D49" s="75" t="inlineStr">
+      <c r="D70" s="75" t="inlineStr">
         <is>
           <t>NVIDIA</t>
         </is>
       </c>
-      <c r="E49" s="78" t="n">
+      <c r="E70" s="78" t="n">
         <v>6.3</v>
       </c>
-      <c r="F49" s="75" t="inlineStr">
+      <c r="F70" s="75" t="inlineStr">
         <is>
           <t>Vendor backstop of unsold capacity</t>
         </is>
       </c>
-      <c r="G49" s="75" t="inlineStr">
+      <c r="G70" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H49" s="75" t="inlineStr">
+      <c r="H70" s="75" t="inlineStr">
         <is>
           <t>to 2032</t>
         </is>
       </c>
-      <c r="I49" s="75" t="inlineStr">
+      <c r="I70" s="75" t="inlineStr">
         <is>
           <t>De-risks CoreWeave</t>
         </is>
       </c>
-      <c r="J49" s="79" t="inlineStr">
+      <c r="J70" s="79" t="inlineStr">
         <is>
           <t>theaiinsider</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="14" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr">
         <is>
           <t>8) EQUITY &amp; SOVEREIGN COMMITMENTS (memo — not debt)</t>
         </is>
       </c>
-      <c r="B50" s="15" t="n"/>
-      <c r="C50" s="15" t="n"/>
-      <c r="D50" s="15" t="n"/>
-      <c r="E50" s="15" t="n"/>
-      <c r="F50" s="15" t="n"/>
-      <c r="G50" s="15" t="n"/>
-      <c r="H50" s="15" t="n"/>
-      <c r="I50" s="15" t="n"/>
-      <c r="J50" s="15" t="n"/>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="70" t="inlineStr">
+      <c r="B71" s="15" t="n"/>
+      <c r="C71" s="15" t="n"/>
+      <c r="D71" s="15" t="n"/>
+      <c r="E71" s="15" t="n"/>
+      <c r="F71" s="15" t="n"/>
+      <c r="G71" s="15" t="n"/>
+      <c r="H71" s="15" t="n"/>
+      <c r="I71" s="15" t="n"/>
+      <c r="J71" s="15" t="n"/>
+    </row>
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="70" t="inlineStr">
         <is>
           <t>2024-25</t>
         </is>
       </c>
-      <c r="B51" s="71" t="inlineStr">
+      <c r="B72" s="71" t="inlineStr">
         <is>
           <t>Microsoft — AI Infrastructure Partnership (AIP)</t>
         </is>
       </c>
-      <c r="C51" s="72" t="inlineStr">
+      <c r="C72" s="72" t="inlineStr">
         <is>
           <t>Hyperscaler</t>
         </is>
       </c>
-      <c r="D51" s="70" t="inlineStr">
+      <c r="D72" s="70" t="inlineStr">
         <is>
           <t>Microsoft, BlackRock/GIP, MGX (+ NVIDIA)</t>
         </is>
       </c>
-      <c r="E51" s="73" t="n">
+      <c r="E72" s="73" t="n">
         <v>100</v>
       </c>
-      <c r="F51" s="70" t="inlineStr">
+      <c r="F72" s="70" t="inlineStr">
         <is>
           <t>Co-investment fund (equity sponsor)</t>
         </is>
       </c>
-      <c r="G51" s="70" t="inlineStr">
+      <c r="G72" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H51" s="70" t="inlineStr">
+      <c r="H72" s="70" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I51" s="70" t="inlineStr">
+      <c r="I72" s="70" t="inlineStr">
         <is>
           <t>Up to $100bn incl. debt; first deployment $40bn Aligned (Oct 2025); Microsoft offtake underwrites it</t>
         </is>
       </c>
-      <c r="J51" s="74" t="inlineStr">
+      <c r="J72" s="74" t="inlineStr">
         <is>
           <t>FT; chiragvadhia</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="95" t="inlineStr">
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="95" t="inlineStr">
         <is>
           <t>2025-30</t>
         </is>
       </c>
-      <c r="B52" s="96" t="inlineStr">
+      <c r="B73" s="96" t="inlineStr">
         <is>
           <t>HUMAIN (Saudi PIF)</t>
         </is>
       </c>
-      <c r="C52" s="97" t="inlineStr">
+      <c r="C73" s="97" t="inlineStr">
         <is>
           <t>Sovereign cloud</t>
         </is>
       </c>
-      <c r="D52" s="95" t="inlineStr">
+      <c r="D73" s="95" t="inlineStr">
         <is>
           <t>Public Investment Fund</t>
         </is>
       </c>
-      <c r="E52" s="98" t="n">
+      <c r="E73" s="98" t="n">
         <v>100</v>
       </c>
-      <c r="F52" s="95" t="inlineStr">
+      <c r="F73" s="95" t="inlineStr">
         <is>
           <t>Sovereign equity</t>
         </is>
       </c>
-      <c r="G52" s="95" t="inlineStr">
+      <c r="G73" s="95" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H52" s="95" t="inlineStr">
+      <c r="H73" s="95" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I52" s="95" t="inlineStr">
+      <c r="I73" s="95" t="inlineStr">
         <is>
           <t>11 DCs / 2.2GW; ~600k GPUs</t>
         </is>
       </c>
-      <c r="J52" s="99" t="inlineStr">
+      <c r="J73" s="99" t="inlineStr">
         <is>
           <t>Presenc AI; NYU DRI</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="95" t="inlineStr">
+    <row r="74" ht="30" customHeight="1">
+      <c r="A74" s="95" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="B53" s="96" t="inlineStr">
+      <c r="B74" s="96" t="inlineStr">
         <is>
           <t>MGX / Mubadala (UAE)</t>
         </is>
       </c>
-      <c r="C53" s="97" t="inlineStr">
+      <c r="C74" s="97" t="inlineStr">
         <is>
           <t>Sovereign cloud</t>
         </is>
       </c>
-      <c r="D53" s="95" t="inlineStr">
+      <c r="D74" s="95" t="inlineStr">
         <is>
           <t>Mubadala / MGX</t>
         </is>
       </c>
-      <c r="E53" s="98" t="n">
+      <c r="E74" s="98" t="n">
         <v>40</v>
       </c>
-      <c r="F53" s="95" t="inlineStr">
+      <c r="F74" s="95" t="inlineStr">
         <is>
           <t>Sovereign equity / infra</t>
         </is>
       </c>
-      <c r="G53" s="95" t="inlineStr">
+      <c r="G74" s="95" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H53" s="95" t="inlineStr">
+      <c r="H74" s="95" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I53" s="95" t="inlineStr">
+      <c r="I74" s="95" t="inlineStr">
         <is>
           <t>Anchored Stargate; co-bought Aligned</t>
         </is>
       </c>
-      <c r="J53" s="99" t="inlineStr">
+      <c r="J74" s="99" t="inlineStr">
         <is>
           <t>NYU DRI</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="95" t="inlineStr">
+    <row r="75" ht="30" customHeight="1">
+      <c r="A75" s="95" t="inlineStr">
         <is>
           <t>2025-30</t>
         </is>
       </c>
-      <c r="B54" s="96" t="inlineStr">
+      <c r="B75" s="96" t="inlineStr">
         <is>
           <t>Stargate UAE / G42 / Khazna</t>
         </is>
       </c>
-      <c r="C54" s="97" t="inlineStr">
+      <c r="C75" s="97" t="inlineStr">
         <is>
           <t>Sovereign cloud</t>
         </is>
       </c>
-      <c r="D54" s="95" t="inlineStr">
+      <c r="D75" s="95" t="inlineStr">
         <is>
           <t>Mubadala, MGX, Microsoft, G42</t>
         </is>
       </c>
-      <c r="E54" s="98" t="n">
+      <c r="E75" s="98" t="n">
         <v>30</v>
       </c>
-      <c r="F54" s="95" t="inlineStr">
+      <c r="F75" s="95" t="inlineStr">
         <is>
           <t>Sovereign equity + JV</t>
         </is>
       </c>
-      <c r="G54" s="95" t="inlineStr">
+      <c r="G75" s="95" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H54" s="95" t="inlineStr">
+      <c r="H75" s="95" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I54" s="95" t="inlineStr">
+      <c r="I75" s="95" t="inlineStr">
         <is>
           <t>5GW Abu Dhabi campus</t>
         </is>
       </c>
-      <c r="J54" s="99" t="inlineStr">
+      <c r="J75" s="99" t="inlineStr">
         <is>
           <t>Khaleej Times; dcpulse</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="95" t="inlineStr">
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="95" t="inlineStr">
         <is>
           <t>Late 2025</t>
         </is>
       </c>
-      <c r="B55" s="96" t="inlineStr">
+      <c r="B76" s="96" t="inlineStr">
         <is>
           <t>Qatar (QIA / Qai) + Brookfield</t>
         </is>
       </c>
-      <c r="C55" s="97" t="inlineStr">
+      <c r="C76" s="97" t="inlineStr">
         <is>
           <t>Sovereign cloud</t>
         </is>
       </c>
-      <c r="D55" s="95" t="inlineStr">
+      <c r="D76" s="95" t="inlineStr">
         <is>
           <t>QIA / Qai, Brookfield</t>
         </is>
       </c>
-      <c r="E55" s="98" t="n">
+      <c r="E76" s="98" t="n">
         <v>20</v>
       </c>
-      <c r="F55" s="95" t="inlineStr">
+      <c r="F76" s="95" t="inlineStr">
         <is>
           <t>JV / infra</t>
         </is>
       </c>
-      <c r="G55" s="95" t="inlineStr">
+      <c r="G76" s="95" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H55" s="95" t="inlineStr">
+      <c r="H76" s="95" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I55" s="95" t="inlineStr">
+      <c r="I76" s="95" t="inlineStr">
         <is>
           <t>AI-infrastructure JV</t>
         </is>
       </c>
-      <c r="J55" s="99" t="inlineStr">
+      <c r="J76" s="99" t="inlineStr">
         <is>
           <t>NYU DRI</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="75" t="inlineStr">
+    <row r="77" ht="30" customHeight="1">
+      <c r="A77" s="75" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B56" s="76" t="inlineStr">
+      <c r="B77" s="76" t="inlineStr">
         <is>
           <t>SpaceX / xAI — $10bn raise</t>
         </is>
       </c>
-      <c r="C56" s="77" t="inlineStr">
+      <c r="C77" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D56" s="75" t="inlineStr">
+      <c r="D77" s="75" t="inlineStr">
         <is>
           <t>Morgan Stanley</t>
         </is>
       </c>
-      <c r="E56" s="78" t="n">
+      <c r="E77" s="78" t="n">
         <v>10</v>
       </c>
-      <c r="F56" s="75" t="inlineStr">
+      <c r="F77" s="75" t="inlineStr">
         <is>
           <t>$5bn debt + $5bn equity</t>
         </is>
       </c>
-      <c r="G56" s="75" t="inlineStr">
+      <c r="G77" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H56" s="75" t="inlineStr">
+      <c r="H77" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I56" s="75" t="inlineStr">
+      <c r="I77" s="75" t="inlineStr">
         <is>
           <t>Debt portion also in group 3</t>
         </is>
       </c>
-      <c r="J56" s="79" t="inlineStr">
+      <c r="J77" s="79" t="inlineStr">
         <is>
           <t>CNBC</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="75" t="inlineStr">
+    <row r="78" ht="30" customHeight="1">
+      <c r="A78" s="75" t="inlineStr">
         <is>
           <t>2025-26</t>
         </is>
       </c>
-      <c r="B57" s="76" t="inlineStr">
+      <c r="B78" s="76" t="inlineStr">
         <is>
           <t>CoreWeave — equity</t>
         </is>
       </c>
-      <c r="C57" s="77" t="inlineStr">
+      <c r="C78" s="77" t="inlineStr">
         <is>
           <t>Neocloud / AI-native</t>
         </is>
       </c>
-      <c r="D57" s="75" t="inlineStr">
+      <c r="D78" s="75" t="inlineStr">
         <is>
           <t>NVIDIA; IPO</t>
         </is>
       </c>
-      <c r="E57" s="78" t="n">
+      <c r="E78" s="78" t="n">
         <v>3.5</v>
       </c>
-      <c r="F57" s="75" t="inlineStr">
+      <c r="F78" s="75" t="inlineStr">
         <is>
           <t>IPO ($1.5bn) + NVIDIA strategic ($2bn)</t>
         </is>
       </c>
-      <c r="G57" s="75" t="inlineStr">
+      <c r="G78" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H57" s="75" t="inlineStr">
+      <c r="H78" s="75" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I57" s="75" t="inlineStr">
+      <c r="I78" s="75" t="inlineStr">
         <is>
           <t>Equity (not debt)</t>
         </is>
       </c>
-      <c r="J57" s="79" t="inlineStr">
+      <c r="J78" s="79" t="inlineStr">
         <is>
           <t>CNBC; CoreWeave</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="14" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="14" t="inlineStr">
         <is>
           <t>9) CONTEXT / FRAMEWORKS / PROJECTIONS (memo)</t>
         </is>
       </c>
-      <c r="B58" s="15" t="n"/>
-      <c r="C58" s="15" t="n"/>
-      <c r="D58" s="15" t="n"/>
-      <c r="E58" s="15" t="n"/>
-      <c r="F58" s="15" t="n"/>
-      <c r="G58" s="15" t="n"/>
-      <c r="H58" s="15" t="n"/>
-      <c r="I58" s="15" t="n"/>
-      <c r="J58" s="15" t="n"/>
-    </row>
-    <row r="59" ht="30" customHeight="1">
-      <c r="A59" s="85" t="inlineStr">
+      <c r="B79" s="15" t="n"/>
+      <c r="C79" s="15" t="n"/>
+      <c r="D79" s="15" t="n"/>
+      <c r="E79" s="15" t="n"/>
+      <c r="F79" s="15" t="n"/>
+      <c r="G79" s="15" t="n"/>
+      <c r="H79" s="15" t="n"/>
+      <c r="I79" s="15" t="n"/>
+      <c r="J79" s="15" t="n"/>
+    </row>
+    <row r="80" ht="30" customHeight="1">
+      <c r="A80" s="85" t="inlineStr">
         <is>
           <t>2025-28</t>
         </is>
       </c>
-      <c r="B59" s="86" t="inlineStr">
+      <c r="B80" s="86" t="inlineStr">
         <is>
           <t>Market — private credit for AI data centers</t>
         </is>
       </c>
-      <c r="C59" s="87" t="inlineStr">
+      <c r="C80" s="87" t="inlineStr">
         <is>
           <t>Context / market</t>
         </is>
       </c>
-      <c r="D59" s="85" t="inlineStr">
+      <c r="D80" s="85" t="inlineStr">
         <is>
           <t>Industry-wide</t>
         </is>
       </c>
-      <c r="E59" s="88" t="n">
+      <c r="E80" s="88" t="n">
         <v>800</v>
       </c>
-      <c r="F59" s="85" t="inlineStr">
+      <c r="F80" s="85" t="inlineStr">
         <is>
           <t>Projection</t>
         </is>
       </c>
-      <c r="G59" s="85" t="inlineStr">
+      <c r="G80" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H59" s="85" t="inlineStr">
+      <c r="H80" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I59" s="85" t="inlineStr">
+      <c r="I80" s="85" t="inlineStr">
         <is>
           <t>&gt;$200bn already outstanding</t>
         </is>
       </c>
-      <c r="J59" s="89" t="inlineStr">
+      <c r="J80" s="89" t="inlineStr">
         <is>
           <t>Morgan Stanley; Quinn Emanuel</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="30" customHeight="1">
-      <c r="A60" s="85" t="inlineStr">
+    <row r="81" ht="30" customHeight="1">
+      <c r="A81" s="85" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B60" s="86" t="inlineStr">
+      <c r="B81" s="86" t="inlineStr">
         <is>
           <t>Insurance-linked platforms — private credit</t>
         </is>
       </c>
-      <c r="C60" s="87" t="inlineStr">
+      <c r="C81" s="87" t="inlineStr">
         <is>
           <t>Context / market</t>
         </is>
       </c>
-      <c r="D60" s="85" t="inlineStr">
+      <c r="D81" s="85" t="inlineStr">
         <is>
           <t>Athene, Global Atlantic, etc.</t>
         </is>
       </c>
-      <c r="E60" s="88" t="n">
+      <c r="E81" s="88" t="n">
         <v>180</v>
       </c>
-      <c r="F60" s="85" t="inlineStr">
+      <c r="F81" s="85" t="inlineStr">
         <is>
           <t>Insurance capital into private credit</t>
         </is>
       </c>
-      <c r="G60" s="85" t="inlineStr">
+      <c r="G81" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H60" s="85" t="inlineStr">
+      <c r="H81" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I60" s="85" t="inlineStr">
+      <c r="I81" s="85" t="inlineStr">
         <is>
           <t>~25% of global private credit AUM</t>
         </is>
       </c>
-      <c r="J60" s="89" t="inlineStr">
+      <c r="J81" s="89" t="inlineStr">
         <is>
           <t>McKinsey; ABF Journal</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="30" customHeight="1">
-      <c r="A61" s="85" t="inlineStr">
+    <row r="82" ht="30" customHeight="1">
+      <c r="A82" s="85" t="inlineStr">
         <is>
           <t>2026-28</t>
         </is>
       </c>
-      <c r="B61" s="86" t="inlineStr">
+      <c r="B82" s="86" t="inlineStr">
         <is>
           <t>Colocation — DC securitization supply</t>
         </is>
       </c>
-      <c r="C61" s="87" t="inlineStr">
+      <c r="C82" s="87" t="inlineStr">
         <is>
           <t>Context / market</t>
         </is>
       </c>
-      <c r="D61" s="85" t="inlineStr">
+      <c r="D82" s="85" t="inlineStr">
         <is>
           <t>Industry-wide</t>
         </is>
       </c>
-      <c r="E61" s="88" t="n">
+      <c r="E82" s="88" t="n">
         <v>130</v>
       </c>
-      <c r="F61" s="85" t="inlineStr">
+      <c r="F82" s="85" t="inlineStr">
         <is>
           <t>ABS + CMBS net issuance</t>
         </is>
       </c>
-      <c r="G61" s="85" t="inlineStr">
+      <c r="G82" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H61" s="85" t="inlineStr">
+      <c r="H82" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I61" s="85" t="inlineStr">
+      <c r="I82" s="85" t="inlineStr">
         <is>
           <t>Morgan Stanley estimate</t>
         </is>
       </c>
-      <c r="J61" s="89" t="inlineStr">
+      <c r="J82" s="89" t="inlineStr">
         <is>
           <t>CREFC; Impax</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="30" customHeight="1">
-      <c r="A62" s="85" t="inlineStr">
+    <row r="83" ht="30" customHeight="1">
+      <c r="A83" s="85" t="inlineStr">
         <is>
           <t>to 2026</t>
         </is>
       </c>
-      <c r="B62" s="86" t="inlineStr">
+      <c r="B83" s="86" t="inlineStr">
         <is>
           <t>Sector — HY/unrated AI-infra debt</t>
         </is>
       </c>
-      <c r="C62" s="87" t="inlineStr">
+      <c r="C83" s="87" t="inlineStr">
         <is>
           <t>Context / market</t>
         </is>
       </c>
-      <c r="D62" s="85" t="inlineStr">
+      <c r="D83" s="85" t="inlineStr">
         <is>
           <t>Multiple</t>
         </is>
       </c>
-      <c r="E62" s="88" t="n">
+      <c r="E83" s="88" t="n">
         <v>107</v>
       </c>
-      <c r="F62" s="85" t="inlineStr">
+      <c r="F83" s="85" t="inlineStr">
         <is>
           <t>Funded + committed debt</t>
         </is>
       </c>
-      <c r="G62" s="85" t="inlineStr">
+      <c r="G83" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H62" s="85" t="inlineStr">
+      <c r="H83" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I62" s="85" t="inlineStr">
+      <c r="I83" s="85" t="inlineStr">
         <is>
           <t>$68.7bn neoclouds / $38.7bn AI-native DCs</t>
         </is>
       </c>
-      <c r="J62" s="89" t="inlineStr">
+      <c r="J83" s="89" t="inlineStr">
         <is>
           <t>Octus</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="30" customHeight="1">
-      <c r="A63" s="85" t="inlineStr">
+    <row r="84" ht="30" customHeight="1">
+      <c r="A84" s="85" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="B63" s="86" t="inlineStr">
+      <c r="B84" s="86" t="inlineStr">
         <is>
           <t>KKR + Energy Capital Partners — partnership</t>
         </is>
       </c>
-      <c r="C63" s="87" t="inlineStr">
+      <c r="C84" s="87" t="inlineStr">
         <is>
           <t>Context / market</t>
         </is>
       </c>
-      <c r="D63" s="85" t="inlineStr">
+      <c r="D84" s="85" t="inlineStr">
         <is>
           <t>KKR, ECP</t>
         </is>
       </c>
-      <c r="E63" s="88" t="n">
+      <c r="E84" s="88" t="n">
         <v>50</v>
       </c>
-      <c r="F63" s="85" t="inlineStr">
+      <c r="F84" s="85" t="inlineStr">
         <is>
           <t>Strategic partnership</t>
         </is>
       </c>
-      <c r="G63" s="85" t="inlineStr">
+      <c r="G84" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="H63" s="85" t="inlineStr">
+      <c r="H84" s="85" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="I63" s="85" t="inlineStr">
+      <c r="I84" s="85" t="inlineStr">
         <is>
           <t>Accelerate AI infrastructure</t>
         </is>
       </c>
-      <c r="J63" s="89" t="inlineStr">
+      <c r="J84" s="89" t="inlineStr">
         <is>
           <t>Business Times</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="30" customHeight="1">
-      <c r="A64" s="85" t="inlineStr">
+    <row r="85" ht="30" customHeight="1">
+      <c r="A85" s="85" t="inlineStr">
         <is>
           <t>2025-28</t>
         </is>
       </c>
-      <c r="B64" s="86" t="inlineStr">
+      <c r="B85" s="86" t="inlineStr">
         <is>
           <t>Broadcom + Apollo + Blackstone — platform</t>
         </is>
       </c>
-      <c r="C64" s="87" t="inlineStr">
+      <c r="C85" s="87" t="inlineStr">
         <is>
           <t>Context / market</t>
         </is>
       </c>
-      <c r="D64" s="85" t="inlineStr">
+      <c r="D85" s="85" t="inlineStr">
         <is>
           <t>Apollo, Blackstone, Broadcom</t>
         </is>
       </c>
-      <c r="E64" s="100" t="n"/>
-      <c r="F64" s="85" t="inlineStr">
+      <c r="E85" s="100" t="n"/>
+      <c r="F85" s="85" t="inlineStr">
         <is>
           <t>Platform framework</t>
         </is>
       </c>
-      <c r="G64" s="85" t="inlineStr">
+      <c r="G85" s="85" t="inlineStr">
         <is>
           <t>&gt;20 GW</t>
         </is>
       </c>
-      <c r="H64" s="85" t="inlineStr">
+      <c r="H85" s="85" t="inlineStr">
         <is>
           <t>to 2028</t>
         </is>
       </c>
-      <c r="I64" s="85" t="inlineStr">
+      <c r="I85" s="85" t="inlineStr">
         <is>
           <t>Deploy &gt;20GW compute</t>
         </is>
       </c>
-      <c r="J64" s="89" t="inlineStr">
+      <c r="J85" s="89" t="inlineStr">
         <is>
           <t>privatedebtnews</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="101" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="101" t="inlineStr">
         <is>
           <t>Selected sources:</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="102" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="102" t="inlineStr">
         <is>
           <t>Goldman Sachs Research — ~$5.3tn AI + data-center capex 2025-2030; private markets in DC financing.</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="102" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="102" t="inlineStr">
         <is>
           <t>Morgan Stanley — ~$2tn capex 2025-28 with &gt;$1tn debt; ~$800bn private credit for AI DCs.</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="102" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="102" t="inlineStr">
         <is>
           <t>Bank of America / BofA Securities — hyperscaler bond issuance ($121bn 2025; ~$175bn 2026E).</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="102" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="102" t="inlineStr">
         <is>
           <t>Moody's Ratings — hyperscaler capex (~$785bn 2026, ~$1tn 2027); $662bn off-B/S DC leases.</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="102" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="102" t="inlineStr">
         <is>
           <t>McKinsey — ~$2.7tn US (5.2tn global) data-center capex by 2030; insurance-linked private credit.</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="102" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="102" t="inlineStr">
         <is>
           <t>Octus — HY/unrated AI-infra debt (~$107bn to ~May 2026); ~14GW unfunded ≈ $344bn need.</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="102" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="102" t="inlineStr">
+        <is>
+          <t>Seaport Global (Andrew Cueter) — 'AI Data Centers (HY &amp; IG)' desk note, 12-13 Jun 2026: secured</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  data-center bonds by tenant-credit tier (price/YTW/spread); Bloomberg, rating agencies, filings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="102" t="inlineStr">
         <is>
           <t>Company / press: Meta IR, FT, S&amp;P, IFR (Hyperion); Oracle IR, IFR, Reuters; CoreWeave IR; Blackstone;</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="102" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="102" t="inlineStr">
         <is>
           <t xml:space="preserve">  Apollo Academy; privatedebtnews; Bisnow; Quinn Emanuel; Build.inc; CNBC / WSJ / The Information (xAI).</t>
         </is>

</xml_diff>